<commit_message>
compiled report 2026-06-06: 549 election events, 273 audit entries
</commit_message>
<xml_diff>
--- a/punmonitor-compiled-report.xlsx
+++ b/punmonitor-compiled-report.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2241" uniqueCount="2241">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2324" uniqueCount="2324">
   <si>
     <t>Source Date</t>
   </si>
@@ -6691,22 +6691,58 @@
     <t>2026-06-06</t>
   </si>
   <si>
-    <t>0h 17m 11s</t>
-  </si>
-  <si>
-    <t>1h 14m 49s</t>
-  </si>
-  <si>
-    <t>00:05:00</t>
-  </si>
-  <si>
-    <t>232.0</t>
-  </si>
-  <si>
-    <t>239231.5</t>
-  </si>
-  <si>
-    <t>6873</t>
+    <t>10.0.59</t>
+  </si>
+  <si>
+    <t>2026-06-06 02:12:42</t>
+  </si>
+  <si>
+    <t>2h 50m 9s</t>
+  </si>
+  <si>
+    <t>02:14:57</t>
+  </si>
+  <si>
+    <t>122.0</t>
+  </si>
+  <si>
+    <t>113683.3</t>
+  </si>
+  <si>
+    <t>954</t>
+  </si>
+  <si>
+    <t>2h 49m 44s</t>
+  </si>
+  <si>
+    <t>2026-06-06T02:12:57.4419603+05:30</t>
+  </si>
+  <si>
+    <t>02:12:57.441</t>
+  </si>
+  <si>
+    <t>2026-06-06T02:12:57+05:30 (2m0s ago)</t>
+  </si>
+  <si>
+    <t>520</t>
+  </si>
+  <si>
+    <t>2026-06-05T23:53:04.3464959+05:30</t>
+  </si>
+  <si>
+    <t>23:53:04.346</t>
+  </si>
+  <si>
+    <t>521</t>
+  </si>
+  <si>
+    <t>2026-06-05T23:58:04.4885433+05:30</t>
+  </si>
+  <si>
+    <t>23:58:04.488</t>
+  </si>
+  <si>
+    <t>522</t>
   </si>
   <si>
     <t>2026-06-06T00:03:04.5336367+05:30</t>
@@ -6715,31 +6751,244 @@
     <t>00:03:04.533</t>
   </si>
   <si>
-    <t>2026-06-06T00:03:04+05:30 (1m55s ago)</t>
-  </si>
-  <si>
-    <t>520</t>
-  </si>
-  <si>
-    <t>2026-06-05T23:53:04.3464959+05:30</t>
-  </si>
-  <si>
-    <t>23:53:04.346</t>
-  </si>
-  <si>
-    <t>521</t>
-  </si>
-  <si>
-    <t>2026-06-05T23:58:04.4885433+05:30</t>
-  </si>
-  <si>
-    <t>23:58:04.488</t>
-  </si>
-  <si>
-    <t>522</t>
-  </si>
-  <si>
-    <t>2026-06-06T00:05:00+05:30</t>
+    <t>523</t>
+  </si>
+  <si>
+    <t>2026-06-06T00:08:04.3890711+05:30</t>
+  </si>
+  <si>
+    <t>00:08:04.389</t>
+  </si>
+  <si>
+    <t>524</t>
+  </si>
+  <si>
+    <t>2026-06-06T00:13:04.2945198+05:30</t>
+  </si>
+  <si>
+    <t>00:13:04.294</t>
+  </si>
+  <si>
+    <t>525</t>
+  </si>
+  <si>
+    <t>2026-06-06T00:18:04.349719+05:30</t>
+  </si>
+  <si>
+    <t>00:18:04.349</t>
+  </si>
+  <si>
+    <t>526</t>
+  </si>
+  <si>
+    <t>2026-06-06T00:23:03.2036477+05:30</t>
+  </si>
+  <si>
+    <t>00:23:03.203</t>
+  </si>
+  <si>
+    <t>527</t>
+  </si>
+  <si>
+    <t>2026-06-06T00:23:03.20476+05:30</t>
+  </si>
+  <si>
+    <t>00:23:03.204</t>
+  </si>
+  <si>
+    <t>528</t>
+  </si>
+  <si>
+    <t>2026-06-06T00:28:04.4524866+05:30</t>
+  </si>
+  <si>
+    <t>00:28:04.452</t>
+  </si>
+  <si>
+    <t>529</t>
+  </si>
+  <si>
+    <t>2026-06-06T00:33:04.9882474+05:30</t>
+  </si>
+  <si>
+    <t>00:33:04.988</t>
+  </si>
+  <si>
+    <t>530</t>
+  </si>
+  <si>
+    <t>2026-06-06T00:38:04.4578185+05:30</t>
+  </si>
+  <si>
+    <t>00:38:04.457</t>
+  </si>
+  <si>
+    <t>531</t>
+  </si>
+  <si>
+    <t>2026-06-06T00:43:04.4165849+05:30</t>
+  </si>
+  <si>
+    <t>00:43:04.416</t>
+  </si>
+  <si>
+    <t>532</t>
+  </si>
+  <si>
+    <t>2026-06-06T00:48:04.4972065+05:30</t>
+  </si>
+  <si>
+    <t>00:48:04.497</t>
+  </si>
+  <si>
+    <t>533</t>
+  </si>
+  <si>
+    <t>2026-06-06T00:53:04.4158628+05:30</t>
+  </si>
+  <si>
+    <t>00:53:04.415</t>
+  </si>
+  <si>
+    <t>534</t>
+  </si>
+  <si>
+    <t>2026-06-06T00:58:04.746462+05:30</t>
+  </si>
+  <si>
+    <t>00:58:04.746</t>
+  </si>
+  <si>
+    <t>535</t>
+  </si>
+  <si>
+    <t>2026-06-06T01:03:04.2965606+05:30</t>
+  </si>
+  <si>
+    <t>01:03:04.296</t>
+  </si>
+  <si>
+    <t>536</t>
+  </si>
+  <si>
+    <t>2026-06-06T01:08:04.4870498+05:30</t>
+  </si>
+  <si>
+    <t>01:08:04.487</t>
+  </si>
+  <si>
+    <t>537</t>
+  </si>
+  <si>
+    <t>2026-06-06T01:13:04.3971229+05:30</t>
+  </si>
+  <si>
+    <t>01:13:04.397</t>
+  </si>
+  <si>
+    <t>538</t>
+  </si>
+  <si>
+    <t>2026-06-06T01:18:04.3982097+05:30</t>
+  </si>
+  <si>
+    <t>01:18:04.398</t>
+  </si>
+  <si>
+    <t>539</t>
+  </si>
+  <si>
+    <t>2026-06-06T01:23:04.338193+05:30</t>
+  </si>
+  <si>
+    <t>01:23:04.338</t>
+  </si>
+  <si>
+    <t>540</t>
+  </si>
+  <si>
+    <t>2026-06-06T01:28:04.3749159+05:30</t>
+  </si>
+  <si>
+    <t>01:28:04.374</t>
+  </si>
+  <si>
+    <t>541</t>
+  </si>
+  <si>
+    <t>2026-06-06T01:33:04.3612467+05:30</t>
+  </si>
+  <si>
+    <t>01:33:04.361</t>
+  </si>
+  <si>
+    <t>542</t>
+  </si>
+  <si>
+    <t>2026-06-06T01:38:04.5068535+05:30</t>
+  </si>
+  <si>
+    <t>01:38:04.506</t>
+  </si>
+  <si>
+    <t>543</t>
+  </si>
+  <si>
+    <t>2026-06-06T01:43:04.4507225+05:30</t>
+  </si>
+  <si>
+    <t>01:43:04.450</t>
+  </si>
+  <si>
+    <t>544</t>
+  </si>
+  <si>
+    <t>2026-06-06T01:48:04.4562151+05:30</t>
+  </si>
+  <si>
+    <t>01:48:04.456</t>
+  </si>
+  <si>
+    <t>545</t>
+  </si>
+  <si>
+    <t>2026-06-06T01:53:04.4814572+05:30</t>
+  </si>
+  <si>
+    <t>01:53:04.481</t>
+  </si>
+  <si>
+    <t>546</t>
+  </si>
+  <si>
+    <t>2026-06-06T01:58:04.3490827+05:30</t>
+  </si>
+  <si>
+    <t>01:58:04.349</t>
+  </si>
+  <si>
+    <t>547</t>
+  </si>
+  <si>
+    <t>2026-06-06T02:03:04.395145+05:30</t>
+  </si>
+  <si>
+    <t>02:03:04.395</t>
+  </si>
+  <si>
+    <t>548</t>
+  </si>
+  <si>
+    <t>2026-06-06T02:08:04.4247916+05:30</t>
+  </si>
+  <si>
+    <t>02:08:04.424</t>
+  </si>
+  <si>
+    <t>549</t>
+  </si>
+  <si>
+    <t>2026-06-06T02:14:57+05:30</t>
   </si>
 </sst>
 </file>
@@ -8089,7 +8338,7 @@
         <v>34</v>
       </c>
       <c r="H18" t="s">
-        <v>1183</v>
+        <v>2224</v>
       </c>
       <c r="I18" t="s">
         <v>36</v>
@@ -8113,25 +8362,25 @@
         <v>39</v>
       </c>
       <c r="P18" t="s">
-        <v>2224</v>
+        <v>739</v>
       </c>
       <c r="Q18" t="s">
-        <v>1185</v>
+        <v>2225</v>
       </c>
       <c r="R18" t="s">
         <v>1186</v>
       </c>
       <c r="S18" t="s">
-        <v>1185</v>
+        <v>2225</v>
       </c>
       <c r="T18" t="s">
-        <v>2225</v>
+        <v>2226</v>
       </c>
       <c r="U18" t="s">
         <v>2223</v>
       </c>
       <c r="V18" t="s">
-        <v>2226</v>
+        <v>2227</v>
       </c>
     </row>
     <row r="19">
@@ -8157,7 +8406,7 @@
         <v>34</v>
       </c>
       <c r="H19" t="s">
-        <v>1183</v>
+        <v>2224</v>
       </c>
       <c r="I19" t="s">
         <v>45</v>
@@ -8169,13 +8418,13 @@
         <v>241</v>
       </c>
       <c r="L19" t="s">
-        <v>2227</v>
+        <v>2228</v>
       </c>
       <c r="M19" t="s">
-        <v>2228</v>
+        <v>2229</v>
       </c>
       <c r="N19" t="s">
-        <v>2229</v>
+        <v>2230</v>
       </c>
       <c r="O19" t="s">
         <v>245</v>
@@ -8190,16 +8439,16 @@
         <v>1186</v>
       </c>
       <c r="S19" t="s">
-        <v>1185</v>
+        <v>2225</v>
       </c>
       <c r="T19" t="s">
-        <v>1192</v>
+        <v>2231</v>
       </c>
       <c r="U19" t="s">
         <v>2223</v>
       </c>
       <c r="V19" t="s">
-        <v>2226</v>
+        <v>2227</v>
       </c>
     </row>
     <row r="20">
@@ -8263,13 +8512,13 @@
         <v>51</v>
       </c>
       <c r="C21" t="s">
-        <v>2230</v>
+        <v>2232</v>
       </c>
       <c r="D21" t="s">
         <v>2223</v>
       </c>
       <c r="E21" t="s">
-        <v>2231</v>
+        <v>2233</v>
       </c>
       <c r="F21" t="s">
         <v>54</v>
@@ -67721,7 +67970,7 @@
         <v>162</v>
       </c>
       <c r="C1103" t="s">
-        <v>2232</v>
+        <v>2234</v>
       </c>
       <c r="D1103" t="s">
         <v>50</v>
@@ -67785,7 +68034,7 @@
         <v>166</v>
       </c>
       <c r="C1105" t="s">
-        <v>2232</v>
+        <v>2234</v>
       </c>
       <c r="D1105" t="s">
         <v>50</v>
@@ -67817,7 +68066,7 @@
         <v>167</v>
       </c>
       <c r="C1106" t="s">
-        <v>190</v>
+        <v>168</v>
       </c>
       <c r="D1106" t="s">
         <v>50</v>
@@ -87819,16 +88068,16 @@
         <v>2223</v>
       </c>
       <c r="B1630" t="s">
-        <v>2233</v>
+        <v>2235</v>
       </c>
       <c r="C1630" t="s">
-        <v>2234</v>
+        <v>2236</v>
       </c>
       <c r="D1630" t="s">
         <v>1181</v>
       </c>
       <c r="E1630" t="s">
-        <v>2235</v>
+        <v>2237</v>
       </c>
       <c r="F1630" t="s">
         <v>54</v>
@@ -87857,16 +88106,16 @@
         <v>2223</v>
       </c>
       <c r="B1631" t="s">
-        <v>2236</v>
+        <v>2238</v>
       </c>
       <c r="C1631" t="s">
-        <v>2237</v>
+        <v>2239</v>
       </c>
       <c r="D1631" t="s">
         <v>1181</v>
       </c>
       <c r="E1631" t="s">
-        <v>2238</v>
+        <v>2240</v>
       </c>
       <c r="F1631" t="s">
         <v>54</v>
@@ -87895,16 +88144,16 @@
         <v>2223</v>
       </c>
       <c r="B1632" t="s">
-        <v>2239</v>
+        <v>2241</v>
       </c>
       <c r="C1632" t="s">
-        <v>2230</v>
+        <v>2242</v>
       </c>
       <c r="D1632" t="s">
         <v>2223</v>
       </c>
       <c r="E1632" t="s">
-        <v>2231</v>
+        <v>2243</v>
       </c>
       <c r="F1632" t="s">
         <v>54</v>
@@ -87933,31 +88182,37 @@
         <v>2223</v>
       </c>
       <c r="B1633" t="s">
-        <v>50</v>
+        <v>2244</v>
       </c>
       <c r="C1633" t="s">
-        <v>50</v>
+        <v>2245</v>
       </c>
       <c r="D1633" t="s">
-        <v>50</v>
+        <v>2223</v>
       </c>
       <c r="E1633" t="s">
-        <v>50</v>
+        <v>2246</v>
       </c>
       <c r="F1633" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="G1633" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="H1633" t="s">
-        <v>50</v>
+        <v>29</v>
       </c>
       <c r="I1633" t="s">
-        <v>50</v>
+        <v>30</v>
       </c>
       <c r="J1633" t="s">
-        <v>50</v>
+        <v>29</v>
+      </c>
+      <c r="K1633" t="s">
+        <v>39</v>
+      </c>
+      <c r="L1633" t="s">
+        <v>54</v>
       </c>
     </row>
     <row r="1634">
@@ -87965,30 +88220,1056 @@
         <v>2223</v>
       </c>
       <c r="B1634" t="s">
+        <v>2247</v>
+      </c>
+      <c r="C1634" t="s">
+        <v>2248</v>
+      </c>
+      <c r="D1634" t="s">
+        <v>2223</v>
+      </c>
+      <c r="E1634" t="s">
+        <v>2249</v>
+      </c>
+      <c r="F1634" t="s">
+        <v>54</v>
+      </c>
+      <c r="G1634" t="s">
+        <v>55</v>
+      </c>
+      <c r="H1634" t="s">
+        <v>29</v>
+      </c>
+      <c r="I1634" t="s">
+        <v>30</v>
+      </c>
+      <c r="J1634" t="s">
+        <v>29</v>
+      </c>
+      <c r="K1634" t="s">
+        <v>39</v>
+      </c>
+      <c r="L1634" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="1635">
+      <c r="A1635" t="s">
+        <v>2223</v>
+      </c>
+      <c r="B1635" t="s">
+        <v>2250</v>
+      </c>
+      <c r="C1635" t="s">
+        <v>2251</v>
+      </c>
+      <c r="D1635" t="s">
+        <v>2223</v>
+      </c>
+      <c r="E1635" t="s">
+        <v>2252</v>
+      </c>
+      <c r="F1635" t="s">
+        <v>54</v>
+      </c>
+      <c r="G1635" t="s">
+        <v>55</v>
+      </c>
+      <c r="H1635" t="s">
+        <v>29</v>
+      </c>
+      <c r="I1635" t="s">
+        <v>30</v>
+      </c>
+      <c r="J1635" t="s">
+        <v>29</v>
+      </c>
+      <c r="K1635" t="s">
+        <v>39</v>
+      </c>
+      <c r="L1635" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="1636">
+      <c r="A1636" t="s">
+        <v>2223</v>
+      </c>
+      <c r="B1636" t="s">
+        <v>2253</v>
+      </c>
+      <c r="C1636" t="s">
+        <v>2254</v>
+      </c>
+      <c r="D1636" t="s">
+        <v>2223</v>
+      </c>
+      <c r="E1636" t="s">
+        <v>2255</v>
+      </c>
+      <c r="F1636" t="s">
+        <v>180</v>
+      </c>
+      <c r="G1636" t="s">
+        <v>55</v>
+      </c>
+      <c r="H1636" t="s">
+        <v>29</v>
+      </c>
+      <c r="I1636" t="s">
+        <v>30</v>
+      </c>
+      <c r="J1636" t="s">
+        <v>50</v>
+      </c>
+      <c r="K1636" t="s">
+        <v>181</v>
+      </c>
+      <c r="L1636" t="s">
+        <v>180</v>
+      </c>
+      <c r="M1636" t="s">
+        <v>587</v>
+      </c>
+    </row>
+    <row r="1637">
+      <c r="A1637" t="s">
+        <v>2223</v>
+      </c>
+      <c r="B1637" t="s">
+        <v>2256</v>
+      </c>
+      <c r="C1637" t="s">
+        <v>2257</v>
+      </c>
+      <c r="D1637" t="s">
+        <v>2223</v>
+      </c>
+      <c r="E1637" t="s">
+        <v>2258</v>
+      </c>
+      <c r="F1637" t="s">
+        <v>180</v>
+      </c>
+      <c r="G1637" t="s">
+        <v>55</v>
+      </c>
+      <c r="H1637" t="s">
+        <v>29</v>
+      </c>
+      <c r="I1637" t="s">
+        <v>30</v>
+      </c>
+      <c r="J1637" t="s">
+        <v>50</v>
+      </c>
+      <c r="K1637" t="s">
+        <v>181</v>
+      </c>
+      <c r="L1637" t="s">
+        <v>180</v>
+      </c>
+      <c r="M1637" t="s">
+        <v>587</v>
+      </c>
+    </row>
+    <row r="1638">
+      <c r="A1638" t="s">
+        <v>2223</v>
+      </c>
+      <c r="B1638" t="s">
+        <v>2259</v>
+      </c>
+      <c r="C1638" t="s">
+        <v>2260</v>
+      </c>
+      <c r="D1638" t="s">
+        <v>2223</v>
+      </c>
+      <c r="E1638" t="s">
+        <v>2261</v>
+      </c>
+      <c r="F1638" t="s">
+        <v>54</v>
+      </c>
+      <c r="G1638" t="s">
+        <v>55</v>
+      </c>
+      <c r="H1638" t="s">
+        <v>29</v>
+      </c>
+      <c r="I1638" t="s">
+        <v>30</v>
+      </c>
+      <c r="J1638" t="s">
+        <v>29</v>
+      </c>
+      <c r="K1638" t="s">
+        <v>39</v>
+      </c>
+      <c r="L1638" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="1639">
+      <c r="A1639" t="s">
+        <v>2223</v>
+      </c>
+      <c r="B1639" t="s">
+        <v>2262</v>
+      </c>
+      <c r="C1639" t="s">
+        <v>2263</v>
+      </c>
+      <c r="D1639" t="s">
+        <v>2223</v>
+      </c>
+      <c r="E1639" t="s">
+        <v>2264</v>
+      </c>
+      <c r="F1639" t="s">
+        <v>54</v>
+      </c>
+      <c r="G1639" t="s">
+        <v>55</v>
+      </c>
+      <c r="H1639" t="s">
+        <v>29</v>
+      </c>
+      <c r="I1639" t="s">
+        <v>30</v>
+      </c>
+      <c r="J1639" t="s">
+        <v>29</v>
+      </c>
+      <c r="K1639" t="s">
+        <v>39</v>
+      </c>
+      <c r="L1639" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="1640">
+      <c r="A1640" t="s">
+        <v>2223</v>
+      </c>
+      <c r="B1640" t="s">
+        <v>2265</v>
+      </c>
+      <c r="C1640" t="s">
+        <v>2266</v>
+      </c>
+      <c r="D1640" t="s">
+        <v>2223</v>
+      </c>
+      <c r="E1640" t="s">
+        <v>2267</v>
+      </c>
+      <c r="F1640" t="s">
+        <v>54</v>
+      </c>
+      <c r="G1640" t="s">
+        <v>55</v>
+      </c>
+      <c r="H1640" t="s">
+        <v>29</v>
+      </c>
+      <c r="I1640" t="s">
+        <v>30</v>
+      </c>
+      <c r="J1640" t="s">
+        <v>29</v>
+      </c>
+      <c r="K1640" t="s">
+        <v>39</v>
+      </c>
+      <c r="L1640" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="1641">
+      <c r="A1641" t="s">
+        <v>2223</v>
+      </c>
+      <c r="B1641" t="s">
+        <v>2268</v>
+      </c>
+      <c r="C1641" t="s">
+        <v>2269</v>
+      </c>
+      <c r="D1641" t="s">
+        <v>2223</v>
+      </c>
+      <c r="E1641" t="s">
+        <v>2270</v>
+      </c>
+      <c r="F1641" t="s">
+        <v>54</v>
+      </c>
+      <c r="G1641" t="s">
+        <v>55</v>
+      </c>
+      <c r="H1641" t="s">
+        <v>29</v>
+      </c>
+      <c r="I1641" t="s">
+        <v>30</v>
+      </c>
+      <c r="J1641" t="s">
+        <v>29</v>
+      </c>
+      <c r="K1641" t="s">
+        <v>39</v>
+      </c>
+      <c r="L1641" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="1642">
+      <c r="A1642" t="s">
+        <v>2223</v>
+      </c>
+      <c r="B1642" t="s">
+        <v>2271</v>
+      </c>
+      <c r="C1642" t="s">
+        <v>2272</v>
+      </c>
+      <c r="D1642" t="s">
+        <v>2223</v>
+      </c>
+      <c r="E1642" t="s">
+        <v>2273</v>
+      </c>
+      <c r="F1642" t="s">
+        <v>54</v>
+      </c>
+      <c r="G1642" t="s">
+        <v>55</v>
+      </c>
+      <c r="H1642" t="s">
+        <v>29</v>
+      </c>
+      <c r="I1642" t="s">
+        <v>30</v>
+      </c>
+      <c r="J1642" t="s">
+        <v>29</v>
+      </c>
+      <c r="K1642" t="s">
+        <v>39</v>
+      </c>
+      <c r="L1642" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="1643">
+      <c r="A1643" t="s">
+        <v>2223</v>
+      </c>
+      <c r="B1643" t="s">
+        <v>2274</v>
+      </c>
+      <c r="C1643" t="s">
+        <v>2275</v>
+      </c>
+      <c r="D1643" t="s">
+        <v>2223</v>
+      </c>
+      <c r="E1643" t="s">
+        <v>2276</v>
+      </c>
+      <c r="F1643" t="s">
+        <v>54</v>
+      </c>
+      <c r="G1643" t="s">
+        <v>55</v>
+      </c>
+      <c r="H1643" t="s">
+        <v>29</v>
+      </c>
+      <c r="I1643" t="s">
+        <v>30</v>
+      </c>
+      <c r="J1643" t="s">
+        <v>29</v>
+      </c>
+      <c r="K1643" t="s">
+        <v>39</v>
+      </c>
+      <c r="L1643" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="1644">
+      <c r="A1644" t="s">
+        <v>2223</v>
+      </c>
+      <c r="B1644" t="s">
+        <v>2277</v>
+      </c>
+      <c r="C1644" t="s">
+        <v>2278</v>
+      </c>
+      <c r="D1644" t="s">
+        <v>2223</v>
+      </c>
+      <c r="E1644" t="s">
+        <v>2279</v>
+      </c>
+      <c r="F1644" t="s">
+        <v>54</v>
+      </c>
+      <c r="G1644" t="s">
+        <v>55</v>
+      </c>
+      <c r="H1644" t="s">
+        <v>29</v>
+      </c>
+      <c r="I1644" t="s">
+        <v>30</v>
+      </c>
+      <c r="J1644" t="s">
+        <v>29</v>
+      </c>
+      <c r="K1644" t="s">
+        <v>39</v>
+      </c>
+      <c r="L1644" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="1645">
+      <c r="A1645" t="s">
+        <v>2223</v>
+      </c>
+      <c r="B1645" t="s">
+        <v>2280</v>
+      </c>
+      <c r="C1645" t="s">
+        <v>2281</v>
+      </c>
+      <c r="D1645" t="s">
+        <v>2223</v>
+      </c>
+      <c r="E1645" t="s">
+        <v>2282</v>
+      </c>
+      <c r="F1645" t="s">
+        <v>54</v>
+      </c>
+      <c r="G1645" t="s">
+        <v>55</v>
+      </c>
+      <c r="H1645" t="s">
+        <v>29</v>
+      </c>
+      <c r="I1645" t="s">
+        <v>30</v>
+      </c>
+      <c r="J1645" t="s">
+        <v>29</v>
+      </c>
+      <c r="K1645" t="s">
+        <v>39</v>
+      </c>
+      <c r="L1645" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="1646">
+      <c r="A1646" t="s">
+        <v>2223</v>
+      </c>
+      <c r="B1646" t="s">
+        <v>2283</v>
+      </c>
+      <c r="C1646" t="s">
+        <v>2284</v>
+      </c>
+      <c r="D1646" t="s">
+        <v>2223</v>
+      </c>
+      <c r="E1646" t="s">
+        <v>2285</v>
+      </c>
+      <c r="F1646" t="s">
+        <v>54</v>
+      </c>
+      <c r="G1646" t="s">
+        <v>55</v>
+      </c>
+      <c r="H1646" t="s">
+        <v>29</v>
+      </c>
+      <c r="I1646" t="s">
+        <v>30</v>
+      </c>
+      <c r="J1646" t="s">
+        <v>29</v>
+      </c>
+      <c r="K1646" t="s">
+        <v>39</v>
+      </c>
+      <c r="L1646" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="1647">
+      <c r="A1647" t="s">
+        <v>2223</v>
+      </c>
+      <c r="B1647" t="s">
+        <v>2286</v>
+      </c>
+      <c r="C1647" t="s">
+        <v>2287</v>
+      </c>
+      <c r="D1647" t="s">
+        <v>2223</v>
+      </c>
+      <c r="E1647" t="s">
+        <v>2288</v>
+      </c>
+      <c r="F1647" t="s">
+        <v>54</v>
+      </c>
+      <c r="G1647" t="s">
+        <v>55</v>
+      </c>
+      <c r="H1647" t="s">
+        <v>29</v>
+      </c>
+      <c r="I1647" t="s">
+        <v>30</v>
+      </c>
+      <c r="J1647" t="s">
+        <v>29</v>
+      </c>
+      <c r="K1647" t="s">
+        <v>39</v>
+      </c>
+      <c r="L1647" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="1648">
+      <c r="A1648" t="s">
+        <v>2223</v>
+      </c>
+      <c r="B1648" t="s">
+        <v>2289</v>
+      </c>
+      <c r="C1648" t="s">
+        <v>2290</v>
+      </c>
+      <c r="D1648" t="s">
+        <v>2223</v>
+      </c>
+      <c r="E1648" t="s">
+        <v>2291</v>
+      </c>
+      <c r="F1648" t="s">
+        <v>54</v>
+      </c>
+      <c r="G1648" t="s">
+        <v>55</v>
+      </c>
+      <c r="H1648" t="s">
+        <v>29</v>
+      </c>
+      <c r="I1648" t="s">
+        <v>30</v>
+      </c>
+      <c r="J1648" t="s">
+        <v>29</v>
+      </c>
+      <c r="K1648" t="s">
+        <v>39</v>
+      </c>
+      <c r="L1648" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="1649">
+      <c r="A1649" t="s">
+        <v>2223</v>
+      </c>
+      <c r="B1649" t="s">
+        <v>2292</v>
+      </c>
+      <c r="C1649" t="s">
+        <v>2293</v>
+      </c>
+      <c r="D1649" t="s">
+        <v>2223</v>
+      </c>
+      <c r="E1649" t="s">
+        <v>2294</v>
+      </c>
+      <c r="F1649" t="s">
+        <v>54</v>
+      </c>
+      <c r="G1649" t="s">
+        <v>55</v>
+      </c>
+      <c r="H1649" t="s">
+        <v>29</v>
+      </c>
+      <c r="I1649" t="s">
+        <v>30</v>
+      </c>
+      <c r="J1649" t="s">
+        <v>29</v>
+      </c>
+      <c r="K1649" t="s">
+        <v>39</v>
+      </c>
+      <c r="L1649" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="1650">
+      <c r="A1650" t="s">
+        <v>2223</v>
+      </c>
+      <c r="B1650" t="s">
+        <v>2295</v>
+      </c>
+      <c r="C1650" t="s">
+        <v>2296</v>
+      </c>
+      <c r="D1650" t="s">
+        <v>2223</v>
+      </c>
+      <c r="E1650" t="s">
+        <v>2297</v>
+      </c>
+      <c r="F1650" t="s">
+        <v>54</v>
+      </c>
+      <c r="G1650" t="s">
+        <v>55</v>
+      </c>
+      <c r="H1650" t="s">
+        <v>29</v>
+      </c>
+      <c r="I1650" t="s">
+        <v>30</v>
+      </c>
+      <c r="J1650" t="s">
+        <v>29</v>
+      </c>
+      <c r="K1650" t="s">
+        <v>39</v>
+      </c>
+      <c r="L1650" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="1651">
+      <c r="A1651" t="s">
+        <v>2223</v>
+      </c>
+      <c r="B1651" t="s">
+        <v>2298</v>
+      </c>
+      <c r="C1651" t="s">
+        <v>2299</v>
+      </c>
+      <c r="D1651" t="s">
+        <v>2223</v>
+      </c>
+      <c r="E1651" t="s">
+        <v>2300</v>
+      </c>
+      <c r="F1651" t="s">
+        <v>54</v>
+      </c>
+      <c r="G1651" t="s">
+        <v>55</v>
+      </c>
+      <c r="H1651" t="s">
+        <v>29</v>
+      </c>
+      <c r="I1651" t="s">
+        <v>30</v>
+      </c>
+      <c r="J1651" t="s">
+        <v>29</v>
+      </c>
+      <c r="K1651" t="s">
+        <v>39</v>
+      </c>
+      <c r="L1651" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="1652">
+      <c r="A1652" t="s">
+        <v>2223</v>
+      </c>
+      <c r="B1652" t="s">
+        <v>2301</v>
+      </c>
+      <c r="C1652" t="s">
+        <v>2302</v>
+      </c>
+      <c r="D1652" t="s">
+        <v>2223</v>
+      </c>
+      <c r="E1652" t="s">
+        <v>2303</v>
+      </c>
+      <c r="F1652" t="s">
+        <v>54</v>
+      </c>
+      <c r="G1652" t="s">
+        <v>55</v>
+      </c>
+      <c r="H1652" t="s">
+        <v>29</v>
+      </c>
+      <c r="I1652" t="s">
+        <v>30</v>
+      </c>
+      <c r="J1652" t="s">
+        <v>29</v>
+      </c>
+      <c r="K1652" t="s">
+        <v>39</v>
+      </c>
+      <c r="L1652" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="1653">
+      <c r="A1653" t="s">
+        <v>2223</v>
+      </c>
+      <c r="B1653" t="s">
+        <v>2304</v>
+      </c>
+      <c r="C1653" t="s">
+        <v>2305</v>
+      </c>
+      <c r="D1653" t="s">
+        <v>2223</v>
+      </c>
+      <c r="E1653" t="s">
+        <v>2306</v>
+      </c>
+      <c r="F1653" t="s">
+        <v>54</v>
+      </c>
+      <c r="G1653" t="s">
+        <v>55</v>
+      </c>
+      <c r="H1653" t="s">
+        <v>29</v>
+      </c>
+      <c r="I1653" t="s">
+        <v>30</v>
+      </c>
+      <c r="J1653" t="s">
+        <v>29</v>
+      </c>
+      <c r="K1653" t="s">
+        <v>39</v>
+      </c>
+      <c r="L1653" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="1654">
+      <c r="A1654" t="s">
+        <v>2223</v>
+      </c>
+      <c r="B1654" t="s">
+        <v>2307</v>
+      </c>
+      <c r="C1654" t="s">
+        <v>2308</v>
+      </c>
+      <c r="D1654" t="s">
+        <v>2223</v>
+      </c>
+      <c r="E1654" t="s">
+        <v>2309</v>
+      </c>
+      <c r="F1654" t="s">
+        <v>54</v>
+      </c>
+      <c r="G1654" t="s">
+        <v>55</v>
+      </c>
+      <c r="H1654" t="s">
+        <v>29</v>
+      </c>
+      <c r="I1654" t="s">
+        <v>30</v>
+      </c>
+      <c r="J1654" t="s">
+        <v>29</v>
+      </c>
+      <c r="K1654" t="s">
+        <v>39</v>
+      </c>
+      <c r="L1654" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="1655">
+      <c r="A1655" t="s">
+        <v>2223</v>
+      </c>
+      <c r="B1655" t="s">
+        <v>2310</v>
+      </c>
+      <c r="C1655" t="s">
+        <v>2311</v>
+      </c>
+      <c r="D1655" t="s">
+        <v>2223</v>
+      </c>
+      <c r="E1655" t="s">
+        <v>2312</v>
+      </c>
+      <c r="F1655" t="s">
+        <v>54</v>
+      </c>
+      <c r="G1655" t="s">
+        <v>55</v>
+      </c>
+      <c r="H1655" t="s">
+        <v>29</v>
+      </c>
+      <c r="I1655" t="s">
+        <v>30</v>
+      </c>
+      <c r="J1655" t="s">
+        <v>29</v>
+      </c>
+      <c r="K1655" t="s">
+        <v>39</v>
+      </c>
+      <c r="L1655" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="1656">
+      <c r="A1656" t="s">
+        <v>2223</v>
+      </c>
+      <c r="B1656" t="s">
+        <v>2313</v>
+      </c>
+      <c r="C1656" t="s">
+        <v>2314</v>
+      </c>
+      <c r="D1656" t="s">
+        <v>2223</v>
+      </c>
+      <c r="E1656" t="s">
+        <v>2315</v>
+      </c>
+      <c r="F1656" t="s">
+        <v>54</v>
+      </c>
+      <c r="G1656" t="s">
+        <v>55</v>
+      </c>
+      <c r="H1656" t="s">
+        <v>29</v>
+      </c>
+      <c r="I1656" t="s">
+        <v>30</v>
+      </c>
+      <c r="J1656" t="s">
+        <v>29</v>
+      </c>
+      <c r="K1656" t="s">
+        <v>39</v>
+      </c>
+      <c r="L1656" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="1657">
+      <c r="A1657" t="s">
+        <v>2223</v>
+      </c>
+      <c r="B1657" t="s">
+        <v>2316</v>
+      </c>
+      <c r="C1657" t="s">
+        <v>2317</v>
+      </c>
+      <c r="D1657" t="s">
+        <v>2223</v>
+      </c>
+      <c r="E1657" t="s">
+        <v>2318</v>
+      </c>
+      <c r="F1657" t="s">
+        <v>54</v>
+      </c>
+      <c r="G1657" t="s">
+        <v>55</v>
+      </c>
+      <c r="H1657" t="s">
+        <v>29</v>
+      </c>
+      <c r="I1657" t="s">
+        <v>30</v>
+      </c>
+      <c r="J1657" t="s">
+        <v>29</v>
+      </c>
+      <c r="K1657" t="s">
+        <v>39</v>
+      </c>
+      <c r="L1657" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="1658">
+      <c r="A1658" t="s">
+        <v>2223</v>
+      </c>
+      <c r="B1658" t="s">
+        <v>2319</v>
+      </c>
+      <c r="C1658" t="s">
+        <v>2320</v>
+      </c>
+      <c r="D1658" t="s">
+        <v>2223</v>
+      </c>
+      <c r="E1658" t="s">
+        <v>2321</v>
+      </c>
+      <c r="F1658" t="s">
+        <v>54</v>
+      </c>
+      <c r="G1658" t="s">
+        <v>55</v>
+      </c>
+      <c r="H1658" t="s">
+        <v>29</v>
+      </c>
+      <c r="I1658" t="s">
+        <v>30</v>
+      </c>
+      <c r="J1658" t="s">
+        <v>29</v>
+      </c>
+      <c r="K1658" t="s">
+        <v>39</v>
+      </c>
+      <c r="L1658" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="1659">
+      <c r="A1659" t="s">
+        <v>2223</v>
+      </c>
+      <c r="B1659" t="s">
+        <v>2322</v>
+      </c>
+      <c r="C1659" t="s">
+        <v>2232</v>
+      </c>
+      <c r="D1659" t="s">
+        <v>2223</v>
+      </c>
+      <c r="E1659" t="s">
+        <v>2233</v>
+      </c>
+      <c r="F1659" t="s">
+        <v>54</v>
+      </c>
+      <c r="G1659" t="s">
+        <v>55</v>
+      </c>
+      <c r="H1659" t="s">
+        <v>29</v>
+      </c>
+      <c r="I1659" t="s">
+        <v>30</v>
+      </c>
+      <c r="J1659" t="s">
+        <v>29</v>
+      </c>
+      <c r="K1659" t="s">
+        <v>39</v>
+      </c>
+      <c r="L1659" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="1660">
+      <c r="A1660" t="s">
+        <v>2223</v>
+      </c>
+      <c r="B1660" t="s">
+        <v>50</v>
+      </c>
+      <c r="C1660" t="s">
+        <v>50</v>
+      </c>
+      <c r="D1660" t="s">
+        <v>50</v>
+      </c>
+      <c r="E1660" t="s">
+        <v>50</v>
+      </c>
+      <c r="F1660" t="s">
+        <v>50</v>
+      </c>
+      <c r="G1660" t="s">
+        <v>50</v>
+      </c>
+      <c r="H1660" t="s">
+        <v>50</v>
+      </c>
+      <c r="I1660" t="s">
+        <v>50</v>
+      </c>
+      <c r="J1660" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="1661">
+      <c r="A1661" t="s">
+        <v>2223</v>
+      </c>
+      <c r="B1661" t="s">
         <v>230</v>
       </c>
-      <c r="C1634" t="s">
-        <v>2240</v>
-      </c>
-      <c r="D1634" t="s">
-        <v>50</v>
-      </c>
-      <c r="E1634" t="s">
+      <c r="C1661" t="s">
+        <v>2323</v>
+      </c>
+      <c r="D1661" t="s">
+        <v>50</v>
+      </c>
+      <c r="E1661" t="s">
         <v>232</v>
       </c>
-      <c r="F1634" t="s">
-        <v>2239</v>
-      </c>
-      <c r="G1634" t="s">
-        <v>50</v>
-      </c>
-      <c r="H1634" t="s">
-        <v>50</v>
-      </c>
-      <c r="I1634" t="s">
-        <v>50</v>
-      </c>
-      <c r="J1634" t="s">
+      <c r="F1661" t="s">
+        <v>2322</v>
+      </c>
+      <c r="G1661" t="s">
+        <v>50</v>
+      </c>
+      <c r="H1661" t="s">
+        <v>50</v>
+      </c>
+      <c r="I1661" t="s">
+        <v>50</v>
+      </c>
+      <c r="J1661" t="s">
         <v>50</v>
       </c>
     </row>

</xml_diff>

<commit_message>
compiled report 2026-06-06: 551 election events, 279 audit entries
</commit_message>
<xml_diff>
--- a/punmonitor-compiled-report.xlsx
+++ b/punmonitor-compiled-report.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2324" uniqueCount="2324">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2343" uniqueCount="2343">
   <si>
     <t>Source Date</t>
   </si>
@@ -6691,28 +6691,340 @@
     <t>2026-06-06</t>
   </si>
   <si>
-    <t>10.0.59</t>
-  </si>
-  <si>
-    <t>2026-06-06 02:12:42</t>
-  </si>
-  <si>
-    <t>2h 50m 9s</t>
-  </si>
-  <si>
-    <t>02:14:57</t>
-  </si>
-  <si>
-    <t>122.0</t>
-  </si>
-  <si>
-    <t>113683.3</t>
-  </si>
-  <si>
-    <t>954</t>
-  </si>
-  <si>
-    <t>2h 49m 44s</t>
+    <t>10.0.60</t>
+  </si>
+  <si>
+    <t>2026-06-06 02:18:47</t>
+  </si>
+  <si>
+    <t>2h 54m 14s</t>
+  </si>
+  <si>
+    <t>02:21:01</t>
+  </si>
+  <si>
+    <t>100.0</t>
+  </si>
+  <si>
+    <t>110214.7</t>
+  </si>
+  <si>
+    <t>1148</t>
+  </si>
+  <si>
+    <t>2h 52m 59s</t>
+  </si>
+  <si>
+    <t>2026-06-06T02:19:01.3448451+05:30</t>
+  </si>
+  <si>
+    <t>02:19:01.344</t>
+  </si>
+  <si>
+    <t>1780692604499</t>
+  </si>
+  <si>
+    <t>02:20:04</t>
+  </si>
+  <si>
+    <t>72MYabHy</t>
+  </si>
+  <si>
+    <t>1780692604755</t>
+  </si>
+  <si>
+    <t>1780692606976</t>
+  </si>
+  <si>
+    <t>02:20:06</t>
+  </si>
+  <si>
+    <t>gGIz8GGT</t>
+  </si>
+  <si>
+    <t>1780692607134</t>
+  </si>
+  <si>
+    <t>02:20:07</t>
+  </si>
+  <si>
+    <t>1780692607886</t>
+  </si>
+  <si>
+    <t>prYYq3pj</t>
+  </si>
+  <si>
+    <t>1780692608129</t>
+  </si>
+  <si>
+    <t>02:20:08</t>
+  </si>
+  <si>
+    <t>2026-06-06T02:19:01+05:30 (2m0s ago)</t>
+  </si>
+  <si>
+    <t>520</t>
+  </si>
+  <si>
+    <t>2026-06-05T23:53:04.3464959+05:30</t>
+  </si>
+  <si>
+    <t>23:53:04.346</t>
+  </si>
+  <si>
+    <t>521</t>
+  </si>
+  <si>
+    <t>2026-06-05T23:58:04.4885433+05:30</t>
+  </si>
+  <si>
+    <t>23:58:04.488</t>
+  </si>
+  <si>
+    <t>522</t>
+  </si>
+  <si>
+    <t>2026-06-06T00:03:04.5336367+05:30</t>
+  </si>
+  <si>
+    <t>00:03:04.533</t>
+  </si>
+  <si>
+    <t>523</t>
+  </si>
+  <si>
+    <t>2026-06-06T00:08:04.3890711+05:30</t>
+  </si>
+  <si>
+    <t>00:08:04.389</t>
+  </si>
+  <si>
+    <t>524</t>
+  </si>
+  <si>
+    <t>2026-06-06T00:13:04.2945198+05:30</t>
+  </si>
+  <si>
+    <t>00:13:04.294</t>
+  </si>
+  <si>
+    <t>525</t>
+  </si>
+  <si>
+    <t>2026-06-06T00:18:04.349719+05:30</t>
+  </si>
+  <si>
+    <t>00:18:04.349</t>
+  </si>
+  <si>
+    <t>526</t>
+  </si>
+  <si>
+    <t>2026-06-06T00:23:03.2036477+05:30</t>
+  </si>
+  <si>
+    <t>00:23:03.203</t>
+  </si>
+  <si>
+    <t>527</t>
+  </si>
+  <si>
+    <t>2026-06-06T00:23:03.20476+05:30</t>
+  </si>
+  <si>
+    <t>00:23:03.204</t>
+  </si>
+  <si>
+    <t>528</t>
+  </si>
+  <si>
+    <t>2026-06-06T00:28:04.4524866+05:30</t>
+  </si>
+  <si>
+    <t>00:28:04.452</t>
+  </si>
+  <si>
+    <t>529</t>
+  </si>
+  <si>
+    <t>2026-06-06T00:33:04.9882474+05:30</t>
+  </si>
+  <si>
+    <t>00:33:04.988</t>
+  </si>
+  <si>
+    <t>530</t>
+  </si>
+  <si>
+    <t>2026-06-06T00:38:04.4578185+05:30</t>
+  </si>
+  <si>
+    <t>00:38:04.457</t>
+  </si>
+  <si>
+    <t>531</t>
+  </si>
+  <si>
+    <t>2026-06-06T00:43:04.4165849+05:30</t>
+  </si>
+  <si>
+    <t>00:43:04.416</t>
+  </si>
+  <si>
+    <t>532</t>
+  </si>
+  <si>
+    <t>2026-06-06T00:48:04.4972065+05:30</t>
+  </si>
+  <si>
+    <t>00:48:04.497</t>
+  </si>
+  <si>
+    <t>533</t>
+  </si>
+  <si>
+    <t>2026-06-06T00:53:04.4158628+05:30</t>
+  </si>
+  <si>
+    <t>00:53:04.415</t>
+  </si>
+  <si>
+    <t>534</t>
+  </si>
+  <si>
+    <t>2026-06-06T00:58:04.746462+05:30</t>
+  </si>
+  <si>
+    <t>00:58:04.746</t>
+  </si>
+  <si>
+    <t>535</t>
+  </si>
+  <si>
+    <t>2026-06-06T01:03:04.2965606+05:30</t>
+  </si>
+  <si>
+    <t>01:03:04.296</t>
+  </si>
+  <si>
+    <t>536</t>
+  </si>
+  <si>
+    <t>2026-06-06T01:08:04.4870498+05:30</t>
+  </si>
+  <si>
+    <t>01:08:04.487</t>
+  </si>
+  <si>
+    <t>537</t>
+  </si>
+  <si>
+    <t>2026-06-06T01:13:04.3971229+05:30</t>
+  </si>
+  <si>
+    <t>01:13:04.397</t>
+  </si>
+  <si>
+    <t>538</t>
+  </si>
+  <si>
+    <t>2026-06-06T01:18:04.3982097+05:30</t>
+  </si>
+  <si>
+    <t>01:18:04.398</t>
+  </si>
+  <si>
+    <t>539</t>
+  </si>
+  <si>
+    <t>2026-06-06T01:23:04.338193+05:30</t>
+  </si>
+  <si>
+    <t>01:23:04.338</t>
+  </si>
+  <si>
+    <t>540</t>
+  </si>
+  <si>
+    <t>2026-06-06T01:28:04.3749159+05:30</t>
+  </si>
+  <si>
+    <t>01:28:04.374</t>
+  </si>
+  <si>
+    <t>541</t>
+  </si>
+  <si>
+    <t>2026-06-06T01:33:04.3612467+05:30</t>
+  </si>
+  <si>
+    <t>01:33:04.361</t>
+  </si>
+  <si>
+    <t>542</t>
+  </si>
+  <si>
+    <t>2026-06-06T01:38:04.5068535+05:30</t>
+  </si>
+  <si>
+    <t>01:38:04.506</t>
+  </si>
+  <si>
+    <t>543</t>
+  </si>
+  <si>
+    <t>2026-06-06T01:43:04.4507225+05:30</t>
+  </si>
+  <si>
+    <t>01:43:04.450</t>
+  </si>
+  <si>
+    <t>544</t>
+  </si>
+  <si>
+    <t>2026-06-06T01:48:04.4562151+05:30</t>
+  </si>
+  <si>
+    <t>01:48:04.456</t>
+  </si>
+  <si>
+    <t>545</t>
+  </si>
+  <si>
+    <t>2026-06-06T01:53:04.4814572+05:30</t>
+  </si>
+  <si>
+    <t>01:53:04.481</t>
+  </si>
+  <si>
+    <t>546</t>
+  </si>
+  <si>
+    <t>2026-06-06T01:58:04.3490827+05:30</t>
+  </si>
+  <si>
+    <t>01:58:04.349</t>
+  </si>
+  <si>
+    <t>547</t>
+  </si>
+  <si>
+    <t>2026-06-06T02:03:04.395145+05:30</t>
+  </si>
+  <si>
+    <t>02:03:04.395</t>
+  </si>
+  <si>
+    <t>548</t>
+  </si>
+  <si>
+    <t>2026-06-06T02:08:04.4247916+05:30</t>
+  </si>
+  <si>
+    <t>02:08:04.424</t>
+  </si>
+  <si>
+    <t>549</t>
   </si>
   <si>
     <t>2026-06-06T02:12:57.4419603+05:30</t>
@@ -6721,274 +7033,19 @@
     <t>02:12:57.441</t>
   </si>
   <si>
-    <t>2026-06-06T02:12:57+05:30 (2m0s ago)</t>
-  </si>
-  <si>
-    <t>520</t>
-  </si>
-  <si>
-    <t>2026-06-05T23:53:04.3464959+05:30</t>
-  </si>
-  <si>
-    <t>23:53:04.346</t>
-  </si>
-  <si>
-    <t>521</t>
-  </si>
-  <si>
-    <t>2026-06-05T23:58:04.4885433+05:30</t>
-  </si>
-  <si>
-    <t>23:58:04.488</t>
-  </si>
-  <si>
-    <t>522</t>
-  </si>
-  <si>
-    <t>2026-06-06T00:03:04.5336367+05:30</t>
-  </si>
-  <si>
-    <t>00:03:04.533</t>
-  </si>
-  <si>
-    <t>523</t>
-  </si>
-  <si>
-    <t>2026-06-06T00:08:04.3890711+05:30</t>
-  </si>
-  <si>
-    <t>00:08:04.389</t>
-  </si>
-  <si>
-    <t>524</t>
-  </si>
-  <si>
-    <t>2026-06-06T00:13:04.2945198+05:30</t>
-  </si>
-  <si>
-    <t>00:13:04.294</t>
-  </si>
-  <si>
-    <t>525</t>
-  </si>
-  <si>
-    <t>2026-06-06T00:18:04.349719+05:30</t>
-  </si>
-  <si>
-    <t>00:18:04.349</t>
-  </si>
-  <si>
-    <t>526</t>
-  </si>
-  <si>
-    <t>2026-06-06T00:23:03.2036477+05:30</t>
-  </si>
-  <si>
-    <t>00:23:03.203</t>
-  </si>
-  <si>
-    <t>527</t>
-  </si>
-  <si>
-    <t>2026-06-06T00:23:03.20476+05:30</t>
-  </si>
-  <si>
-    <t>00:23:03.204</t>
-  </si>
-  <si>
-    <t>528</t>
-  </si>
-  <si>
-    <t>2026-06-06T00:28:04.4524866+05:30</t>
-  </si>
-  <si>
-    <t>00:28:04.452</t>
-  </si>
-  <si>
-    <t>529</t>
-  </si>
-  <si>
-    <t>2026-06-06T00:33:04.9882474+05:30</t>
-  </si>
-  <si>
-    <t>00:33:04.988</t>
-  </si>
-  <si>
-    <t>530</t>
-  </si>
-  <si>
-    <t>2026-06-06T00:38:04.4578185+05:30</t>
-  </si>
-  <si>
-    <t>00:38:04.457</t>
-  </si>
-  <si>
-    <t>531</t>
-  </si>
-  <si>
-    <t>2026-06-06T00:43:04.4165849+05:30</t>
-  </si>
-  <si>
-    <t>00:43:04.416</t>
-  </si>
-  <si>
-    <t>532</t>
-  </si>
-  <si>
-    <t>2026-06-06T00:48:04.4972065+05:30</t>
-  </si>
-  <si>
-    <t>00:48:04.497</t>
-  </si>
-  <si>
-    <t>533</t>
-  </si>
-  <si>
-    <t>2026-06-06T00:53:04.4158628+05:30</t>
-  </si>
-  <si>
-    <t>00:53:04.415</t>
-  </si>
-  <si>
-    <t>534</t>
-  </si>
-  <si>
-    <t>2026-06-06T00:58:04.746462+05:30</t>
-  </si>
-  <si>
-    <t>00:58:04.746</t>
-  </si>
-  <si>
-    <t>535</t>
-  </si>
-  <si>
-    <t>2026-06-06T01:03:04.2965606+05:30</t>
-  </si>
-  <si>
-    <t>01:03:04.296</t>
-  </si>
-  <si>
-    <t>536</t>
-  </si>
-  <si>
-    <t>2026-06-06T01:08:04.4870498+05:30</t>
-  </si>
-  <si>
-    <t>01:08:04.487</t>
-  </si>
-  <si>
-    <t>537</t>
-  </si>
-  <si>
-    <t>2026-06-06T01:13:04.3971229+05:30</t>
-  </si>
-  <si>
-    <t>01:13:04.397</t>
-  </si>
-  <si>
-    <t>538</t>
-  </si>
-  <si>
-    <t>2026-06-06T01:18:04.3982097+05:30</t>
-  </si>
-  <si>
-    <t>01:18:04.398</t>
-  </si>
-  <si>
-    <t>539</t>
-  </si>
-  <si>
-    <t>2026-06-06T01:23:04.338193+05:30</t>
-  </si>
-  <si>
-    <t>01:23:04.338</t>
-  </si>
-  <si>
-    <t>540</t>
-  </si>
-  <si>
-    <t>2026-06-06T01:28:04.3749159+05:30</t>
-  </si>
-  <si>
-    <t>01:28:04.374</t>
-  </si>
-  <si>
-    <t>541</t>
-  </si>
-  <si>
-    <t>2026-06-06T01:33:04.3612467+05:30</t>
-  </si>
-  <si>
-    <t>01:33:04.361</t>
-  </si>
-  <si>
-    <t>542</t>
-  </si>
-  <si>
-    <t>2026-06-06T01:38:04.5068535+05:30</t>
-  </si>
-  <si>
-    <t>01:38:04.506</t>
-  </si>
-  <si>
-    <t>543</t>
-  </si>
-  <si>
-    <t>2026-06-06T01:43:04.4507225+05:30</t>
-  </si>
-  <si>
-    <t>01:43:04.450</t>
-  </si>
-  <si>
-    <t>544</t>
-  </si>
-  <si>
-    <t>2026-06-06T01:48:04.4562151+05:30</t>
-  </si>
-  <si>
-    <t>01:48:04.456</t>
-  </si>
-  <si>
-    <t>545</t>
-  </si>
-  <si>
-    <t>2026-06-06T01:53:04.4814572+05:30</t>
-  </si>
-  <si>
-    <t>01:53:04.481</t>
-  </si>
-  <si>
-    <t>546</t>
-  </si>
-  <si>
-    <t>2026-06-06T01:58:04.3490827+05:30</t>
-  </si>
-  <si>
-    <t>01:58:04.349</t>
-  </si>
-  <si>
-    <t>547</t>
-  </si>
-  <si>
-    <t>2026-06-06T02:03:04.395145+05:30</t>
-  </si>
-  <si>
-    <t>02:03:04.395</t>
-  </si>
-  <si>
-    <t>548</t>
-  </si>
-  <si>
-    <t>2026-06-06T02:08:04.4247916+05:30</t>
-  </si>
-  <si>
-    <t>02:08:04.424</t>
-  </si>
-  <si>
-    <t>549</t>
-  </si>
-  <si>
-    <t>2026-06-06T02:14:57+05:30</t>
+    <t>550</t>
+  </si>
+  <si>
+    <t>2026-06-06T02:17:58.646138+05:30</t>
+  </si>
+  <si>
+    <t>02:17:58.646</t>
+  </si>
+  <si>
+    <t>551</t>
+  </si>
+  <si>
+    <t>2026-06-06T02:21:01+05:30</t>
   </si>
 </sst>
 </file>
@@ -8362,7 +8419,7 @@
         <v>39</v>
       </c>
       <c r="P18" t="s">
-        <v>739</v>
+        <v>1184</v>
       </c>
       <c r="Q18" t="s">
         <v>2225</v>
@@ -8430,7 +8487,7 @@
         <v>245</v>
       </c>
       <c r="P19" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
       <c r="Q19" t="s">
         <v>46</v>
@@ -26219,6 +26276,162 @@
         <v>50</v>
       </c>
     </row>
+    <row r="680">
+      <c r="A680" t="s">
+        <v>2223</v>
+      </c>
+      <c r="B680" t="s">
+        <v>2234</v>
+      </c>
+      <c r="C680" t="s">
+        <v>2235</v>
+      </c>
+      <c r="D680" t="s">
+        <v>2223</v>
+      </c>
+      <c r="E680" t="s">
+        <v>58</v>
+      </c>
+      <c r="F680" t="s">
+        <v>50</v>
+      </c>
+      <c r="G680" t="s">
+        <v>59</v>
+      </c>
+      <c r="H680" t="s">
+        <v>2236</v>
+      </c>
+    </row>
+    <row r="681">
+      <c r="A681" t="s">
+        <v>2223</v>
+      </c>
+      <c r="B681" t="s">
+        <v>2237</v>
+      </c>
+      <c r="C681" t="s">
+        <v>2235</v>
+      </c>
+      <c r="D681" t="s">
+        <v>2223</v>
+      </c>
+      <c r="E681" t="s">
+        <v>62</v>
+      </c>
+      <c r="F681" t="s">
+        <v>2236</v>
+      </c>
+      <c r="G681" t="s">
+        <v>59</v>
+      </c>
+      <c r="H681" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="682">
+      <c r="A682" t="s">
+        <v>2223</v>
+      </c>
+      <c r="B682" t="s">
+        <v>2238</v>
+      </c>
+      <c r="C682" t="s">
+        <v>2239</v>
+      </c>
+      <c r="D682" t="s">
+        <v>2223</v>
+      </c>
+      <c r="E682" t="s">
+        <v>58</v>
+      </c>
+      <c r="F682" t="s">
+        <v>50</v>
+      </c>
+      <c r="G682" t="s">
+        <v>59</v>
+      </c>
+      <c r="H682" t="s">
+        <v>2240</v>
+      </c>
+    </row>
+    <row r="683">
+      <c r="A683" t="s">
+        <v>2223</v>
+      </c>
+      <c r="B683" t="s">
+        <v>2241</v>
+      </c>
+      <c r="C683" t="s">
+        <v>2242</v>
+      </c>
+      <c r="D683" t="s">
+        <v>2223</v>
+      </c>
+      <c r="E683" t="s">
+        <v>62</v>
+      </c>
+      <c r="F683" t="s">
+        <v>2240</v>
+      </c>
+      <c r="G683" t="s">
+        <v>59</v>
+      </c>
+      <c r="H683" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="684">
+      <c r="A684" t="s">
+        <v>2223</v>
+      </c>
+      <c r="B684" t="s">
+        <v>2243</v>
+      </c>
+      <c r="C684" t="s">
+        <v>2242</v>
+      </c>
+      <c r="D684" t="s">
+        <v>2223</v>
+      </c>
+      <c r="E684" t="s">
+        <v>58</v>
+      </c>
+      <c r="F684" t="s">
+        <v>50</v>
+      </c>
+      <c r="G684" t="s">
+        <v>59</v>
+      </c>
+      <c r="H684" t="s">
+        <v>2244</v>
+      </c>
+    </row>
+    <row r="685">
+      <c r="A685" t="s">
+        <v>2223</v>
+      </c>
+      <c r="B685" t="s">
+        <v>2245</v>
+      </c>
+      <c r="C685" t="s">
+        <v>2246</v>
+      </c>
+      <c r="D685" t="s">
+        <v>2223</v>
+      </c>
+      <c r="E685" t="s">
+        <v>62</v>
+      </c>
+      <c r="F685" t="s">
+        <v>2244</v>
+      </c>
+      <c r="G685" t="s">
+        <v>59</v>
+      </c>
+      <c r="H685" t="s">
+        <v>50</v>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
@@ -67970,7 +68183,7 @@
         <v>162</v>
       </c>
       <c r="C1103" t="s">
-        <v>2234</v>
+        <v>2247</v>
       </c>
       <c r="D1103" t="s">
         <v>50</v>
@@ -68034,7 +68247,7 @@
         <v>166</v>
       </c>
       <c r="C1105" t="s">
-        <v>2234</v>
+        <v>2247</v>
       </c>
       <c r="D1105" t="s">
         <v>50</v>
@@ -88068,16 +88281,16 @@
         <v>2223</v>
       </c>
       <c r="B1630" t="s">
-        <v>2235</v>
+        <v>2248</v>
       </c>
       <c r="C1630" t="s">
-        <v>2236</v>
+        <v>2249</v>
       </c>
       <c r="D1630" t="s">
         <v>1181</v>
       </c>
       <c r="E1630" t="s">
-        <v>2237</v>
+        <v>2250</v>
       </c>
       <c r="F1630" t="s">
         <v>54</v>
@@ -88106,16 +88319,16 @@
         <v>2223</v>
       </c>
       <c r="B1631" t="s">
-        <v>2238</v>
+        <v>2251</v>
       </c>
       <c r="C1631" t="s">
-        <v>2239</v>
+        <v>2252</v>
       </c>
       <c r="D1631" t="s">
         <v>1181</v>
       </c>
       <c r="E1631" t="s">
-        <v>2240</v>
+        <v>2253</v>
       </c>
       <c r="F1631" t="s">
         <v>54</v>
@@ -88144,16 +88357,16 @@
         <v>2223</v>
       </c>
       <c r="B1632" t="s">
-        <v>2241</v>
+        <v>2254</v>
       </c>
       <c r="C1632" t="s">
-        <v>2242</v>
+        <v>2255</v>
       </c>
       <c r="D1632" t="s">
         <v>2223</v>
       </c>
       <c r="E1632" t="s">
-        <v>2243</v>
+        <v>2256</v>
       </c>
       <c r="F1632" t="s">
         <v>54</v>
@@ -88182,16 +88395,16 @@
         <v>2223</v>
       </c>
       <c r="B1633" t="s">
-        <v>2244</v>
+        <v>2257</v>
       </c>
       <c r="C1633" t="s">
-        <v>2245</v>
+        <v>2258</v>
       </c>
       <c r="D1633" t="s">
         <v>2223</v>
       </c>
       <c r="E1633" t="s">
-        <v>2246</v>
+        <v>2259</v>
       </c>
       <c r="F1633" t="s">
         <v>54</v>
@@ -88220,16 +88433,16 @@
         <v>2223</v>
       </c>
       <c r="B1634" t="s">
-        <v>2247</v>
+        <v>2260</v>
       </c>
       <c r="C1634" t="s">
-        <v>2248</v>
+        <v>2261</v>
       </c>
       <c r="D1634" t="s">
         <v>2223</v>
       </c>
       <c r="E1634" t="s">
-        <v>2249</v>
+        <v>2262</v>
       </c>
       <c r="F1634" t="s">
         <v>54</v>
@@ -88258,16 +88471,16 @@
         <v>2223</v>
       </c>
       <c r="B1635" t="s">
-        <v>2250</v>
+        <v>2263</v>
       </c>
       <c r="C1635" t="s">
-        <v>2251</v>
+        <v>2264</v>
       </c>
       <c r="D1635" t="s">
         <v>2223</v>
       </c>
       <c r="E1635" t="s">
-        <v>2252</v>
+        <v>2265</v>
       </c>
       <c r="F1635" t="s">
         <v>54</v>
@@ -88296,16 +88509,16 @@
         <v>2223</v>
       </c>
       <c r="B1636" t="s">
-        <v>2253</v>
+        <v>2266</v>
       </c>
       <c r="C1636" t="s">
-        <v>2254</v>
+        <v>2267</v>
       </c>
       <c r="D1636" t="s">
         <v>2223</v>
       </c>
       <c r="E1636" t="s">
-        <v>2255</v>
+        <v>2268</v>
       </c>
       <c r="F1636" t="s">
         <v>180</v>
@@ -88337,16 +88550,16 @@
         <v>2223</v>
       </c>
       <c r="B1637" t="s">
-        <v>2256</v>
+        <v>2269</v>
       </c>
       <c r="C1637" t="s">
-        <v>2257</v>
+        <v>2270</v>
       </c>
       <c r="D1637" t="s">
         <v>2223</v>
       </c>
       <c r="E1637" t="s">
-        <v>2258</v>
+        <v>2271</v>
       </c>
       <c r="F1637" t="s">
         <v>180</v>
@@ -88378,16 +88591,16 @@
         <v>2223</v>
       </c>
       <c r="B1638" t="s">
-        <v>2259</v>
+        <v>2272</v>
       </c>
       <c r="C1638" t="s">
-        <v>2260</v>
+        <v>2273</v>
       </c>
       <c r="D1638" t="s">
         <v>2223</v>
       </c>
       <c r="E1638" t="s">
-        <v>2261</v>
+        <v>2274</v>
       </c>
       <c r="F1638" t="s">
         <v>54</v>
@@ -88416,16 +88629,16 @@
         <v>2223</v>
       </c>
       <c r="B1639" t="s">
-        <v>2262</v>
+        <v>2275</v>
       </c>
       <c r="C1639" t="s">
-        <v>2263</v>
+        <v>2276</v>
       </c>
       <c r="D1639" t="s">
         <v>2223</v>
       </c>
       <c r="E1639" t="s">
-        <v>2264</v>
+        <v>2277</v>
       </c>
       <c r="F1639" t="s">
         <v>54</v>
@@ -88454,16 +88667,16 @@
         <v>2223</v>
       </c>
       <c r="B1640" t="s">
-        <v>2265</v>
+        <v>2278</v>
       </c>
       <c r="C1640" t="s">
-        <v>2266</v>
+        <v>2279</v>
       </c>
       <c r="D1640" t="s">
         <v>2223</v>
       </c>
       <c r="E1640" t="s">
-        <v>2267</v>
+        <v>2280</v>
       </c>
       <c r="F1640" t="s">
         <v>54</v>
@@ -88492,16 +88705,16 @@
         <v>2223</v>
       </c>
       <c r="B1641" t="s">
-        <v>2268</v>
+        <v>2281</v>
       </c>
       <c r="C1641" t="s">
-        <v>2269</v>
+        <v>2282</v>
       </c>
       <c r="D1641" t="s">
         <v>2223</v>
       </c>
       <c r="E1641" t="s">
-        <v>2270</v>
+        <v>2283</v>
       </c>
       <c r="F1641" t="s">
         <v>54</v>
@@ -88530,16 +88743,16 @@
         <v>2223</v>
       </c>
       <c r="B1642" t="s">
-        <v>2271</v>
+        <v>2284</v>
       </c>
       <c r="C1642" t="s">
-        <v>2272</v>
+        <v>2285</v>
       </c>
       <c r="D1642" t="s">
         <v>2223</v>
       </c>
       <c r="E1642" t="s">
-        <v>2273</v>
+        <v>2286</v>
       </c>
       <c r="F1642" t="s">
         <v>54</v>
@@ -88568,16 +88781,16 @@
         <v>2223</v>
       </c>
       <c r="B1643" t="s">
-        <v>2274</v>
+        <v>2287</v>
       </c>
       <c r="C1643" t="s">
-        <v>2275</v>
+        <v>2288</v>
       </c>
       <c r="D1643" t="s">
         <v>2223</v>
       </c>
       <c r="E1643" t="s">
-        <v>2276</v>
+        <v>2289</v>
       </c>
       <c r="F1643" t="s">
         <v>54</v>
@@ -88606,16 +88819,16 @@
         <v>2223</v>
       </c>
       <c r="B1644" t="s">
-        <v>2277</v>
+        <v>2290</v>
       </c>
       <c r="C1644" t="s">
-        <v>2278</v>
+        <v>2291</v>
       </c>
       <c r="D1644" t="s">
         <v>2223</v>
       </c>
       <c r="E1644" t="s">
-        <v>2279</v>
+        <v>2292</v>
       </c>
       <c r="F1644" t="s">
         <v>54</v>
@@ -88644,16 +88857,16 @@
         <v>2223</v>
       </c>
       <c r="B1645" t="s">
-        <v>2280</v>
+        <v>2293</v>
       </c>
       <c r="C1645" t="s">
-        <v>2281</v>
+        <v>2294</v>
       </c>
       <c r="D1645" t="s">
         <v>2223</v>
       </c>
       <c r="E1645" t="s">
-        <v>2282</v>
+        <v>2295</v>
       </c>
       <c r="F1645" t="s">
         <v>54</v>
@@ -88682,16 +88895,16 @@
         <v>2223</v>
       </c>
       <c r="B1646" t="s">
-        <v>2283</v>
+        <v>2296</v>
       </c>
       <c r="C1646" t="s">
-        <v>2284</v>
+        <v>2297</v>
       </c>
       <c r="D1646" t="s">
         <v>2223</v>
       </c>
       <c r="E1646" t="s">
-        <v>2285</v>
+        <v>2298</v>
       </c>
       <c r="F1646" t="s">
         <v>54</v>
@@ -88720,16 +88933,16 @@
         <v>2223</v>
       </c>
       <c r="B1647" t="s">
-        <v>2286</v>
+        <v>2299</v>
       </c>
       <c r="C1647" t="s">
-        <v>2287</v>
+        <v>2300</v>
       </c>
       <c r="D1647" t="s">
         <v>2223</v>
       </c>
       <c r="E1647" t="s">
-        <v>2288</v>
+        <v>2301</v>
       </c>
       <c r="F1647" t="s">
         <v>54</v>
@@ -88758,16 +88971,16 @@
         <v>2223</v>
       </c>
       <c r="B1648" t="s">
-        <v>2289</v>
+        <v>2302</v>
       </c>
       <c r="C1648" t="s">
-        <v>2290</v>
+        <v>2303</v>
       </c>
       <c r="D1648" t="s">
         <v>2223</v>
       </c>
       <c r="E1648" t="s">
-        <v>2291</v>
+        <v>2304</v>
       </c>
       <c r="F1648" t="s">
         <v>54</v>
@@ -88796,16 +89009,16 @@
         <v>2223</v>
       </c>
       <c r="B1649" t="s">
-        <v>2292</v>
+        <v>2305</v>
       </c>
       <c r="C1649" t="s">
-        <v>2293</v>
+        <v>2306</v>
       </c>
       <c r="D1649" t="s">
         <v>2223</v>
       </c>
       <c r="E1649" t="s">
-        <v>2294</v>
+        <v>2307</v>
       </c>
       <c r="F1649" t="s">
         <v>54</v>
@@ -88834,16 +89047,16 @@
         <v>2223</v>
       </c>
       <c r="B1650" t="s">
-        <v>2295</v>
+        <v>2308</v>
       </c>
       <c r="C1650" t="s">
-        <v>2296</v>
+        <v>2309</v>
       </c>
       <c r="D1650" t="s">
         <v>2223</v>
       </c>
       <c r="E1650" t="s">
-        <v>2297</v>
+        <v>2310</v>
       </c>
       <c r="F1650" t="s">
         <v>54</v>
@@ -88872,16 +89085,16 @@
         <v>2223</v>
       </c>
       <c r="B1651" t="s">
-        <v>2298</v>
+        <v>2311</v>
       </c>
       <c r="C1651" t="s">
-        <v>2299</v>
+        <v>2312</v>
       </c>
       <c r="D1651" t="s">
         <v>2223</v>
       </c>
       <c r="E1651" t="s">
-        <v>2300</v>
+        <v>2313</v>
       </c>
       <c r="F1651" t="s">
         <v>54</v>
@@ -88910,16 +89123,16 @@
         <v>2223</v>
       </c>
       <c r="B1652" t="s">
-        <v>2301</v>
+        <v>2314</v>
       </c>
       <c r="C1652" t="s">
-        <v>2302</v>
+        <v>2315</v>
       </c>
       <c r="D1652" t="s">
         <v>2223</v>
       </c>
       <c r="E1652" t="s">
-        <v>2303</v>
+        <v>2316</v>
       </c>
       <c r="F1652" t="s">
         <v>54</v>
@@ -88948,16 +89161,16 @@
         <v>2223</v>
       </c>
       <c r="B1653" t="s">
-        <v>2304</v>
+        <v>2317</v>
       </c>
       <c r="C1653" t="s">
-        <v>2305</v>
+        <v>2318</v>
       </c>
       <c r="D1653" t="s">
         <v>2223</v>
       </c>
       <c r="E1653" t="s">
-        <v>2306</v>
+        <v>2319</v>
       </c>
       <c r="F1653" t="s">
         <v>54</v>
@@ -88986,16 +89199,16 @@
         <v>2223</v>
       </c>
       <c r="B1654" t="s">
-        <v>2307</v>
+        <v>2320</v>
       </c>
       <c r="C1654" t="s">
-        <v>2308</v>
+        <v>2321</v>
       </c>
       <c r="D1654" t="s">
         <v>2223</v>
       </c>
       <c r="E1654" t="s">
-        <v>2309</v>
+        <v>2322</v>
       </c>
       <c r="F1654" t="s">
         <v>54</v>
@@ -89024,16 +89237,16 @@
         <v>2223</v>
       </c>
       <c r="B1655" t="s">
-        <v>2310</v>
+        <v>2323</v>
       </c>
       <c r="C1655" t="s">
-        <v>2311</v>
+        <v>2324</v>
       </c>
       <c r="D1655" t="s">
         <v>2223</v>
       </c>
       <c r="E1655" t="s">
-        <v>2312</v>
+        <v>2325</v>
       </c>
       <c r="F1655" t="s">
         <v>54</v>
@@ -89062,16 +89275,16 @@
         <v>2223</v>
       </c>
       <c r="B1656" t="s">
-        <v>2313</v>
+        <v>2326</v>
       </c>
       <c r="C1656" t="s">
-        <v>2314</v>
+        <v>2327</v>
       </c>
       <c r="D1656" t="s">
         <v>2223</v>
       </c>
       <c r="E1656" t="s">
-        <v>2315</v>
+        <v>2328</v>
       </c>
       <c r="F1656" t="s">
         <v>54</v>
@@ -89100,16 +89313,16 @@
         <v>2223</v>
       </c>
       <c r="B1657" t="s">
-        <v>2316</v>
+        <v>2329</v>
       </c>
       <c r="C1657" t="s">
-        <v>2317</v>
+        <v>2330</v>
       </c>
       <c r="D1657" t="s">
         <v>2223</v>
       </c>
       <c r="E1657" t="s">
-        <v>2318</v>
+        <v>2331</v>
       </c>
       <c r="F1657" t="s">
         <v>54</v>
@@ -89138,16 +89351,16 @@
         <v>2223</v>
       </c>
       <c r="B1658" t="s">
-        <v>2319</v>
+        <v>2332</v>
       </c>
       <c r="C1658" t="s">
-        <v>2320</v>
+        <v>2333</v>
       </c>
       <c r="D1658" t="s">
         <v>2223</v>
       </c>
       <c r="E1658" t="s">
-        <v>2321</v>
+        <v>2334</v>
       </c>
       <c r="F1658" t="s">
         <v>54</v>
@@ -89176,16 +89389,16 @@
         <v>2223</v>
       </c>
       <c r="B1659" t="s">
-        <v>2322</v>
+        <v>2335</v>
       </c>
       <c r="C1659" t="s">
-        <v>2232</v>
+        <v>2336</v>
       </c>
       <c r="D1659" t="s">
         <v>2223</v>
       </c>
       <c r="E1659" t="s">
-        <v>2233</v>
+        <v>2337</v>
       </c>
       <c r="F1659" t="s">
         <v>54</v>
@@ -89214,31 +89427,37 @@
         <v>2223</v>
       </c>
       <c r="B1660" t="s">
-        <v>50</v>
+        <v>2338</v>
       </c>
       <c r="C1660" t="s">
-        <v>50</v>
+        <v>2339</v>
       </c>
       <c r="D1660" t="s">
-        <v>50</v>
+        <v>2223</v>
       </c>
       <c r="E1660" t="s">
-        <v>50</v>
+        <v>2340</v>
       </c>
       <c r="F1660" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="G1660" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="H1660" t="s">
-        <v>50</v>
+        <v>29</v>
       </c>
       <c r="I1660" t="s">
-        <v>50</v>
+        <v>30</v>
       </c>
       <c r="J1660" t="s">
-        <v>50</v>
+        <v>29</v>
+      </c>
+      <c r="K1660" t="s">
+        <v>39</v>
+      </c>
+      <c r="L1660" t="s">
+        <v>54</v>
       </c>
     </row>
     <row r="1661">
@@ -89246,30 +89465,100 @@
         <v>2223</v>
       </c>
       <c r="B1661" t="s">
+        <v>2341</v>
+      </c>
+      <c r="C1661" t="s">
+        <v>2232</v>
+      </c>
+      <c r="D1661" t="s">
+        <v>2223</v>
+      </c>
+      <c r="E1661" t="s">
+        <v>2233</v>
+      </c>
+      <c r="F1661" t="s">
+        <v>54</v>
+      </c>
+      <c r="G1661" t="s">
+        <v>55</v>
+      </c>
+      <c r="H1661" t="s">
+        <v>29</v>
+      </c>
+      <c r="I1661" t="s">
+        <v>30</v>
+      </c>
+      <c r="J1661" t="s">
+        <v>29</v>
+      </c>
+      <c r="K1661" t="s">
+        <v>39</v>
+      </c>
+      <c r="L1661" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="1662">
+      <c r="A1662" t="s">
+        <v>2223</v>
+      </c>
+      <c r="B1662" t="s">
+        <v>50</v>
+      </c>
+      <c r="C1662" t="s">
+        <v>50</v>
+      </c>
+      <c r="D1662" t="s">
+        <v>50</v>
+      </c>
+      <c r="E1662" t="s">
+        <v>50</v>
+      </c>
+      <c r="F1662" t="s">
+        <v>50</v>
+      </c>
+      <c r="G1662" t="s">
+        <v>50</v>
+      </c>
+      <c r="H1662" t="s">
+        <v>50</v>
+      </c>
+      <c r="I1662" t="s">
+        <v>50</v>
+      </c>
+      <c r="J1662" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="1663">
+      <c r="A1663" t="s">
+        <v>2223</v>
+      </c>
+      <c r="B1663" t="s">
         <v>230</v>
       </c>
-      <c r="C1661" t="s">
-        <v>2323</v>
-      </c>
-      <c r="D1661" t="s">
-        <v>50</v>
-      </c>
-      <c r="E1661" t="s">
+      <c r="C1663" t="s">
+        <v>2342</v>
+      </c>
+      <c r="D1663" t="s">
+        <v>50</v>
+      </c>
+      <c r="E1663" t="s">
         <v>232</v>
       </c>
-      <c r="F1661" t="s">
-        <v>2322</v>
-      </c>
-      <c r="G1661" t="s">
-        <v>50</v>
-      </c>
-      <c r="H1661" t="s">
-        <v>50</v>
-      </c>
-      <c r="I1661" t="s">
-        <v>50</v>
-      </c>
-      <c r="J1661" t="s">
+      <c r="F1663" t="s">
+        <v>2341</v>
+      </c>
+      <c r="G1663" t="s">
+        <v>50</v>
+      </c>
+      <c r="H1663" t="s">
+        <v>50</v>
+      </c>
+      <c r="I1663" t="s">
+        <v>50</v>
+      </c>
+      <c r="J1663" t="s">
         <v>50</v>
       </c>
     </row>

</xml_diff>

<commit_message>
compiled report 2026-06-06: 573 election events, 279 audit entries
</commit_message>
<xml_diff>
--- a/punmonitor-compiled-report.xlsx
+++ b/punmonitor-compiled-report.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2343" uniqueCount="2343">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2418" uniqueCount="2418">
   <si>
     <t>Source Date</t>
   </si>
@@ -6691,28 +6691,385 @@
     <t>2026-06-06</t>
   </si>
   <si>
+    <t>192.168.0.164</t>
+  </si>
+  <si>
+    <t>43.247.40.101</t>
+  </si>
+  <si>
     <t>10.0.60</t>
   </si>
   <si>
-    <t>2026-06-06 02:18:47</t>
-  </si>
-  <si>
-    <t>2h 54m 14s</t>
-  </si>
-  <si>
-    <t>02:21:01</t>
-  </si>
-  <si>
-    <t>100.0</t>
-  </si>
-  <si>
-    <t>110214.7</t>
-  </si>
-  <si>
-    <t>1148</t>
-  </si>
-  <si>
-    <t>2h 52m 59s</t>
+    <t>2026-06-06 12:41:31</t>
+  </si>
+  <si>
+    <t>3h 58m 34s</t>
+  </si>
+  <si>
+    <t>12:43:45</t>
+  </si>
+  <si>
+    <t>330.0</t>
+  </si>
+  <si>
+    <t>113638.3</t>
+  </si>
+  <si>
+    <t>671</t>
+  </si>
+  <si>
+    <t>3h 58m 19s</t>
+  </si>
+  <si>
+    <t>Dual-89e4fa7c</t>
+  </si>
+  <si>
+    <t>Dual</t>
+  </si>
+  <si>
+    <t>192.168.31.110</t>
+  </si>
+  <si>
+    <t>49.36.213.176</t>
+  </si>
+  <si>
+    <t>websocket</t>
+  </si>
+  <si>
+    <t>1060.0</t>
+  </si>
+  <si>
+    <t>239784.0</t>
+  </si>
+  <si>
+    <t>2026-06-06T12:41:45.8254272+05:30</t>
+  </si>
+  <si>
+    <t>12:41:45.825</t>
+  </si>
+  <si>
+    <t>1780692604499</t>
+  </si>
+  <si>
+    <t>02:20:04</t>
+  </si>
+  <si>
+    <t>72MYabHy</t>
+  </si>
+  <si>
+    <t>1780692604755</t>
+  </si>
+  <si>
+    <t>1780692606976</t>
+  </si>
+  <si>
+    <t>02:20:06</t>
+  </si>
+  <si>
+    <t>gGIz8GGT</t>
+  </si>
+  <si>
+    <t>1780692607134</t>
+  </si>
+  <si>
+    <t>02:20:07</t>
+  </si>
+  <si>
+    <t>1780692607886</t>
+  </si>
+  <si>
+    <t>prYYq3pj</t>
+  </si>
+  <si>
+    <t>1780692608129</t>
+  </si>
+  <si>
+    <t>02:20:08</t>
+  </si>
+  <si>
+    <t>2026-06-06T12:41:45+05:30 (2m0s ago)</t>
+  </si>
+  <si>
+    <t>520</t>
+  </si>
+  <si>
+    <t>2026-06-05T23:53:04.3464959+05:30</t>
+  </si>
+  <si>
+    <t>23:53:04.346</t>
+  </si>
+  <si>
+    <t>521</t>
+  </si>
+  <si>
+    <t>2026-06-05T23:58:04.4885433+05:30</t>
+  </si>
+  <si>
+    <t>23:58:04.488</t>
+  </si>
+  <si>
+    <t>522</t>
+  </si>
+  <si>
+    <t>2026-06-06T00:03:04.5336367+05:30</t>
+  </si>
+  <si>
+    <t>00:03:04.533</t>
+  </si>
+  <si>
+    <t>523</t>
+  </si>
+  <si>
+    <t>2026-06-06T00:08:04.3890711+05:30</t>
+  </si>
+  <si>
+    <t>00:08:04.389</t>
+  </si>
+  <si>
+    <t>524</t>
+  </si>
+  <si>
+    <t>2026-06-06T00:13:04.2945198+05:30</t>
+  </si>
+  <si>
+    <t>00:13:04.294</t>
+  </si>
+  <si>
+    <t>525</t>
+  </si>
+  <si>
+    <t>2026-06-06T00:18:04.349719+05:30</t>
+  </si>
+  <si>
+    <t>00:18:04.349</t>
+  </si>
+  <si>
+    <t>526</t>
+  </si>
+  <si>
+    <t>2026-06-06T00:23:03.2036477+05:30</t>
+  </si>
+  <si>
+    <t>00:23:03.203</t>
+  </si>
+  <si>
+    <t>527</t>
+  </si>
+  <si>
+    <t>2026-06-06T00:23:03.20476+05:30</t>
+  </si>
+  <si>
+    <t>00:23:03.204</t>
+  </si>
+  <si>
+    <t>528</t>
+  </si>
+  <si>
+    <t>2026-06-06T00:28:04.4524866+05:30</t>
+  </si>
+  <si>
+    <t>00:28:04.452</t>
+  </si>
+  <si>
+    <t>529</t>
+  </si>
+  <si>
+    <t>2026-06-06T00:33:04.9882474+05:30</t>
+  </si>
+  <si>
+    <t>00:33:04.988</t>
+  </si>
+  <si>
+    <t>530</t>
+  </si>
+  <si>
+    <t>2026-06-06T00:38:04.4578185+05:30</t>
+  </si>
+  <si>
+    <t>00:38:04.457</t>
+  </si>
+  <si>
+    <t>531</t>
+  </si>
+  <si>
+    <t>2026-06-06T00:43:04.4165849+05:30</t>
+  </si>
+  <si>
+    <t>00:43:04.416</t>
+  </si>
+  <si>
+    <t>532</t>
+  </si>
+  <si>
+    <t>2026-06-06T00:48:04.4972065+05:30</t>
+  </si>
+  <si>
+    <t>00:48:04.497</t>
+  </si>
+  <si>
+    <t>533</t>
+  </si>
+  <si>
+    <t>2026-06-06T00:53:04.4158628+05:30</t>
+  </si>
+  <si>
+    <t>00:53:04.415</t>
+  </si>
+  <si>
+    <t>534</t>
+  </si>
+  <si>
+    <t>2026-06-06T00:58:04.746462+05:30</t>
+  </si>
+  <si>
+    <t>00:58:04.746</t>
+  </si>
+  <si>
+    <t>535</t>
+  </si>
+  <si>
+    <t>2026-06-06T01:03:04.2965606+05:30</t>
+  </si>
+  <si>
+    <t>01:03:04.296</t>
+  </si>
+  <si>
+    <t>536</t>
+  </si>
+  <si>
+    <t>2026-06-06T01:08:04.4870498+05:30</t>
+  </si>
+  <si>
+    <t>01:08:04.487</t>
+  </si>
+  <si>
+    <t>537</t>
+  </si>
+  <si>
+    <t>2026-06-06T01:13:04.3971229+05:30</t>
+  </si>
+  <si>
+    <t>01:13:04.397</t>
+  </si>
+  <si>
+    <t>538</t>
+  </si>
+  <si>
+    <t>2026-06-06T01:18:04.3982097+05:30</t>
+  </si>
+  <si>
+    <t>01:18:04.398</t>
+  </si>
+  <si>
+    <t>539</t>
+  </si>
+  <si>
+    <t>2026-06-06T01:23:04.338193+05:30</t>
+  </si>
+  <si>
+    <t>01:23:04.338</t>
+  </si>
+  <si>
+    <t>540</t>
+  </si>
+  <si>
+    <t>2026-06-06T01:28:04.3749159+05:30</t>
+  </si>
+  <si>
+    <t>01:28:04.374</t>
+  </si>
+  <si>
+    <t>541</t>
+  </si>
+  <si>
+    <t>2026-06-06T01:33:04.3612467+05:30</t>
+  </si>
+  <si>
+    <t>01:33:04.361</t>
+  </si>
+  <si>
+    <t>542</t>
+  </si>
+  <si>
+    <t>2026-06-06T01:38:04.5068535+05:30</t>
+  </si>
+  <si>
+    <t>01:38:04.506</t>
+  </si>
+  <si>
+    <t>543</t>
+  </si>
+  <si>
+    <t>2026-06-06T01:43:04.4507225+05:30</t>
+  </si>
+  <si>
+    <t>01:43:04.450</t>
+  </si>
+  <si>
+    <t>544</t>
+  </si>
+  <si>
+    <t>2026-06-06T01:48:04.4562151+05:30</t>
+  </si>
+  <si>
+    <t>01:48:04.456</t>
+  </si>
+  <si>
+    <t>545</t>
+  </si>
+  <si>
+    <t>2026-06-06T01:53:04.4814572+05:30</t>
+  </si>
+  <si>
+    <t>01:53:04.481</t>
+  </si>
+  <si>
+    <t>546</t>
+  </si>
+  <si>
+    <t>2026-06-06T01:58:04.3490827+05:30</t>
+  </si>
+  <si>
+    <t>01:58:04.349</t>
+  </si>
+  <si>
+    <t>547</t>
+  </si>
+  <si>
+    <t>2026-06-06T02:03:04.395145+05:30</t>
+  </si>
+  <si>
+    <t>02:03:04.395</t>
+  </si>
+  <si>
+    <t>548</t>
+  </si>
+  <si>
+    <t>2026-06-06T02:08:04.4247916+05:30</t>
+  </si>
+  <si>
+    <t>02:08:04.424</t>
+  </si>
+  <si>
+    <t>549</t>
+  </si>
+  <si>
+    <t>2026-06-06T02:12:57.4419603+05:30</t>
+  </si>
+  <si>
+    <t>02:12:57.441</t>
+  </si>
+  <si>
+    <t>550</t>
+  </si>
+  <si>
+    <t>2026-06-06T02:17:58.646138+05:30</t>
+  </si>
+  <si>
+    <t>02:17:58.646</t>
+  </si>
+  <si>
+    <t>551</t>
   </si>
   <si>
     <t>2026-06-06T02:19:01.3448451+05:30</t>
@@ -6721,331 +7078,199 @@
     <t>02:19:01.344</t>
   </si>
   <si>
-    <t>1780692604499</t>
-  </si>
-  <si>
-    <t>02:20:04</t>
-  </si>
-  <si>
-    <t>72MYabHy</t>
-  </si>
-  <si>
-    <t>1780692604755</t>
-  </si>
-  <si>
-    <t>1780692606976</t>
-  </si>
-  <si>
-    <t>02:20:06</t>
-  </si>
-  <si>
-    <t>gGIz8GGT</t>
-  </si>
-  <si>
-    <t>1780692607134</t>
-  </si>
-  <si>
-    <t>02:20:07</t>
-  </si>
-  <si>
-    <t>1780692607886</t>
-  </si>
-  <si>
-    <t>prYYq3pj</t>
-  </si>
-  <si>
-    <t>1780692608129</t>
-  </si>
-  <si>
-    <t>02:20:08</t>
-  </si>
-  <si>
-    <t>2026-06-06T02:19:01+05:30 (2m0s ago)</t>
-  </si>
-  <si>
-    <t>520</t>
-  </si>
-  <si>
-    <t>2026-06-05T23:53:04.3464959+05:30</t>
-  </si>
-  <si>
-    <t>23:53:04.346</t>
-  </si>
-  <si>
-    <t>521</t>
-  </si>
-  <si>
-    <t>2026-06-05T23:58:04.4885433+05:30</t>
-  </si>
-  <si>
-    <t>23:58:04.488</t>
-  </si>
-  <si>
-    <t>522</t>
-  </si>
-  <si>
-    <t>2026-06-06T00:03:04.5336367+05:30</t>
-  </si>
-  <si>
-    <t>00:03:04.533</t>
-  </si>
-  <si>
-    <t>523</t>
-  </si>
-  <si>
-    <t>2026-06-06T00:08:04.3890711+05:30</t>
-  </si>
-  <si>
-    <t>00:08:04.389</t>
-  </si>
-  <si>
-    <t>524</t>
-  </si>
-  <si>
-    <t>2026-06-06T00:13:04.2945198+05:30</t>
-  </si>
-  <si>
-    <t>00:13:04.294</t>
-  </si>
-  <si>
-    <t>525</t>
-  </si>
-  <si>
-    <t>2026-06-06T00:18:04.349719+05:30</t>
-  </si>
-  <si>
-    <t>00:18:04.349</t>
-  </si>
-  <si>
-    <t>526</t>
-  </si>
-  <si>
-    <t>2026-06-06T00:23:03.2036477+05:30</t>
-  </si>
-  <si>
-    <t>00:23:03.203</t>
-  </si>
-  <si>
-    <t>527</t>
-  </si>
-  <si>
-    <t>2026-06-06T00:23:03.20476+05:30</t>
-  </si>
-  <si>
-    <t>00:23:03.204</t>
-  </si>
-  <si>
-    <t>528</t>
-  </si>
-  <si>
-    <t>2026-06-06T00:28:04.4524866+05:30</t>
-  </si>
-  <si>
-    <t>00:28:04.452</t>
-  </si>
-  <si>
-    <t>529</t>
-  </si>
-  <si>
-    <t>2026-06-06T00:33:04.9882474+05:30</t>
-  </si>
-  <si>
-    <t>00:33:04.988</t>
-  </si>
-  <si>
-    <t>530</t>
-  </si>
-  <si>
-    <t>2026-06-06T00:38:04.4578185+05:30</t>
-  </si>
-  <si>
-    <t>00:38:04.457</t>
-  </si>
-  <si>
-    <t>531</t>
-  </si>
-  <si>
-    <t>2026-06-06T00:43:04.4165849+05:30</t>
-  </si>
-  <si>
-    <t>00:43:04.416</t>
-  </si>
-  <si>
-    <t>532</t>
-  </si>
-  <si>
-    <t>2026-06-06T00:48:04.4972065+05:30</t>
-  </si>
-  <si>
-    <t>00:48:04.497</t>
-  </si>
-  <si>
-    <t>533</t>
-  </si>
-  <si>
-    <t>2026-06-06T00:53:04.4158628+05:30</t>
-  </si>
-  <si>
-    <t>00:53:04.415</t>
-  </si>
-  <si>
-    <t>534</t>
-  </si>
-  <si>
-    <t>2026-06-06T00:58:04.746462+05:30</t>
-  </si>
-  <si>
-    <t>00:58:04.746</t>
-  </si>
-  <si>
-    <t>535</t>
-  </si>
-  <si>
-    <t>2026-06-06T01:03:04.2965606+05:30</t>
-  </si>
-  <si>
-    <t>01:03:04.296</t>
-  </si>
-  <si>
-    <t>536</t>
-  </si>
-  <si>
-    <t>2026-06-06T01:08:04.4870498+05:30</t>
-  </si>
-  <si>
-    <t>01:08:04.487</t>
-  </si>
-  <si>
-    <t>537</t>
-  </si>
-  <si>
-    <t>2026-06-06T01:13:04.3971229+05:30</t>
-  </si>
-  <si>
-    <t>01:13:04.397</t>
-  </si>
-  <si>
-    <t>538</t>
-  </si>
-  <si>
-    <t>2026-06-06T01:18:04.3982097+05:30</t>
-  </si>
-  <si>
-    <t>01:18:04.398</t>
-  </si>
-  <si>
-    <t>539</t>
-  </si>
-  <si>
-    <t>2026-06-06T01:23:04.338193+05:30</t>
-  </si>
-  <si>
-    <t>01:23:04.338</t>
-  </si>
-  <si>
-    <t>540</t>
-  </si>
-  <si>
-    <t>2026-06-06T01:28:04.3749159+05:30</t>
-  </si>
-  <si>
-    <t>01:28:04.374</t>
-  </si>
-  <si>
-    <t>541</t>
-  </si>
-  <si>
-    <t>2026-06-06T01:33:04.3612467+05:30</t>
-  </si>
-  <si>
-    <t>01:33:04.361</t>
-  </si>
-  <si>
-    <t>542</t>
-  </si>
-  <si>
-    <t>2026-06-06T01:38:04.5068535+05:30</t>
-  </si>
-  <si>
-    <t>01:38:04.506</t>
-  </si>
-  <si>
-    <t>543</t>
-  </si>
-  <si>
-    <t>2026-06-06T01:43:04.4507225+05:30</t>
-  </si>
-  <si>
-    <t>01:43:04.450</t>
-  </si>
-  <si>
-    <t>544</t>
-  </si>
-  <si>
-    <t>2026-06-06T01:48:04.4562151+05:30</t>
-  </si>
-  <si>
-    <t>01:48:04.456</t>
-  </si>
-  <si>
-    <t>545</t>
-  </si>
-  <si>
-    <t>2026-06-06T01:53:04.4814572+05:30</t>
-  </si>
-  <si>
-    <t>01:53:04.481</t>
-  </si>
-  <si>
-    <t>546</t>
-  </si>
-  <si>
-    <t>2026-06-06T01:58:04.3490827+05:30</t>
-  </si>
-  <si>
-    <t>01:58:04.349</t>
-  </si>
-  <si>
-    <t>547</t>
-  </si>
-  <si>
-    <t>2026-06-06T02:03:04.395145+05:30</t>
-  </si>
-  <si>
-    <t>02:03:04.395</t>
-  </si>
-  <si>
-    <t>548</t>
-  </si>
-  <si>
-    <t>2026-06-06T02:08:04.4247916+05:30</t>
-  </si>
-  <si>
-    <t>02:08:04.424</t>
-  </si>
-  <si>
-    <t>549</t>
-  </si>
-  <si>
-    <t>2026-06-06T02:12:57.4419603+05:30</t>
-  </si>
-  <si>
-    <t>02:12:57.441</t>
-  </si>
-  <si>
-    <t>550</t>
-  </si>
-  <si>
-    <t>2026-06-06T02:17:58.646138+05:30</t>
-  </si>
-  <si>
-    <t>02:17:58.646</t>
-  </si>
-  <si>
-    <t>551</t>
-  </si>
-  <si>
-    <t>2026-06-06T02:21:01+05:30</t>
+    <t>552</t>
+  </si>
+  <si>
+    <t>2026-06-06T02:24:02.6039292+05:30</t>
+  </si>
+  <si>
+    <t>02:24:02.603</t>
+  </si>
+  <si>
+    <t>553</t>
+  </si>
+  <si>
+    <t>2026-06-06T02:29:02.5972012+05:30</t>
+  </si>
+  <si>
+    <t>02:29:02.597</t>
+  </si>
+  <si>
+    <t>554</t>
+  </si>
+  <si>
+    <t>2026-06-06T02:34:02.754349+05:30</t>
+  </si>
+  <si>
+    <t>02:34:02.754</t>
+  </si>
+  <si>
+    <t>555</t>
+  </si>
+  <si>
+    <t>2026-06-06T02:39:02.6088993+05:30</t>
+  </si>
+  <si>
+    <t>02:39:02.608</t>
+  </si>
+  <si>
+    <t>556</t>
+  </si>
+  <si>
+    <t>2026-06-06T02:44:02.6738715+05:30</t>
+  </si>
+  <si>
+    <t>02:44:02.673</t>
+  </si>
+  <si>
+    <t>557</t>
+  </si>
+  <si>
+    <t>2026-06-06T02:49:02.6003314+05:30</t>
+  </si>
+  <si>
+    <t>02:49:02.600</t>
+  </si>
+  <si>
+    <t>558</t>
+  </si>
+  <si>
+    <t>2026-06-06T02:54:02.634182+05:30</t>
+  </si>
+  <si>
+    <t>02:54:02.634</t>
+  </si>
+  <si>
+    <t>559</t>
+  </si>
+  <si>
+    <t>2026-06-06T02:59:02.5326307+05:30</t>
+  </si>
+  <si>
+    <t>02:59:02.532</t>
+  </si>
+  <si>
+    <t>560</t>
+  </si>
+  <si>
+    <t>2026-06-06T03:04:02.4988555+05:30</t>
+  </si>
+  <si>
+    <t>03:04:02.498</t>
+  </si>
+  <si>
+    <t>561</t>
+  </si>
+  <si>
+    <t>2026-06-06T03:09:02.5174213+05:30</t>
+  </si>
+  <si>
+    <t>03:09:02.517</t>
+  </si>
+  <si>
+    <t>562</t>
+  </si>
+  <si>
+    <t>2026-06-06T03:14:03.0156796+05:30</t>
+  </si>
+  <si>
+    <t>03:14:03.015</t>
+  </si>
+  <si>
+    <t>563</t>
+  </si>
+  <si>
+    <t>2026-06-06T03:19:02.6230539+05:30</t>
+  </si>
+  <si>
+    <t>03:19:02.623</t>
+  </si>
+  <si>
+    <t>564</t>
+  </si>
+  <si>
+    <t>2026-06-06T03:24:02.5271236+05:30</t>
+  </si>
+  <si>
+    <t>03:24:02.527</t>
+  </si>
+  <si>
+    <t>565</t>
+  </si>
+  <si>
+    <t>2026-06-06T03:29:02.5720525+05:30</t>
+  </si>
+  <si>
+    <t>03:29:02.572</t>
+  </si>
+  <si>
+    <t>566</t>
+  </si>
+  <si>
+    <t>2026-06-06T03:34:02.5814869+05:30</t>
+  </si>
+  <si>
+    <t>03:34:02.581</t>
+  </si>
+  <si>
+    <t>567</t>
+  </si>
+  <si>
+    <t>2026-06-06T03:39:02.5788422+05:30</t>
+  </si>
+  <si>
+    <t>03:39:02.578</t>
+  </si>
+  <si>
+    <t>568</t>
+  </si>
+  <si>
+    <t>2026-06-06T03:44:02.633002+05:30</t>
+  </si>
+  <si>
+    <t>03:44:02.633</t>
+  </si>
+  <si>
+    <t>569</t>
+  </si>
+  <si>
+    <t>2026-06-06T03:49:02.566586+05:30</t>
+  </si>
+  <si>
+    <t>03:49:02.566</t>
+  </si>
+  <si>
+    <t>570</t>
+  </si>
+  <si>
+    <t>2026-06-06T03:54:02.8834141+05:30</t>
+  </si>
+  <si>
+    <t>03:54:02.883</t>
+  </si>
+  <si>
+    <t>571</t>
+  </si>
+  <si>
+    <t>2026-06-06T12:37:31.4976556+05:30</t>
+  </si>
+  <si>
+    <t>12:37:31.497</t>
+  </si>
+  <si>
+    <t>572</t>
+  </si>
+  <si>
+    <t>2026-06-06T12:40:03.0204921+05:30</t>
+  </si>
+  <si>
+    <t>12:40:03.020</t>
+  </si>
+  <si>
+    <t>573</t>
+  </si>
+  <si>
+    <t>2026-06-06T12:43:46+05:30</t>
   </si>
 </sst>
 </file>
@@ -8383,10 +8608,10 @@
         <v>30</v>
       </c>
       <c r="D18" t="s">
-        <v>1182</v>
+        <v>2224</v>
       </c>
       <c r="E18" t="s">
-        <v>32</v>
+        <v>2225</v>
       </c>
       <c r="F18" t="s">
         <v>33</v>
@@ -8395,7 +8620,7 @@
         <v>34</v>
       </c>
       <c r="H18" t="s">
-        <v>2224</v>
+        <v>2226</v>
       </c>
       <c r="I18" t="s">
         <v>36</v>
@@ -8422,22 +8647,22 @@
         <v>1184</v>
       </c>
       <c r="Q18" t="s">
-        <v>2225</v>
+        <v>2227</v>
       </c>
       <c r="R18" t="s">
         <v>1186</v>
       </c>
       <c r="S18" t="s">
-        <v>2225</v>
+        <v>2227</v>
       </c>
       <c r="T18" t="s">
-        <v>2226</v>
+        <v>2228</v>
       </c>
       <c r="U18" t="s">
         <v>2223</v>
       </c>
       <c r="V18" t="s">
-        <v>2227</v>
+        <v>2229</v>
       </c>
     </row>
     <row r="19">
@@ -8451,10 +8676,10 @@
         <v>30</v>
       </c>
       <c r="D19" t="s">
-        <v>1182</v>
+        <v>2224</v>
       </c>
       <c r="E19" t="s">
-        <v>32</v>
+        <v>2225</v>
       </c>
       <c r="F19" t="s">
         <v>33</v>
@@ -8463,7 +8688,7 @@
         <v>34</v>
       </c>
       <c r="H19" t="s">
-        <v>2224</v>
+        <v>2226</v>
       </c>
       <c r="I19" t="s">
         <v>45</v>
@@ -8475,19 +8700,19 @@
         <v>241</v>
       </c>
       <c r="L19" t="s">
-        <v>2228</v>
+        <v>2230</v>
       </c>
       <c r="M19" t="s">
-        <v>2229</v>
+        <v>2231</v>
       </c>
       <c r="N19" t="s">
-        <v>2230</v>
+        <v>2232</v>
       </c>
       <c r="O19" t="s">
         <v>245</v>
       </c>
       <c r="P19" t="s">
-        <v>220</v>
+        <v>223</v>
       </c>
       <c r="Q19" t="s">
         <v>46</v>
@@ -8496,16 +8721,16 @@
         <v>1186</v>
       </c>
       <c r="S19" t="s">
-        <v>2225</v>
+        <v>2227</v>
       </c>
       <c r="T19" t="s">
-        <v>2231</v>
+        <v>2233</v>
       </c>
       <c r="U19" t="s">
         <v>2223</v>
       </c>
       <c r="V19" t="s">
-        <v>2227</v>
+        <v>2229</v>
       </c>
     </row>
     <row r="20">
@@ -8513,52 +8738,67 @@
         <v>2223</v>
       </c>
       <c r="B20" t="s">
-        <v>49</v>
+        <v>2234</v>
       </c>
       <c r="C20" t="s">
-        <v>50</v>
+        <v>2235</v>
       </c>
       <c r="D20" t="s">
-        <v>50</v>
+        <v>2236</v>
       </c>
       <c r="E20" t="s">
-        <v>50</v>
+        <v>2237</v>
       </c>
       <c r="F20" t="s">
-        <v>50</v>
+        <v>33</v>
       </c>
       <c r="G20" t="s">
-        <v>50</v>
+        <v>34</v>
       </c>
       <c r="H20" t="s">
-        <v>50</v>
+        <v>1183</v>
       </c>
       <c r="I20" t="s">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="J20" t="s">
-        <v>50</v>
+        <v>2238</v>
       </c>
       <c r="K20" t="s">
-        <v>50</v>
+        <v>241</v>
       </c>
       <c r="L20" t="s">
-        <v>50</v>
+        <v>2239</v>
       </c>
       <c r="M20" t="s">
-        <v>50</v>
+        <v>2240</v>
       </c>
       <c r="N20" t="s">
-        <v>50</v>
+        <v>470</v>
       </c>
       <c r="O20" t="s">
-        <v>50</v>
+        <v>245</v>
       </c>
       <c r="P20" t="s">
-        <v>50</v>
+        <v>627</v>
       </c>
       <c r="Q20" t="s">
-        <v>50</v>
+        <v>46</v>
+      </c>
+      <c r="R20" t="s">
+        <v>46</v>
+      </c>
+      <c r="S20" t="s">
+        <v>46</v>
+      </c>
+      <c r="T20" t="s">
+        <v>46</v>
+      </c>
+      <c r="U20" t="s">
+        <v>2223</v>
+      </c>
+      <c r="V20" t="s">
+        <v>2229</v>
       </c>
     </row>
     <row r="21">
@@ -8566,51 +8806,104 @@
         <v>2223</v>
       </c>
       <c r="B21" t="s">
+        <v>49</v>
+      </c>
+      <c r="C21" t="s">
+        <v>50</v>
+      </c>
+      <c r="D21" t="s">
+        <v>50</v>
+      </c>
+      <c r="E21" t="s">
+        <v>50</v>
+      </c>
+      <c r="F21" t="s">
+        <v>50</v>
+      </c>
+      <c r="G21" t="s">
+        <v>50</v>
+      </c>
+      <c r="H21" t="s">
+        <v>50</v>
+      </c>
+      <c r="I21" t="s">
+        <v>50</v>
+      </c>
+      <c r="J21" t="s">
+        <v>50</v>
+      </c>
+      <c r="K21" t="s">
+        <v>50</v>
+      </c>
+      <c r="L21" t="s">
+        <v>50</v>
+      </c>
+      <c r="M21" t="s">
+        <v>50</v>
+      </c>
+      <c r="N21" t="s">
+        <v>50</v>
+      </c>
+      <c r="O21" t="s">
+        <v>50</v>
+      </c>
+      <c r="P21" t="s">
+        <v>50</v>
+      </c>
+      <c r="Q21" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="s">
+        <v>2223</v>
+      </c>
+      <c r="B22" t="s">
         <v>51</v>
       </c>
-      <c r="C21" t="s">
-        <v>2232</v>
-      </c>
-      <c r="D21" t="s">
-        <v>2223</v>
-      </c>
-      <c r="E21" t="s">
-        <v>2233</v>
-      </c>
-      <c r="F21" t="s">
-        <v>54</v>
-      </c>
-      <c r="G21" t="s">
-        <v>55</v>
-      </c>
-      <c r="H21" t="s">
-        <v>29</v>
-      </c>
-      <c r="I21" t="s">
-        <v>30</v>
-      </c>
-      <c r="J21" t="s">
-        <v>29</v>
-      </c>
-      <c r="K21" t="s">
-        <v>39</v>
-      </c>
-      <c r="L21" t="s">
-        <v>54</v>
-      </c>
-      <c r="M21" t="s">
-        <v>50</v>
-      </c>
-      <c r="N21" t="s">
-        <v>50</v>
-      </c>
-      <c r="O21" t="s">
-        <v>50</v>
-      </c>
-      <c r="P21" t="s">
-        <v>50</v>
-      </c>
-      <c r="Q21" t="s">
+      <c r="C22" t="s">
+        <v>2241</v>
+      </c>
+      <c r="D22" t="s">
+        <v>2223</v>
+      </c>
+      <c r="E22" t="s">
+        <v>2242</v>
+      </c>
+      <c r="F22" t="s">
+        <v>54</v>
+      </c>
+      <c r="G22" t="s">
+        <v>55</v>
+      </c>
+      <c r="H22" t="s">
+        <v>29</v>
+      </c>
+      <c r="I22" t="s">
+        <v>30</v>
+      </c>
+      <c r="J22" t="s">
+        <v>29</v>
+      </c>
+      <c r="K22" t="s">
+        <v>39</v>
+      </c>
+      <c r="L22" t="s">
+        <v>54</v>
+      </c>
+      <c r="M22" t="s">
+        <v>50</v>
+      </c>
+      <c r="N22" t="s">
+        <v>50</v>
+      </c>
+      <c r="O22" t="s">
+        <v>50</v>
+      </c>
+      <c r="P22" t="s">
+        <v>50</v>
+      </c>
+      <c r="Q22" t="s">
         <v>50</v>
       </c>
     </row>
@@ -26281,10 +26574,10 @@
         <v>2223</v>
       </c>
       <c r="B680" t="s">
-        <v>2234</v>
+        <v>2243</v>
       </c>
       <c r="C680" t="s">
-        <v>2235</v>
+        <v>2244</v>
       </c>
       <c r="D680" t="s">
         <v>2223</v>
@@ -26299,7 +26592,7 @@
         <v>59</v>
       </c>
       <c r="H680" t="s">
-        <v>2236</v>
+        <v>2245</v>
       </c>
     </row>
     <row r="681">
@@ -26307,10 +26600,10 @@
         <v>2223</v>
       </c>
       <c r="B681" t="s">
-        <v>2237</v>
+        <v>2246</v>
       </c>
       <c r="C681" t="s">
-        <v>2235</v>
+        <v>2244</v>
       </c>
       <c r="D681" t="s">
         <v>2223</v>
@@ -26319,7 +26612,7 @@
         <v>62</v>
       </c>
       <c r="F681" t="s">
-        <v>2236</v>
+        <v>2245</v>
       </c>
       <c r="G681" t="s">
         <v>59</v>
@@ -26333,10 +26626,10 @@
         <v>2223</v>
       </c>
       <c r="B682" t="s">
-        <v>2238</v>
+        <v>2247</v>
       </c>
       <c r="C682" t="s">
-        <v>2239</v>
+        <v>2248</v>
       </c>
       <c r="D682" t="s">
         <v>2223</v>
@@ -26351,7 +26644,7 @@
         <v>59</v>
       </c>
       <c r="H682" t="s">
-        <v>2240</v>
+        <v>2249</v>
       </c>
     </row>
     <row r="683">
@@ -26359,10 +26652,10 @@
         <v>2223</v>
       </c>
       <c r="B683" t="s">
-        <v>2241</v>
+        <v>2250</v>
       </c>
       <c r="C683" t="s">
-        <v>2242</v>
+        <v>2251</v>
       </c>
       <c r="D683" t="s">
         <v>2223</v>
@@ -26371,7 +26664,7 @@
         <v>62</v>
       </c>
       <c r="F683" t="s">
-        <v>2240</v>
+        <v>2249</v>
       </c>
       <c r="G683" t="s">
         <v>59</v>
@@ -26385,10 +26678,10 @@
         <v>2223</v>
       </c>
       <c r="B684" t="s">
-        <v>2243</v>
+        <v>2252</v>
       </c>
       <c r="C684" t="s">
-        <v>2242</v>
+        <v>2251</v>
       </c>
       <c r="D684" t="s">
         <v>2223</v>
@@ -26403,7 +26696,7 @@
         <v>59</v>
       </c>
       <c r="H684" t="s">
-        <v>2244</v>
+        <v>2253</v>
       </c>
     </row>
     <row r="685">
@@ -26411,10 +26704,10 @@
         <v>2223</v>
       </c>
       <c r="B685" t="s">
-        <v>2245</v>
+        <v>2254</v>
       </c>
       <c r="C685" t="s">
-        <v>2246</v>
+        <v>2255</v>
       </c>
       <c r="D685" t="s">
         <v>2223</v>
@@ -26423,7 +26716,7 @@
         <v>62</v>
       </c>
       <c r="F685" t="s">
-        <v>2244</v>
+        <v>2253</v>
       </c>
       <c r="G685" t="s">
         <v>59</v>
@@ -68183,7 +68476,7 @@
         <v>162</v>
       </c>
       <c r="C1103" t="s">
-        <v>2247</v>
+        <v>2256</v>
       </c>
       <c r="D1103" t="s">
         <v>50</v>
@@ -68247,7 +68540,7 @@
         <v>166</v>
       </c>
       <c r="C1105" t="s">
-        <v>2247</v>
+        <v>2256</v>
       </c>
       <c r="D1105" t="s">
         <v>50</v>
@@ -88281,16 +88574,16 @@
         <v>2223</v>
       </c>
       <c r="B1630" t="s">
-        <v>2248</v>
+        <v>2257</v>
       </c>
       <c r="C1630" t="s">
-        <v>2249</v>
+        <v>2258</v>
       </c>
       <c r="D1630" t="s">
         <v>1181</v>
       </c>
       <c r="E1630" t="s">
-        <v>2250</v>
+        <v>2259</v>
       </c>
       <c r="F1630" t="s">
         <v>54</v>
@@ -88319,16 +88612,16 @@
         <v>2223</v>
       </c>
       <c r="B1631" t="s">
-        <v>2251</v>
+        <v>2260</v>
       </c>
       <c r="C1631" t="s">
-        <v>2252</v>
+        <v>2261</v>
       </c>
       <c r="D1631" t="s">
         <v>1181</v>
       </c>
       <c r="E1631" t="s">
-        <v>2253</v>
+        <v>2262</v>
       </c>
       <c r="F1631" t="s">
         <v>54</v>
@@ -88357,16 +88650,16 @@
         <v>2223</v>
       </c>
       <c r="B1632" t="s">
-        <v>2254</v>
+        <v>2263</v>
       </c>
       <c r="C1632" t="s">
-        <v>2255</v>
+        <v>2264</v>
       </c>
       <c r="D1632" t="s">
         <v>2223</v>
       </c>
       <c r="E1632" t="s">
-        <v>2256</v>
+        <v>2265</v>
       </c>
       <c r="F1632" t="s">
         <v>54</v>
@@ -88395,16 +88688,16 @@
         <v>2223</v>
       </c>
       <c r="B1633" t="s">
-        <v>2257</v>
+        <v>2266</v>
       </c>
       <c r="C1633" t="s">
-        <v>2258</v>
+        <v>2267</v>
       </c>
       <c r="D1633" t="s">
         <v>2223</v>
       </c>
       <c r="E1633" t="s">
-        <v>2259</v>
+        <v>2268</v>
       </c>
       <c r="F1633" t="s">
         <v>54</v>
@@ -88433,16 +88726,16 @@
         <v>2223</v>
       </c>
       <c r="B1634" t="s">
-        <v>2260</v>
+        <v>2269</v>
       </c>
       <c r="C1634" t="s">
-        <v>2261</v>
+        <v>2270</v>
       </c>
       <c r="D1634" t="s">
         <v>2223</v>
       </c>
       <c r="E1634" t="s">
-        <v>2262</v>
+        <v>2271</v>
       </c>
       <c r="F1634" t="s">
         <v>54</v>
@@ -88471,16 +88764,16 @@
         <v>2223</v>
       </c>
       <c r="B1635" t="s">
-        <v>2263</v>
+        <v>2272</v>
       </c>
       <c r="C1635" t="s">
-        <v>2264</v>
+        <v>2273</v>
       </c>
       <c r="D1635" t="s">
         <v>2223</v>
       </c>
       <c r="E1635" t="s">
-        <v>2265</v>
+        <v>2274</v>
       </c>
       <c r="F1635" t="s">
         <v>54</v>
@@ -88509,16 +88802,16 @@
         <v>2223</v>
       </c>
       <c r="B1636" t="s">
-        <v>2266</v>
+        <v>2275</v>
       </c>
       <c r="C1636" t="s">
-        <v>2267</v>
+        <v>2276</v>
       </c>
       <c r="D1636" t="s">
         <v>2223</v>
       </c>
       <c r="E1636" t="s">
-        <v>2268</v>
+        <v>2277</v>
       </c>
       <c r="F1636" t="s">
         <v>180</v>
@@ -88550,16 +88843,16 @@
         <v>2223</v>
       </c>
       <c r="B1637" t="s">
-        <v>2269</v>
+        <v>2278</v>
       </c>
       <c r="C1637" t="s">
-        <v>2270</v>
+        <v>2279</v>
       </c>
       <c r="D1637" t="s">
         <v>2223</v>
       </c>
       <c r="E1637" t="s">
-        <v>2271</v>
+        <v>2280</v>
       </c>
       <c r="F1637" t="s">
         <v>180</v>
@@ -88591,16 +88884,16 @@
         <v>2223</v>
       </c>
       <c r="B1638" t="s">
-        <v>2272</v>
+        <v>2281</v>
       </c>
       <c r="C1638" t="s">
-        <v>2273</v>
+        <v>2282</v>
       </c>
       <c r="D1638" t="s">
         <v>2223</v>
       </c>
       <c r="E1638" t="s">
-        <v>2274</v>
+        <v>2283</v>
       </c>
       <c r="F1638" t="s">
         <v>54</v>
@@ -88629,16 +88922,16 @@
         <v>2223</v>
       </c>
       <c r="B1639" t="s">
-        <v>2275</v>
+        <v>2284</v>
       </c>
       <c r="C1639" t="s">
-        <v>2276</v>
+        <v>2285</v>
       </c>
       <c r="D1639" t="s">
         <v>2223</v>
       </c>
       <c r="E1639" t="s">
-        <v>2277</v>
+        <v>2286</v>
       </c>
       <c r="F1639" t="s">
         <v>54</v>
@@ -88667,16 +88960,16 @@
         <v>2223</v>
       </c>
       <c r="B1640" t="s">
-        <v>2278</v>
+        <v>2287</v>
       </c>
       <c r="C1640" t="s">
-        <v>2279</v>
+        <v>2288</v>
       </c>
       <c r="D1640" t="s">
         <v>2223</v>
       </c>
       <c r="E1640" t="s">
-        <v>2280</v>
+        <v>2289</v>
       </c>
       <c r="F1640" t="s">
         <v>54</v>
@@ -88705,16 +88998,16 @@
         <v>2223</v>
       </c>
       <c r="B1641" t="s">
-        <v>2281</v>
+        <v>2290</v>
       </c>
       <c r="C1641" t="s">
-        <v>2282</v>
+        <v>2291</v>
       </c>
       <c r="D1641" t="s">
         <v>2223</v>
       </c>
       <c r="E1641" t="s">
-        <v>2283</v>
+        <v>2292</v>
       </c>
       <c r="F1641" t="s">
         <v>54</v>
@@ -88743,16 +89036,16 @@
         <v>2223</v>
       </c>
       <c r="B1642" t="s">
-        <v>2284</v>
+        <v>2293</v>
       </c>
       <c r="C1642" t="s">
-        <v>2285</v>
+        <v>2294</v>
       </c>
       <c r="D1642" t="s">
         <v>2223</v>
       </c>
       <c r="E1642" t="s">
-        <v>2286</v>
+        <v>2295</v>
       </c>
       <c r="F1642" t="s">
         <v>54</v>
@@ -88781,16 +89074,16 @@
         <v>2223</v>
       </c>
       <c r="B1643" t="s">
-        <v>2287</v>
+        <v>2296</v>
       </c>
       <c r="C1643" t="s">
-        <v>2288</v>
+        <v>2297</v>
       </c>
       <c r="D1643" t="s">
         <v>2223</v>
       </c>
       <c r="E1643" t="s">
-        <v>2289</v>
+        <v>2298</v>
       </c>
       <c r="F1643" t="s">
         <v>54</v>
@@ -88819,16 +89112,16 @@
         <v>2223</v>
       </c>
       <c r="B1644" t="s">
-        <v>2290</v>
+        <v>2299</v>
       </c>
       <c r="C1644" t="s">
-        <v>2291</v>
+        <v>2300</v>
       </c>
       <c r="D1644" t="s">
         <v>2223</v>
       </c>
       <c r="E1644" t="s">
-        <v>2292</v>
+        <v>2301</v>
       </c>
       <c r="F1644" t="s">
         <v>54</v>
@@ -88857,16 +89150,16 @@
         <v>2223</v>
       </c>
       <c r="B1645" t="s">
-        <v>2293</v>
+        <v>2302</v>
       </c>
       <c r="C1645" t="s">
-        <v>2294</v>
+        <v>2303</v>
       </c>
       <c r="D1645" t="s">
         <v>2223</v>
       </c>
       <c r="E1645" t="s">
-        <v>2295</v>
+        <v>2304</v>
       </c>
       <c r="F1645" t="s">
         <v>54</v>
@@ -88895,16 +89188,16 @@
         <v>2223</v>
       </c>
       <c r="B1646" t="s">
-        <v>2296</v>
+        <v>2305</v>
       </c>
       <c r="C1646" t="s">
-        <v>2297</v>
+        <v>2306</v>
       </c>
       <c r="D1646" t="s">
         <v>2223</v>
       </c>
       <c r="E1646" t="s">
-        <v>2298</v>
+        <v>2307</v>
       </c>
       <c r="F1646" t="s">
         <v>54</v>
@@ -88933,16 +89226,16 @@
         <v>2223</v>
       </c>
       <c r="B1647" t="s">
-        <v>2299</v>
+        <v>2308</v>
       </c>
       <c r="C1647" t="s">
-        <v>2300</v>
+        <v>2309</v>
       </c>
       <c r="D1647" t="s">
         <v>2223</v>
       </c>
       <c r="E1647" t="s">
-        <v>2301</v>
+        <v>2310</v>
       </c>
       <c r="F1647" t="s">
         <v>54</v>
@@ -88971,16 +89264,16 @@
         <v>2223</v>
       </c>
       <c r="B1648" t="s">
-        <v>2302</v>
+        <v>2311</v>
       </c>
       <c r="C1648" t="s">
-        <v>2303</v>
+        <v>2312</v>
       </c>
       <c r="D1648" t="s">
         <v>2223</v>
       </c>
       <c r="E1648" t="s">
-        <v>2304</v>
+        <v>2313</v>
       </c>
       <c r="F1648" t="s">
         <v>54</v>
@@ -89009,16 +89302,16 @@
         <v>2223</v>
       </c>
       <c r="B1649" t="s">
-        <v>2305</v>
+        <v>2314</v>
       </c>
       <c r="C1649" t="s">
-        <v>2306</v>
+        <v>2315</v>
       </c>
       <c r="D1649" t="s">
         <v>2223</v>
       </c>
       <c r="E1649" t="s">
-        <v>2307</v>
+        <v>2316</v>
       </c>
       <c r="F1649" t="s">
         <v>54</v>
@@ -89047,16 +89340,16 @@
         <v>2223</v>
       </c>
       <c r="B1650" t="s">
-        <v>2308</v>
+        <v>2317</v>
       </c>
       <c r="C1650" t="s">
-        <v>2309</v>
+        <v>2318</v>
       </c>
       <c r="D1650" t="s">
         <v>2223</v>
       </c>
       <c r="E1650" t="s">
-        <v>2310</v>
+        <v>2319</v>
       </c>
       <c r="F1650" t="s">
         <v>54</v>
@@ -89085,16 +89378,16 @@
         <v>2223</v>
       </c>
       <c r="B1651" t="s">
-        <v>2311</v>
+        <v>2320</v>
       </c>
       <c r="C1651" t="s">
-        <v>2312</v>
+        <v>2321</v>
       </c>
       <c r="D1651" t="s">
         <v>2223</v>
       </c>
       <c r="E1651" t="s">
-        <v>2313</v>
+        <v>2322</v>
       </c>
       <c r="F1651" t="s">
         <v>54</v>
@@ -89123,16 +89416,16 @@
         <v>2223</v>
       </c>
       <c r="B1652" t="s">
-        <v>2314</v>
+        <v>2323</v>
       </c>
       <c r="C1652" t="s">
-        <v>2315</v>
+        <v>2324</v>
       </c>
       <c r="D1652" t="s">
         <v>2223</v>
       </c>
       <c r="E1652" t="s">
-        <v>2316</v>
+        <v>2325</v>
       </c>
       <c r="F1652" t="s">
         <v>54</v>
@@ -89161,16 +89454,16 @@
         <v>2223</v>
       </c>
       <c r="B1653" t="s">
-        <v>2317</v>
+        <v>2326</v>
       </c>
       <c r="C1653" t="s">
-        <v>2318</v>
+        <v>2327</v>
       </c>
       <c r="D1653" t="s">
         <v>2223</v>
       </c>
       <c r="E1653" t="s">
-        <v>2319</v>
+        <v>2328</v>
       </c>
       <c r="F1653" t="s">
         <v>54</v>
@@ -89199,16 +89492,16 @@
         <v>2223</v>
       </c>
       <c r="B1654" t="s">
-        <v>2320</v>
+        <v>2329</v>
       </c>
       <c r="C1654" t="s">
-        <v>2321</v>
+        <v>2330</v>
       </c>
       <c r="D1654" t="s">
         <v>2223</v>
       </c>
       <c r="E1654" t="s">
-        <v>2322</v>
+        <v>2331</v>
       </c>
       <c r="F1654" t="s">
         <v>54</v>
@@ -89237,16 +89530,16 @@
         <v>2223</v>
       </c>
       <c r="B1655" t="s">
-        <v>2323</v>
+        <v>2332</v>
       </c>
       <c r="C1655" t="s">
-        <v>2324</v>
+        <v>2333</v>
       </c>
       <c r="D1655" t="s">
         <v>2223</v>
       </c>
       <c r="E1655" t="s">
-        <v>2325</v>
+        <v>2334</v>
       </c>
       <c r="F1655" t="s">
         <v>54</v>
@@ -89275,16 +89568,16 @@
         <v>2223</v>
       </c>
       <c r="B1656" t="s">
-        <v>2326</v>
+        <v>2335</v>
       </c>
       <c r="C1656" t="s">
-        <v>2327</v>
+        <v>2336</v>
       </c>
       <c r="D1656" t="s">
         <v>2223</v>
       </c>
       <c r="E1656" t="s">
-        <v>2328</v>
+        <v>2337</v>
       </c>
       <c r="F1656" t="s">
         <v>54</v>
@@ -89313,16 +89606,16 @@
         <v>2223</v>
       </c>
       <c r="B1657" t="s">
-        <v>2329</v>
+        <v>2338</v>
       </c>
       <c r="C1657" t="s">
-        <v>2330</v>
+        <v>2339</v>
       </c>
       <c r="D1657" t="s">
         <v>2223</v>
       </c>
       <c r="E1657" t="s">
-        <v>2331</v>
+        <v>2340</v>
       </c>
       <c r="F1657" t="s">
         <v>54</v>
@@ -89351,16 +89644,16 @@
         <v>2223</v>
       </c>
       <c r="B1658" t="s">
-        <v>2332</v>
+        <v>2341</v>
       </c>
       <c r="C1658" t="s">
-        <v>2333</v>
+        <v>2342</v>
       </c>
       <c r="D1658" t="s">
         <v>2223</v>
       </c>
       <c r="E1658" t="s">
-        <v>2334</v>
+        <v>2343</v>
       </c>
       <c r="F1658" t="s">
         <v>54</v>
@@ -89389,16 +89682,16 @@
         <v>2223</v>
       </c>
       <c r="B1659" t="s">
-        <v>2335</v>
+        <v>2344</v>
       </c>
       <c r="C1659" t="s">
-        <v>2336</v>
+        <v>2345</v>
       </c>
       <c r="D1659" t="s">
         <v>2223</v>
       </c>
       <c r="E1659" t="s">
-        <v>2337</v>
+        <v>2346</v>
       </c>
       <c r="F1659" t="s">
         <v>54</v>
@@ -89427,16 +89720,16 @@
         <v>2223</v>
       </c>
       <c r="B1660" t="s">
-        <v>2338</v>
+        <v>2347</v>
       </c>
       <c r="C1660" t="s">
-        <v>2339</v>
+        <v>2348</v>
       </c>
       <c r="D1660" t="s">
         <v>2223</v>
       </c>
       <c r="E1660" t="s">
-        <v>2340</v>
+        <v>2349</v>
       </c>
       <c r="F1660" t="s">
         <v>54</v>
@@ -89465,16 +89758,16 @@
         <v>2223</v>
       </c>
       <c r="B1661" t="s">
-        <v>2341</v>
+        <v>2350</v>
       </c>
       <c r="C1661" t="s">
-        <v>2232</v>
+        <v>2351</v>
       </c>
       <c r="D1661" t="s">
         <v>2223</v>
       </c>
       <c r="E1661" t="s">
-        <v>2233</v>
+        <v>2352</v>
       </c>
       <c r="F1661" t="s">
         <v>54</v>
@@ -89503,31 +89796,37 @@
         <v>2223</v>
       </c>
       <c r="B1662" t="s">
-        <v>50</v>
+        <v>2353</v>
       </c>
       <c r="C1662" t="s">
-        <v>50</v>
+        <v>2354</v>
       </c>
       <c r="D1662" t="s">
-        <v>50</v>
+        <v>2223</v>
       </c>
       <c r="E1662" t="s">
-        <v>50</v>
+        <v>2355</v>
       </c>
       <c r="F1662" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="G1662" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="H1662" t="s">
-        <v>50</v>
+        <v>29</v>
       </c>
       <c r="I1662" t="s">
-        <v>50</v>
+        <v>30</v>
       </c>
       <c r="J1662" t="s">
-        <v>50</v>
+        <v>29</v>
+      </c>
+      <c r="K1662" t="s">
+        <v>39</v>
+      </c>
+      <c r="L1662" t="s">
+        <v>54</v>
       </c>
     </row>
     <row r="1663">
@@ -89535,30 +89834,860 @@
         <v>2223</v>
       </c>
       <c r="B1663" t="s">
+        <v>2356</v>
+      </c>
+      <c r="C1663" t="s">
+        <v>2357</v>
+      </c>
+      <c r="D1663" t="s">
+        <v>2223</v>
+      </c>
+      <c r="E1663" t="s">
+        <v>2358</v>
+      </c>
+      <c r="F1663" t="s">
+        <v>54</v>
+      </c>
+      <c r="G1663" t="s">
+        <v>55</v>
+      </c>
+      <c r="H1663" t="s">
+        <v>29</v>
+      </c>
+      <c r="I1663" t="s">
+        <v>30</v>
+      </c>
+      <c r="J1663" t="s">
+        <v>29</v>
+      </c>
+      <c r="K1663" t="s">
+        <v>39</v>
+      </c>
+      <c r="L1663" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="1664">
+      <c r="A1664" t="s">
+        <v>2223</v>
+      </c>
+      <c r="B1664" t="s">
+        <v>2359</v>
+      </c>
+      <c r="C1664" t="s">
+        <v>2360</v>
+      </c>
+      <c r="D1664" t="s">
+        <v>2223</v>
+      </c>
+      <c r="E1664" t="s">
+        <v>2361</v>
+      </c>
+      <c r="F1664" t="s">
+        <v>54</v>
+      </c>
+      <c r="G1664" t="s">
+        <v>55</v>
+      </c>
+      <c r="H1664" t="s">
+        <v>29</v>
+      </c>
+      <c r="I1664" t="s">
+        <v>30</v>
+      </c>
+      <c r="J1664" t="s">
+        <v>29</v>
+      </c>
+      <c r="K1664" t="s">
+        <v>39</v>
+      </c>
+      <c r="L1664" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="1665">
+      <c r="A1665" t="s">
+        <v>2223</v>
+      </c>
+      <c r="B1665" t="s">
+        <v>2362</v>
+      </c>
+      <c r="C1665" t="s">
+        <v>2363</v>
+      </c>
+      <c r="D1665" t="s">
+        <v>2223</v>
+      </c>
+      <c r="E1665" t="s">
+        <v>2364</v>
+      </c>
+      <c r="F1665" t="s">
+        <v>54</v>
+      </c>
+      <c r="G1665" t="s">
+        <v>55</v>
+      </c>
+      <c r="H1665" t="s">
+        <v>29</v>
+      </c>
+      <c r="I1665" t="s">
+        <v>30</v>
+      </c>
+      <c r="J1665" t="s">
+        <v>29</v>
+      </c>
+      <c r="K1665" t="s">
+        <v>39</v>
+      </c>
+      <c r="L1665" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="1666">
+      <c r="A1666" t="s">
+        <v>2223</v>
+      </c>
+      <c r="B1666" t="s">
+        <v>2365</v>
+      </c>
+      <c r="C1666" t="s">
+        <v>2366</v>
+      </c>
+      <c r="D1666" t="s">
+        <v>2223</v>
+      </c>
+      <c r="E1666" t="s">
+        <v>2367</v>
+      </c>
+      <c r="F1666" t="s">
+        <v>54</v>
+      </c>
+      <c r="G1666" t="s">
+        <v>55</v>
+      </c>
+      <c r="H1666" t="s">
+        <v>29</v>
+      </c>
+      <c r="I1666" t="s">
+        <v>30</v>
+      </c>
+      <c r="J1666" t="s">
+        <v>29</v>
+      </c>
+      <c r="K1666" t="s">
+        <v>39</v>
+      </c>
+      <c r="L1666" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="1667">
+      <c r="A1667" t="s">
+        <v>2223</v>
+      </c>
+      <c r="B1667" t="s">
+        <v>2368</v>
+      </c>
+      <c r="C1667" t="s">
+        <v>2369</v>
+      </c>
+      <c r="D1667" t="s">
+        <v>2223</v>
+      </c>
+      <c r="E1667" t="s">
+        <v>2370</v>
+      </c>
+      <c r="F1667" t="s">
+        <v>54</v>
+      </c>
+      <c r="G1667" t="s">
+        <v>55</v>
+      </c>
+      <c r="H1667" t="s">
+        <v>29</v>
+      </c>
+      <c r="I1667" t="s">
+        <v>30</v>
+      </c>
+      <c r="J1667" t="s">
+        <v>29</v>
+      </c>
+      <c r="K1667" t="s">
+        <v>39</v>
+      </c>
+      <c r="L1667" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="1668">
+      <c r="A1668" t="s">
+        <v>2223</v>
+      </c>
+      <c r="B1668" t="s">
+        <v>2371</v>
+      </c>
+      <c r="C1668" t="s">
+        <v>2372</v>
+      </c>
+      <c r="D1668" t="s">
+        <v>2223</v>
+      </c>
+      <c r="E1668" t="s">
+        <v>2373</v>
+      </c>
+      <c r="F1668" t="s">
+        <v>54</v>
+      </c>
+      <c r="G1668" t="s">
+        <v>55</v>
+      </c>
+      <c r="H1668" t="s">
+        <v>29</v>
+      </c>
+      <c r="I1668" t="s">
+        <v>30</v>
+      </c>
+      <c r="J1668" t="s">
+        <v>29</v>
+      </c>
+      <c r="K1668" t="s">
+        <v>39</v>
+      </c>
+      <c r="L1668" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="1669">
+      <c r="A1669" t="s">
+        <v>2223</v>
+      </c>
+      <c r="B1669" t="s">
+        <v>2374</v>
+      </c>
+      <c r="C1669" t="s">
+        <v>2375</v>
+      </c>
+      <c r="D1669" t="s">
+        <v>2223</v>
+      </c>
+      <c r="E1669" t="s">
+        <v>2376</v>
+      </c>
+      <c r="F1669" t="s">
+        <v>54</v>
+      </c>
+      <c r="G1669" t="s">
+        <v>55</v>
+      </c>
+      <c r="H1669" t="s">
+        <v>29</v>
+      </c>
+      <c r="I1669" t="s">
+        <v>30</v>
+      </c>
+      <c r="J1669" t="s">
+        <v>29</v>
+      </c>
+      <c r="K1669" t="s">
+        <v>39</v>
+      </c>
+      <c r="L1669" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="1670">
+      <c r="A1670" t="s">
+        <v>2223</v>
+      </c>
+      <c r="B1670" t="s">
+        <v>2377</v>
+      </c>
+      <c r="C1670" t="s">
+        <v>2378</v>
+      </c>
+      <c r="D1670" t="s">
+        <v>2223</v>
+      </c>
+      <c r="E1670" t="s">
+        <v>2379</v>
+      </c>
+      <c r="F1670" t="s">
+        <v>54</v>
+      </c>
+      <c r="G1670" t="s">
+        <v>55</v>
+      </c>
+      <c r="H1670" t="s">
+        <v>29</v>
+      </c>
+      <c r="I1670" t="s">
+        <v>30</v>
+      </c>
+      <c r="J1670" t="s">
+        <v>29</v>
+      </c>
+      <c r="K1670" t="s">
+        <v>39</v>
+      </c>
+      <c r="L1670" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="1671">
+      <c r="A1671" t="s">
+        <v>2223</v>
+      </c>
+      <c r="B1671" t="s">
+        <v>2380</v>
+      </c>
+      <c r="C1671" t="s">
+        <v>2381</v>
+      </c>
+      <c r="D1671" t="s">
+        <v>2223</v>
+      </c>
+      <c r="E1671" t="s">
+        <v>2382</v>
+      </c>
+      <c r="F1671" t="s">
+        <v>54</v>
+      </c>
+      <c r="G1671" t="s">
+        <v>55</v>
+      </c>
+      <c r="H1671" t="s">
+        <v>29</v>
+      </c>
+      <c r="I1671" t="s">
+        <v>30</v>
+      </c>
+      <c r="J1671" t="s">
+        <v>29</v>
+      </c>
+      <c r="K1671" t="s">
+        <v>39</v>
+      </c>
+      <c r="L1671" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="1672">
+      <c r="A1672" t="s">
+        <v>2223</v>
+      </c>
+      <c r="B1672" t="s">
+        <v>2383</v>
+      </c>
+      <c r="C1672" t="s">
+        <v>2384</v>
+      </c>
+      <c r="D1672" t="s">
+        <v>2223</v>
+      </c>
+      <c r="E1672" t="s">
+        <v>2385</v>
+      </c>
+      <c r="F1672" t="s">
+        <v>54</v>
+      </c>
+      <c r="G1672" t="s">
+        <v>55</v>
+      </c>
+      <c r="H1672" t="s">
+        <v>29</v>
+      </c>
+      <c r="I1672" t="s">
+        <v>30</v>
+      </c>
+      <c r="J1672" t="s">
+        <v>29</v>
+      </c>
+      <c r="K1672" t="s">
+        <v>39</v>
+      </c>
+      <c r="L1672" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="1673">
+      <c r="A1673" t="s">
+        <v>2223</v>
+      </c>
+      <c r="B1673" t="s">
+        <v>2386</v>
+      </c>
+      <c r="C1673" t="s">
+        <v>2387</v>
+      </c>
+      <c r="D1673" t="s">
+        <v>2223</v>
+      </c>
+      <c r="E1673" t="s">
+        <v>2388</v>
+      </c>
+      <c r="F1673" t="s">
+        <v>54</v>
+      </c>
+      <c r="G1673" t="s">
+        <v>55</v>
+      </c>
+      <c r="H1673" t="s">
+        <v>29</v>
+      </c>
+      <c r="I1673" t="s">
+        <v>30</v>
+      </c>
+      <c r="J1673" t="s">
+        <v>29</v>
+      </c>
+      <c r="K1673" t="s">
+        <v>39</v>
+      </c>
+      <c r="L1673" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="1674">
+      <c r="A1674" t="s">
+        <v>2223</v>
+      </c>
+      <c r="B1674" t="s">
+        <v>2389</v>
+      </c>
+      <c r="C1674" t="s">
+        <v>2390</v>
+      </c>
+      <c r="D1674" t="s">
+        <v>2223</v>
+      </c>
+      <c r="E1674" t="s">
+        <v>2391</v>
+      </c>
+      <c r="F1674" t="s">
+        <v>54</v>
+      </c>
+      <c r="G1674" t="s">
+        <v>55</v>
+      </c>
+      <c r="H1674" t="s">
+        <v>29</v>
+      </c>
+      <c r="I1674" t="s">
+        <v>30</v>
+      </c>
+      <c r="J1674" t="s">
+        <v>29</v>
+      </c>
+      <c r="K1674" t="s">
+        <v>39</v>
+      </c>
+      <c r="L1674" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="1675">
+      <c r="A1675" t="s">
+        <v>2223</v>
+      </c>
+      <c r="B1675" t="s">
+        <v>2392</v>
+      </c>
+      <c r="C1675" t="s">
+        <v>2393</v>
+      </c>
+      <c r="D1675" t="s">
+        <v>2223</v>
+      </c>
+      <c r="E1675" t="s">
+        <v>2394</v>
+      </c>
+      <c r="F1675" t="s">
+        <v>54</v>
+      </c>
+      <c r="G1675" t="s">
+        <v>55</v>
+      </c>
+      <c r="H1675" t="s">
+        <v>29</v>
+      </c>
+      <c r="I1675" t="s">
+        <v>30</v>
+      </c>
+      <c r="J1675" t="s">
+        <v>29</v>
+      </c>
+      <c r="K1675" t="s">
+        <v>39</v>
+      </c>
+      <c r="L1675" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="1676">
+      <c r="A1676" t="s">
+        <v>2223</v>
+      </c>
+      <c r="B1676" t="s">
+        <v>2395</v>
+      </c>
+      <c r="C1676" t="s">
+        <v>2396</v>
+      </c>
+      <c r="D1676" t="s">
+        <v>2223</v>
+      </c>
+      <c r="E1676" t="s">
+        <v>2397</v>
+      </c>
+      <c r="F1676" t="s">
+        <v>54</v>
+      </c>
+      <c r="G1676" t="s">
+        <v>55</v>
+      </c>
+      <c r="H1676" t="s">
+        <v>29</v>
+      </c>
+      <c r="I1676" t="s">
+        <v>30</v>
+      </c>
+      <c r="J1676" t="s">
+        <v>29</v>
+      </c>
+      <c r="K1676" t="s">
+        <v>39</v>
+      </c>
+      <c r="L1676" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="1677">
+      <c r="A1677" t="s">
+        <v>2223</v>
+      </c>
+      <c r="B1677" t="s">
+        <v>2398</v>
+      </c>
+      <c r="C1677" t="s">
+        <v>2399</v>
+      </c>
+      <c r="D1677" t="s">
+        <v>2223</v>
+      </c>
+      <c r="E1677" t="s">
+        <v>2400</v>
+      </c>
+      <c r="F1677" t="s">
+        <v>54</v>
+      </c>
+      <c r="G1677" t="s">
+        <v>55</v>
+      </c>
+      <c r="H1677" t="s">
+        <v>29</v>
+      </c>
+      <c r="I1677" t="s">
+        <v>30</v>
+      </c>
+      <c r="J1677" t="s">
+        <v>29</v>
+      </c>
+      <c r="K1677" t="s">
+        <v>39</v>
+      </c>
+      <c r="L1677" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="1678">
+      <c r="A1678" t="s">
+        <v>2223</v>
+      </c>
+      <c r="B1678" t="s">
+        <v>2401</v>
+      </c>
+      <c r="C1678" t="s">
+        <v>2402</v>
+      </c>
+      <c r="D1678" t="s">
+        <v>2223</v>
+      </c>
+      <c r="E1678" t="s">
+        <v>2403</v>
+      </c>
+      <c r="F1678" t="s">
+        <v>54</v>
+      </c>
+      <c r="G1678" t="s">
+        <v>55</v>
+      </c>
+      <c r="H1678" t="s">
+        <v>29</v>
+      </c>
+      <c r="I1678" t="s">
+        <v>30</v>
+      </c>
+      <c r="J1678" t="s">
+        <v>29</v>
+      </c>
+      <c r="K1678" t="s">
+        <v>39</v>
+      </c>
+      <c r="L1678" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="1679">
+      <c r="A1679" t="s">
+        <v>2223</v>
+      </c>
+      <c r="B1679" t="s">
+        <v>2404</v>
+      </c>
+      <c r="C1679" t="s">
+        <v>2405</v>
+      </c>
+      <c r="D1679" t="s">
+        <v>2223</v>
+      </c>
+      <c r="E1679" t="s">
+        <v>2406</v>
+      </c>
+      <c r="F1679" t="s">
+        <v>54</v>
+      </c>
+      <c r="G1679" t="s">
+        <v>55</v>
+      </c>
+      <c r="H1679" t="s">
+        <v>29</v>
+      </c>
+      <c r="I1679" t="s">
+        <v>30</v>
+      </c>
+      <c r="J1679" t="s">
+        <v>29</v>
+      </c>
+      <c r="K1679" t="s">
+        <v>39</v>
+      </c>
+      <c r="L1679" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="1680">
+      <c r="A1680" t="s">
+        <v>2223</v>
+      </c>
+      <c r="B1680" t="s">
+        <v>2407</v>
+      </c>
+      <c r="C1680" t="s">
+        <v>2408</v>
+      </c>
+      <c r="D1680" t="s">
+        <v>2223</v>
+      </c>
+      <c r="E1680" t="s">
+        <v>2409</v>
+      </c>
+      <c r="F1680" t="s">
+        <v>54</v>
+      </c>
+      <c r="G1680" t="s">
+        <v>55</v>
+      </c>
+      <c r="H1680" t="s">
+        <v>29</v>
+      </c>
+      <c r="I1680" t="s">
+        <v>30</v>
+      </c>
+      <c r="J1680" t="s">
+        <v>29</v>
+      </c>
+      <c r="K1680" t="s">
+        <v>39</v>
+      </c>
+      <c r="L1680" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="1681">
+      <c r="A1681" t="s">
+        <v>2223</v>
+      </c>
+      <c r="B1681" t="s">
+        <v>2410</v>
+      </c>
+      <c r="C1681" t="s">
+        <v>2411</v>
+      </c>
+      <c r="D1681" t="s">
+        <v>2223</v>
+      </c>
+      <c r="E1681" t="s">
+        <v>2412</v>
+      </c>
+      <c r="F1681" t="s">
+        <v>54</v>
+      </c>
+      <c r="G1681" t="s">
+        <v>55</v>
+      </c>
+      <c r="H1681" t="s">
+        <v>29</v>
+      </c>
+      <c r="I1681" t="s">
+        <v>30</v>
+      </c>
+      <c r="J1681" t="s">
+        <v>29</v>
+      </c>
+      <c r="K1681" t="s">
+        <v>39</v>
+      </c>
+      <c r="L1681" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="1682">
+      <c r="A1682" t="s">
+        <v>2223</v>
+      </c>
+      <c r="B1682" t="s">
+        <v>2413</v>
+      </c>
+      <c r="C1682" t="s">
+        <v>2414</v>
+      </c>
+      <c r="D1682" t="s">
+        <v>2223</v>
+      </c>
+      <c r="E1682" t="s">
+        <v>2415</v>
+      </c>
+      <c r="F1682" t="s">
+        <v>54</v>
+      </c>
+      <c r="G1682" t="s">
+        <v>55</v>
+      </c>
+      <c r="H1682" t="s">
+        <v>29</v>
+      </c>
+      <c r="I1682" t="s">
+        <v>30</v>
+      </c>
+      <c r="J1682" t="s">
+        <v>29</v>
+      </c>
+      <c r="K1682" t="s">
+        <v>39</v>
+      </c>
+      <c r="L1682" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="1683">
+      <c r="A1683" t="s">
+        <v>2223</v>
+      </c>
+      <c r="B1683" t="s">
+        <v>2416</v>
+      </c>
+      <c r="C1683" t="s">
+        <v>2241</v>
+      </c>
+      <c r="D1683" t="s">
+        <v>2223</v>
+      </c>
+      <c r="E1683" t="s">
+        <v>2242</v>
+      </c>
+      <c r="F1683" t="s">
+        <v>54</v>
+      </c>
+      <c r="G1683" t="s">
+        <v>55</v>
+      </c>
+      <c r="H1683" t="s">
+        <v>29</v>
+      </c>
+      <c r="I1683" t="s">
+        <v>30</v>
+      </c>
+      <c r="J1683" t="s">
+        <v>29</v>
+      </c>
+      <c r="K1683" t="s">
+        <v>39</v>
+      </c>
+      <c r="L1683" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="1684">
+      <c r="A1684" t="s">
+        <v>2223</v>
+      </c>
+      <c r="B1684" t="s">
+        <v>50</v>
+      </c>
+      <c r="C1684" t="s">
+        <v>50</v>
+      </c>
+      <c r="D1684" t="s">
+        <v>50</v>
+      </c>
+      <c r="E1684" t="s">
+        <v>50</v>
+      </c>
+      <c r="F1684" t="s">
+        <v>50</v>
+      </c>
+      <c r="G1684" t="s">
+        <v>50</v>
+      </c>
+      <c r="H1684" t="s">
+        <v>50</v>
+      </c>
+      <c r="I1684" t="s">
+        <v>50</v>
+      </c>
+      <c r="J1684" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="1685">
+      <c r="A1685" t="s">
+        <v>2223</v>
+      </c>
+      <c r="B1685" t="s">
         <v>230</v>
       </c>
-      <c r="C1663" t="s">
-        <v>2342</v>
-      </c>
-      <c r="D1663" t="s">
-        <v>50</v>
-      </c>
-      <c r="E1663" t="s">
+      <c r="C1685" t="s">
+        <v>2417</v>
+      </c>
+      <c r="D1685" t="s">
+        <v>50</v>
+      </c>
+      <c r="E1685" t="s">
         <v>232</v>
       </c>
-      <c r="F1663" t="s">
-        <v>2341</v>
-      </c>
-      <c r="G1663" t="s">
-        <v>50</v>
-      </c>
-      <c r="H1663" t="s">
-        <v>50</v>
-      </c>
-      <c r="I1663" t="s">
-        <v>50</v>
-      </c>
-      <c r="J1663" t="s">
+      <c r="F1685" t="s">
+        <v>2416</v>
+      </c>
+      <c r="G1685" t="s">
+        <v>50</v>
+      </c>
+      <c r="H1685" t="s">
+        <v>50</v>
+      </c>
+      <c r="I1685" t="s">
+        <v>50</v>
+      </c>
+      <c r="J1685" t="s">
         <v>50</v>
       </c>
     </row>

</xml_diff>

<commit_message>
compiled report 2026-06-06: 615 election events, 279 audit entries
</commit_message>
<xml_diff>
--- a/punmonitor-compiled-report.xlsx
+++ b/punmonitor-compiled-report.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2418" uniqueCount="2418">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2538" uniqueCount="2538">
   <si>
     <t>Source Date</t>
   </si>
@@ -6697,49 +6697,559 @@
     <t>43.247.40.101</t>
   </si>
   <si>
-    <t>10.0.60</t>
-  </si>
-  <si>
-    <t>2026-06-06 12:41:31</t>
-  </si>
-  <si>
-    <t>3h 58m 34s</t>
-  </si>
-  <si>
-    <t>12:43:45</t>
-  </si>
-  <si>
-    <t>330.0</t>
-  </si>
-  <si>
-    <t>113638.3</t>
-  </si>
-  <si>
-    <t>671</t>
-  </si>
-  <si>
-    <t>3h 58m 19s</t>
-  </si>
-  <si>
-    <t>Dual-89e4fa7c</t>
-  </si>
-  <si>
-    <t>Dual</t>
-  </si>
-  <si>
-    <t>192.168.31.110</t>
-  </si>
-  <si>
-    <t>49.36.213.176</t>
-  </si>
-  <si>
-    <t>websocket</t>
-  </si>
-  <si>
-    <t>1060.0</t>
-  </si>
-  <si>
-    <t>239784.0</t>
+    <t>10.0.61</t>
+  </si>
+  <si>
+    <t>0h 2m 19s</t>
+  </si>
+  <si>
+    <t>2026-06-06 21:31:33</t>
+  </si>
+  <si>
+    <t>Jun 6 03:12 PM</t>
+  </si>
+  <si>
+    <t>1h 25m 36s</t>
+  </si>
+  <si>
+    <t>21:33:52</t>
+  </si>
+  <si>
+    <t>301.0</t>
+  </si>
+  <si>
+    <t>118930.3</t>
+  </si>
+  <si>
+    <t>1h 23m 36s</t>
+  </si>
+  <si>
+    <t>2026-06-06T21:31:52.053887+05:30</t>
+  </si>
+  <si>
+    <t>21:31:52.053</t>
+  </si>
+  <si>
+    <t>1780692604499</t>
+  </si>
+  <si>
+    <t>02:20:04</t>
+  </si>
+  <si>
+    <t>72MYabHy</t>
+  </si>
+  <si>
+    <t>1780692604755</t>
+  </si>
+  <si>
+    <t>1780692606976</t>
+  </si>
+  <si>
+    <t>02:20:06</t>
+  </si>
+  <si>
+    <t>gGIz8GGT</t>
+  </si>
+  <si>
+    <t>1780692607134</t>
+  </si>
+  <si>
+    <t>02:20:07</t>
+  </si>
+  <si>
+    <t>1780692607886</t>
+  </si>
+  <si>
+    <t>prYYq3pj</t>
+  </si>
+  <si>
+    <t>1780692608129</t>
+  </si>
+  <si>
+    <t>02:20:08</t>
+  </si>
+  <si>
+    <t>2026-06-06T21:31:52+05:30 (2m0s ago)</t>
+  </si>
+  <si>
+    <t>520</t>
+  </si>
+  <si>
+    <t>2026-06-05T23:53:04.3464959+05:30</t>
+  </si>
+  <si>
+    <t>23:53:04.346</t>
+  </si>
+  <si>
+    <t>521</t>
+  </si>
+  <si>
+    <t>2026-06-05T23:58:04.4885433+05:30</t>
+  </si>
+  <si>
+    <t>23:58:04.488</t>
+  </si>
+  <si>
+    <t>522</t>
+  </si>
+  <si>
+    <t>2026-06-06T00:03:04.5336367+05:30</t>
+  </si>
+  <si>
+    <t>00:03:04.533</t>
+  </si>
+  <si>
+    <t>523</t>
+  </si>
+  <si>
+    <t>2026-06-06T00:08:04.3890711+05:30</t>
+  </si>
+  <si>
+    <t>00:08:04.389</t>
+  </si>
+  <si>
+    <t>524</t>
+  </si>
+  <si>
+    <t>2026-06-06T00:13:04.2945198+05:30</t>
+  </si>
+  <si>
+    <t>00:13:04.294</t>
+  </si>
+  <si>
+    <t>525</t>
+  </si>
+  <si>
+    <t>2026-06-06T00:18:04.349719+05:30</t>
+  </si>
+  <si>
+    <t>00:18:04.349</t>
+  </si>
+  <si>
+    <t>526</t>
+  </si>
+  <si>
+    <t>2026-06-06T00:23:03.2036477+05:30</t>
+  </si>
+  <si>
+    <t>00:23:03.203</t>
+  </si>
+  <si>
+    <t>527</t>
+  </si>
+  <si>
+    <t>2026-06-06T00:23:03.20476+05:30</t>
+  </si>
+  <si>
+    <t>00:23:03.204</t>
+  </si>
+  <si>
+    <t>528</t>
+  </si>
+  <si>
+    <t>2026-06-06T00:28:04.4524866+05:30</t>
+  </si>
+  <si>
+    <t>00:28:04.452</t>
+  </si>
+  <si>
+    <t>529</t>
+  </si>
+  <si>
+    <t>2026-06-06T00:33:04.9882474+05:30</t>
+  </si>
+  <si>
+    <t>00:33:04.988</t>
+  </si>
+  <si>
+    <t>530</t>
+  </si>
+  <si>
+    <t>2026-06-06T00:38:04.4578185+05:30</t>
+  </si>
+  <si>
+    <t>00:38:04.457</t>
+  </si>
+  <si>
+    <t>531</t>
+  </si>
+  <si>
+    <t>2026-06-06T00:43:04.4165849+05:30</t>
+  </si>
+  <si>
+    <t>00:43:04.416</t>
+  </si>
+  <si>
+    <t>532</t>
+  </si>
+  <si>
+    <t>2026-06-06T00:48:04.4972065+05:30</t>
+  </si>
+  <si>
+    <t>00:48:04.497</t>
+  </si>
+  <si>
+    <t>533</t>
+  </si>
+  <si>
+    <t>2026-06-06T00:53:04.4158628+05:30</t>
+  </si>
+  <si>
+    <t>00:53:04.415</t>
+  </si>
+  <si>
+    <t>534</t>
+  </si>
+  <si>
+    <t>2026-06-06T00:58:04.746462+05:30</t>
+  </si>
+  <si>
+    <t>00:58:04.746</t>
+  </si>
+  <si>
+    <t>535</t>
+  </si>
+  <si>
+    <t>2026-06-06T01:03:04.2965606+05:30</t>
+  </si>
+  <si>
+    <t>01:03:04.296</t>
+  </si>
+  <si>
+    <t>536</t>
+  </si>
+  <si>
+    <t>2026-06-06T01:08:04.4870498+05:30</t>
+  </si>
+  <si>
+    <t>01:08:04.487</t>
+  </si>
+  <si>
+    <t>537</t>
+  </si>
+  <si>
+    <t>2026-06-06T01:13:04.3971229+05:30</t>
+  </si>
+  <si>
+    <t>01:13:04.397</t>
+  </si>
+  <si>
+    <t>538</t>
+  </si>
+  <si>
+    <t>2026-06-06T01:18:04.3982097+05:30</t>
+  </si>
+  <si>
+    <t>01:18:04.398</t>
+  </si>
+  <si>
+    <t>539</t>
+  </si>
+  <si>
+    <t>2026-06-06T01:23:04.338193+05:30</t>
+  </si>
+  <si>
+    <t>01:23:04.338</t>
+  </si>
+  <si>
+    <t>540</t>
+  </si>
+  <si>
+    <t>2026-06-06T01:28:04.3749159+05:30</t>
+  </si>
+  <si>
+    <t>01:28:04.374</t>
+  </si>
+  <si>
+    <t>541</t>
+  </si>
+  <si>
+    <t>2026-06-06T01:33:04.3612467+05:30</t>
+  </si>
+  <si>
+    <t>01:33:04.361</t>
+  </si>
+  <si>
+    <t>542</t>
+  </si>
+  <si>
+    <t>2026-06-06T01:38:04.5068535+05:30</t>
+  </si>
+  <si>
+    <t>01:38:04.506</t>
+  </si>
+  <si>
+    <t>543</t>
+  </si>
+  <si>
+    <t>2026-06-06T01:43:04.4507225+05:30</t>
+  </si>
+  <si>
+    <t>01:43:04.450</t>
+  </si>
+  <si>
+    <t>544</t>
+  </si>
+  <si>
+    <t>2026-06-06T01:48:04.4562151+05:30</t>
+  </si>
+  <si>
+    <t>01:48:04.456</t>
+  </si>
+  <si>
+    <t>545</t>
+  </si>
+  <si>
+    <t>2026-06-06T01:53:04.4814572+05:30</t>
+  </si>
+  <si>
+    <t>01:53:04.481</t>
+  </si>
+  <si>
+    <t>546</t>
+  </si>
+  <si>
+    <t>2026-06-06T01:58:04.3490827+05:30</t>
+  </si>
+  <si>
+    <t>01:58:04.349</t>
+  </si>
+  <si>
+    <t>547</t>
+  </si>
+  <si>
+    <t>2026-06-06T02:03:04.395145+05:30</t>
+  </si>
+  <si>
+    <t>02:03:04.395</t>
+  </si>
+  <si>
+    <t>548</t>
+  </si>
+  <si>
+    <t>2026-06-06T02:08:04.4247916+05:30</t>
+  </si>
+  <si>
+    <t>02:08:04.424</t>
+  </si>
+  <si>
+    <t>549</t>
+  </si>
+  <si>
+    <t>2026-06-06T02:12:57.4419603+05:30</t>
+  </si>
+  <si>
+    <t>02:12:57.441</t>
+  </si>
+  <si>
+    <t>550</t>
+  </si>
+  <si>
+    <t>2026-06-06T02:17:58.646138+05:30</t>
+  </si>
+  <si>
+    <t>02:17:58.646</t>
+  </si>
+  <si>
+    <t>551</t>
+  </si>
+  <si>
+    <t>2026-06-06T02:19:01.3448451+05:30</t>
+  </si>
+  <si>
+    <t>02:19:01.344</t>
+  </si>
+  <si>
+    <t>552</t>
+  </si>
+  <si>
+    <t>2026-06-06T02:24:02.6039292+05:30</t>
+  </si>
+  <si>
+    <t>02:24:02.603</t>
+  </si>
+  <si>
+    <t>553</t>
+  </si>
+  <si>
+    <t>2026-06-06T02:29:02.5972012+05:30</t>
+  </si>
+  <si>
+    <t>02:29:02.597</t>
+  </si>
+  <si>
+    <t>554</t>
+  </si>
+  <si>
+    <t>2026-06-06T02:34:02.754349+05:30</t>
+  </si>
+  <si>
+    <t>02:34:02.754</t>
+  </si>
+  <si>
+    <t>555</t>
+  </si>
+  <si>
+    <t>2026-06-06T02:39:02.6088993+05:30</t>
+  </si>
+  <si>
+    <t>02:39:02.608</t>
+  </si>
+  <si>
+    <t>556</t>
+  </si>
+  <si>
+    <t>2026-06-06T02:44:02.6738715+05:30</t>
+  </si>
+  <si>
+    <t>02:44:02.673</t>
+  </si>
+  <si>
+    <t>557</t>
+  </si>
+  <si>
+    <t>2026-06-06T02:49:02.6003314+05:30</t>
+  </si>
+  <si>
+    <t>02:49:02.600</t>
+  </si>
+  <si>
+    <t>558</t>
+  </si>
+  <si>
+    <t>2026-06-06T02:54:02.634182+05:30</t>
+  </si>
+  <si>
+    <t>02:54:02.634</t>
+  </si>
+  <si>
+    <t>559</t>
+  </si>
+  <si>
+    <t>2026-06-06T02:59:02.5326307+05:30</t>
+  </si>
+  <si>
+    <t>02:59:02.532</t>
+  </si>
+  <si>
+    <t>560</t>
+  </si>
+  <si>
+    <t>2026-06-06T03:04:02.4988555+05:30</t>
+  </si>
+  <si>
+    <t>03:04:02.498</t>
+  </si>
+  <si>
+    <t>561</t>
+  </si>
+  <si>
+    <t>2026-06-06T03:09:02.5174213+05:30</t>
+  </si>
+  <si>
+    <t>03:09:02.517</t>
+  </si>
+  <si>
+    <t>562</t>
+  </si>
+  <si>
+    <t>2026-06-06T03:14:03.0156796+05:30</t>
+  </si>
+  <si>
+    <t>03:14:03.015</t>
+  </si>
+  <si>
+    <t>563</t>
+  </si>
+  <si>
+    <t>2026-06-06T03:19:02.6230539+05:30</t>
+  </si>
+  <si>
+    <t>03:19:02.623</t>
+  </si>
+  <si>
+    <t>564</t>
+  </si>
+  <si>
+    <t>2026-06-06T03:24:02.5271236+05:30</t>
+  </si>
+  <si>
+    <t>03:24:02.527</t>
+  </si>
+  <si>
+    <t>565</t>
+  </si>
+  <si>
+    <t>2026-06-06T03:29:02.5720525+05:30</t>
+  </si>
+  <si>
+    <t>03:29:02.572</t>
+  </si>
+  <si>
+    <t>566</t>
+  </si>
+  <si>
+    <t>2026-06-06T03:34:02.5814869+05:30</t>
+  </si>
+  <si>
+    <t>03:34:02.581</t>
+  </si>
+  <si>
+    <t>567</t>
+  </si>
+  <si>
+    <t>2026-06-06T03:39:02.5788422+05:30</t>
+  </si>
+  <si>
+    <t>03:39:02.578</t>
+  </si>
+  <si>
+    <t>568</t>
+  </si>
+  <si>
+    <t>2026-06-06T03:44:02.633002+05:30</t>
+  </si>
+  <si>
+    <t>03:44:02.633</t>
+  </si>
+  <si>
+    <t>569</t>
+  </si>
+  <si>
+    <t>2026-06-06T03:49:02.566586+05:30</t>
+  </si>
+  <si>
+    <t>03:49:02.566</t>
+  </si>
+  <si>
+    <t>570</t>
+  </si>
+  <si>
+    <t>2026-06-06T03:54:02.8834141+05:30</t>
+  </si>
+  <si>
+    <t>03:54:02.883</t>
+  </si>
+  <si>
+    <t>571</t>
+  </si>
+  <si>
+    <t>2026-06-06T12:37:31.4976556+05:30</t>
+  </si>
+  <si>
+    <t>12:37:31.497</t>
+  </si>
+  <si>
+    <t>572</t>
+  </si>
+  <si>
+    <t>2026-06-06T12:40:03.0204921+05:30</t>
+  </si>
+  <si>
+    <t>12:40:03.020</t>
+  </si>
+  <si>
+    <t>573</t>
   </si>
   <si>
     <t>2026-06-06T12:41:45.8254272+05:30</t>
@@ -6748,529 +7258,379 @@
     <t>12:41:45.825</t>
   </si>
   <si>
-    <t>1780692604499</t>
-  </si>
-  <si>
-    <t>02:20:04</t>
-  </si>
-  <si>
-    <t>72MYabHy</t>
-  </si>
-  <si>
-    <t>1780692604755</t>
-  </si>
-  <si>
-    <t>1780692606976</t>
-  </si>
-  <si>
-    <t>02:20:06</t>
-  </si>
-  <si>
-    <t>gGIz8GGT</t>
-  </si>
-  <si>
-    <t>1780692607134</t>
-  </si>
-  <si>
-    <t>02:20:07</t>
-  </si>
-  <si>
-    <t>1780692607886</t>
-  </si>
-  <si>
-    <t>prYYq3pj</t>
-  </si>
-  <si>
-    <t>1780692608129</t>
-  </si>
-  <si>
-    <t>02:20:08</t>
-  </si>
-  <si>
-    <t>2026-06-06T12:41:45+05:30 (2m0s ago)</t>
-  </si>
-  <si>
-    <t>520</t>
-  </si>
-  <si>
-    <t>2026-06-05T23:53:04.3464959+05:30</t>
-  </si>
-  <si>
-    <t>23:53:04.346</t>
-  </si>
-  <si>
-    <t>521</t>
-  </si>
-  <si>
-    <t>2026-06-05T23:58:04.4885433+05:30</t>
-  </si>
-  <si>
-    <t>23:58:04.488</t>
-  </si>
-  <si>
-    <t>522</t>
-  </si>
-  <si>
-    <t>2026-06-06T00:03:04.5336367+05:30</t>
-  </si>
-  <si>
-    <t>00:03:04.533</t>
-  </si>
-  <si>
-    <t>523</t>
-  </si>
-  <si>
-    <t>2026-06-06T00:08:04.3890711+05:30</t>
-  </si>
-  <si>
-    <t>00:08:04.389</t>
-  </si>
-  <si>
-    <t>524</t>
-  </si>
-  <si>
-    <t>2026-06-06T00:13:04.2945198+05:30</t>
-  </si>
-  <si>
-    <t>00:13:04.294</t>
-  </si>
-  <si>
-    <t>525</t>
-  </si>
-  <si>
-    <t>2026-06-06T00:18:04.349719+05:30</t>
-  </si>
-  <si>
-    <t>00:18:04.349</t>
-  </si>
-  <si>
-    <t>526</t>
-  </si>
-  <si>
-    <t>2026-06-06T00:23:03.2036477+05:30</t>
-  </si>
-  <si>
-    <t>00:23:03.203</t>
-  </si>
-  <si>
-    <t>527</t>
-  </si>
-  <si>
-    <t>2026-06-06T00:23:03.20476+05:30</t>
-  </si>
-  <si>
-    <t>00:23:03.204</t>
-  </si>
-  <si>
-    <t>528</t>
-  </si>
-  <si>
-    <t>2026-06-06T00:28:04.4524866+05:30</t>
-  </si>
-  <si>
-    <t>00:28:04.452</t>
-  </si>
-  <si>
-    <t>529</t>
-  </si>
-  <si>
-    <t>2026-06-06T00:33:04.9882474+05:30</t>
-  </si>
-  <si>
-    <t>00:33:04.988</t>
-  </si>
-  <si>
-    <t>530</t>
-  </si>
-  <si>
-    <t>2026-06-06T00:38:04.4578185+05:30</t>
-  </si>
-  <si>
-    <t>00:38:04.457</t>
-  </si>
-  <si>
-    <t>531</t>
-  </si>
-  <si>
-    <t>2026-06-06T00:43:04.4165849+05:30</t>
-  </si>
-  <si>
-    <t>00:43:04.416</t>
-  </si>
-  <si>
-    <t>532</t>
-  </si>
-  <si>
-    <t>2026-06-06T00:48:04.4972065+05:30</t>
-  </si>
-  <si>
-    <t>00:48:04.497</t>
-  </si>
-  <si>
-    <t>533</t>
-  </si>
-  <si>
-    <t>2026-06-06T00:53:04.4158628+05:30</t>
-  </si>
-  <si>
-    <t>00:53:04.415</t>
-  </si>
-  <si>
-    <t>534</t>
-  </si>
-  <si>
-    <t>2026-06-06T00:58:04.746462+05:30</t>
-  </si>
-  <si>
-    <t>00:58:04.746</t>
-  </si>
-  <si>
-    <t>535</t>
-  </si>
-  <si>
-    <t>2026-06-06T01:03:04.2965606+05:30</t>
-  </si>
-  <si>
-    <t>01:03:04.296</t>
-  </si>
-  <si>
-    <t>536</t>
-  </si>
-  <si>
-    <t>2026-06-06T01:08:04.4870498+05:30</t>
-  </si>
-  <si>
-    <t>01:08:04.487</t>
-  </si>
-  <si>
-    <t>537</t>
-  </si>
-  <si>
-    <t>2026-06-06T01:13:04.3971229+05:30</t>
-  </si>
-  <si>
-    <t>01:13:04.397</t>
-  </si>
-  <si>
-    <t>538</t>
-  </si>
-  <si>
-    <t>2026-06-06T01:18:04.3982097+05:30</t>
-  </si>
-  <si>
-    <t>01:18:04.398</t>
-  </si>
-  <si>
-    <t>539</t>
-  </si>
-  <si>
-    <t>2026-06-06T01:23:04.338193+05:30</t>
-  </si>
-  <si>
-    <t>01:23:04.338</t>
-  </si>
-  <si>
-    <t>540</t>
-  </si>
-  <si>
-    <t>2026-06-06T01:28:04.3749159+05:30</t>
-  </si>
-  <si>
-    <t>01:28:04.374</t>
-  </si>
-  <si>
-    <t>541</t>
-  </si>
-  <si>
-    <t>2026-06-06T01:33:04.3612467+05:30</t>
-  </si>
-  <si>
-    <t>01:33:04.361</t>
-  </si>
-  <si>
-    <t>542</t>
-  </si>
-  <si>
-    <t>2026-06-06T01:38:04.5068535+05:30</t>
-  </si>
-  <si>
-    <t>01:38:04.506</t>
-  </si>
-  <si>
-    <t>543</t>
-  </si>
-  <si>
-    <t>2026-06-06T01:43:04.4507225+05:30</t>
-  </si>
-  <si>
-    <t>01:43:04.450</t>
-  </si>
-  <si>
-    <t>544</t>
-  </si>
-  <si>
-    <t>2026-06-06T01:48:04.4562151+05:30</t>
-  </si>
-  <si>
-    <t>01:48:04.456</t>
-  </si>
-  <si>
-    <t>545</t>
-  </si>
-  <si>
-    <t>2026-06-06T01:53:04.4814572+05:30</t>
-  </si>
-  <si>
-    <t>01:53:04.481</t>
-  </si>
-  <si>
-    <t>546</t>
-  </si>
-  <si>
-    <t>2026-06-06T01:58:04.3490827+05:30</t>
-  </si>
-  <si>
-    <t>01:58:04.349</t>
-  </si>
-  <si>
-    <t>547</t>
-  </si>
-  <si>
-    <t>2026-06-06T02:03:04.395145+05:30</t>
-  </si>
-  <si>
-    <t>02:03:04.395</t>
-  </si>
-  <si>
-    <t>548</t>
-  </si>
-  <si>
-    <t>2026-06-06T02:08:04.4247916+05:30</t>
-  </si>
-  <si>
-    <t>02:08:04.424</t>
-  </si>
-  <si>
-    <t>549</t>
-  </si>
-  <si>
-    <t>2026-06-06T02:12:57.4419603+05:30</t>
-  </si>
-  <si>
-    <t>02:12:57.441</t>
-  </si>
-  <si>
-    <t>550</t>
-  </si>
-  <si>
-    <t>2026-06-06T02:17:58.646138+05:30</t>
-  </si>
-  <si>
-    <t>02:17:58.646</t>
-  </si>
-  <si>
-    <t>551</t>
-  </si>
-  <si>
-    <t>2026-06-06T02:19:01.3448451+05:30</t>
-  </si>
-  <si>
-    <t>02:19:01.344</t>
-  </si>
-  <si>
-    <t>552</t>
-  </si>
-  <si>
-    <t>2026-06-06T02:24:02.6039292+05:30</t>
-  </si>
-  <si>
-    <t>02:24:02.603</t>
-  </si>
-  <si>
-    <t>553</t>
-  </si>
-  <si>
-    <t>2026-06-06T02:29:02.5972012+05:30</t>
-  </si>
-  <si>
-    <t>02:29:02.597</t>
-  </si>
-  <si>
-    <t>554</t>
-  </si>
-  <si>
-    <t>2026-06-06T02:34:02.754349+05:30</t>
-  </si>
-  <si>
-    <t>02:34:02.754</t>
-  </si>
-  <si>
-    <t>555</t>
-  </si>
-  <si>
-    <t>2026-06-06T02:39:02.6088993+05:30</t>
-  </si>
-  <si>
-    <t>02:39:02.608</t>
-  </si>
-  <si>
-    <t>556</t>
-  </si>
-  <si>
-    <t>2026-06-06T02:44:02.6738715+05:30</t>
-  </si>
-  <si>
-    <t>02:44:02.673</t>
-  </si>
-  <si>
-    <t>557</t>
-  </si>
-  <si>
-    <t>2026-06-06T02:49:02.6003314+05:30</t>
-  </si>
-  <si>
-    <t>02:49:02.600</t>
-  </si>
-  <si>
-    <t>558</t>
-  </si>
-  <si>
-    <t>2026-06-06T02:54:02.634182+05:30</t>
-  </si>
-  <si>
-    <t>02:54:02.634</t>
-  </si>
-  <si>
-    <t>559</t>
-  </si>
-  <si>
-    <t>2026-06-06T02:59:02.5326307+05:30</t>
-  </si>
-  <si>
-    <t>02:59:02.532</t>
-  </si>
-  <si>
-    <t>560</t>
-  </si>
-  <si>
-    <t>2026-06-06T03:04:02.4988555+05:30</t>
-  </si>
-  <si>
-    <t>03:04:02.498</t>
-  </si>
-  <si>
-    <t>561</t>
-  </si>
-  <si>
-    <t>2026-06-06T03:09:02.5174213+05:30</t>
-  </si>
-  <si>
-    <t>03:09:02.517</t>
-  </si>
-  <si>
-    <t>562</t>
-  </si>
-  <si>
-    <t>2026-06-06T03:14:03.0156796+05:30</t>
-  </si>
-  <si>
-    <t>03:14:03.015</t>
-  </si>
-  <si>
-    <t>563</t>
-  </si>
-  <si>
-    <t>2026-06-06T03:19:02.6230539+05:30</t>
-  </si>
-  <si>
-    <t>03:19:02.623</t>
-  </si>
-  <si>
-    <t>564</t>
-  </si>
-  <si>
-    <t>2026-06-06T03:24:02.5271236+05:30</t>
-  </si>
-  <si>
-    <t>03:24:02.527</t>
-  </si>
-  <si>
-    <t>565</t>
-  </si>
-  <si>
-    <t>2026-06-06T03:29:02.5720525+05:30</t>
-  </si>
-  <si>
-    <t>03:29:02.572</t>
-  </si>
-  <si>
-    <t>566</t>
-  </si>
-  <si>
-    <t>2026-06-06T03:34:02.5814869+05:30</t>
-  </si>
-  <si>
-    <t>03:34:02.581</t>
-  </si>
-  <si>
-    <t>567</t>
-  </si>
-  <si>
-    <t>2026-06-06T03:39:02.5788422+05:30</t>
-  </si>
-  <si>
-    <t>03:39:02.578</t>
-  </si>
-  <si>
-    <t>568</t>
-  </si>
-  <si>
-    <t>2026-06-06T03:44:02.633002+05:30</t>
-  </si>
-  <si>
-    <t>03:44:02.633</t>
-  </si>
-  <si>
-    <t>569</t>
-  </si>
-  <si>
-    <t>2026-06-06T03:49:02.566586+05:30</t>
-  </si>
-  <si>
-    <t>03:49:02.566</t>
-  </si>
-  <si>
-    <t>570</t>
-  </si>
-  <si>
-    <t>2026-06-06T03:54:02.8834141+05:30</t>
-  </si>
-  <si>
-    <t>03:54:02.883</t>
-  </si>
-  <si>
-    <t>571</t>
-  </si>
-  <si>
-    <t>2026-06-06T12:37:31.4976556+05:30</t>
-  </si>
-  <si>
-    <t>12:37:31.497</t>
-  </si>
-  <si>
-    <t>572</t>
-  </si>
-  <si>
-    <t>2026-06-06T12:40:03.0204921+05:30</t>
-  </si>
-  <si>
-    <t>12:40:03.020</t>
-  </si>
-  <si>
-    <t>573</t>
-  </si>
-  <si>
-    <t>2026-06-06T12:43:46+05:30</t>
+    <t>574</t>
+  </si>
+  <si>
+    <t>2026-06-06T12:46:47.2560864+05:30</t>
+  </si>
+  <si>
+    <t>12:46:47.256</t>
+  </si>
+  <si>
+    <t>575</t>
+  </si>
+  <si>
+    <t>2026-06-06T12:51:47.1244945+05:30</t>
+  </si>
+  <si>
+    <t>12:51:47.124</t>
+  </si>
+  <si>
+    <t>576</t>
+  </si>
+  <si>
+    <t>2026-06-06T12:56:47.2292248+05:30</t>
+  </si>
+  <si>
+    <t>12:56:47.229</t>
+  </si>
+  <si>
+    <t>577</t>
+  </si>
+  <si>
+    <t>2026-06-06T13:01:47.7179577+05:30</t>
+  </si>
+  <si>
+    <t>13:01:47.717</t>
+  </si>
+  <si>
+    <t>578</t>
+  </si>
+  <si>
+    <t>2026-06-06T13:06:47.4441712+05:30</t>
+  </si>
+  <si>
+    <t>13:06:47.444</t>
+  </si>
+  <si>
+    <t>579</t>
+  </si>
+  <si>
+    <t>2026-06-06T13:11:47.2557786+05:30</t>
+  </si>
+  <si>
+    <t>13:11:47.255</t>
+  </si>
+  <si>
+    <t>580</t>
+  </si>
+  <si>
+    <t>2026-06-06T13:16:48.7631823+05:30</t>
+  </si>
+  <si>
+    <t>13:16:48.763</t>
+  </si>
+  <si>
+    <t>581</t>
+  </si>
+  <si>
+    <t>2026-06-06T13:21:49.4635515+05:30</t>
+  </si>
+  <si>
+    <t>13:21:49.463</t>
+  </si>
+  <si>
+    <t>582</t>
+  </si>
+  <si>
+    <t>2026-06-06T13:26:46.9172972+05:30</t>
+  </si>
+  <si>
+    <t>13:26:46.917</t>
+  </si>
+  <si>
+    <t>583</t>
+  </si>
+  <si>
+    <t>2026-06-06T13:31:47.348369+05:30</t>
+  </si>
+  <si>
+    <t>13:31:47.348</t>
+  </si>
+  <si>
+    <t>584</t>
+  </si>
+  <si>
+    <t>2026-06-06T13:36:47.392442+05:30</t>
+  </si>
+  <si>
+    <t>13:36:47.392</t>
+  </si>
+  <si>
+    <t>585</t>
+  </si>
+  <si>
+    <t>2026-06-06T13:41:48.3311396+05:30</t>
+  </si>
+  <si>
+    <t>13:41:48.331</t>
+  </si>
+  <si>
+    <t>586</t>
+  </si>
+  <si>
+    <t>2026-06-06T13:46:47.2396639+05:30</t>
+  </si>
+  <si>
+    <t>13:46:47.239</t>
+  </si>
+  <si>
+    <t>587</t>
+  </si>
+  <si>
+    <t>2026-06-06T13:51:51.0832952+05:30</t>
+  </si>
+  <si>
+    <t>13:51:51.083</t>
+  </si>
+  <si>
+    <t>588</t>
+  </si>
+  <si>
+    <t>2026-06-06T13:56:47.101891+05:30</t>
+  </si>
+  <si>
+    <t>13:56:47.101</t>
+  </si>
+  <si>
+    <t>589</t>
+  </si>
+  <si>
+    <t>2026-06-06T14:01:47.0489808+05:30</t>
+  </si>
+  <si>
+    <t>14:01:47.048</t>
+  </si>
+  <si>
+    <t>590</t>
+  </si>
+  <si>
+    <t>2026-06-06T15:14:14.354455+05:30</t>
+  </si>
+  <si>
+    <t>15:14:14.354</t>
+  </si>
+  <si>
+    <t>591</t>
+  </si>
+  <si>
+    <t>2026-06-06T15:14:19.3587347+05:30</t>
+  </si>
+  <si>
+    <t>15:14:19.358</t>
+  </si>
+  <si>
+    <t>592</t>
+  </si>
+  <si>
+    <t>2026-06-06T15:14:26.3679956+05:30</t>
+  </si>
+  <si>
+    <t>15:14:26.367</t>
+  </si>
+  <si>
+    <t>593</t>
+  </si>
+  <si>
+    <t>2026-06-06T15:20:38.5562603+05:30</t>
+  </si>
+  <si>
+    <t>15:20:38.556</t>
+  </si>
+  <si>
+    <t>594</t>
+  </si>
+  <si>
+    <t>2026-06-06T15:25:38.5558976+05:30</t>
+  </si>
+  <si>
+    <t>15:25:38.555</t>
+  </si>
+  <si>
+    <t>595</t>
+  </si>
+  <si>
+    <t>2026-06-06T15:30:38.5562188+05:30</t>
+  </si>
+  <si>
+    <t>15:30:38.556</t>
+  </si>
+  <si>
+    <t>596</t>
+  </si>
+  <si>
+    <t>2026-06-06T18:32:51.8844302+05:30</t>
+  </si>
+  <si>
+    <t>18:32:51.884</t>
+  </si>
+  <si>
+    <t>597</t>
+  </si>
+  <si>
+    <t>2026-06-06T18:35:33.1574356+05:30</t>
+  </si>
+  <si>
+    <t>18:35:33.157</t>
+  </si>
+  <si>
+    <t>598</t>
+  </si>
+  <si>
+    <t>2026-06-06T18:40:30.4555118+05:30</t>
+  </si>
+  <si>
+    <t>18:40:30.455</t>
+  </si>
+  <si>
+    <t>599</t>
+  </si>
+  <si>
+    <t>2026-06-06T18:45:38.5555278+05:30</t>
+  </si>
+  <si>
+    <t>18:45:38.555</t>
+  </si>
+  <si>
+    <t>600</t>
+  </si>
+  <si>
+    <t>2026-06-06T18:45:40.5835175+05:30</t>
+  </si>
+  <si>
+    <t>18:45:40.583</t>
+  </si>
+  <si>
+    <t>601</t>
+  </si>
+  <si>
+    <t>2026-06-06T18:50:31.2008843+05:30</t>
+  </si>
+  <si>
+    <t>18:50:31.200</t>
+  </si>
+  <si>
+    <t>602</t>
+  </si>
+  <si>
+    <t>2026-06-06T18:55:29.8174079+05:30</t>
+  </si>
+  <si>
+    <t>18:55:29.817</t>
+  </si>
+  <si>
+    <t>603</t>
+  </si>
+  <si>
+    <t>2026-06-06T19:00:38.5549153+05:30</t>
+  </si>
+  <si>
+    <t>19:00:38.554</t>
+  </si>
+  <si>
+    <t>604</t>
+  </si>
+  <si>
+    <t>2026-06-06T19:05:38.5558702+05:30</t>
+  </si>
+  <si>
+    <t>19:05:38.555</t>
+  </si>
+  <si>
+    <t>605</t>
+  </si>
+  <si>
+    <t>2026-06-06T19:10:38.5551272+05:30</t>
+  </si>
+  <si>
+    <t>19:10:38.555</t>
+  </si>
+  <si>
+    <t>606</t>
+  </si>
+  <si>
+    <t>2026-06-06T19:47:29.2654343+05:30</t>
+  </si>
+  <si>
+    <t>19:47:29.265</t>
+  </si>
+  <si>
+    <t>607</t>
+  </si>
+  <si>
+    <t>2026-06-06T19:50:29.9532522+05:30</t>
+  </si>
+  <si>
+    <t>19:50:29.953</t>
+  </si>
+  <si>
+    <t>608</t>
+  </si>
+  <si>
+    <t>2026-06-06T19:55:29.834916+05:30</t>
+  </si>
+  <si>
+    <t>19:55:29.834</t>
+  </si>
+  <si>
+    <t>609</t>
+  </si>
+  <si>
+    <t>2026-06-06T20:00:38.5548904+05:30</t>
+  </si>
+  <si>
+    <t>20:00:38.554</t>
+  </si>
+  <si>
+    <t>610</t>
+  </si>
+  <si>
+    <t>2026-06-06T20:00:48.5552444+05:30</t>
+  </si>
+  <si>
+    <t>20:00:48.555</t>
+  </si>
+  <si>
+    <t>611</t>
+  </si>
+  <si>
+    <t>2026-06-06T20:05:30.0395294+05:30</t>
+  </si>
+  <si>
+    <t>20:05:30.039</t>
+  </si>
+  <si>
+    <t>612</t>
+  </si>
+  <si>
+    <t>2026-06-06T20:10:30.0757021+05:30</t>
+  </si>
+  <si>
+    <t>20:10:30.075</t>
+  </si>
+  <si>
+    <t>613</t>
+  </si>
+  <si>
+    <t>2026-06-06T20:15:31.1592802+05:30</t>
+  </si>
+  <si>
+    <t>20:15:31.159</t>
+  </si>
+  <si>
+    <t>614</t>
+  </si>
+  <si>
+    <t>2026-06-06T21:08:03.4430969+05:30</t>
+  </si>
+  <si>
+    <t>21:08:03.443</t>
+  </si>
+  <si>
+    <t>615</t>
+  </si>
+  <si>
+    <t>2026-06-06T21:33:52+05:30</t>
   </si>
 </sst>
 </file>
@@ -8644,25 +9004,25 @@
         <v>39</v>
       </c>
       <c r="P18" t="s">
-        <v>1184</v>
+        <v>2227</v>
       </c>
       <c r="Q18" t="s">
-        <v>2227</v>
+        <v>2228</v>
       </c>
       <c r="R18" t="s">
-        <v>1186</v>
+        <v>2229</v>
       </c>
       <c r="S18" t="s">
-        <v>2227</v>
+        <v>2228</v>
       </c>
       <c r="T18" t="s">
-        <v>2228</v>
+        <v>2230</v>
       </c>
       <c r="U18" t="s">
         <v>2223</v>
       </c>
       <c r="V18" t="s">
-        <v>2229</v>
+        <v>2231</v>
       </c>
     </row>
     <row r="19">
@@ -8700,37 +9060,37 @@
         <v>241</v>
       </c>
       <c r="L19" t="s">
-        <v>2230</v>
+        <v>2232</v>
       </c>
       <c r="M19" t="s">
-        <v>2231</v>
+        <v>2233</v>
       </c>
       <c r="N19" t="s">
-        <v>2232</v>
+        <v>2065</v>
       </c>
       <c r="O19" t="s">
         <v>245</v>
       </c>
       <c r="P19" t="s">
-        <v>223</v>
+        <v>275</v>
       </c>
       <c r="Q19" t="s">
         <v>46</v>
       </c>
       <c r="R19" t="s">
-        <v>1186</v>
+        <v>2229</v>
       </c>
       <c r="S19" t="s">
-        <v>2227</v>
+        <v>2228</v>
       </c>
       <c r="T19" t="s">
-        <v>2233</v>
+        <v>2234</v>
       </c>
       <c r="U19" t="s">
         <v>2223</v>
       </c>
       <c r="V19" t="s">
-        <v>2229</v>
+        <v>2231</v>
       </c>
     </row>
     <row r="20">
@@ -8738,67 +9098,52 @@
         <v>2223</v>
       </c>
       <c r="B20" t="s">
-        <v>2234</v>
+        <v>49</v>
       </c>
       <c r="C20" t="s">
-        <v>2235</v>
+        <v>50</v>
       </c>
       <c r="D20" t="s">
-        <v>2236</v>
+        <v>50</v>
       </c>
       <c r="E20" t="s">
-        <v>2237</v>
+        <v>50</v>
       </c>
       <c r="F20" t="s">
-        <v>33</v>
+        <v>50</v>
       </c>
       <c r="G20" t="s">
-        <v>34</v>
+        <v>50</v>
       </c>
       <c r="H20" t="s">
-        <v>1183</v>
+        <v>50</v>
       </c>
       <c r="I20" t="s">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="J20" t="s">
-        <v>2238</v>
+        <v>50</v>
       </c>
       <c r="K20" t="s">
-        <v>241</v>
+        <v>50</v>
       </c>
       <c r="L20" t="s">
-        <v>2239</v>
+        <v>50</v>
       </c>
       <c r="M20" t="s">
-        <v>2240</v>
+        <v>50</v>
       </c>
       <c r="N20" t="s">
-        <v>470</v>
+        <v>50</v>
       </c>
       <c r="O20" t="s">
-        <v>245</v>
+        <v>50</v>
       </c>
       <c r="P20" t="s">
-        <v>627</v>
+        <v>50</v>
       </c>
       <c r="Q20" t="s">
-        <v>46</v>
-      </c>
-      <c r="R20" t="s">
-        <v>46</v>
-      </c>
-      <c r="S20" t="s">
-        <v>46</v>
-      </c>
-      <c r="T20" t="s">
-        <v>46</v>
-      </c>
-      <c r="U20" t="s">
-        <v>2223</v>
-      </c>
-      <c r="V20" t="s">
-        <v>2229</v>
+        <v>50</v>
       </c>
     </row>
     <row r="21">
@@ -8806,37 +9151,37 @@
         <v>2223</v>
       </c>
       <c r="B21" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="C21" t="s">
-        <v>50</v>
+        <v>2235</v>
       </c>
       <c r="D21" t="s">
-        <v>50</v>
+        <v>2223</v>
       </c>
       <c r="E21" t="s">
-        <v>50</v>
+        <v>2236</v>
       </c>
       <c r="F21" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="G21" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="H21" t="s">
-        <v>50</v>
+        <v>29</v>
       </c>
       <c r="I21" t="s">
-        <v>50</v>
+        <v>30</v>
       </c>
       <c r="J21" t="s">
-        <v>50</v>
+        <v>29</v>
       </c>
       <c r="K21" t="s">
-        <v>50</v>
+        <v>39</v>
       </c>
       <c r="L21" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="M21" t="s">
         <v>50</v>
@@ -8851,59 +9196,6 @@
         <v>50</v>
       </c>
       <c r="Q21" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="s">
-        <v>2223</v>
-      </c>
-      <c r="B22" t="s">
-        <v>51</v>
-      </c>
-      <c r="C22" t="s">
-        <v>2241</v>
-      </c>
-      <c r="D22" t="s">
-        <v>2223</v>
-      </c>
-      <c r="E22" t="s">
-        <v>2242</v>
-      </c>
-      <c r="F22" t="s">
-        <v>54</v>
-      </c>
-      <c r="G22" t="s">
-        <v>55</v>
-      </c>
-      <c r="H22" t="s">
-        <v>29</v>
-      </c>
-      <c r="I22" t="s">
-        <v>30</v>
-      </c>
-      <c r="J22" t="s">
-        <v>29</v>
-      </c>
-      <c r="K22" t="s">
-        <v>39</v>
-      </c>
-      <c r="L22" t="s">
-        <v>54</v>
-      </c>
-      <c r="M22" t="s">
-        <v>50</v>
-      </c>
-      <c r="N22" t="s">
-        <v>50</v>
-      </c>
-      <c r="O22" t="s">
-        <v>50</v>
-      </c>
-      <c r="P22" t="s">
-        <v>50</v>
-      </c>
-      <c r="Q22" t="s">
         <v>50</v>
       </c>
     </row>
@@ -26574,10 +26866,10 @@
         <v>2223</v>
       </c>
       <c r="B680" t="s">
-        <v>2243</v>
+        <v>2237</v>
       </c>
       <c r="C680" t="s">
-        <v>2244</v>
+        <v>2238</v>
       </c>
       <c r="D680" t="s">
         <v>2223</v>
@@ -26592,7 +26884,7 @@
         <v>59</v>
       </c>
       <c r="H680" t="s">
-        <v>2245</v>
+        <v>2239</v>
       </c>
     </row>
     <row r="681">
@@ -26600,10 +26892,10 @@
         <v>2223</v>
       </c>
       <c r="B681" t="s">
-        <v>2246</v>
+        <v>2240</v>
       </c>
       <c r="C681" t="s">
-        <v>2244</v>
+        <v>2238</v>
       </c>
       <c r="D681" t="s">
         <v>2223</v>
@@ -26612,7 +26904,7 @@
         <v>62</v>
       </c>
       <c r="F681" t="s">
-        <v>2245</v>
+        <v>2239</v>
       </c>
       <c r="G681" t="s">
         <v>59</v>
@@ -26626,10 +26918,10 @@
         <v>2223</v>
       </c>
       <c r="B682" t="s">
-        <v>2247</v>
+        <v>2241</v>
       </c>
       <c r="C682" t="s">
-        <v>2248</v>
+        <v>2242</v>
       </c>
       <c r="D682" t="s">
         <v>2223</v>
@@ -26644,7 +26936,7 @@
         <v>59</v>
       </c>
       <c r="H682" t="s">
-        <v>2249</v>
+        <v>2243</v>
       </c>
     </row>
     <row r="683">
@@ -26652,10 +26944,10 @@
         <v>2223</v>
       </c>
       <c r="B683" t="s">
-        <v>2250</v>
+        <v>2244</v>
       </c>
       <c r="C683" t="s">
-        <v>2251</v>
+        <v>2245</v>
       </c>
       <c r="D683" t="s">
         <v>2223</v>
@@ -26664,7 +26956,7 @@
         <v>62</v>
       </c>
       <c r="F683" t="s">
-        <v>2249</v>
+        <v>2243</v>
       </c>
       <c r="G683" t="s">
         <v>59</v>
@@ -26678,10 +26970,10 @@
         <v>2223</v>
       </c>
       <c r="B684" t="s">
-        <v>2252</v>
+        <v>2246</v>
       </c>
       <c r="C684" t="s">
-        <v>2251</v>
+        <v>2245</v>
       </c>
       <c r="D684" t="s">
         <v>2223</v>
@@ -26696,7 +26988,7 @@
         <v>59</v>
       </c>
       <c r="H684" t="s">
-        <v>2253</v>
+        <v>2247</v>
       </c>
     </row>
     <row r="685">
@@ -26704,10 +26996,10 @@
         <v>2223</v>
       </c>
       <c r="B685" t="s">
-        <v>2254</v>
+        <v>2248</v>
       </c>
       <c r="C685" t="s">
-        <v>2255</v>
+        <v>2249</v>
       </c>
       <c r="D685" t="s">
         <v>2223</v>
@@ -26716,7 +27008,7 @@
         <v>62</v>
       </c>
       <c r="F685" t="s">
-        <v>2253</v>
+        <v>2247</v>
       </c>
       <c r="G685" t="s">
         <v>59</v>
@@ -68476,7 +68768,7 @@
         <v>162</v>
       </c>
       <c r="C1103" t="s">
-        <v>2256</v>
+        <v>2250</v>
       </c>
       <c r="D1103" t="s">
         <v>50</v>
@@ -68540,7 +68832,7 @@
         <v>166</v>
       </c>
       <c r="C1105" t="s">
-        <v>2256</v>
+        <v>2250</v>
       </c>
       <c r="D1105" t="s">
         <v>50</v>
@@ -88574,16 +88866,16 @@
         <v>2223</v>
       </c>
       <c r="B1630" t="s">
-        <v>2257</v>
+        <v>2251</v>
       </c>
       <c r="C1630" t="s">
-        <v>2258</v>
+        <v>2252</v>
       </c>
       <c r="D1630" t="s">
         <v>1181</v>
       </c>
       <c r="E1630" t="s">
-        <v>2259</v>
+        <v>2253</v>
       </c>
       <c r="F1630" t="s">
         <v>54</v>
@@ -88612,16 +88904,16 @@
         <v>2223</v>
       </c>
       <c r="B1631" t="s">
-        <v>2260</v>
+        <v>2254</v>
       </c>
       <c r="C1631" t="s">
-        <v>2261</v>
+        <v>2255</v>
       </c>
       <c r="D1631" t="s">
         <v>1181</v>
       </c>
       <c r="E1631" t="s">
-        <v>2262</v>
+        <v>2256</v>
       </c>
       <c r="F1631" t="s">
         <v>54</v>
@@ -88650,16 +88942,16 @@
         <v>2223</v>
       </c>
       <c r="B1632" t="s">
-        <v>2263</v>
+        <v>2257</v>
       </c>
       <c r="C1632" t="s">
-        <v>2264</v>
+        <v>2258</v>
       </c>
       <c r="D1632" t="s">
         <v>2223</v>
       </c>
       <c r="E1632" t="s">
-        <v>2265</v>
+        <v>2259</v>
       </c>
       <c r="F1632" t="s">
         <v>54</v>
@@ -88688,16 +88980,16 @@
         <v>2223</v>
       </c>
       <c r="B1633" t="s">
-        <v>2266</v>
+        <v>2260</v>
       </c>
       <c r="C1633" t="s">
-        <v>2267</v>
+        <v>2261</v>
       </c>
       <c r="D1633" t="s">
         <v>2223</v>
       </c>
       <c r="E1633" t="s">
-        <v>2268</v>
+        <v>2262</v>
       </c>
       <c r="F1633" t="s">
         <v>54</v>
@@ -88726,16 +89018,16 @@
         <v>2223</v>
       </c>
       <c r="B1634" t="s">
-        <v>2269</v>
+        <v>2263</v>
       </c>
       <c r="C1634" t="s">
-        <v>2270</v>
+        <v>2264</v>
       </c>
       <c r="D1634" t="s">
         <v>2223</v>
       </c>
       <c r="E1634" t="s">
-        <v>2271</v>
+        <v>2265</v>
       </c>
       <c r="F1634" t="s">
         <v>54</v>
@@ -88764,16 +89056,16 @@
         <v>2223</v>
       </c>
       <c r="B1635" t="s">
-        <v>2272</v>
+        <v>2266</v>
       </c>
       <c r="C1635" t="s">
-        <v>2273</v>
+        <v>2267</v>
       </c>
       <c r="D1635" t="s">
         <v>2223</v>
       </c>
       <c r="E1635" t="s">
-        <v>2274</v>
+        <v>2268</v>
       </c>
       <c r="F1635" t="s">
         <v>54</v>
@@ -88802,16 +89094,16 @@
         <v>2223</v>
       </c>
       <c r="B1636" t="s">
-        <v>2275</v>
+        <v>2269</v>
       </c>
       <c r="C1636" t="s">
-        <v>2276</v>
+        <v>2270</v>
       </c>
       <c r="D1636" t="s">
         <v>2223</v>
       </c>
       <c r="E1636" t="s">
-        <v>2277</v>
+        <v>2271</v>
       </c>
       <c r="F1636" t="s">
         <v>180</v>
@@ -88843,16 +89135,16 @@
         <v>2223</v>
       </c>
       <c r="B1637" t="s">
-        <v>2278</v>
+        <v>2272</v>
       </c>
       <c r="C1637" t="s">
-        <v>2279</v>
+        <v>2273</v>
       </c>
       <c r="D1637" t="s">
         <v>2223</v>
       </c>
       <c r="E1637" t="s">
-        <v>2280</v>
+        <v>2274</v>
       </c>
       <c r="F1637" t="s">
         <v>180</v>
@@ -88884,16 +89176,16 @@
         <v>2223</v>
       </c>
       <c r="B1638" t="s">
-        <v>2281</v>
+        <v>2275</v>
       </c>
       <c r="C1638" t="s">
-        <v>2282</v>
+        <v>2276</v>
       </c>
       <c r="D1638" t="s">
         <v>2223</v>
       </c>
       <c r="E1638" t="s">
-        <v>2283</v>
+        <v>2277</v>
       </c>
       <c r="F1638" t="s">
         <v>54</v>
@@ -88922,16 +89214,16 @@
         <v>2223</v>
       </c>
       <c r="B1639" t="s">
-        <v>2284</v>
+        <v>2278</v>
       </c>
       <c r="C1639" t="s">
-        <v>2285</v>
+        <v>2279</v>
       </c>
       <c r="D1639" t="s">
         <v>2223</v>
       </c>
       <c r="E1639" t="s">
-        <v>2286</v>
+        <v>2280</v>
       </c>
       <c r="F1639" t="s">
         <v>54</v>
@@ -88960,16 +89252,16 @@
         <v>2223</v>
       </c>
       <c r="B1640" t="s">
-        <v>2287</v>
+        <v>2281</v>
       </c>
       <c r="C1640" t="s">
-        <v>2288</v>
+        <v>2282</v>
       </c>
       <c r="D1640" t="s">
         <v>2223</v>
       </c>
       <c r="E1640" t="s">
-        <v>2289</v>
+        <v>2283</v>
       </c>
       <c r="F1640" t="s">
         <v>54</v>
@@ -88998,16 +89290,16 @@
         <v>2223</v>
       </c>
       <c r="B1641" t="s">
-        <v>2290</v>
+        <v>2284</v>
       </c>
       <c r="C1641" t="s">
-        <v>2291</v>
+        <v>2285</v>
       </c>
       <c r="D1641" t="s">
         <v>2223</v>
       </c>
       <c r="E1641" t="s">
-        <v>2292</v>
+        <v>2286</v>
       </c>
       <c r="F1641" t="s">
         <v>54</v>
@@ -89036,16 +89328,16 @@
         <v>2223</v>
       </c>
       <c r="B1642" t="s">
-        <v>2293</v>
+        <v>2287</v>
       </c>
       <c r="C1642" t="s">
-        <v>2294</v>
+        <v>2288</v>
       </c>
       <c r="D1642" t="s">
         <v>2223</v>
       </c>
       <c r="E1642" t="s">
-        <v>2295</v>
+        <v>2289</v>
       </c>
       <c r="F1642" t="s">
         <v>54</v>
@@ -89074,16 +89366,16 @@
         <v>2223</v>
       </c>
       <c r="B1643" t="s">
-        <v>2296</v>
+        <v>2290</v>
       </c>
       <c r="C1643" t="s">
-        <v>2297</v>
+        <v>2291</v>
       </c>
       <c r="D1643" t="s">
         <v>2223</v>
       </c>
       <c r="E1643" t="s">
-        <v>2298</v>
+        <v>2292</v>
       </c>
       <c r="F1643" t="s">
         <v>54</v>
@@ -89112,16 +89404,16 @@
         <v>2223</v>
       </c>
       <c r="B1644" t="s">
-        <v>2299</v>
+        <v>2293</v>
       </c>
       <c r="C1644" t="s">
-        <v>2300</v>
+        <v>2294</v>
       </c>
       <c r="D1644" t="s">
         <v>2223</v>
       </c>
       <c r="E1644" t="s">
-        <v>2301</v>
+        <v>2295</v>
       </c>
       <c r="F1644" t="s">
         <v>54</v>
@@ -89150,16 +89442,16 @@
         <v>2223</v>
       </c>
       <c r="B1645" t="s">
-        <v>2302</v>
+        <v>2296</v>
       </c>
       <c r="C1645" t="s">
-        <v>2303</v>
+        <v>2297</v>
       </c>
       <c r="D1645" t="s">
         <v>2223</v>
       </c>
       <c r="E1645" t="s">
-        <v>2304</v>
+        <v>2298</v>
       </c>
       <c r="F1645" t="s">
         <v>54</v>
@@ -89188,16 +89480,16 @@
         <v>2223</v>
       </c>
       <c r="B1646" t="s">
-        <v>2305</v>
+        <v>2299</v>
       </c>
       <c r="C1646" t="s">
-        <v>2306</v>
+        <v>2300</v>
       </c>
       <c r="D1646" t="s">
         <v>2223</v>
       </c>
       <c r="E1646" t="s">
-        <v>2307</v>
+        <v>2301</v>
       </c>
       <c r="F1646" t="s">
         <v>54</v>
@@ -89226,16 +89518,16 @@
         <v>2223</v>
       </c>
       <c r="B1647" t="s">
-        <v>2308</v>
+        <v>2302</v>
       </c>
       <c r="C1647" t="s">
-        <v>2309</v>
+        <v>2303</v>
       </c>
       <c r="D1647" t="s">
         <v>2223</v>
       </c>
       <c r="E1647" t="s">
-        <v>2310</v>
+        <v>2304</v>
       </c>
       <c r="F1647" t="s">
         <v>54</v>
@@ -89264,16 +89556,16 @@
         <v>2223</v>
       </c>
       <c r="B1648" t="s">
-        <v>2311</v>
+        <v>2305</v>
       </c>
       <c r="C1648" t="s">
-        <v>2312</v>
+        <v>2306</v>
       </c>
       <c r="D1648" t="s">
         <v>2223</v>
       </c>
       <c r="E1648" t="s">
-        <v>2313</v>
+        <v>2307</v>
       </c>
       <c r="F1648" t="s">
         <v>54</v>
@@ -89302,16 +89594,16 @@
         <v>2223</v>
       </c>
       <c r="B1649" t="s">
-        <v>2314</v>
+        <v>2308</v>
       </c>
       <c r="C1649" t="s">
-        <v>2315</v>
+        <v>2309</v>
       </c>
       <c r="D1649" t="s">
         <v>2223</v>
       </c>
       <c r="E1649" t="s">
-        <v>2316</v>
+        <v>2310</v>
       </c>
       <c r="F1649" t="s">
         <v>54</v>
@@ -89340,16 +89632,16 @@
         <v>2223</v>
       </c>
       <c r="B1650" t="s">
-        <v>2317</v>
+        <v>2311</v>
       </c>
       <c r="C1650" t="s">
-        <v>2318</v>
+        <v>2312</v>
       </c>
       <c r="D1650" t="s">
         <v>2223</v>
       </c>
       <c r="E1650" t="s">
-        <v>2319</v>
+        <v>2313</v>
       </c>
       <c r="F1650" t="s">
         <v>54</v>
@@ -89378,16 +89670,16 @@
         <v>2223</v>
       </c>
       <c r="B1651" t="s">
-        <v>2320</v>
+        <v>2314</v>
       </c>
       <c r="C1651" t="s">
-        <v>2321</v>
+        <v>2315</v>
       </c>
       <c r="D1651" t="s">
         <v>2223</v>
       </c>
       <c r="E1651" t="s">
-        <v>2322</v>
+        <v>2316</v>
       </c>
       <c r="F1651" t="s">
         <v>54</v>
@@ -89416,16 +89708,16 @@
         <v>2223</v>
       </c>
       <c r="B1652" t="s">
-        <v>2323</v>
+        <v>2317</v>
       </c>
       <c r="C1652" t="s">
-        <v>2324</v>
+        <v>2318</v>
       </c>
       <c r="D1652" t="s">
         <v>2223</v>
       </c>
       <c r="E1652" t="s">
-        <v>2325</v>
+        <v>2319</v>
       </c>
       <c r="F1652" t="s">
         <v>54</v>
@@ -89454,16 +89746,16 @@
         <v>2223</v>
       </c>
       <c r="B1653" t="s">
-        <v>2326</v>
+        <v>2320</v>
       </c>
       <c r="C1653" t="s">
-        <v>2327</v>
+        <v>2321</v>
       </c>
       <c r="D1653" t="s">
         <v>2223</v>
       </c>
       <c r="E1653" t="s">
-        <v>2328</v>
+        <v>2322</v>
       </c>
       <c r="F1653" t="s">
         <v>54</v>
@@ -89492,16 +89784,16 @@
         <v>2223</v>
       </c>
       <c r="B1654" t="s">
-        <v>2329</v>
+        <v>2323</v>
       </c>
       <c r="C1654" t="s">
-        <v>2330</v>
+        <v>2324</v>
       </c>
       <c r="D1654" t="s">
         <v>2223</v>
       </c>
       <c r="E1654" t="s">
-        <v>2331</v>
+        <v>2325</v>
       </c>
       <c r="F1654" t="s">
         <v>54</v>
@@ -89530,16 +89822,16 @@
         <v>2223</v>
       </c>
       <c r="B1655" t="s">
-        <v>2332</v>
+        <v>2326</v>
       </c>
       <c r="C1655" t="s">
-        <v>2333</v>
+        <v>2327</v>
       </c>
       <c r="D1655" t="s">
         <v>2223</v>
       </c>
       <c r="E1655" t="s">
-        <v>2334</v>
+        <v>2328</v>
       </c>
       <c r="F1655" t="s">
         <v>54</v>
@@ -89568,16 +89860,16 @@
         <v>2223</v>
       </c>
       <c r="B1656" t="s">
-        <v>2335</v>
+        <v>2329</v>
       </c>
       <c r="C1656" t="s">
-        <v>2336</v>
+        <v>2330</v>
       </c>
       <c r="D1656" t="s">
         <v>2223</v>
       </c>
       <c r="E1656" t="s">
-        <v>2337</v>
+        <v>2331</v>
       </c>
       <c r="F1656" t="s">
         <v>54</v>
@@ -89606,16 +89898,16 @@
         <v>2223</v>
       </c>
       <c r="B1657" t="s">
-        <v>2338</v>
+        <v>2332</v>
       </c>
       <c r="C1657" t="s">
-        <v>2339</v>
+        <v>2333</v>
       </c>
       <c r="D1657" t="s">
         <v>2223</v>
       </c>
       <c r="E1657" t="s">
-        <v>2340</v>
+        <v>2334</v>
       </c>
       <c r="F1657" t="s">
         <v>54</v>
@@ -89644,16 +89936,16 @@
         <v>2223</v>
       </c>
       <c r="B1658" t="s">
-        <v>2341</v>
+        <v>2335</v>
       </c>
       <c r="C1658" t="s">
-        <v>2342</v>
+        <v>2336</v>
       </c>
       <c r="D1658" t="s">
         <v>2223</v>
       </c>
       <c r="E1658" t="s">
-        <v>2343</v>
+        <v>2337</v>
       </c>
       <c r="F1658" t="s">
         <v>54</v>
@@ -89682,16 +89974,16 @@
         <v>2223</v>
       </c>
       <c r="B1659" t="s">
-        <v>2344</v>
+        <v>2338</v>
       </c>
       <c r="C1659" t="s">
-        <v>2345</v>
+        <v>2339</v>
       </c>
       <c r="D1659" t="s">
         <v>2223</v>
       </c>
       <c r="E1659" t="s">
-        <v>2346</v>
+        <v>2340</v>
       </c>
       <c r="F1659" t="s">
         <v>54</v>
@@ -89720,16 +90012,16 @@
         <v>2223</v>
       </c>
       <c r="B1660" t="s">
-        <v>2347</v>
+        <v>2341</v>
       </c>
       <c r="C1660" t="s">
-        <v>2348</v>
+        <v>2342</v>
       </c>
       <c r="D1660" t="s">
         <v>2223</v>
       </c>
       <c r="E1660" t="s">
-        <v>2349</v>
+        <v>2343</v>
       </c>
       <c r="F1660" t="s">
         <v>54</v>
@@ -89758,16 +90050,16 @@
         <v>2223</v>
       </c>
       <c r="B1661" t="s">
-        <v>2350</v>
+        <v>2344</v>
       </c>
       <c r="C1661" t="s">
-        <v>2351</v>
+        <v>2345</v>
       </c>
       <c r="D1661" t="s">
         <v>2223</v>
       </c>
       <c r="E1661" t="s">
-        <v>2352</v>
+        <v>2346</v>
       </c>
       <c r="F1661" t="s">
         <v>54</v>
@@ -89796,16 +90088,16 @@
         <v>2223</v>
       </c>
       <c r="B1662" t="s">
-        <v>2353</v>
+        <v>2347</v>
       </c>
       <c r="C1662" t="s">
-        <v>2354</v>
+        <v>2348</v>
       </c>
       <c r="D1662" t="s">
         <v>2223</v>
       </c>
       <c r="E1662" t="s">
-        <v>2355</v>
+        <v>2349</v>
       </c>
       <c r="F1662" t="s">
         <v>54</v>
@@ -89834,16 +90126,16 @@
         <v>2223</v>
       </c>
       <c r="B1663" t="s">
-        <v>2356</v>
+        <v>2350</v>
       </c>
       <c r="C1663" t="s">
-        <v>2357</v>
+        <v>2351</v>
       </c>
       <c r="D1663" t="s">
         <v>2223</v>
       </c>
       <c r="E1663" t="s">
-        <v>2358</v>
+        <v>2352</v>
       </c>
       <c r="F1663" t="s">
         <v>54</v>
@@ -89872,16 +90164,16 @@
         <v>2223</v>
       </c>
       <c r="B1664" t="s">
-        <v>2359</v>
+        <v>2353</v>
       </c>
       <c r="C1664" t="s">
-        <v>2360</v>
+        <v>2354</v>
       </c>
       <c r="D1664" t="s">
         <v>2223</v>
       </c>
       <c r="E1664" t="s">
-        <v>2361</v>
+        <v>2355</v>
       </c>
       <c r="F1664" t="s">
         <v>54</v>
@@ -89910,16 +90202,16 @@
         <v>2223</v>
       </c>
       <c r="B1665" t="s">
-        <v>2362</v>
+        <v>2356</v>
       </c>
       <c r="C1665" t="s">
-        <v>2363</v>
+        <v>2357</v>
       </c>
       <c r="D1665" t="s">
         <v>2223</v>
       </c>
       <c r="E1665" t="s">
-        <v>2364</v>
+        <v>2358</v>
       </c>
       <c r="F1665" t="s">
         <v>54</v>
@@ -89948,16 +90240,16 @@
         <v>2223</v>
       </c>
       <c r="B1666" t="s">
-        <v>2365</v>
+        <v>2359</v>
       </c>
       <c r="C1666" t="s">
-        <v>2366</v>
+        <v>2360</v>
       </c>
       <c r="D1666" t="s">
         <v>2223</v>
       </c>
       <c r="E1666" t="s">
-        <v>2367</v>
+        <v>2361</v>
       </c>
       <c r="F1666" t="s">
         <v>54</v>
@@ -89986,16 +90278,16 @@
         <v>2223</v>
       </c>
       <c r="B1667" t="s">
-        <v>2368</v>
+        <v>2362</v>
       </c>
       <c r="C1667" t="s">
-        <v>2369</v>
+        <v>2363</v>
       </c>
       <c r="D1667" t="s">
         <v>2223</v>
       </c>
       <c r="E1667" t="s">
-        <v>2370</v>
+        <v>2364</v>
       </c>
       <c r="F1667" t="s">
         <v>54</v>
@@ -90024,16 +90316,16 @@
         <v>2223</v>
       </c>
       <c r="B1668" t="s">
-        <v>2371</v>
+        <v>2365</v>
       </c>
       <c r="C1668" t="s">
-        <v>2372</v>
+        <v>2366</v>
       </c>
       <c r="D1668" t="s">
         <v>2223</v>
       </c>
       <c r="E1668" t="s">
-        <v>2373</v>
+        <v>2367</v>
       </c>
       <c r="F1668" t="s">
         <v>54</v>
@@ -90062,16 +90354,16 @@
         <v>2223</v>
       </c>
       <c r="B1669" t="s">
-        <v>2374</v>
+        <v>2368</v>
       </c>
       <c r="C1669" t="s">
-        <v>2375</v>
+        <v>2369</v>
       </c>
       <c r="D1669" t="s">
         <v>2223</v>
       </c>
       <c r="E1669" t="s">
-        <v>2376</v>
+        <v>2370</v>
       </c>
       <c r="F1669" t="s">
         <v>54</v>
@@ -90100,16 +90392,16 @@
         <v>2223</v>
       </c>
       <c r="B1670" t="s">
-        <v>2377</v>
+        <v>2371</v>
       </c>
       <c r="C1670" t="s">
-        <v>2378</v>
+        <v>2372</v>
       </c>
       <c r="D1670" t="s">
         <v>2223</v>
       </c>
       <c r="E1670" t="s">
-        <v>2379</v>
+        <v>2373</v>
       </c>
       <c r="F1670" t="s">
         <v>54</v>
@@ -90138,16 +90430,16 @@
         <v>2223</v>
       </c>
       <c r="B1671" t="s">
-        <v>2380</v>
+        <v>2374</v>
       </c>
       <c r="C1671" t="s">
-        <v>2381</v>
+        <v>2375</v>
       </c>
       <c r="D1671" t="s">
         <v>2223</v>
       </c>
       <c r="E1671" t="s">
-        <v>2382</v>
+        <v>2376</v>
       </c>
       <c r="F1671" t="s">
         <v>54</v>
@@ -90176,16 +90468,16 @@
         <v>2223</v>
       </c>
       <c r="B1672" t="s">
-        <v>2383</v>
+        <v>2377</v>
       </c>
       <c r="C1672" t="s">
-        <v>2384</v>
+        <v>2378</v>
       </c>
       <c r="D1672" t="s">
         <v>2223</v>
       </c>
       <c r="E1672" t="s">
-        <v>2385</v>
+        <v>2379</v>
       </c>
       <c r="F1672" t="s">
         <v>54</v>
@@ -90214,16 +90506,16 @@
         <v>2223</v>
       </c>
       <c r="B1673" t="s">
-        <v>2386</v>
+        <v>2380</v>
       </c>
       <c r="C1673" t="s">
-        <v>2387</v>
+        <v>2381</v>
       </c>
       <c r="D1673" t="s">
         <v>2223</v>
       </c>
       <c r="E1673" t="s">
-        <v>2388</v>
+        <v>2382</v>
       </c>
       <c r="F1673" t="s">
         <v>54</v>
@@ -90252,16 +90544,16 @@
         <v>2223</v>
       </c>
       <c r="B1674" t="s">
-        <v>2389</v>
+        <v>2383</v>
       </c>
       <c r="C1674" t="s">
-        <v>2390</v>
+        <v>2384</v>
       </c>
       <c r="D1674" t="s">
         <v>2223</v>
       </c>
       <c r="E1674" t="s">
-        <v>2391</v>
+        <v>2385</v>
       </c>
       <c r="F1674" t="s">
         <v>54</v>
@@ -90290,16 +90582,16 @@
         <v>2223</v>
       </c>
       <c r="B1675" t="s">
-        <v>2392</v>
+        <v>2386</v>
       </c>
       <c r="C1675" t="s">
-        <v>2393</v>
+        <v>2387</v>
       </c>
       <c r="D1675" t="s">
         <v>2223</v>
       </c>
       <c r="E1675" t="s">
-        <v>2394</v>
+        <v>2388</v>
       </c>
       <c r="F1675" t="s">
         <v>54</v>
@@ -90328,16 +90620,16 @@
         <v>2223</v>
       </c>
       <c r="B1676" t="s">
-        <v>2395</v>
+        <v>2389</v>
       </c>
       <c r="C1676" t="s">
-        <v>2396</v>
+        <v>2390</v>
       </c>
       <c r="D1676" t="s">
         <v>2223</v>
       </c>
       <c r="E1676" t="s">
-        <v>2397</v>
+        <v>2391</v>
       </c>
       <c r="F1676" t="s">
         <v>54</v>
@@ -90366,16 +90658,16 @@
         <v>2223</v>
       </c>
       <c r="B1677" t="s">
-        <v>2398</v>
+        <v>2392</v>
       </c>
       <c r="C1677" t="s">
-        <v>2399</v>
+        <v>2393</v>
       </c>
       <c r="D1677" t="s">
         <v>2223</v>
       </c>
       <c r="E1677" t="s">
-        <v>2400</v>
+        <v>2394</v>
       </c>
       <c r="F1677" t="s">
         <v>54</v>
@@ -90404,16 +90696,16 @@
         <v>2223</v>
       </c>
       <c r="B1678" t="s">
-        <v>2401</v>
+        <v>2395</v>
       </c>
       <c r="C1678" t="s">
-        <v>2402</v>
+        <v>2396</v>
       </c>
       <c r="D1678" t="s">
         <v>2223</v>
       </c>
       <c r="E1678" t="s">
-        <v>2403</v>
+        <v>2397</v>
       </c>
       <c r="F1678" t="s">
         <v>54</v>
@@ -90442,16 +90734,16 @@
         <v>2223</v>
       </c>
       <c r="B1679" t="s">
-        <v>2404</v>
+        <v>2398</v>
       </c>
       <c r="C1679" t="s">
-        <v>2405</v>
+        <v>2399</v>
       </c>
       <c r="D1679" t="s">
         <v>2223</v>
       </c>
       <c r="E1679" t="s">
-        <v>2406</v>
+        <v>2400</v>
       </c>
       <c r="F1679" t="s">
         <v>54</v>
@@ -90480,16 +90772,16 @@
         <v>2223</v>
       </c>
       <c r="B1680" t="s">
-        <v>2407</v>
+        <v>2401</v>
       </c>
       <c r="C1680" t="s">
-        <v>2408</v>
+        <v>2402</v>
       </c>
       <c r="D1680" t="s">
         <v>2223</v>
       </c>
       <c r="E1680" t="s">
-        <v>2409</v>
+        <v>2403</v>
       </c>
       <c r="F1680" t="s">
         <v>54</v>
@@ -90518,16 +90810,16 @@
         <v>2223</v>
       </c>
       <c r="B1681" t="s">
-        <v>2410</v>
+        <v>2404</v>
       </c>
       <c r="C1681" t="s">
-        <v>2411</v>
+        <v>2405</v>
       </c>
       <c r="D1681" t="s">
         <v>2223</v>
       </c>
       <c r="E1681" t="s">
-        <v>2412</v>
+        <v>2406</v>
       </c>
       <c r="F1681" t="s">
         <v>54</v>
@@ -90556,16 +90848,16 @@
         <v>2223</v>
       </c>
       <c r="B1682" t="s">
-        <v>2413</v>
+        <v>2407</v>
       </c>
       <c r="C1682" t="s">
-        <v>2414</v>
+        <v>2408</v>
       </c>
       <c r="D1682" t="s">
         <v>2223</v>
       </c>
       <c r="E1682" t="s">
-        <v>2415</v>
+        <v>2409</v>
       </c>
       <c r="F1682" t="s">
         <v>54</v>
@@ -90594,16 +90886,16 @@
         <v>2223</v>
       </c>
       <c r="B1683" t="s">
-        <v>2416</v>
+        <v>2410</v>
       </c>
       <c r="C1683" t="s">
-        <v>2241</v>
+        <v>2411</v>
       </c>
       <c r="D1683" t="s">
         <v>2223</v>
       </c>
       <c r="E1683" t="s">
-        <v>2242</v>
+        <v>2412</v>
       </c>
       <c r="F1683" t="s">
         <v>54</v>
@@ -90632,31 +90924,37 @@
         <v>2223</v>
       </c>
       <c r="B1684" t="s">
-        <v>50</v>
+        <v>2413</v>
       </c>
       <c r="C1684" t="s">
-        <v>50</v>
+        <v>2414</v>
       </c>
       <c r="D1684" t="s">
-        <v>50</v>
+        <v>2223</v>
       </c>
       <c r="E1684" t="s">
-        <v>50</v>
+        <v>2415</v>
       </c>
       <c r="F1684" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="G1684" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="H1684" t="s">
-        <v>50</v>
+        <v>29</v>
       </c>
       <c r="I1684" t="s">
-        <v>50</v>
+        <v>30</v>
       </c>
       <c r="J1684" t="s">
-        <v>50</v>
+        <v>29</v>
+      </c>
+      <c r="K1684" t="s">
+        <v>39</v>
+      </c>
+      <c r="L1684" t="s">
+        <v>54</v>
       </c>
     </row>
     <row r="1685">
@@ -90664,30 +90962,1665 @@
         <v>2223</v>
       </c>
       <c r="B1685" t="s">
-        <v>230</v>
+        <v>2416</v>
       </c>
       <c r="C1685" t="s">
         <v>2417</v>
       </c>
       <c r="D1685" t="s">
-        <v>50</v>
+        <v>2223</v>
       </c>
       <c r="E1685" t="s">
+        <v>2418</v>
+      </c>
+      <c r="F1685" t="s">
+        <v>54</v>
+      </c>
+      <c r="G1685" t="s">
+        <v>55</v>
+      </c>
+      <c r="H1685" t="s">
+        <v>29</v>
+      </c>
+      <c r="I1685" t="s">
+        <v>30</v>
+      </c>
+      <c r="J1685" t="s">
+        <v>29</v>
+      </c>
+      <c r="K1685" t="s">
+        <v>39</v>
+      </c>
+      <c r="L1685" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="1686">
+      <c r="A1686" t="s">
+        <v>2223</v>
+      </c>
+      <c r="B1686" t="s">
+        <v>2419</v>
+      </c>
+      <c r="C1686" t="s">
+        <v>2420</v>
+      </c>
+      <c r="D1686" t="s">
+        <v>2223</v>
+      </c>
+      <c r="E1686" t="s">
+        <v>2421</v>
+      </c>
+      <c r="F1686" t="s">
+        <v>54</v>
+      </c>
+      <c r="G1686" t="s">
+        <v>55</v>
+      </c>
+      <c r="H1686" t="s">
+        <v>29</v>
+      </c>
+      <c r="I1686" t="s">
+        <v>30</v>
+      </c>
+      <c r="J1686" t="s">
+        <v>29</v>
+      </c>
+      <c r="K1686" t="s">
+        <v>39</v>
+      </c>
+      <c r="L1686" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="1687">
+      <c r="A1687" t="s">
+        <v>2223</v>
+      </c>
+      <c r="B1687" t="s">
+        <v>2422</v>
+      </c>
+      <c r="C1687" t="s">
+        <v>2423</v>
+      </c>
+      <c r="D1687" t="s">
+        <v>2223</v>
+      </c>
+      <c r="E1687" t="s">
+        <v>2424</v>
+      </c>
+      <c r="F1687" t="s">
+        <v>54</v>
+      </c>
+      <c r="G1687" t="s">
+        <v>55</v>
+      </c>
+      <c r="H1687" t="s">
+        <v>29</v>
+      </c>
+      <c r="I1687" t="s">
+        <v>30</v>
+      </c>
+      <c r="J1687" t="s">
+        <v>29</v>
+      </c>
+      <c r="K1687" t="s">
+        <v>39</v>
+      </c>
+      <c r="L1687" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="1688">
+      <c r="A1688" t="s">
+        <v>2223</v>
+      </c>
+      <c r="B1688" t="s">
+        <v>2425</v>
+      </c>
+      <c r="C1688" t="s">
+        <v>2426</v>
+      </c>
+      <c r="D1688" t="s">
+        <v>2223</v>
+      </c>
+      <c r="E1688" t="s">
+        <v>2427</v>
+      </c>
+      <c r="F1688" t="s">
+        <v>54</v>
+      </c>
+      <c r="G1688" t="s">
+        <v>55</v>
+      </c>
+      <c r="H1688" t="s">
+        <v>29</v>
+      </c>
+      <c r="I1688" t="s">
+        <v>30</v>
+      </c>
+      <c r="J1688" t="s">
+        <v>29</v>
+      </c>
+      <c r="K1688" t="s">
+        <v>39</v>
+      </c>
+      <c r="L1688" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="1689">
+      <c r="A1689" t="s">
+        <v>2223</v>
+      </c>
+      <c r="B1689" t="s">
+        <v>2428</v>
+      </c>
+      <c r="C1689" t="s">
+        <v>2429</v>
+      </c>
+      <c r="D1689" t="s">
+        <v>2223</v>
+      </c>
+      <c r="E1689" t="s">
+        <v>2430</v>
+      </c>
+      <c r="F1689" t="s">
+        <v>54</v>
+      </c>
+      <c r="G1689" t="s">
+        <v>55</v>
+      </c>
+      <c r="H1689" t="s">
+        <v>29</v>
+      </c>
+      <c r="I1689" t="s">
+        <v>30</v>
+      </c>
+      <c r="J1689" t="s">
+        <v>29</v>
+      </c>
+      <c r="K1689" t="s">
+        <v>39</v>
+      </c>
+      <c r="L1689" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="1690">
+      <c r="A1690" t="s">
+        <v>2223</v>
+      </c>
+      <c r="B1690" t="s">
+        <v>2431</v>
+      </c>
+      <c r="C1690" t="s">
+        <v>2432</v>
+      </c>
+      <c r="D1690" t="s">
+        <v>2223</v>
+      </c>
+      <c r="E1690" t="s">
+        <v>2433</v>
+      </c>
+      <c r="F1690" t="s">
+        <v>54</v>
+      </c>
+      <c r="G1690" t="s">
+        <v>55</v>
+      </c>
+      <c r="H1690" t="s">
+        <v>29</v>
+      </c>
+      <c r="I1690" t="s">
+        <v>30</v>
+      </c>
+      <c r="J1690" t="s">
+        <v>29</v>
+      </c>
+      <c r="K1690" t="s">
+        <v>39</v>
+      </c>
+      <c r="L1690" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="1691">
+      <c r="A1691" t="s">
+        <v>2223</v>
+      </c>
+      <c r="B1691" t="s">
+        <v>2434</v>
+      </c>
+      <c r="C1691" t="s">
+        <v>2435</v>
+      </c>
+      <c r="D1691" t="s">
+        <v>2223</v>
+      </c>
+      <c r="E1691" t="s">
+        <v>2436</v>
+      </c>
+      <c r="F1691" t="s">
+        <v>54</v>
+      </c>
+      <c r="G1691" t="s">
+        <v>55</v>
+      </c>
+      <c r="H1691" t="s">
+        <v>29</v>
+      </c>
+      <c r="I1691" t="s">
+        <v>30</v>
+      </c>
+      <c r="J1691" t="s">
+        <v>29</v>
+      </c>
+      <c r="K1691" t="s">
+        <v>39</v>
+      </c>
+      <c r="L1691" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="1692">
+      <c r="A1692" t="s">
+        <v>2223</v>
+      </c>
+      <c r="B1692" t="s">
+        <v>2437</v>
+      </c>
+      <c r="C1692" t="s">
+        <v>2438</v>
+      </c>
+      <c r="D1692" t="s">
+        <v>2223</v>
+      </c>
+      <c r="E1692" t="s">
+        <v>2439</v>
+      </c>
+      <c r="F1692" t="s">
+        <v>54</v>
+      </c>
+      <c r="G1692" t="s">
+        <v>55</v>
+      </c>
+      <c r="H1692" t="s">
+        <v>29</v>
+      </c>
+      <c r="I1692" t="s">
+        <v>30</v>
+      </c>
+      <c r="J1692" t="s">
+        <v>29</v>
+      </c>
+      <c r="K1692" t="s">
+        <v>39</v>
+      </c>
+      <c r="L1692" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="1693">
+      <c r="A1693" t="s">
+        <v>2223</v>
+      </c>
+      <c r="B1693" t="s">
+        <v>2440</v>
+      </c>
+      <c r="C1693" t="s">
+        <v>2441</v>
+      </c>
+      <c r="D1693" t="s">
+        <v>2223</v>
+      </c>
+      <c r="E1693" t="s">
+        <v>2442</v>
+      </c>
+      <c r="F1693" t="s">
+        <v>54</v>
+      </c>
+      <c r="G1693" t="s">
+        <v>55</v>
+      </c>
+      <c r="H1693" t="s">
+        <v>29</v>
+      </c>
+      <c r="I1693" t="s">
+        <v>30</v>
+      </c>
+      <c r="J1693" t="s">
+        <v>29</v>
+      </c>
+      <c r="K1693" t="s">
+        <v>39</v>
+      </c>
+      <c r="L1693" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="1694">
+      <c r="A1694" t="s">
+        <v>2223</v>
+      </c>
+      <c r="B1694" t="s">
+        <v>2443</v>
+      </c>
+      <c r="C1694" t="s">
+        <v>2444</v>
+      </c>
+      <c r="D1694" t="s">
+        <v>2223</v>
+      </c>
+      <c r="E1694" t="s">
+        <v>2445</v>
+      </c>
+      <c r="F1694" t="s">
+        <v>54</v>
+      </c>
+      <c r="G1694" t="s">
+        <v>55</v>
+      </c>
+      <c r="H1694" t="s">
+        <v>29</v>
+      </c>
+      <c r="I1694" t="s">
+        <v>30</v>
+      </c>
+      <c r="J1694" t="s">
+        <v>29</v>
+      </c>
+      <c r="K1694" t="s">
+        <v>39</v>
+      </c>
+      <c r="L1694" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="1695">
+      <c r="A1695" t="s">
+        <v>2223</v>
+      </c>
+      <c r="B1695" t="s">
+        <v>2446</v>
+      </c>
+      <c r="C1695" t="s">
+        <v>2447</v>
+      </c>
+      <c r="D1695" t="s">
+        <v>2223</v>
+      </c>
+      <c r="E1695" t="s">
+        <v>2448</v>
+      </c>
+      <c r="F1695" t="s">
+        <v>54</v>
+      </c>
+      <c r="G1695" t="s">
+        <v>55</v>
+      </c>
+      <c r="H1695" t="s">
+        <v>29</v>
+      </c>
+      <c r="I1695" t="s">
+        <v>30</v>
+      </c>
+      <c r="J1695" t="s">
+        <v>29</v>
+      </c>
+      <c r="K1695" t="s">
+        <v>39</v>
+      </c>
+      <c r="L1695" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="1696">
+      <c r="A1696" t="s">
+        <v>2223</v>
+      </c>
+      <c r="B1696" t="s">
+        <v>2449</v>
+      </c>
+      <c r="C1696" t="s">
+        <v>2450</v>
+      </c>
+      <c r="D1696" t="s">
+        <v>2223</v>
+      </c>
+      <c r="E1696" t="s">
+        <v>2451</v>
+      </c>
+      <c r="F1696" t="s">
+        <v>54</v>
+      </c>
+      <c r="G1696" t="s">
+        <v>55</v>
+      </c>
+      <c r="H1696" t="s">
+        <v>29</v>
+      </c>
+      <c r="I1696" t="s">
+        <v>30</v>
+      </c>
+      <c r="J1696" t="s">
+        <v>29</v>
+      </c>
+      <c r="K1696" t="s">
+        <v>39</v>
+      </c>
+      <c r="L1696" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="1697">
+      <c r="A1697" t="s">
+        <v>2223</v>
+      </c>
+      <c r="B1697" t="s">
+        <v>2452</v>
+      </c>
+      <c r="C1697" t="s">
+        <v>2453</v>
+      </c>
+      <c r="D1697" t="s">
+        <v>2223</v>
+      </c>
+      <c r="E1697" t="s">
+        <v>2454</v>
+      </c>
+      <c r="F1697" t="s">
+        <v>54</v>
+      </c>
+      <c r="G1697" t="s">
+        <v>55</v>
+      </c>
+      <c r="H1697" t="s">
+        <v>29</v>
+      </c>
+      <c r="I1697" t="s">
+        <v>30</v>
+      </c>
+      <c r="J1697" t="s">
+        <v>29</v>
+      </c>
+      <c r="K1697" t="s">
+        <v>39</v>
+      </c>
+      <c r="L1697" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="1698">
+      <c r="A1698" t="s">
+        <v>2223</v>
+      </c>
+      <c r="B1698" t="s">
+        <v>2455</v>
+      </c>
+      <c r="C1698" t="s">
+        <v>2456</v>
+      </c>
+      <c r="D1698" t="s">
+        <v>2223</v>
+      </c>
+      <c r="E1698" t="s">
+        <v>2457</v>
+      </c>
+      <c r="F1698" t="s">
+        <v>54</v>
+      </c>
+      <c r="G1698" t="s">
+        <v>55</v>
+      </c>
+      <c r="H1698" t="s">
+        <v>29</v>
+      </c>
+      <c r="I1698" t="s">
+        <v>30</v>
+      </c>
+      <c r="J1698" t="s">
+        <v>29</v>
+      </c>
+      <c r="K1698" t="s">
+        <v>39</v>
+      </c>
+      <c r="L1698" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="1699">
+      <c r="A1699" t="s">
+        <v>2223</v>
+      </c>
+      <c r="B1699" t="s">
+        <v>2458</v>
+      </c>
+      <c r="C1699" t="s">
+        <v>2459</v>
+      </c>
+      <c r="D1699" t="s">
+        <v>2223</v>
+      </c>
+      <c r="E1699" t="s">
+        <v>2460</v>
+      </c>
+      <c r="F1699" t="s">
+        <v>54</v>
+      </c>
+      <c r="G1699" t="s">
+        <v>55</v>
+      </c>
+      <c r="H1699" t="s">
+        <v>29</v>
+      </c>
+      <c r="I1699" t="s">
+        <v>30</v>
+      </c>
+      <c r="J1699" t="s">
+        <v>29</v>
+      </c>
+      <c r="K1699" t="s">
+        <v>39</v>
+      </c>
+      <c r="L1699" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="1700">
+      <c r="A1700" t="s">
+        <v>2223</v>
+      </c>
+      <c r="B1700" t="s">
+        <v>2461</v>
+      </c>
+      <c r="C1700" t="s">
+        <v>2462</v>
+      </c>
+      <c r="D1700" t="s">
+        <v>2223</v>
+      </c>
+      <c r="E1700" t="s">
+        <v>2463</v>
+      </c>
+      <c r="F1700" t="s">
+        <v>180</v>
+      </c>
+      <c r="G1700" t="s">
+        <v>55</v>
+      </c>
+      <c r="H1700" t="s">
+        <v>29</v>
+      </c>
+      <c r="I1700" t="s">
+        <v>30</v>
+      </c>
+      <c r="J1700" t="s">
+        <v>50</v>
+      </c>
+      <c r="K1700" t="s">
+        <v>181</v>
+      </c>
+      <c r="L1700" t="s">
+        <v>180</v>
+      </c>
+      <c r="M1700" t="s">
+        <v>587</v>
+      </c>
+    </row>
+    <row r="1701">
+      <c r="A1701" t="s">
+        <v>2223</v>
+      </c>
+      <c r="B1701" t="s">
+        <v>2464</v>
+      </c>
+      <c r="C1701" t="s">
+        <v>2465</v>
+      </c>
+      <c r="D1701" t="s">
+        <v>2223</v>
+      </c>
+      <c r="E1701" t="s">
+        <v>2466</v>
+      </c>
+      <c r="F1701" t="s">
+        <v>180</v>
+      </c>
+      <c r="G1701" t="s">
+        <v>55</v>
+      </c>
+      <c r="H1701" t="s">
+        <v>29</v>
+      </c>
+      <c r="I1701" t="s">
+        <v>30</v>
+      </c>
+      <c r="J1701" t="s">
+        <v>50</v>
+      </c>
+      <c r="K1701" t="s">
+        <v>181</v>
+      </c>
+      <c r="L1701" t="s">
+        <v>180</v>
+      </c>
+      <c r="M1701" t="s">
+        <v>587</v>
+      </c>
+    </row>
+    <row r="1702">
+      <c r="A1702" t="s">
+        <v>2223</v>
+      </c>
+      <c r="B1702" t="s">
+        <v>2467</v>
+      </c>
+      <c r="C1702" t="s">
+        <v>2468</v>
+      </c>
+      <c r="D1702" t="s">
+        <v>2223</v>
+      </c>
+      <c r="E1702" t="s">
+        <v>2469</v>
+      </c>
+      <c r="F1702" t="s">
+        <v>180</v>
+      </c>
+      <c r="G1702" t="s">
+        <v>55</v>
+      </c>
+      <c r="H1702" t="s">
+        <v>29</v>
+      </c>
+      <c r="I1702" t="s">
+        <v>30</v>
+      </c>
+      <c r="J1702" t="s">
+        <v>50</v>
+      </c>
+      <c r="K1702" t="s">
+        <v>181</v>
+      </c>
+      <c r="L1702" t="s">
+        <v>180</v>
+      </c>
+      <c r="M1702" t="s">
+        <v>587</v>
+      </c>
+    </row>
+    <row r="1703">
+      <c r="A1703" t="s">
+        <v>2223</v>
+      </c>
+      <c r="B1703" t="s">
+        <v>2470</v>
+      </c>
+      <c r="C1703" t="s">
+        <v>2471</v>
+      </c>
+      <c r="D1703" t="s">
+        <v>2223</v>
+      </c>
+      <c r="E1703" t="s">
+        <v>2472</v>
+      </c>
+      <c r="F1703" t="s">
+        <v>180</v>
+      </c>
+      <c r="G1703" t="s">
+        <v>55</v>
+      </c>
+      <c r="H1703" t="s">
+        <v>29</v>
+      </c>
+      <c r="I1703" t="s">
+        <v>30</v>
+      </c>
+      <c r="J1703" t="s">
+        <v>50</v>
+      </c>
+      <c r="K1703" t="s">
+        <v>181</v>
+      </c>
+      <c r="L1703" t="s">
+        <v>180</v>
+      </c>
+      <c r="M1703" t="s">
+        <v>956</v>
+      </c>
+    </row>
+    <row r="1704">
+      <c r="A1704" t="s">
+        <v>2223</v>
+      </c>
+      <c r="B1704" t="s">
+        <v>2473</v>
+      </c>
+      <c r="C1704" t="s">
+        <v>2474</v>
+      </c>
+      <c r="D1704" t="s">
+        <v>2223</v>
+      </c>
+      <c r="E1704" t="s">
+        <v>2475</v>
+      </c>
+      <c r="F1704" t="s">
+        <v>180</v>
+      </c>
+      <c r="G1704" t="s">
+        <v>55</v>
+      </c>
+      <c r="H1704" t="s">
+        <v>29</v>
+      </c>
+      <c r="I1704" t="s">
+        <v>30</v>
+      </c>
+      <c r="J1704" t="s">
+        <v>50</v>
+      </c>
+      <c r="K1704" t="s">
+        <v>181</v>
+      </c>
+      <c r="L1704" t="s">
+        <v>180</v>
+      </c>
+      <c r="M1704" t="s">
+        <v>956</v>
+      </c>
+    </row>
+    <row r="1705">
+      <c r="A1705" t="s">
+        <v>2223</v>
+      </c>
+      <c r="B1705" t="s">
+        <v>2476</v>
+      </c>
+      <c r="C1705" t="s">
+        <v>2477</v>
+      </c>
+      <c r="D1705" t="s">
+        <v>2223</v>
+      </c>
+      <c r="E1705" t="s">
+        <v>2478</v>
+      </c>
+      <c r="F1705" t="s">
+        <v>180</v>
+      </c>
+      <c r="G1705" t="s">
+        <v>55</v>
+      </c>
+      <c r="H1705" t="s">
+        <v>29</v>
+      </c>
+      <c r="I1705" t="s">
+        <v>30</v>
+      </c>
+      <c r="J1705" t="s">
+        <v>50</v>
+      </c>
+      <c r="K1705" t="s">
+        <v>181</v>
+      </c>
+      <c r="L1705" t="s">
+        <v>180</v>
+      </c>
+      <c r="M1705" t="s">
+        <v>956</v>
+      </c>
+    </row>
+    <row r="1706">
+      <c r="A1706" t="s">
+        <v>2223</v>
+      </c>
+      <c r="B1706" t="s">
+        <v>2479</v>
+      </c>
+      <c r="C1706" t="s">
+        <v>2480</v>
+      </c>
+      <c r="D1706" t="s">
+        <v>2223</v>
+      </c>
+      <c r="E1706" t="s">
+        <v>2481</v>
+      </c>
+      <c r="F1706" t="s">
+        <v>180</v>
+      </c>
+      <c r="G1706" t="s">
+        <v>55</v>
+      </c>
+      <c r="H1706" t="s">
+        <v>29</v>
+      </c>
+      <c r="I1706" t="s">
+        <v>30</v>
+      </c>
+      <c r="J1706" t="s">
+        <v>50</v>
+      </c>
+      <c r="K1706" t="s">
+        <v>181</v>
+      </c>
+      <c r="L1706" t="s">
+        <v>180</v>
+      </c>
+      <c r="M1706" t="s">
+        <v>587</v>
+      </c>
+    </row>
+    <row r="1707">
+      <c r="A1707" t="s">
+        <v>2223</v>
+      </c>
+      <c r="B1707" t="s">
+        <v>2482</v>
+      </c>
+      <c r="C1707" t="s">
+        <v>2483</v>
+      </c>
+      <c r="D1707" t="s">
+        <v>2223</v>
+      </c>
+      <c r="E1707" t="s">
+        <v>2484</v>
+      </c>
+      <c r="F1707" t="s">
+        <v>54</v>
+      </c>
+      <c r="G1707" t="s">
+        <v>55</v>
+      </c>
+      <c r="H1707" t="s">
+        <v>29</v>
+      </c>
+      <c r="I1707" t="s">
+        <v>30</v>
+      </c>
+      <c r="J1707" t="s">
+        <v>29</v>
+      </c>
+      <c r="K1707" t="s">
+        <v>39</v>
+      </c>
+      <c r="L1707" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="1708">
+      <c r="A1708" t="s">
+        <v>2223</v>
+      </c>
+      <c r="B1708" t="s">
+        <v>2485</v>
+      </c>
+      <c r="C1708" t="s">
+        <v>2486</v>
+      </c>
+      <c r="D1708" t="s">
+        <v>2223</v>
+      </c>
+      <c r="E1708" t="s">
+        <v>2487</v>
+      </c>
+      <c r="F1708" t="s">
+        <v>54</v>
+      </c>
+      <c r="G1708" t="s">
+        <v>55</v>
+      </c>
+      <c r="H1708" t="s">
+        <v>29</v>
+      </c>
+      <c r="I1708" t="s">
+        <v>30</v>
+      </c>
+      <c r="J1708" t="s">
+        <v>29</v>
+      </c>
+      <c r="K1708" t="s">
+        <v>39</v>
+      </c>
+      <c r="L1708" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="1709">
+      <c r="A1709" t="s">
+        <v>2223</v>
+      </c>
+      <c r="B1709" t="s">
+        <v>2488</v>
+      </c>
+      <c r="C1709" t="s">
+        <v>2489</v>
+      </c>
+      <c r="D1709" t="s">
+        <v>2223</v>
+      </c>
+      <c r="E1709" t="s">
+        <v>2490</v>
+      </c>
+      <c r="F1709" t="s">
+        <v>180</v>
+      </c>
+      <c r="G1709" t="s">
+        <v>55</v>
+      </c>
+      <c r="H1709" t="s">
+        <v>29</v>
+      </c>
+      <c r="I1709" t="s">
+        <v>30</v>
+      </c>
+      <c r="J1709" t="s">
+        <v>50</v>
+      </c>
+      <c r="K1709" t="s">
+        <v>181</v>
+      </c>
+      <c r="L1709" t="s">
+        <v>180</v>
+      </c>
+      <c r="M1709" t="s">
+        <v>956</v>
+      </c>
+    </row>
+    <row r="1710">
+      <c r="A1710" t="s">
+        <v>2223</v>
+      </c>
+      <c r="B1710" t="s">
+        <v>2491</v>
+      </c>
+      <c r="C1710" t="s">
+        <v>2492</v>
+      </c>
+      <c r="D1710" t="s">
+        <v>2223</v>
+      </c>
+      <c r="E1710" t="s">
+        <v>2493</v>
+      </c>
+      <c r="F1710" t="s">
+        <v>180</v>
+      </c>
+      <c r="G1710" t="s">
+        <v>55</v>
+      </c>
+      <c r="H1710" t="s">
+        <v>29</v>
+      </c>
+      <c r="I1710" t="s">
+        <v>30</v>
+      </c>
+      <c r="J1710" t="s">
+        <v>50</v>
+      </c>
+      <c r="K1710" t="s">
+        <v>181</v>
+      </c>
+      <c r="L1710" t="s">
+        <v>180</v>
+      </c>
+      <c r="M1710" t="s">
+        <v>587</v>
+      </c>
+    </row>
+    <row r="1711">
+      <c r="A1711" t="s">
+        <v>2223</v>
+      </c>
+      <c r="B1711" t="s">
+        <v>2494</v>
+      </c>
+      <c r="C1711" t="s">
+        <v>2495</v>
+      </c>
+      <c r="D1711" t="s">
+        <v>2223</v>
+      </c>
+      <c r="E1711" t="s">
+        <v>2496</v>
+      </c>
+      <c r="F1711" t="s">
+        <v>54</v>
+      </c>
+      <c r="G1711" t="s">
+        <v>55</v>
+      </c>
+      <c r="H1711" t="s">
+        <v>29</v>
+      </c>
+      <c r="I1711" t="s">
+        <v>30</v>
+      </c>
+      <c r="J1711" t="s">
+        <v>29</v>
+      </c>
+      <c r="K1711" t="s">
+        <v>39</v>
+      </c>
+      <c r="L1711" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="1712">
+      <c r="A1712" t="s">
+        <v>2223</v>
+      </c>
+      <c r="B1712" t="s">
+        <v>2497</v>
+      </c>
+      <c r="C1712" t="s">
+        <v>2498</v>
+      </c>
+      <c r="D1712" t="s">
+        <v>2223</v>
+      </c>
+      <c r="E1712" t="s">
+        <v>2499</v>
+      </c>
+      <c r="F1712" t="s">
+        <v>54</v>
+      </c>
+      <c r="G1712" t="s">
+        <v>55</v>
+      </c>
+      <c r="H1712" t="s">
+        <v>29</v>
+      </c>
+      <c r="I1712" t="s">
+        <v>30</v>
+      </c>
+      <c r="J1712" t="s">
+        <v>29</v>
+      </c>
+      <c r="K1712" t="s">
+        <v>39</v>
+      </c>
+      <c r="L1712" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="1713">
+      <c r="A1713" t="s">
+        <v>2223</v>
+      </c>
+      <c r="B1713" t="s">
+        <v>2500</v>
+      </c>
+      <c r="C1713" t="s">
+        <v>2501</v>
+      </c>
+      <c r="D1713" t="s">
+        <v>2223</v>
+      </c>
+      <c r="E1713" t="s">
+        <v>2502</v>
+      </c>
+      <c r="F1713" t="s">
+        <v>180</v>
+      </c>
+      <c r="G1713" t="s">
+        <v>55</v>
+      </c>
+      <c r="H1713" t="s">
+        <v>29</v>
+      </c>
+      <c r="I1713" t="s">
+        <v>30</v>
+      </c>
+      <c r="J1713" t="s">
+        <v>50</v>
+      </c>
+      <c r="K1713" t="s">
+        <v>181</v>
+      </c>
+      <c r="L1713" t="s">
+        <v>180</v>
+      </c>
+      <c r="M1713" t="s">
+        <v>956</v>
+      </c>
+    </row>
+    <row r="1714">
+      <c r="A1714" t="s">
+        <v>2223</v>
+      </c>
+      <c r="B1714" t="s">
+        <v>2503</v>
+      </c>
+      <c r="C1714" t="s">
+        <v>2504</v>
+      </c>
+      <c r="D1714" t="s">
+        <v>2223</v>
+      </c>
+      <c r="E1714" t="s">
+        <v>2505</v>
+      </c>
+      <c r="F1714" t="s">
+        <v>180</v>
+      </c>
+      <c r="G1714" t="s">
+        <v>55</v>
+      </c>
+      <c r="H1714" t="s">
+        <v>29</v>
+      </c>
+      <c r="I1714" t="s">
+        <v>30</v>
+      </c>
+      <c r="J1714" t="s">
+        <v>50</v>
+      </c>
+      <c r="K1714" t="s">
+        <v>181</v>
+      </c>
+      <c r="L1714" t="s">
+        <v>180</v>
+      </c>
+      <c r="M1714" t="s">
+        <v>956</v>
+      </c>
+    </row>
+    <row r="1715">
+      <c r="A1715" t="s">
+        <v>2223</v>
+      </c>
+      <c r="B1715" t="s">
+        <v>2506</v>
+      </c>
+      <c r="C1715" t="s">
+        <v>2507</v>
+      </c>
+      <c r="D1715" t="s">
+        <v>2223</v>
+      </c>
+      <c r="E1715" t="s">
+        <v>2508</v>
+      </c>
+      <c r="F1715" t="s">
+        <v>180</v>
+      </c>
+      <c r="G1715" t="s">
+        <v>55</v>
+      </c>
+      <c r="H1715" t="s">
+        <v>29</v>
+      </c>
+      <c r="I1715" t="s">
+        <v>30</v>
+      </c>
+      <c r="J1715" t="s">
+        <v>50</v>
+      </c>
+      <c r="K1715" t="s">
+        <v>181</v>
+      </c>
+      <c r="L1715" t="s">
+        <v>180</v>
+      </c>
+      <c r="M1715" t="s">
+        <v>956</v>
+      </c>
+    </row>
+    <row r="1716">
+      <c r="A1716" t="s">
+        <v>2223</v>
+      </c>
+      <c r="B1716" t="s">
+        <v>2509</v>
+      </c>
+      <c r="C1716" t="s">
+        <v>2510</v>
+      </c>
+      <c r="D1716" t="s">
+        <v>2223</v>
+      </c>
+      <c r="E1716" t="s">
+        <v>2511</v>
+      </c>
+      <c r="F1716" t="s">
+        <v>180</v>
+      </c>
+      <c r="G1716" t="s">
+        <v>55</v>
+      </c>
+      <c r="H1716" t="s">
+        <v>29</v>
+      </c>
+      <c r="I1716" t="s">
+        <v>30</v>
+      </c>
+      <c r="J1716" t="s">
+        <v>50</v>
+      </c>
+      <c r="K1716" t="s">
+        <v>181</v>
+      </c>
+      <c r="L1716" t="s">
+        <v>180</v>
+      </c>
+      <c r="M1716" t="s">
+        <v>587</v>
+      </c>
+    </row>
+    <row r="1717">
+      <c r="A1717" t="s">
+        <v>2223</v>
+      </c>
+      <c r="B1717" t="s">
+        <v>2512</v>
+      </c>
+      <c r="C1717" t="s">
+        <v>2513</v>
+      </c>
+      <c r="D1717" t="s">
+        <v>2223</v>
+      </c>
+      <c r="E1717" t="s">
+        <v>2514</v>
+      </c>
+      <c r="F1717" t="s">
+        <v>54</v>
+      </c>
+      <c r="G1717" t="s">
+        <v>55</v>
+      </c>
+      <c r="H1717" t="s">
+        <v>29</v>
+      </c>
+      <c r="I1717" t="s">
+        <v>30</v>
+      </c>
+      <c r="J1717" t="s">
+        <v>29</v>
+      </c>
+      <c r="K1717" t="s">
+        <v>39</v>
+      </c>
+      <c r="L1717" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="1718">
+      <c r="A1718" t="s">
+        <v>2223</v>
+      </c>
+      <c r="B1718" t="s">
+        <v>2515</v>
+      </c>
+      <c r="C1718" t="s">
+        <v>2516</v>
+      </c>
+      <c r="D1718" t="s">
+        <v>2223</v>
+      </c>
+      <c r="E1718" t="s">
+        <v>2517</v>
+      </c>
+      <c r="F1718" t="s">
+        <v>54</v>
+      </c>
+      <c r="G1718" t="s">
+        <v>55</v>
+      </c>
+      <c r="H1718" t="s">
+        <v>29</v>
+      </c>
+      <c r="I1718" t="s">
+        <v>30</v>
+      </c>
+      <c r="J1718" t="s">
+        <v>29</v>
+      </c>
+      <c r="K1718" t="s">
+        <v>39</v>
+      </c>
+      <c r="L1718" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="1719">
+      <c r="A1719" t="s">
+        <v>2223</v>
+      </c>
+      <c r="B1719" t="s">
+        <v>2518</v>
+      </c>
+      <c r="C1719" t="s">
+        <v>2519</v>
+      </c>
+      <c r="D1719" t="s">
+        <v>2223</v>
+      </c>
+      <c r="E1719" t="s">
+        <v>2520</v>
+      </c>
+      <c r="F1719" t="s">
+        <v>180</v>
+      </c>
+      <c r="G1719" t="s">
+        <v>55</v>
+      </c>
+      <c r="H1719" t="s">
+        <v>29</v>
+      </c>
+      <c r="I1719" t="s">
+        <v>30</v>
+      </c>
+      <c r="J1719" t="s">
+        <v>50</v>
+      </c>
+      <c r="K1719" t="s">
+        <v>181</v>
+      </c>
+      <c r="L1719" t="s">
+        <v>180</v>
+      </c>
+      <c r="M1719" t="s">
+        <v>956</v>
+      </c>
+    </row>
+    <row r="1720">
+      <c r="A1720" t="s">
+        <v>2223</v>
+      </c>
+      <c r="B1720" t="s">
+        <v>2521</v>
+      </c>
+      <c r="C1720" t="s">
+        <v>2522</v>
+      </c>
+      <c r="D1720" t="s">
+        <v>2223</v>
+      </c>
+      <c r="E1720" t="s">
+        <v>2523</v>
+      </c>
+      <c r="F1720" t="s">
+        <v>180</v>
+      </c>
+      <c r="G1720" t="s">
+        <v>55</v>
+      </c>
+      <c r="H1720" t="s">
+        <v>29</v>
+      </c>
+      <c r="I1720" t="s">
+        <v>30</v>
+      </c>
+      <c r="J1720" t="s">
+        <v>50</v>
+      </c>
+      <c r="K1720" t="s">
+        <v>181</v>
+      </c>
+      <c r="L1720" t="s">
+        <v>180</v>
+      </c>
+      <c r="M1720" t="s">
+        <v>956</v>
+      </c>
+    </row>
+    <row r="1721">
+      <c r="A1721" t="s">
+        <v>2223</v>
+      </c>
+      <c r="B1721" t="s">
+        <v>2524</v>
+      </c>
+      <c r="C1721" t="s">
+        <v>2525</v>
+      </c>
+      <c r="D1721" t="s">
+        <v>2223</v>
+      </c>
+      <c r="E1721" t="s">
+        <v>2526</v>
+      </c>
+      <c r="F1721" t="s">
+        <v>54</v>
+      </c>
+      <c r="G1721" t="s">
+        <v>55</v>
+      </c>
+      <c r="H1721" t="s">
+        <v>29</v>
+      </c>
+      <c r="I1721" t="s">
+        <v>30</v>
+      </c>
+      <c r="J1721" t="s">
+        <v>29</v>
+      </c>
+      <c r="K1721" t="s">
+        <v>39</v>
+      </c>
+      <c r="L1721" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="1722">
+      <c r="A1722" t="s">
+        <v>2223</v>
+      </c>
+      <c r="B1722" t="s">
+        <v>2527</v>
+      </c>
+      <c r="C1722" t="s">
+        <v>2528</v>
+      </c>
+      <c r="D1722" t="s">
+        <v>2223</v>
+      </c>
+      <c r="E1722" t="s">
+        <v>2529</v>
+      </c>
+      <c r="F1722" t="s">
+        <v>54</v>
+      </c>
+      <c r="G1722" t="s">
+        <v>55</v>
+      </c>
+      <c r="H1722" t="s">
+        <v>29</v>
+      </c>
+      <c r="I1722" t="s">
+        <v>30</v>
+      </c>
+      <c r="J1722" t="s">
+        <v>29</v>
+      </c>
+      <c r="K1722" t="s">
+        <v>39</v>
+      </c>
+      <c r="L1722" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="1723">
+      <c r="A1723" t="s">
+        <v>2223</v>
+      </c>
+      <c r="B1723" t="s">
+        <v>2530</v>
+      </c>
+      <c r="C1723" t="s">
+        <v>2531</v>
+      </c>
+      <c r="D1723" t="s">
+        <v>2223</v>
+      </c>
+      <c r="E1723" t="s">
+        <v>2532</v>
+      </c>
+      <c r="F1723" t="s">
+        <v>54</v>
+      </c>
+      <c r="G1723" t="s">
+        <v>55</v>
+      </c>
+      <c r="H1723" t="s">
+        <v>29</v>
+      </c>
+      <c r="I1723" t="s">
+        <v>30</v>
+      </c>
+      <c r="J1723" t="s">
+        <v>29</v>
+      </c>
+      <c r="K1723" t="s">
+        <v>39</v>
+      </c>
+      <c r="L1723" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="1724">
+      <c r="A1724" t="s">
+        <v>2223</v>
+      </c>
+      <c r="B1724" t="s">
+        <v>2533</v>
+      </c>
+      <c r="C1724" t="s">
+        <v>2534</v>
+      </c>
+      <c r="D1724" t="s">
+        <v>2223</v>
+      </c>
+      <c r="E1724" t="s">
+        <v>2535</v>
+      </c>
+      <c r="F1724" t="s">
+        <v>54</v>
+      </c>
+      <c r="G1724" t="s">
+        <v>55</v>
+      </c>
+      <c r="H1724" t="s">
+        <v>29</v>
+      </c>
+      <c r="I1724" t="s">
+        <v>30</v>
+      </c>
+      <c r="J1724" t="s">
+        <v>29</v>
+      </c>
+      <c r="K1724" t="s">
+        <v>39</v>
+      </c>
+      <c r="L1724" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="1725">
+      <c r="A1725" t="s">
+        <v>2223</v>
+      </c>
+      <c r="B1725" t="s">
+        <v>2536</v>
+      </c>
+      <c r="C1725" t="s">
+        <v>2235</v>
+      </c>
+      <c r="D1725" t="s">
+        <v>2223</v>
+      </c>
+      <c r="E1725" t="s">
+        <v>2236</v>
+      </c>
+      <c r="F1725" t="s">
+        <v>54</v>
+      </c>
+      <c r="G1725" t="s">
+        <v>55</v>
+      </c>
+      <c r="H1725" t="s">
+        <v>29</v>
+      </c>
+      <c r="I1725" t="s">
+        <v>30</v>
+      </c>
+      <c r="J1725" t="s">
+        <v>29</v>
+      </c>
+      <c r="K1725" t="s">
+        <v>39</v>
+      </c>
+      <c r="L1725" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="1726">
+      <c r="A1726" t="s">
+        <v>2223</v>
+      </c>
+      <c r="B1726" t="s">
+        <v>50</v>
+      </c>
+      <c r="C1726" t="s">
+        <v>50</v>
+      </c>
+      <c r="D1726" t="s">
+        <v>50</v>
+      </c>
+      <c r="E1726" t="s">
+        <v>50</v>
+      </c>
+      <c r="F1726" t="s">
+        <v>50</v>
+      </c>
+      <c r="G1726" t="s">
+        <v>50</v>
+      </c>
+      <c r="H1726" t="s">
+        <v>50</v>
+      </c>
+      <c r="I1726" t="s">
+        <v>50</v>
+      </c>
+      <c r="J1726" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="1727">
+      <c r="A1727" t="s">
+        <v>2223</v>
+      </c>
+      <c r="B1727" t="s">
+        <v>230</v>
+      </c>
+      <c r="C1727" t="s">
+        <v>2537</v>
+      </c>
+      <c r="D1727" t="s">
+        <v>50</v>
+      </c>
+      <c r="E1727" t="s">
         <v>232</v>
       </c>
-      <c r="F1685" t="s">
-        <v>2416</v>
-      </c>
-      <c r="G1685" t="s">
-        <v>50</v>
-      </c>
-      <c r="H1685" t="s">
-        <v>50</v>
-      </c>
-      <c r="I1685" t="s">
-        <v>50</v>
-      </c>
-      <c r="J1685" t="s">
+      <c r="F1727" t="s">
+        <v>2536</v>
+      </c>
+      <c r="G1727" t="s">
+        <v>50</v>
+      </c>
+      <c r="H1727" t="s">
+        <v>50</v>
+      </c>
+      <c r="I1727" t="s">
+        <v>50</v>
+      </c>
+      <c r="J1727" t="s">
         <v>50</v>
       </c>
     </row>

</xml_diff>

<commit_message>
compiled report 2026-06-08: 14 election events, 11 audit entries
</commit_message>
<xml_diff>
--- a/punmonitor-compiled-report.xlsx
+++ b/punmonitor-compiled-report.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="125" uniqueCount="125">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="163" uniqueCount="163">
   <si>
     <t>Source Date</t>
   </si>
@@ -123,7 +123,7 @@
     <t>amd64</t>
   </si>
   <si>
-    <t>10.0.58</t>
+    <t>10.0.59</t>
   </si>
   <si>
     <t>server+agent</t>
@@ -138,19 +138,19 @@
     <t>0</t>
   </si>
   <si>
-    <t>0h 2m 23s</t>
-  </si>
-  <si>
-    <t>2026-06-08 23:39:54</t>
+    <t>0h 2m 41s</t>
+  </si>
+  <si>
+    <t>2026-06-08 23:55:21</t>
   </si>
   <si>
     <t>Jun 8 12:55 PM</t>
   </si>
   <si>
-    <t>0h 1m 36s</t>
-  </si>
-  <si>
-    <t>23:42:18</t>
+    <t>0h 3m 26s</t>
+  </si>
+  <si>
+    <t>23:58:03</t>
   </si>
   <si>
     <t>agent</t>
@@ -162,31 +162,292 @@
     <t>good</t>
   </si>
   <si>
-    <t>110.0</t>
-  </si>
-  <si>
-    <t>109146.2</t>
-  </si>
-  <si>
-    <t>1114</t>
+    <t>57.0</t>
+  </si>
+  <si>
+    <t>94066.6</t>
+  </si>
+  <si>
+    <t>1201</t>
   </si>
   <si>
     <t>0.5</t>
   </si>
   <si>
-    <t>24</t>
+    <t>42</t>
   </si>
   <si>
     <t>—</t>
   </si>
   <si>
+    <t>0h 3m 11s</t>
+  </si>
+  <si>
     <t>── LATEST GITHUB ELECTION EVENT ──</t>
   </si>
   <si>
     <t/>
   </si>
   <si>
-    <t>[stale-takeover]</t>
+    <t>[renewed]</t>
+  </si>
+  <si>
+    <t>2026-06-08T23:55:37.4511138+05:30</t>
+  </si>
+  <si>
+    <t>23:55:37.451</t>
+  </si>
+  <si>
+    <t>renewed</t>
+  </si>
+  <si>
+    <t>github</t>
+  </si>
+  <si>
+    <t>1780940945054</t>
+  </si>
+  <si>
+    <t>23:19:05</t>
+  </si>
+  <si>
+    <t>promote_to_server</t>
+  </si>
+  <si>
+    <t>admin</t>
+  </si>
+  <si>
+    <t>1780941240320</t>
+  </si>
+  <si>
+    <t>23:24:00</t>
+  </si>
+  <si>
+    <t>1780943233682</t>
+  </si>
+  <si>
+    <t>23:57:13</t>
+  </si>
+  <si>
+    <t>assist_created</t>
+  </si>
+  <si>
+    <t>kRx060GX</t>
+  </si>
+  <si>
+    <t>1780943233790</t>
+  </si>
+  <si>
+    <t>assist_view</t>
+  </si>
+  <si>
+    <t>1780943234407</t>
+  </si>
+  <si>
+    <t>23:57:14</t>
+  </si>
+  <si>
+    <t>apzw9sxr</t>
+  </si>
+  <si>
+    <t>1780943234507</t>
+  </si>
+  <si>
+    <t>1780943235211</t>
+  </si>
+  <si>
+    <t>23:57:15</t>
+  </si>
+  <si>
+    <t>62OYvYNz</t>
+  </si>
+  <si>
+    <t>1780943235306</t>
+  </si>
+  <si>
+    <t>1780943241868</t>
+  </si>
+  <si>
+    <t>23:57:21</t>
+  </si>
+  <si>
+    <t>assist_closed</t>
+  </si>
+  <si>
+    <t>1780943242590</t>
+  </si>
+  <si>
+    <t>23:57:22</t>
+  </si>
+  <si>
+    <t>1780943244346</t>
+  </si>
+  <si>
+    <t>23:57:24</t>
+  </si>
+  <si>
+    <t>Election method</t>
+  </si>
+  <si>
+    <t>GitHub configured</t>
+  </si>
+  <si>
+    <t>Yes</t>
+  </si>
+  <si>
+    <t>GitHub repo</t>
+  </si>
+  <si>
+    <t>puniteswra-spec/PU</t>
+  </si>
+  <si>
+    <t>Self AgentID</t>
+  </si>
+  <si>
+    <t>Self hostname</t>
+  </si>
+  <si>
+    <t>Mode / Role</t>
+  </si>
+  <si>
+    <t>SERVER+LEADER (this instance is the GitHub primary)</t>
+  </si>
+  <si>
+    <t>Self is leader</t>
+  </si>
+  <si>
+    <t>YES — this instance is the primary server</t>
+  </si>
+  <si>
+    <t>Current leader</t>
+  </si>
+  <si>
+    <t>Leader last update</t>
+  </si>
+  <si>
+    <t>2026-06-08T23:55:37+05:30 (2m25s ago)</t>
+  </si>
+  <si>
+    <t>Leader stale?</t>
+  </si>
+  <si>
+    <t>No</t>
+  </si>
+  <si>
+    <t>Last check</t>
+  </si>
+  <si>
+    <t>Check count</t>
+  </si>
+  <si>
+    <t>1</t>
+  </si>
+  <si>
+    <t>Last error</t>
+  </si>
+  <si>
+    <t>(none)</t>
+  </si>
+  <si>
+    <t>Election History (row-wise — latest first)</t>
+  </si>
+  <si>
+    <t>#</t>
+  </si>
+  <si>
+    <t>Timestamp</t>
+  </si>
+  <si>
+    <t>Date</t>
+  </si>
+  <si>
+    <t>Time</t>
+  </si>
+  <si>
+    <t>Agent ID (self)</t>
+  </si>
+  <si>
+    <t>Leader Age (sec)</t>
+  </si>
+  <si>
+    <t>2026-06-08T23:18:21.1575718+05:30</t>
+  </si>
+  <si>
+    <t>23:18:21.157</t>
+  </si>
+  <si>
+    <t>checking</t>
+  </si>
+  <si>
+    <t>relay</t>
+  </si>
+  <si>
+    <t>9223372036</t>
+  </si>
+  <si>
+    <t>2</t>
+  </si>
+  <si>
+    <t>2026-06-08T23:19:40.0639784+05:30</t>
+  </si>
+  <si>
+    <t>23:19:40.063</t>
+  </si>
+  <si>
+    <t>3</t>
+  </si>
+  <si>
+    <t>2026-06-08T23:22:10.5651401+05:30</t>
+  </si>
+  <si>
+    <t>23:22:10.565</t>
+  </si>
+  <si>
+    <t>4</t>
+  </si>
+  <si>
+    <t>2026-06-08T23:23:21.8314433+05:30</t>
+  </si>
+  <si>
+    <t>23:23:21.831</t>
+  </si>
+  <si>
+    <t>5</t>
+  </si>
+  <si>
+    <t>2026-06-08T23:26:30.4757625+05:30</t>
+  </si>
+  <si>
+    <t>23:26:30.475</t>
+  </si>
+  <si>
+    <t>6</t>
+  </si>
+  <si>
+    <t>2026-06-08T23:28:53.5745305+05:30</t>
+  </si>
+  <si>
+    <t>23:28:53.574</t>
+  </si>
+  <si>
+    <t>7</t>
+  </si>
+  <si>
+    <t>2026-06-08T23:30:51.2403981+05:30</t>
+  </si>
+  <si>
+    <t>23:30:51.240</t>
+  </si>
+  <si>
+    <t>8</t>
+  </si>
+  <si>
+    <t>2026-06-08T23:32:14.1980002+05:30</t>
+  </si>
+  <si>
+    <t>23:32:14.198</t>
+  </si>
+  <si>
+    <t>9</t>
   </si>
   <si>
     <t>2026-06-08T23:40:10.5495809+05:30</t>
@@ -198,196 +459,49 @@
     <t>stale-takeover</t>
   </si>
   <si>
-    <t>github</t>
-  </si>
-  <si>
-    <t>1780940945054</t>
-  </si>
-  <si>
-    <t>23:19:05</t>
-  </si>
-  <si>
-    <t>promote_to_server</t>
-  </si>
-  <si>
-    <t>admin</t>
-  </si>
-  <si>
-    <t>1780941240320</t>
-  </si>
-  <si>
-    <t>23:24:00</t>
-  </si>
-  <si>
-    <t>Election method</t>
-  </si>
-  <si>
-    <t>GitHub configured</t>
-  </si>
-  <si>
-    <t>Yes</t>
-  </si>
-  <si>
-    <t>GitHub repo</t>
-  </si>
-  <si>
-    <t>puniteswra-spec/PU</t>
-  </si>
-  <si>
-    <t>Self AgentID</t>
-  </si>
-  <si>
-    <t>Self hostname</t>
-  </si>
-  <si>
-    <t>Mode / Role</t>
-  </si>
-  <si>
-    <t>SERVER+LEADER (this instance is the GitHub primary)</t>
-  </si>
-  <si>
-    <t>Self is leader</t>
-  </si>
-  <si>
-    <t>YES — this instance is the primary server</t>
-  </si>
-  <si>
-    <t>Current leader</t>
-  </si>
-  <si>
-    <t>Leader last update</t>
-  </si>
-  <si>
-    <t>2026-06-08T23:40:10+05:30 (2m8s ago)</t>
-  </si>
-  <si>
-    <t>Leader stale?</t>
-  </si>
-  <si>
-    <t>No</t>
-  </si>
-  <si>
-    <t>Last check</t>
-  </si>
-  <si>
-    <t>Check count</t>
-  </si>
-  <si>
-    <t>1</t>
-  </si>
-  <si>
-    <t>Last error</t>
-  </si>
-  <si>
-    <t>(none)</t>
-  </si>
-  <si>
-    <t>Election History (row-wise — latest first)</t>
-  </si>
-  <si>
-    <t>#</t>
-  </si>
-  <si>
-    <t>Timestamp</t>
-  </si>
-  <si>
-    <t>Date</t>
-  </si>
-  <si>
-    <t>Time</t>
-  </si>
-  <si>
-    <t>Agent ID (self)</t>
-  </si>
-  <si>
-    <t>Leader Age (sec)</t>
-  </si>
-  <si>
-    <t>2026-06-08T23:18:21.1575718+05:30</t>
-  </si>
-  <si>
-    <t>23:18:21.157</t>
-  </si>
-  <si>
-    <t>checking</t>
-  </si>
-  <si>
-    <t>relay</t>
-  </si>
-  <si>
-    <t>9223372036</t>
-  </si>
-  <si>
-    <t>2</t>
-  </si>
-  <si>
-    <t>2026-06-08T23:19:40.0639784+05:30</t>
-  </si>
-  <si>
-    <t>23:19:40.063</t>
-  </si>
-  <si>
-    <t>3</t>
-  </si>
-  <si>
-    <t>2026-06-08T23:22:10.5651401+05:30</t>
-  </si>
-  <si>
-    <t>23:22:10.565</t>
-  </si>
-  <si>
-    <t>4</t>
-  </si>
-  <si>
-    <t>2026-06-08T23:23:21.8314433+05:30</t>
-  </si>
-  <si>
-    <t>23:23:21.831</t>
-  </si>
-  <si>
-    <t>5</t>
-  </si>
-  <si>
-    <t>2026-06-08T23:26:30.4757625+05:30</t>
-  </si>
-  <si>
-    <t>23:26:30.475</t>
-  </si>
-  <si>
-    <t>6</t>
-  </si>
-  <si>
-    <t>2026-06-08T23:28:53.5745305+05:30</t>
-  </si>
-  <si>
-    <t>23:28:53.574</t>
-  </si>
-  <si>
-    <t>7</t>
-  </si>
-  <si>
-    <t>2026-06-08T23:30:51.2403981+05:30</t>
-  </si>
-  <si>
-    <t>23:30:51.240</t>
-  </si>
-  <si>
-    <t>8</t>
-  </si>
-  <si>
-    <t>2026-06-08T23:32:14.1980002+05:30</t>
-  </si>
-  <si>
-    <t>23:32:14.198</t>
-  </si>
-  <si>
-    <t>9</t>
+    <t>10</t>
+  </si>
+  <si>
+    <t>2026-06-08T23:45:21.045245+05:30</t>
+  </si>
+  <si>
+    <t>23:45:21.045</t>
+  </si>
+  <si>
+    <t>11</t>
+  </si>
+  <si>
+    <t>2026-06-08T23:50:20.3164757+05:30</t>
+  </si>
+  <si>
+    <t>23:50:20.316</t>
+  </si>
+  <si>
+    <t>12</t>
+  </si>
+  <si>
+    <t>2026-06-08T23:51:53.3444626+05:30</t>
+  </si>
+  <si>
+    <t>23:51:53.344</t>
+  </si>
+  <si>
+    <t>13</t>
+  </si>
+  <si>
+    <t>2026-06-08T23:53:00.5826369+05:30</t>
+  </si>
+  <si>
+    <t>23:53:00.582</t>
+  </si>
+  <si>
+    <t>14</t>
   </si>
   <si>
     <t>Generated</t>
   </si>
   <si>
-    <t>2026-06-08T23:42:18+05:30</t>
+    <t>2026-06-08T23:58:03+05:30</t>
   </si>
   <si>
     <t>Total events</t>
@@ -876,7 +990,7 @@
         <v>41</v>
       </c>
       <c r="T3" t="s">
-        <v>43</v>
+        <v>54</v>
       </c>
       <c r="U3" t="s">
         <v>28</v>
@@ -890,52 +1004,52 @@
         <v>28</v>
       </c>
       <c r="B4" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="C4" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="D4" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="E4" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="F4" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="G4" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="H4" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="I4" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="J4" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="K4" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="L4" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="M4" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="N4" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="O4" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="P4" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="Q4" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="5">
@@ -943,22 +1057,22 @@
         <v>28</v>
       </c>
       <c r="B5" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="C5" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="D5" t="s">
         <v>28</v>
       </c>
       <c r="E5" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="F5" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="G5" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="H5" t="s">
         <v>29</v>
@@ -973,22 +1087,22 @@
         <v>39</v>
       </c>
       <c r="L5" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="M5" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="N5" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="O5" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="P5" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="Q5" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
   </sheetData>
@@ -1030,25 +1144,25 @@
         <v>28</v>
       </c>
       <c r="B2" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="C2" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D2" t="s">
         <v>28</v>
       </c>
       <c r="E2" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="F2" t="s">
         <v>29</v>
       </c>
       <c r="G2" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="H2" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="3">
@@ -1056,25 +1170,259 @@
         <v>28</v>
       </c>
       <c r="B3" t="s">
+        <v>66</v>
+      </c>
+      <c r="C3" t="s">
+        <v>67</v>
+      </c>
+      <c r="D3" t="s">
+        <v>28</v>
+      </c>
+      <c r="E3" t="s">
+        <v>64</v>
+      </c>
+      <c r="F3" t="s">
+        <v>29</v>
+      </c>
+      <c r="G3" t="s">
         <v>65</v>
       </c>
-      <c r="C3" t="s">
-        <v>66</v>
-      </c>
-      <c r="D3" t="s">
-        <v>28</v>
-      </c>
-      <c r="E3" t="s">
-        <v>63</v>
-      </c>
-      <c r="F3" t="s">
-        <v>29</v>
-      </c>
-      <c r="G3" t="s">
-        <v>64</v>
-      </c>
       <c r="H3" t="s">
-        <v>55</v>
+        <v>56</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s">
+        <v>28</v>
+      </c>
+      <c r="B4" t="s">
+        <v>68</v>
+      </c>
+      <c r="C4" t="s">
+        <v>69</v>
+      </c>
+      <c r="D4" t="s">
+        <v>28</v>
+      </c>
+      <c r="E4" t="s">
+        <v>70</v>
+      </c>
+      <c r="F4" t="s">
+        <v>56</v>
+      </c>
+      <c r="G4" t="s">
+        <v>65</v>
+      </c>
+      <c r="H4" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="s">
+        <v>28</v>
+      </c>
+      <c r="B5" t="s">
+        <v>72</v>
+      </c>
+      <c r="C5" t="s">
+        <v>69</v>
+      </c>
+      <c r="D5" t="s">
+        <v>28</v>
+      </c>
+      <c r="E5" t="s">
+        <v>73</v>
+      </c>
+      <c r="F5" t="s">
+        <v>71</v>
+      </c>
+      <c r="G5" t="s">
+        <v>65</v>
+      </c>
+      <c r="H5" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="s">
+        <v>28</v>
+      </c>
+      <c r="B6" t="s">
+        <v>74</v>
+      </c>
+      <c r="C6" t="s">
+        <v>75</v>
+      </c>
+      <c r="D6" t="s">
+        <v>28</v>
+      </c>
+      <c r="E6" t="s">
+        <v>70</v>
+      </c>
+      <c r="F6" t="s">
+        <v>56</v>
+      </c>
+      <c r="G6" t="s">
+        <v>65</v>
+      </c>
+      <c r="H6" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="s">
+        <v>28</v>
+      </c>
+      <c r="B7" t="s">
+        <v>77</v>
+      </c>
+      <c r="C7" t="s">
+        <v>75</v>
+      </c>
+      <c r="D7" t="s">
+        <v>28</v>
+      </c>
+      <c r="E7" t="s">
+        <v>73</v>
+      </c>
+      <c r="F7" t="s">
+        <v>76</v>
+      </c>
+      <c r="G7" t="s">
+        <v>65</v>
+      </c>
+      <c r="H7" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="s">
+        <v>28</v>
+      </c>
+      <c r="B8" t="s">
+        <v>78</v>
+      </c>
+      <c r="C8" t="s">
+        <v>79</v>
+      </c>
+      <c r="D8" t="s">
+        <v>28</v>
+      </c>
+      <c r="E8" t="s">
+        <v>70</v>
+      </c>
+      <c r="F8" t="s">
+        <v>56</v>
+      </c>
+      <c r="G8" t="s">
+        <v>65</v>
+      </c>
+      <c r="H8" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="s">
+        <v>28</v>
+      </c>
+      <c r="B9" t="s">
+        <v>81</v>
+      </c>
+      <c r="C9" t="s">
+        <v>79</v>
+      </c>
+      <c r="D9" t="s">
+        <v>28</v>
+      </c>
+      <c r="E9" t="s">
+        <v>73</v>
+      </c>
+      <c r="F9" t="s">
+        <v>80</v>
+      </c>
+      <c r="G9" t="s">
+        <v>65</v>
+      </c>
+      <c r="H9" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="s">
+        <v>28</v>
+      </c>
+      <c r="B10" t="s">
+        <v>82</v>
+      </c>
+      <c r="C10" t="s">
+        <v>83</v>
+      </c>
+      <c r="D10" t="s">
+        <v>28</v>
+      </c>
+      <c r="E10" t="s">
+        <v>84</v>
+      </c>
+      <c r="F10" t="s">
+        <v>56</v>
+      </c>
+      <c r="G10" t="s">
+        <v>65</v>
+      </c>
+      <c r="H10" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="s">
+        <v>28</v>
+      </c>
+      <c r="B11" t="s">
+        <v>85</v>
+      </c>
+      <c r="C11" t="s">
+        <v>86</v>
+      </c>
+      <c r="D11" t="s">
+        <v>28</v>
+      </c>
+      <c r="E11" t="s">
+        <v>84</v>
+      </c>
+      <c r="F11" t="s">
+        <v>56</v>
+      </c>
+      <c r="G11" t="s">
+        <v>65</v>
+      </c>
+      <c r="H11" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="s">
+        <v>28</v>
+      </c>
+      <c r="B12" t="s">
+        <v>87</v>
+      </c>
+      <c r="C12" t="s">
+        <v>88</v>
+      </c>
+      <c r="D12" t="s">
+        <v>28</v>
+      </c>
+      <c r="E12" t="s">
+        <v>84</v>
+      </c>
+      <c r="F12" t="s">
+        <v>56</v>
+      </c>
+      <c r="G12" t="s">
+        <v>65</v>
+      </c>
+      <c r="H12" t="s">
+        <v>80</v>
       </c>
     </row>
   </sheetData>
@@ -1122,31 +1470,31 @@
         <v>28</v>
       </c>
       <c r="B2" t="s">
-        <v>67</v>
+        <v>89</v>
       </c>
       <c r="C2" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="D2" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="E2" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="F2" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="G2" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="H2" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="I2" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="J2" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="3">
@@ -1154,31 +1502,31 @@
         <v>28</v>
       </c>
       <c r="B3" t="s">
-        <v>68</v>
+        <v>90</v>
       </c>
       <c r="C3" t="s">
-        <v>69</v>
+        <v>91</v>
       </c>
       <c r="D3" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="E3" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="F3" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="G3" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="H3" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="I3" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="J3" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="4">
@@ -1186,31 +1534,31 @@
         <v>28</v>
       </c>
       <c r="B4" t="s">
-        <v>70</v>
+        <v>92</v>
       </c>
       <c r="C4" t="s">
-        <v>71</v>
+        <v>93</v>
       </c>
       <c r="D4" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="E4" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="F4" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="G4" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="H4" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="I4" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="J4" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="5">
@@ -1218,31 +1566,31 @@
         <v>28</v>
       </c>
       <c r="B5" t="s">
-        <v>72</v>
+        <v>94</v>
       </c>
       <c r="C5" t="s">
         <v>29</v>
       </c>
       <c r="D5" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="E5" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="F5" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="G5" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="H5" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="I5" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="J5" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="6">
@@ -1250,31 +1598,31 @@
         <v>28</v>
       </c>
       <c r="B6" t="s">
-        <v>73</v>
+        <v>95</v>
       </c>
       <c r="C6" t="s">
         <v>30</v>
       </c>
       <c r="D6" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="E6" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="F6" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="G6" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="H6" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="I6" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="J6" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="7">
@@ -1282,31 +1630,31 @@
         <v>28</v>
       </c>
       <c r="B7" t="s">
-        <v>74</v>
+        <v>96</v>
       </c>
       <c r="C7" t="s">
-        <v>75</v>
+        <v>97</v>
       </c>
       <c r="D7" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="E7" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="F7" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="G7" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="H7" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="I7" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="J7" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="8">
@@ -1314,31 +1662,31 @@
         <v>28</v>
       </c>
       <c r="B8" t="s">
-        <v>76</v>
+        <v>98</v>
       </c>
       <c r="C8" t="s">
-        <v>77</v>
+        <v>99</v>
       </c>
       <c r="D8" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="E8" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="F8" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="G8" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="H8" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="I8" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="J8" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="9">
@@ -1346,31 +1694,31 @@
         <v>28</v>
       </c>
       <c r="B9" t="s">
-        <v>78</v>
+        <v>100</v>
       </c>
       <c r="C9" t="s">
         <v>29</v>
       </c>
       <c r="D9" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="E9" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="F9" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="G9" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="H9" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="I9" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="J9" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="10">
@@ -1378,31 +1726,31 @@
         <v>28</v>
       </c>
       <c r="B10" t="s">
-        <v>79</v>
+        <v>101</v>
       </c>
       <c r="C10" t="s">
-        <v>80</v>
+        <v>102</v>
       </c>
       <c r="D10" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="E10" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="F10" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="G10" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="H10" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="I10" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="J10" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="11">
@@ -1410,31 +1758,31 @@
         <v>28</v>
       </c>
       <c r="B11" t="s">
-        <v>81</v>
+        <v>103</v>
       </c>
       <c r="C11" t="s">
-        <v>82</v>
+        <v>104</v>
       </c>
       <c r="D11" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="E11" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="F11" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="G11" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="H11" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="I11" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="J11" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="12">
@@ -1442,31 +1790,31 @@
         <v>28</v>
       </c>
       <c r="B12" t="s">
-        <v>83</v>
+        <v>105</v>
       </c>
       <c r="C12" t="s">
-        <v>80</v>
+        <v>102</v>
       </c>
       <c r="D12" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="E12" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="F12" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="G12" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="H12" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="I12" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="J12" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="13">
@@ -1474,31 +1822,31 @@
         <v>28</v>
       </c>
       <c r="B13" t="s">
-        <v>84</v>
+        <v>106</v>
       </c>
       <c r="C13" t="s">
-        <v>85</v>
+        <v>107</v>
       </c>
       <c r="D13" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="E13" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="F13" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="G13" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="H13" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="I13" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="J13" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="14">
@@ -1506,31 +1854,31 @@
         <v>28</v>
       </c>
       <c r="B14" t="s">
-        <v>86</v>
+        <v>108</v>
       </c>
       <c r="C14" t="s">
-        <v>87</v>
+        <v>109</v>
       </c>
       <c r="D14" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="E14" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="F14" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="G14" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="H14" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="I14" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="J14" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="15">
@@ -1538,31 +1886,31 @@
         <v>28</v>
       </c>
       <c r="B15" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C15" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="D15" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="E15" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="F15" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="G15" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="H15" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="I15" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="J15" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="16">
@@ -1570,31 +1918,31 @@
         <v>28</v>
       </c>
       <c r="B16" t="s">
-        <v>88</v>
+        <v>110</v>
       </c>
       <c r="C16" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="D16" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="E16" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="F16" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="G16" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="H16" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="I16" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="J16" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="17">
@@ -1602,16 +1950,16 @@
         <v>28</v>
       </c>
       <c r="B17" t="s">
-        <v>89</v>
+        <v>111</v>
       </c>
       <c r="C17" t="s">
-        <v>90</v>
+        <v>112</v>
       </c>
       <c r="D17" t="s">
-        <v>91</v>
+        <v>113</v>
       </c>
       <c r="E17" t="s">
-        <v>92</v>
+        <v>114</v>
       </c>
       <c r="F17" t="s">
         <v>19</v>
@@ -1620,7 +1968,7 @@
         <v>23</v>
       </c>
       <c r="H17" t="s">
-        <v>93</v>
+        <v>115</v>
       </c>
       <c r="I17" t="s">
         <v>2</v>
@@ -1629,7 +1977,7 @@
         <v>24</v>
       </c>
       <c r="K17" t="s">
-        <v>94</v>
+        <v>116</v>
       </c>
       <c r="L17" t="s">
         <v>26</v>
@@ -1643,22 +1991,22 @@
         <v>28</v>
       </c>
       <c r="B18" t="s">
-        <v>85</v>
+        <v>107</v>
       </c>
       <c r="C18" t="s">
-        <v>95</v>
+        <v>117</v>
       </c>
       <c r="D18" t="s">
         <v>28</v>
       </c>
       <c r="E18" t="s">
-        <v>96</v>
+        <v>118</v>
       </c>
       <c r="F18" t="s">
-        <v>97</v>
+        <v>119</v>
       </c>
       <c r="G18" t="s">
-        <v>98</v>
+        <v>120</v>
       </c>
       <c r="H18" t="s">
         <v>29</v>
@@ -1667,13 +2015,13 @@
         <v>30</v>
       </c>
       <c r="J18" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="K18" t="s">
-        <v>99</v>
+        <v>121</v>
       </c>
       <c r="L18" t="s">
-        <v>97</v>
+        <v>119</v>
       </c>
     </row>
     <row r="19">
@@ -1681,22 +2029,22 @@
         <v>28</v>
       </c>
       <c r="B19" t="s">
-        <v>100</v>
+        <v>122</v>
       </c>
       <c r="C19" t="s">
-        <v>101</v>
+        <v>123</v>
       </c>
       <c r="D19" t="s">
         <v>28</v>
       </c>
       <c r="E19" t="s">
-        <v>102</v>
+        <v>124</v>
       </c>
       <c r="F19" t="s">
-        <v>97</v>
+        <v>119</v>
       </c>
       <c r="G19" t="s">
-        <v>98</v>
+        <v>120</v>
       </c>
       <c r="H19" t="s">
         <v>29</v>
@@ -1705,13 +2053,13 @@
         <v>30</v>
       </c>
       <c r="J19" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="K19" t="s">
-        <v>99</v>
+        <v>121</v>
       </c>
       <c r="L19" t="s">
-        <v>97</v>
+        <v>119</v>
       </c>
     </row>
     <row r="20">
@@ -1719,22 +2067,22 @@
         <v>28</v>
       </c>
       <c r="B20" t="s">
-        <v>103</v>
+        <v>125</v>
       </c>
       <c r="C20" t="s">
-        <v>104</v>
+        <v>126</v>
       </c>
       <c r="D20" t="s">
         <v>28</v>
       </c>
       <c r="E20" t="s">
-        <v>105</v>
+        <v>127</v>
       </c>
       <c r="F20" t="s">
-        <v>97</v>
+        <v>119</v>
       </c>
       <c r="G20" t="s">
-        <v>98</v>
+        <v>120</v>
       </c>
       <c r="H20" t="s">
         <v>29</v>
@@ -1743,13 +2091,13 @@
         <v>30</v>
       </c>
       <c r="J20" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="K20" t="s">
-        <v>99</v>
+        <v>121</v>
       </c>
       <c r="L20" t="s">
-        <v>97</v>
+        <v>119</v>
       </c>
     </row>
     <row r="21">
@@ -1757,22 +2105,22 @@
         <v>28</v>
       </c>
       <c r="B21" t="s">
-        <v>106</v>
+        <v>128</v>
       </c>
       <c r="C21" t="s">
-        <v>107</v>
+        <v>129</v>
       </c>
       <c r="D21" t="s">
         <v>28</v>
       </c>
       <c r="E21" t="s">
-        <v>108</v>
+        <v>130</v>
       </c>
       <c r="F21" t="s">
-        <v>97</v>
+        <v>119</v>
       </c>
       <c r="G21" t="s">
-        <v>98</v>
+        <v>120</v>
       </c>
       <c r="H21" t="s">
         <v>29</v>
@@ -1781,13 +2129,13 @@
         <v>30</v>
       </c>
       <c r="J21" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="K21" t="s">
-        <v>99</v>
+        <v>121</v>
       </c>
       <c r="L21" t="s">
-        <v>97</v>
+        <v>119</v>
       </c>
     </row>
     <row r="22">
@@ -1795,22 +2143,22 @@
         <v>28</v>
       </c>
       <c r="B22" t="s">
-        <v>109</v>
+        <v>131</v>
       </c>
       <c r="C22" t="s">
-        <v>110</v>
+        <v>132</v>
       </c>
       <c r="D22" t="s">
         <v>28</v>
       </c>
       <c r="E22" t="s">
-        <v>111</v>
+        <v>133</v>
       </c>
       <c r="F22" t="s">
-        <v>97</v>
+        <v>119</v>
       </c>
       <c r="G22" t="s">
-        <v>98</v>
+        <v>120</v>
       </c>
       <c r="H22" t="s">
         <v>29</v>
@@ -1819,13 +2167,13 @@
         <v>30</v>
       </c>
       <c r="J22" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="K22" t="s">
-        <v>99</v>
+        <v>121</v>
       </c>
       <c r="L22" t="s">
-        <v>97</v>
+        <v>119</v>
       </c>
     </row>
     <row r="23">
@@ -1833,22 +2181,22 @@
         <v>28</v>
       </c>
       <c r="B23" t="s">
-        <v>112</v>
+        <v>134</v>
       </c>
       <c r="C23" t="s">
-        <v>113</v>
+        <v>135</v>
       </c>
       <c r="D23" t="s">
         <v>28</v>
       </c>
       <c r="E23" t="s">
-        <v>114</v>
+        <v>136</v>
       </c>
       <c r="F23" t="s">
-        <v>97</v>
+        <v>119</v>
       </c>
       <c r="G23" t="s">
-        <v>98</v>
+        <v>120</v>
       </c>
       <c r="H23" t="s">
         <v>29</v>
@@ -1857,13 +2205,13 @@
         <v>30</v>
       </c>
       <c r="J23" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="K23" t="s">
-        <v>99</v>
+        <v>121</v>
       </c>
       <c r="L23" t="s">
-        <v>97</v>
+        <v>119</v>
       </c>
     </row>
     <row r="24">
@@ -1871,22 +2219,22 @@
         <v>28</v>
       </c>
       <c r="B24" t="s">
-        <v>115</v>
+        <v>137</v>
       </c>
       <c r="C24" t="s">
-        <v>116</v>
+        <v>138</v>
       </c>
       <c r="D24" t="s">
         <v>28</v>
       </c>
       <c r="E24" t="s">
-        <v>117</v>
+        <v>139</v>
       </c>
       <c r="F24" t="s">
-        <v>97</v>
+        <v>119</v>
       </c>
       <c r="G24" t="s">
-        <v>98</v>
+        <v>120</v>
       </c>
       <c r="H24" t="s">
         <v>29</v>
@@ -1895,13 +2243,13 @@
         <v>30</v>
       </c>
       <c r="J24" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="K24" t="s">
-        <v>99</v>
+        <v>121</v>
       </c>
       <c r="L24" t="s">
-        <v>97</v>
+        <v>119</v>
       </c>
     </row>
     <row r="25">
@@ -1909,22 +2257,22 @@
         <v>28</v>
       </c>
       <c r="B25" t="s">
-        <v>118</v>
+        <v>140</v>
       </c>
       <c r="C25" t="s">
+        <v>141</v>
+      </c>
+      <c r="D25" t="s">
+        <v>28</v>
+      </c>
+      <c r="E25" t="s">
+        <v>142</v>
+      </c>
+      <c r="F25" t="s">
         <v>119</v>
       </c>
-      <c r="D25" t="s">
-        <v>28</v>
-      </c>
-      <c r="E25" t="s">
+      <c r="G25" t="s">
         <v>120</v>
-      </c>
-      <c r="F25" t="s">
-        <v>97</v>
-      </c>
-      <c r="G25" t="s">
-        <v>98</v>
       </c>
       <c r="H25" t="s">
         <v>29</v>
@@ -1933,13 +2281,13 @@
         <v>30</v>
       </c>
       <c r="J25" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="K25" t="s">
-        <v>99</v>
+        <v>121</v>
       </c>
       <c r="L25" t="s">
-        <v>97</v>
+        <v>119</v>
       </c>
     </row>
     <row r="26">
@@ -1947,22 +2295,22 @@
         <v>28</v>
       </c>
       <c r="B26" t="s">
-        <v>121</v>
+        <v>143</v>
       </c>
       <c r="C26" t="s">
-        <v>57</v>
+        <v>144</v>
       </c>
       <c r="D26" t="s">
         <v>28</v>
       </c>
       <c r="E26" t="s">
-        <v>58</v>
+        <v>145</v>
       </c>
       <c r="F26" t="s">
-        <v>59</v>
+        <v>146</v>
       </c>
       <c r="G26" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="H26" t="s">
         <v>29</v>
@@ -1977,7 +2325,7 @@
         <v>39</v>
       </c>
       <c r="L26" t="s">
-        <v>59</v>
+        <v>146</v>
       </c>
     </row>
     <row r="27">
@@ -1985,31 +2333,37 @@
         <v>28</v>
       </c>
       <c r="B27" t="s">
-        <v>55</v>
+        <v>147</v>
       </c>
       <c r="C27" t="s">
-        <v>55</v>
+        <v>148</v>
       </c>
       <c r="D27" t="s">
-        <v>55</v>
+        <v>28</v>
       </c>
       <c r="E27" t="s">
-        <v>55</v>
+        <v>149</v>
       </c>
       <c r="F27" t="s">
-        <v>55</v>
+        <v>60</v>
       </c>
       <c r="G27" t="s">
-        <v>55</v>
+        <v>61</v>
       </c>
       <c r="H27" t="s">
-        <v>55</v>
+        <v>29</v>
       </c>
       <c r="I27" t="s">
-        <v>55</v>
+        <v>30</v>
       </c>
       <c r="J27" t="s">
-        <v>55</v>
+        <v>29</v>
+      </c>
+      <c r="K27" t="s">
+        <v>39</v>
+      </c>
+      <c r="L27" t="s">
+        <v>60</v>
       </c>
     </row>
     <row r="28">
@@ -2017,31 +2371,215 @@
         <v>28</v>
       </c>
       <c r="B28" t="s">
-        <v>122</v>
+        <v>150</v>
       </c>
       <c r="C28" t="s">
-        <v>123</v>
+        <v>151</v>
       </c>
       <c r="D28" t="s">
-        <v>55</v>
+        <v>28</v>
       </c>
       <c r="E28" t="s">
-        <v>124</v>
+        <v>152</v>
       </c>
       <c r="F28" t="s">
-        <v>121</v>
+        <v>60</v>
       </c>
       <c r="G28" t="s">
-        <v>55</v>
+        <v>61</v>
       </c>
       <c r="H28" t="s">
-        <v>55</v>
+        <v>29</v>
       </c>
       <c r="I28" t="s">
-        <v>55</v>
+        <v>30</v>
       </c>
       <c r="J28" t="s">
-        <v>55</v>
+        <v>29</v>
+      </c>
+      <c r="K28" t="s">
+        <v>39</v>
+      </c>
+      <c r="L28" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="s">
+        <v>28</v>
+      </c>
+      <c r="B29" t="s">
+        <v>153</v>
+      </c>
+      <c r="C29" t="s">
+        <v>154</v>
+      </c>
+      <c r="D29" t="s">
+        <v>28</v>
+      </c>
+      <c r="E29" t="s">
+        <v>155</v>
+      </c>
+      <c r="F29" t="s">
+        <v>60</v>
+      </c>
+      <c r="G29" t="s">
+        <v>61</v>
+      </c>
+      <c r="H29" t="s">
+        <v>29</v>
+      </c>
+      <c r="I29" t="s">
+        <v>30</v>
+      </c>
+      <c r="J29" t="s">
+        <v>29</v>
+      </c>
+      <c r="K29" t="s">
+        <v>39</v>
+      </c>
+      <c r="L29" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="s">
+        <v>28</v>
+      </c>
+      <c r="B30" t="s">
+        <v>156</v>
+      </c>
+      <c r="C30" t="s">
+        <v>157</v>
+      </c>
+      <c r="D30" t="s">
+        <v>28</v>
+      </c>
+      <c r="E30" t="s">
+        <v>158</v>
+      </c>
+      <c r="F30" t="s">
+        <v>60</v>
+      </c>
+      <c r="G30" t="s">
+        <v>61</v>
+      </c>
+      <c r="H30" t="s">
+        <v>29</v>
+      </c>
+      <c r="I30" t="s">
+        <v>30</v>
+      </c>
+      <c r="J30" t="s">
+        <v>29</v>
+      </c>
+      <c r="K30" t="s">
+        <v>39</v>
+      </c>
+      <c r="L30" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="s">
+        <v>28</v>
+      </c>
+      <c r="B31" t="s">
+        <v>159</v>
+      </c>
+      <c r="C31" t="s">
+        <v>58</v>
+      </c>
+      <c r="D31" t="s">
+        <v>28</v>
+      </c>
+      <c r="E31" t="s">
+        <v>59</v>
+      </c>
+      <c r="F31" t="s">
+        <v>60</v>
+      </c>
+      <c r="G31" t="s">
+        <v>61</v>
+      </c>
+      <c r="H31" t="s">
+        <v>29</v>
+      </c>
+      <c r="I31" t="s">
+        <v>30</v>
+      </c>
+      <c r="J31" t="s">
+        <v>29</v>
+      </c>
+      <c r="K31" t="s">
+        <v>39</v>
+      </c>
+      <c r="L31" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="s">
+        <v>28</v>
+      </c>
+      <c r="B32" t="s">
+        <v>56</v>
+      </c>
+      <c r="C32" t="s">
+        <v>56</v>
+      </c>
+      <c r="D32" t="s">
+        <v>56</v>
+      </c>
+      <c r="E32" t="s">
+        <v>56</v>
+      </c>
+      <c r="F32" t="s">
+        <v>56</v>
+      </c>
+      <c r="G32" t="s">
+        <v>56</v>
+      </c>
+      <c r="H32" t="s">
+        <v>56</v>
+      </c>
+      <c r="I32" t="s">
+        <v>56</v>
+      </c>
+      <c r="J32" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="s">
+        <v>28</v>
+      </c>
+      <c r="B33" t="s">
+        <v>160</v>
+      </c>
+      <c r="C33" t="s">
+        <v>161</v>
+      </c>
+      <c r="D33" t="s">
+        <v>56</v>
+      </c>
+      <c r="E33" t="s">
+        <v>162</v>
+      </c>
+      <c r="F33" t="s">
+        <v>159</v>
+      </c>
+      <c r="G33" t="s">
+        <v>56</v>
+      </c>
+      <c r="H33" t="s">
+        <v>56</v>
+      </c>
+      <c r="I33" t="s">
+        <v>56</v>
+      </c>
+      <c r="J33" t="s">
+        <v>56</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
compiled report 2026-06-09: 16 election events, 11 audit entries
</commit_message>
<xml_diff>
--- a/punmonitor-compiled-report.xlsx
+++ b/punmonitor-compiled-report.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="163" uniqueCount="163">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="181" uniqueCount="181">
   <si>
     <t>Source Date</t>
   </si>
@@ -505,6 +505,60 @@
   </si>
   <si>
     <t>Total events</t>
+  </si>
+  <si>
+    <t>2026-06-09</t>
+  </si>
+  <si>
+    <t>0h 2m 30s</t>
+  </si>
+  <si>
+    <t>2026-06-09 00:05:25</t>
+  </si>
+  <si>
+    <t>0h 7m 51s</t>
+  </si>
+  <si>
+    <t>00:07:55</t>
+  </si>
+  <si>
+    <t>83.0</t>
+  </si>
+  <si>
+    <t>101118.4</t>
+  </si>
+  <si>
+    <t>1168</t>
+  </si>
+  <si>
+    <t>31</t>
+  </si>
+  <si>
+    <t>0h 7m 31s</t>
+  </si>
+  <si>
+    <t>2026-06-09T00:05:42.5586377+05:30</t>
+  </si>
+  <si>
+    <t>00:05:42.558</t>
+  </si>
+  <si>
+    <t>2026-06-09T00:05:42+05:30 (2m13s ago)</t>
+  </si>
+  <si>
+    <t>15</t>
+  </si>
+  <si>
+    <t>2026-06-09T00:01:04.5833579+05:30</t>
+  </si>
+  <si>
+    <t>00:01:04.583</t>
+  </si>
+  <si>
+    <t>16</t>
+  </si>
+  <si>
+    <t>2026-06-09T00:07:55+05:30</t>
   </si>
 </sst>
 </file>
@@ -1105,6 +1159,248 @@
         <v>56</v>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="s">
+        <v>163</v>
+      </c>
+      <c r="B6" t="s">
+        <v>29</v>
+      </c>
+      <c r="C6" t="s">
+        <v>30</v>
+      </c>
+      <c r="D6" t="s">
+        <v>31</v>
+      </c>
+      <c r="E6" t="s">
+        <v>32</v>
+      </c>
+      <c r="F6" t="s">
+        <v>33</v>
+      </c>
+      <c r="G6" t="s">
+        <v>34</v>
+      </c>
+      <c r="H6" t="s">
+        <v>35</v>
+      </c>
+      <c r="I6" t="s">
+        <v>36</v>
+      </c>
+      <c r="J6" t="s">
+        <v>37</v>
+      </c>
+      <c r="K6" t="s">
+        <v>38</v>
+      </c>
+      <c r="L6" t="s">
+        <v>39</v>
+      </c>
+      <c r="M6" t="s">
+        <v>39</v>
+      </c>
+      <c r="N6" t="s">
+        <v>39</v>
+      </c>
+      <c r="O6" t="s">
+        <v>39</v>
+      </c>
+      <c r="P6" t="s">
+        <v>164</v>
+      </c>
+      <c r="Q6" t="s">
+        <v>165</v>
+      </c>
+      <c r="R6" t="s">
+        <v>42</v>
+      </c>
+      <c r="S6" t="s">
+        <v>165</v>
+      </c>
+      <c r="T6" t="s">
+        <v>166</v>
+      </c>
+      <c r="U6" t="s">
+        <v>163</v>
+      </c>
+      <c r="V6" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="s">
+        <v>163</v>
+      </c>
+      <c r="B7" t="s">
+        <v>29</v>
+      </c>
+      <c r="C7" t="s">
+        <v>30</v>
+      </c>
+      <c r="D7" t="s">
+        <v>31</v>
+      </c>
+      <c r="E7" t="s">
+        <v>32</v>
+      </c>
+      <c r="F7" t="s">
+        <v>33</v>
+      </c>
+      <c r="G7" t="s">
+        <v>34</v>
+      </c>
+      <c r="H7" t="s">
+        <v>35</v>
+      </c>
+      <c r="I7" t="s">
+        <v>45</v>
+      </c>
+      <c r="J7" t="s">
+        <v>46</v>
+      </c>
+      <c r="K7" t="s">
+        <v>47</v>
+      </c>
+      <c r="L7" t="s">
+        <v>168</v>
+      </c>
+      <c r="M7" t="s">
+        <v>169</v>
+      </c>
+      <c r="N7" t="s">
+        <v>170</v>
+      </c>
+      <c r="O7" t="s">
+        <v>51</v>
+      </c>
+      <c r="P7" t="s">
+        <v>171</v>
+      </c>
+      <c r="Q7" t="s">
+        <v>53</v>
+      </c>
+      <c r="R7" t="s">
+        <v>42</v>
+      </c>
+      <c r="S7" t="s">
+        <v>165</v>
+      </c>
+      <c r="T7" t="s">
+        <v>172</v>
+      </c>
+      <c r="U7" t="s">
+        <v>163</v>
+      </c>
+      <c r="V7" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="s">
+        <v>163</v>
+      </c>
+      <c r="B8" t="s">
+        <v>55</v>
+      </c>
+      <c r="C8" t="s">
+        <v>56</v>
+      </c>
+      <c r="D8" t="s">
+        <v>56</v>
+      </c>
+      <c r="E8" t="s">
+        <v>56</v>
+      </c>
+      <c r="F8" t="s">
+        <v>56</v>
+      </c>
+      <c r="G8" t="s">
+        <v>56</v>
+      </c>
+      <c r="H8" t="s">
+        <v>56</v>
+      </c>
+      <c r="I8" t="s">
+        <v>56</v>
+      </c>
+      <c r="J8" t="s">
+        <v>56</v>
+      </c>
+      <c r="K8" t="s">
+        <v>56</v>
+      </c>
+      <c r="L8" t="s">
+        <v>56</v>
+      </c>
+      <c r="M8" t="s">
+        <v>56</v>
+      </c>
+      <c r="N8" t="s">
+        <v>56</v>
+      </c>
+      <c r="O8" t="s">
+        <v>56</v>
+      </c>
+      <c r="P8" t="s">
+        <v>56</v>
+      </c>
+      <c r="Q8" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="s">
+        <v>163</v>
+      </c>
+      <c r="B9" t="s">
+        <v>57</v>
+      </c>
+      <c r="C9" t="s">
+        <v>173</v>
+      </c>
+      <c r="D9" t="s">
+        <v>163</v>
+      </c>
+      <c r="E9" t="s">
+        <v>174</v>
+      </c>
+      <c r="F9" t="s">
+        <v>60</v>
+      </c>
+      <c r="G9" t="s">
+        <v>61</v>
+      </c>
+      <c r="H9" t="s">
+        <v>29</v>
+      </c>
+      <c r="I9" t="s">
+        <v>30</v>
+      </c>
+      <c r="J9" t="s">
+        <v>29</v>
+      </c>
+      <c r="K9" t="s">
+        <v>39</v>
+      </c>
+      <c r="L9" t="s">
+        <v>60</v>
+      </c>
+      <c r="M9" t="s">
+        <v>56</v>
+      </c>
+      <c r="N9" t="s">
+        <v>56</v>
+      </c>
+      <c r="O9" t="s">
+        <v>56</v>
+      </c>
+      <c r="P9" t="s">
+        <v>56</v>
+      </c>
+      <c r="Q9" t="s">
+        <v>56</v>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
@@ -1425,6 +1721,292 @@
         <v>80</v>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" t="s">
+        <v>163</v>
+      </c>
+      <c r="B13" t="s">
+        <v>62</v>
+      </c>
+      <c r="C13" t="s">
+        <v>63</v>
+      </c>
+      <c r="D13" t="s">
+        <v>28</v>
+      </c>
+      <c r="E13" t="s">
+        <v>64</v>
+      </c>
+      <c r="F13" t="s">
+        <v>29</v>
+      </c>
+      <c r="G13" t="s">
+        <v>65</v>
+      </c>
+      <c r="H13" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="s">
+        <v>163</v>
+      </c>
+      <c r="B14" t="s">
+        <v>66</v>
+      </c>
+      <c r="C14" t="s">
+        <v>67</v>
+      </c>
+      <c r="D14" t="s">
+        <v>28</v>
+      </c>
+      <c r="E14" t="s">
+        <v>64</v>
+      </c>
+      <c r="F14" t="s">
+        <v>29</v>
+      </c>
+      <c r="G14" t="s">
+        <v>65</v>
+      </c>
+      <c r="H14" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="s">
+        <v>163</v>
+      </c>
+      <c r="B15" t="s">
+        <v>68</v>
+      </c>
+      <c r="C15" t="s">
+        <v>69</v>
+      </c>
+      <c r="D15" t="s">
+        <v>28</v>
+      </c>
+      <c r="E15" t="s">
+        <v>70</v>
+      </c>
+      <c r="F15" t="s">
+        <v>56</v>
+      </c>
+      <c r="G15" t="s">
+        <v>65</v>
+      </c>
+      <c r="H15" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="s">
+        <v>163</v>
+      </c>
+      <c r="B16" t="s">
+        <v>72</v>
+      </c>
+      <c r="C16" t="s">
+        <v>69</v>
+      </c>
+      <c r="D16" t="s">
+        <v>28</v>
+      </c>
+      <c r="E16" t="s">
+        <v>73</v>
+      </c>
+      <c r="F16" t="s">
+        <v>71</v>
+      </c>
+      <c r="G16" t="s">
+        <v>65</v>
+      </c>
+      <c r="H16" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="s">
+        <v>163</v>
+      </c>
+      <c r="B17" t="s">
+        <v>74</v>
+      </c>
+      <c r="C17" t="s">
+        <v>75</v>
+      </c>
+      <c r="D17" t="s">
+        <v>28</v>
+      </c>
+      <c r="E17" t="s">
+        <v>70</v>
+      </c>
+      <c r="F17" t="s">
+        <v>56</v>
+      </c>
+      <c r="G17" t="s">
+        <v>65</v>
+      </c>
+      <c r="H17" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="s">
+        <v>163</v>
+      </c>
+      <c r="B18" t="s">
+        <v>77</v>
+      </c>
+      <c r="C18" t="s">
+        <v>75</v>
+      </c>
+      <c r="D18" t="s">
+        <v>28</v>
+      </c>
+      <c r="E18" t="s">
+        <v>73</v>
+      </c>
+      <c r="F18" t="s">
+        <v>76</v>
+      </c>
+      <c r="G18" t="s">
+        <v>65</v>
+      </c>
+      <c r="H18" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="s">
+        <v>163</v>
+      </c>
+      <c r="B19" t="s">
+        <v>78</v>
+      </c>
+      <c r="C19" t="s">
+        <v>79</v>
+      </c>
+      <c r="D19" t="s">
+        <v>28</v>
+      </c>
+      <c r="E19" t="s">
+        <v>70</v>
+      </c>
+      <c r="F19" t="s">
+        <v>56</v>
+      </c>
+      <c r="G19" t="s">
+        <v>65</v>
+      </c>
+      <c r="H19" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="s">
+        <v>163</v>
+      </c>
+      <c r="B20" t="s">
+        <v>81</v>
+      </c>
+      <c r="C20" t="s">
+        <v>79</v>
+      </c>
+      <c r="D20" t="s">
+        <v>28</v>
+      </c>
+      <c r="E20" t="s">
+        <v>73</v>
+      </c>
+      <c r="F20" t="s">
+        <v>80</v>
+      </c>
+      <c r="G20" t="s">
+        <v>65</v>
+      </c>
+      <c r="H20" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="s">
+        <v>163</v>
+      </c>
+      <c r="B21" t="s">
+        <v>82</v>
+      </c>
+      <c r="C21" t="s">
+        <v>83</v>
+      </c>
+      <c r="D21" t="s">
+        <v>28</v>
+      </c>
+      <c r="E21" t="s">
+        <v>84</v>
+      </c>
+      <c r="F21" t="s">
+        <v>56</v>
+      </c>
+      <c r="G21" t="s">
+        <v>65</v>
+      </c>
+      <c r="H21" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="s">
+        <v>163</v>
+      </c>
+      <c r="B22" t="s">
+        <v>85</v>
+      </c>
+      <c r="C22" t="s">
+        <v>86</v>
+      </c>
+      <c r="D22" t="s">
+        <v>28</v>
+      </c>
+      <c r="E22" t="s">
+        <v>84</v>
+      </c>
+      <c r="F22" t="s">
+        <v>56</v>
+      </c>
+      <c r="G22" t="s">
+        <v>65</v>
+      </c>
+      <c r="H22" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="s">
+        <v>163</v>
+      </c>
+      <c r="B23" t="s">
+        <v>87</v>
+      </c>
+      <c r="C23" t="s">
+        <v>88</v>
+      </c>
+      <c r="D23" t="s">
+        <v>28</v>
+      </c>
+      <c r="E23" t="s">
+        <v>84</v>
+      </c>
+      <c r="F23" t="s">
+        <v>56</v>
+      </c>
+      <c r="G23" t="s">
+        <v>65</v>
+      </c>
+      <c r="H23" t="s">
+        <v>80</v>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
@@ -2582,6 +3164,1199 @@
         <v>56</v>
       </c>
     </row>
+    <row r="34">
+      <c r="A34" t="s">
+        <v>163</v>
+      </c>
+      <c r="B34" t="s">
+        <v>89</v>
+      </c>
+      <c r="C34" t="s">
+        <v>61</v>
+      </c>
+      <c r="D34" t="s">
+        <v>56</v>
+      </c>
+      <c r="E34" t="s">
+        <v>56</v>
+      </c>
+      <c r="F34" t="s">
+        <v>56</v>
+      </c>
+      <c r="G34" t="s">
+        <v>56</v>
+      </c>
+      <c r="H34" t="s">
+        <v>56</v>
+      </c>
+      <c r="I34" t="s">
+        <v>56</v>
+      </c>
+      <c r="J34" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="s">
+        <v>163</v>
+      </c>
+      <c r="B35" t="s">
+        <v>90</v>
+      </c>
+      <c r="C35" t="s">
+        <v>91</v>
+      </c>
+      <c r="D35" t="s">
+        <v>56</v>
+      </c>
+      <c r="E35" t="s">
+        <v>56</v>
+      </c>
+      <c r="F35" t="s">
+        <v>56</v>
+      </c>
+      <c r="G35" t="s">
+        <v>56</v>
+      </c>
+      <c r="H35" t="s">
+        <v>56</v>
+      </c>
+      <c r="I35" t="s">
+        <v>56</v>
+      </c>
+      <c r="J35" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="s">
+        <v>163</v>
+      </c>
+      <c r="B36" t="s">
+        <v>92</v>
+      </c>
+      <c r="C36" t="s">
+        <v>93</v>
+      </c>
+      <c r="D36" t="s">
+        <v>56</v>
+      </c>
+      <c r="E36" t="s">
+        <v>56</v>
+      </c>
+      <c r="F36" t="s">
+        <v>56</v>
+      </c>
+      <c r="G36" t="s">
+        <v>56</v>
+      </c>
+      <c r="H36" t="s">
+        <v>56</v>
+      </c>
+      <c r="I36" t="s">
+        <v>56</v>
+      </c>
+      <c r="J36" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="s">
+        <v>163</v>
+      </c>
+      <c r="B37" t="s">
+        <v>94</v>
+      </c>
+      <c r="C37" t="s">
+        <v>29</v>
+      </c>
+      <c r="D37" t="s">
+        <v>56</v>
+      </c>
+      <c r="E37" t="s">
+        <v>56</v>
+      </c>
+      <c r="F37" t="s">
+        <v>56</v>
+      </c>
+      <c r="G37" t="s">
+        <v>56</v>
+      </c>
+      <c r="H37" t="s">
+        <v>56</v>
+      </c>
+      <c r="I37" t="s">
+        <v>56</v>
+      </c>
+      <c r="J37" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="s">
+        <v>163</v>
+      </c>
+      <c r="B38" t="s">
+        <v>95</v>
+      </c>
+      <c r="C38" t="s">
+        <v>30</v>
+      </c>
+      <c r="D38" t="s">
+        <v>56</v>
+      </c>
+      <c r="E38" t="s">
+        <v>56</v>
+      </c>
+      <c r="F38" t="s">
+        <v>56</v>
+      </c>
+      <c r="G38" t="s">
+        <v>56</v>
+      </c>
+      <c r="H38" t="s">
+        <v>56</v>
+      </c>
+      <c r="I38" t="s">
+        <v>56</v>
+      </c>
+      <c r="J38" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="s">
+        <v>163</v>
+      </c>
+      <c r="B39" t="s">
+        <v>96</v>
+      </c>
+      <c r="C39" t="s">
+        <v>97</v>
+      </c>
+      <c r="D39" t="s">
+        <v>56</v>
+      </c>
+      <c r="E39" t="s">
+        <v>56</v>
+      </c>
+      <c r="F39" t="s">
+        <v>56</v>
+      </c>
+      <c r="G39" t="s">
+        <v>56</v>
+      </c>
+      <c r="H39" t="s">
+        <v>56</v>
+      </c>
+      <c r="I39" t="s">
+        <v>56</v>
+      </c>
+      <c r="J39" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="s">
+        <v>163</v>
+      </c>
+      <c r="B40" t="s">
+        <v>98</v>
+      </c>
+      <c r="C40" t="s">
+        <v>99</v>
+      </c>
+      <c r="D40" t="s">
+        <v>56</v>
+      </c>
+      <c r="E40" t="s">
+        <v>56</v>
+      </c>
+      <c r="F40" t="s">
+        <v>56</v>
+      </c>
+      <c r="G40" t="s">
+        <v>56</v>
+      </c>
+      <c r="H40" t="s">
+        <v>56</v>
+      </c>
+      <c r="I40" t="s">
+        <v>56</v>
+      </c>
+      <c r="J40" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="s">
+        <v>163</v>
+      </c>
+      <c r="B41" t="s">
+        <v>100</v>
+      </c>
+      <c r="C41" t="s">
+        <v>29</v>
+      </c>
+      <c r="D41" t="s">
+        <v>56</v>
+      </c>
+      <c r="E41" t="s">
+        <v>56</v>
+      </c>
+      <c r="F41" t="s">
+        <v>56</v>
+      </c>
+      <c r="G41" t="s">
+        <v>56</v>
+      </c>
+      <c r="H41" t="s">
+        <v>56</v>
+      </c>
+      <c r="I41" t="s">
+        <v>56</v>
+      </c>
+      <c r="J41" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="s">
+        <v>163</v>
+      </c>
+      <c r="B42" t="s">
+        <v>101</v>
+      </c>
+      <c r="C42" t="s">
+        <v>175</v>
+      </c>
+      <c r="D42" t="s">
+        <v>56</v>
+      </c>
+      <c r="E42" t="s">
+        <v>56</v>
+      </c>
+      <c r="F42" t="s">
+        <v>56</v>
+      </c>
+      <c r="G42" t="s">
+        <v>56</v>
+      </c>
+      <c r="H42" t="s">
+        <v>56</v>
+      </c>
+      <c r="I42" t="s">
+        <v>56</v>
+      </c>
+      <c r="J42" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="s">
+        <v>163</v>
+      </c>
+      <c r="B43" t="s">
+        <v>103</v>
+      </c>
+      <c r="C43" t="s">
+        <v>104</v>
+      </c>
+      <c r="D43" t="s">
+        <v>56</v>
+      </c>
+      <c r="E43" t="s">
+        <v>56</v>
+      </c>
+      <c r="F43" t="s">
+        <v>56</v>
+      </c>
+      <c r="G43" t="s">
+        <v>56</v>
+      </c>
+      <c r="H43" t="s">
+        <v>56</v>
+      </c>
+      <c r="I43" t="s">
+        <v>56</v>
+      </c>
+      <c r="J43" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="s">
+        <v>163</v>
+      </c>
+      <c r="B44" t="s">
+        <v>105</v>
+      </c>
+      <c r="C44" t="s">
+        <v>175</v>
+      </c>
+      <c r="D44" t="s">
+        <v>56</v>
+      </c>
+      <c r="E44" t="s">
+        <v>56</v>
+      </c>
+      <c r="F44" t="s">
+        <v>56</v>
+      </c>
+      <c r="G44" t="s">
+        <v>56</v>
+      </c>
+      <c r="H44" t="s">
+        <v>56</v>
+      </c>
+      <c r="I44" t="s">
+        <v>56</v>
+      </c>
+      <c r="J44" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="s">
+        <v>163</v>
+      </c>
+      <c r="B45" t="s">
+        <v>106</v>
+      </c>
+      <c r="C45" t="s">
+        <v>107</v>
+      </c>
+      <c r="D45" t="s">
+        <v>56</v>
+      </c>
+      <c r="E45" t="s">
+        <v>56</v>
+      </c>
+      <c r="F45" t="s">
+        <v>56</v>
+      </c>
+      <c r="G45" t="s">
+        <v>56</v>
+      </c>
+      <c r="H45" t="s">
+        <v>56</v>
+      </c>
+      <c r="I45" t="s">
+        <v>56</v>
+      </c>
+      <c r="J45" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="s">
+        <v>163</v>
+      </c>
+      <c r="B46" t="s">
+        <v>108</v>
+      </c>
+      <c r="C46" t="s">
+        <v>109</v>
+      </c>
+      <c r="D46" t="s">
+        <v>56</v>
+      </c>
+      <c r="E46" t="s">
+        <v>56</v>
+      </c>
+      <c r="F46" t="s">
+        <v>56</v>
+      </c>
+      <c r="G46" t="s">
+        <v>56</v>
+      </c>
+      <c r="H46" t="s">
+        <v>56</v>
+      </c>
+      <c r="I46" t="s">
+        <v>56</v>
+      </c>
+      <c r="J46" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="s">
+        <v>163</v>
+      </c>
+      <c r="B47" t="s">
+        <v>56</v>
+      </c>
+      <c r="C47" t="s">
+        <v>56</v>
+      </c>
+      <c r="D47" t="s">
+        <v>56</v>
+      </c>
+      <c r="E47" t="s">
+        <v>56</v>
+      </c>
+      <c r="F47" t="s">
+        <v>56</v>
+      </c>
+      <c r="G47" t="s">
+        <v>56</v>
+      </c>
+      <c r="H47" t="s">
+        <v>56</v>
+      </c>
+      <c r="I47" t="s">
+        <v>56</v>
+      </c>
+      <c r="J47" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="s">
+        <v>163</v>
+      </c>
+      <c r="B48" t="s">
+        <v>110</v>
+      </c>
+      <c r="C48" t="s">
+        <v>56</v>
+      </c>
+      <c r="D48" t="s">
+        <v>56</v>
+      </c>
+      <c r="E48" t="s">
+        <v>56</v>
+      </c>
+      <c r="F48" t="s">
+        <v>56</v>
+      </c>
+      <c r="G48" t="s">
+        <v>56</v>
+      </c>
+      <c r="H48" t="s">
+        <v>56</v>
+      </c>
+      <c r="I48" t="s">
+        <v>56</v>
+      </c>
+      <c r="J48" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="s">
+        <v>163</v>
+      </c>
+      <c r="B49" t="s">
+        <v>111</v>
+      </c>
+      <c r="C49" t="s">
+        <v>112</v>
+      </c>
+      <c r="D49" t="s">
+        <v>113</v>
+      </c>
+      <c r="E49" t="s">
+        <v>114</v>
+      </c>
+      <c r="F49" t="s">
+        <v>19</v>
+      </c>
+      <c r="G49" t="s">
+        <v>23</v>
+      </c>
+      <c r="H49" t="s">
+        <v>115</v>
+      </c>
+      <c r="I49" t="s">
+        <v>2</v>
+      </c>
+      <c r="J49" t="s">
+        <v>24</v>
+      </c>
+      <c r="K49" t="s">
+        <v>116</v>
+      </c>
+      <c r="L49" t="s">
+        <v>26</v>
+      </c>
+      <c r="M49" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="s">
+        <v>163</v>
+      </c>
+      <c r="B50" t="s">
+        <v>107</v>
+      </c>
+      <c r="C50" t="s">
+        <v>117</v>
+      </c>
+      <c r="D50" t="s">
+        <v>28</v>
+      </c>
+      <c r="E50" t="s">
+        <v>118</v>
+      </c>
+      <c r="F50" t="s">
+        <v>119</v>
+      </c>
+      <c r="G50" t="s">
+        <v>120</v>
+      </c>
+      <c r="H50" t="s">
+        <v>29</v>
+      </c>
+      <c r="I50" t="s">
+        <v>30</v>
+      </c>
+      <c r="J50" t="s">
+        <v>56</v>
+      </c>
+      <c r="K50" t="s">
+        <v>121</v>
+      </c>
+      <c r="L50" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="s">
+        <v>163</v>
+      </c>
+      <c r="B51" t="s">
+        <v>122</v>
+      </c>
+      <c r="C51" t="s">
+        <v>123</v>
+      </c>
+      <c r="D51" t="s">
+        <v>28</v>
+      </c>
+      <c r="E51" t="s">
+        <v>124</v>
+      </c>
+      <c r="F51" t="s">
+        <v>119</v>
+      </c>
+      <c r="G51" t="s">
+        <v>120</v>
+      </c>
+      <c r="H51" t="s">
+        <v>29</v>
+      </c>
+      <c r="I51" t="s">
+        <v>30</v>
+      </c>
+      <c r="J51" t="s">
+        <v>56</v>
+      </c>
+      <c r="K51" t="s">
+        <v>121</v>
+      </c>
+      <c r="L51" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="s">
+        <v>163</v>
+      </c>
+      <c r="B52" t="s">
+        <v>125</v>
+      </c>
+      <c r="C52" t="s">
+        <v>126</v>
+      </c>
+      <c r="D52" t="s">
+        <v>28</v>
+      </c>
+      <c r="E52" t="s">
+        <v>127</v>
+      </c>
+      <c r="F52" t="s">
+        <v>119</v>
+      </c>
+      <c r="G52" t="s">
+        <v>120</v>
+      </c>
+      <c r="H52" t="s">
+        <v>29</v>
+      </c>
+      <c r="I52" t="s">
+        <v>30</v>
+      </c>
+      <c r="J52" t="s">
+        <v>56</v>
+      </c>
+      <c r="K52" t="s">
+        <v>121</v>
+      </c>
+      <c r="L52" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="s">
+        <v>163</v>
+      </c>
+      <c r="B53" t="s">
+        <v>128</v>
+      </c>
+      <c r="C53" t="s">
+        <v>129</v>
+      </c>
+      <c r="D53" t="s">
+        <v>28</v>
+      </c>
+      <c r="E53" t="s">
+        <v>130</v>
+      </c>
+      <c r="F53" t="s">
+        <v>119</v>
+      </c>
+      <c r="G53" t="s">
+        <v>120</v>
+      </c>
+      <c r="H53" t="s">
+        <v>29</v>
+      </c>
+      <c r="I53" t="s">
+        <v>30</v>
+      </c>
+      <c r="J53" t="s">
+        <v>56</v>
+      </c>
+      <c r="K53" t="s">
+        <v>121</v>
+      </c>
+      <c r="L53" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="s">
+        <v>163</v>
+      </c>
+      <c r="B54" t="s">
+        <v>131</v>
+      </c>
+      <c r="C54" t="s">
+        <v>132</v>
+      </c>
+      <c r="D54" t="s">
+        <v>28</v>
+      </c>
+      <c r="E54" t="s">
+        <v>133</v>
+      </c>
+      <c r="F54" t="s">
+        <v>119</v>
+      </c>
+      <c r="G54" t="s">
+        <v>120</v>
+      </c>
+      <c r="H54" t="s">
+        <v>29</v>
+      </c>
+      <c r="I54" t="s">
+        <v>30</v>
+      </c>
+      <c r="J54" t="s">
+        <v>56</v>
+      </c>
+      <c r="K54" t="s">
+        <v>121</v>
+      </c>
+      <c r="L54" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="s">
+        <v>163</v>
+      </c>
+      <c r="B55" t="s">
+        <v>134</v>
+      </c>
+      <c r="C55" t="s">
+        <v>135</v>
+      </c>
+      <c r="D55" t="s">
+        <v>28</v>
+      </c>
+      <c r="E55" t="s">
+        <v>136</v>
+      </c>
+      <c r="F55" t="s">
+        <v>119</v>
+      </c>
+      <c r="G55" t="s">
+        <v>120</v>
+      </c>
+      <c r="H55" t="s">
+        <v>29</v>
+      </c>
+      <c r="I55" t="s">
+        <v>30</v>
+      </c>
+      <c r="J55" t="s">
+        <v>56</v>
+      </c>
+      <c r="K55" t="s">
+        <v>121</v>
+      </c>
+      <c r="L55" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="s">
+        <v>163</v>
+      </c>
+      <c r="B56" t="s">
+        <v>137</v>
+      </c>
+      <c r="C56" t="s">
+        <v>138</v>
+      </c>
+      <c r="D56" t="s">
+        <v>28</v>
+      </c>
+      <c r="E56" t="s">
+        <v>139</v>
+      </c>
+      <c r="F56" t="s">
+        <v>119</v>
+      </c>
+      <c r="G56" t="s">
+        <v>120</v>
+      </c>
+      <c r="H56" t="s">
+        <v>29</v>
+      </c>
+      <c r="I56" t="s">
+        <v>30</v>
+      </c>
+      <c r="J56" t="s">
+        <v>56</v>
+      </c>
+      <c r="K56" t="s">
+        <v>121</v>
+      </c>
+      <c r="L56" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="s">
+        <v>163</v>
+      </c>
+      <c r="B57" t="s">
+        <v>140</v>
+      </c>
+      <c r="C57" t="s">
+        <v>141</v>
+      </c>
+      <c r="D57" t="s">
+        <v>28</v>
+      </c>
+      <c r="E57" t="s">
+        <v>142</v>
+      </c>
+      <c r="F57" t="s">
+        <v>119</v>
+      </c>
+      <c r="G57" t="s">
+        <v>120</v>
+      </c>
+      <c r="H57" t="s">
+        <v>29</v>
+      </c>
+      <c r="I57" t="s">
+        <v>30</v>
+      </c>
+      <c r="J57" t="s">
+        <v>56</v>
+      </c>
+      <c r="K57" t="s">
+        <v>121</v>
+      </c>
+      <c r="L57" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="s">
+        <v>163</v>
+      </c>
+      <c r="B58" t="s">
+        <v>143</v>
+      </c>
+      <c r="C58" t="s">
+        <v>144</v>
+      </c>
+      <c r="D58" t="s">
+        <v>28</v>
+      </c>
+      <c r="E58" t="s">
+        <v>145</v>
+      </c>
+      <c r="F58" t="s">
+        <v>146</v>
+      </c>
+      <c r="G58" t="s">
+        <v>61</v>
+      </c>
+      <c r="H58" t="s">
+        <v>29</v>
+      </c>
+      <c r="I58" t="s">
+        <v>30</v>
+      </c>
+      <c r="J58" t="s">
+        <v>29</v>
+      </c>
+      <c r="K58" t="s">
+        <v>39</v>
+      </c>
+      <c r="L58" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="s">
+        <v>163</v>
+      </c>
+      <c r="B59" t="s">
+        <v>147</v>
+      </c>
+      <c r="C59" t="s">
+        <v>148</v>
+      </c>
+      <c r="D59" t="s">
+        <v>28</v>
+      </c>
+      <c r="E59" t="s">
+        <v>149</v>
+      </c>
+      <c r="F59" t="s">
+        <v>60</v>
+      </c>
+      <c r="G59" t="s">
+        <v>61</v>
+      </c>
+      <c r="H59" t="s">
+        <v>29</v>
+      </c>
+      <c r="I59" t="s">
+        <v>30</v>
+      </c>
+      <c r="J59" t="s">
+        <v>29</v>
+      </c>
+      <c r="K59" t="s">
+        <v>39</v>
+      </c>
+      <c r="L59" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="s">
+        <v>163</v>
+      </c>
+      <c r="B60" t="s">
+        <v>150</v>
+      </c>
+      <c r="C60" t="s">
+        <v>151</v>
+      </c>
+      <c r="D60" t="s">
+        <v>28</v>
+      </c>
+      <c r="E60" t="s">
+        <v>152</v>
+      </c>
+      <c r="F60" t="s">
+        <v>60</v>
+      </c>
+      <c r="G60" t="s">
+        <v>61</v>
+      </c>
+      <c r="H60" t="s">
+        <v>29</v>
+      </c>
+      <c r="I60" t="s">
+        <v>30</v>
+      </c>
+      <c r="J60" t="s">
+        <v>29</v>
+      </c>
+      <c r="K60" t="s">
+        <v>39</v>
+      </c>
+      <c r="L60" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="s">
+        <v>163</v>
+      </c>
+      <c r="B61" t="s">
+        <v>153</v>
+      </c>
+      <c r="C61" t="s">
+        <v>154</v>
+      </c>
+      <c r="D61" t="s">
+        <v>28</v>
+      </c>
+      <c r="E61" t="s">
+        <v>155</v>
+      </c>
+      <c r="F61" t="s">
+        <v>60</v>
+      </c>
+      <c r="G61" t="s">
+        <v>61</v>
+      </c>
+      <c r="H61" t="s">
+        <v>29</v>
+      </c>
+      <c r="I61" t="s">
+        <v>30</v>
+      </c>
+      <c r="J61" t="s">
+        <v>29</v>
+      </c>
+      <c r="K61" t="s">
+        <v>39</v>
+      </c>
+      <c r="L61" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="s">
+        <v>163</v>
+      </c>
+      <c r="B62" t="s">
+        <v>156</v>
+      </c>
+      <c r="C62" t="s">
+        <v>157</v>
+      </c>
+      <c r="D62" t="s">
+        <v>28</v>
+      </c>
+      <c r="E62" t="s">
+        <v>158</v>
+      </c>
+      <c r="F62" t="s">
+        <v>60</v>
+      </c>
+      <c r="G62" t="s">
+        <v>61</v>
+      </c>
+      <c r="H62" t="s">
+        <v>29</v>
+      </c>
+      <c r="I62" t="s">
+        <v>30</v>
+      </c>
+      <c r="J62" t="s">
+        <v>29</v>
+      </c>
+      <c r="K62" t="s">
+        <v>39</v>
+      </c>
+      <c r="L62" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="s">
+        <v>163</v>
+      </c>
+      <c r="B63" t="s">
+        <v>159</v>
+      </c>
+      <c r="C63" t="s">
+        <v>58</v>
+      </c>
+      <c r="D63" t="s">
+        <v>28</v>
+      </c>
+      <c r="E63" t="s">
+        <v>59</v>
+      </c>
+      <c r="F63" t="s">
+        <v>60</v>
+      </c>
+      <c r="G63" t="s">
+        <v>61</v>
+      </c>
+      <c r="H63" t="s">
+        <v>29</v>
+      </c>
+      <c r="I63" t="s">
+        <v>30</v>
+      </c>
+      <c r="J63" t="s">
+        <v>29</v>
+      </c>
+      <c r="K63" t="s">
+        <v>39</v>
+      </c>
+      <c r="L63" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="s">
+        <v>163</v>
+      </c>
+      <c r="B64" t="s">
+        <v>176</v>
+      </c>
+      <c r="C64" t="s">
+        <v>177</v>
+      </c>
+      <c r="D64" t="s">
+        <v>163</v>
+      </c>
+      <c r="E64" t="s">
+        <v>178</v>
+      </c>
+      <c r="F64" t="s">
+        <v>60</v>
+      </c>
+      <c r="G64" t="s">
+        <v>61</v>
+      </c>
+      <c r="H64" t="s">
+        <v>29</v>
+      </c>
+      <c r="I64" t="s">
+        <v>30</v>
+      </c>
+      <c r="J64" t="s">
+        <v>29</v>
+      </c>
+      <c r="K64" t="s">
+        <v>39</v>
+      </c>
+      <c r="L64" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="s">
+        <v>163</v>
+      </c>
+      <c r="B65" t="s">
+        <v>179</v>
+      </c>
+      <c r="C65" t="s">
+        <v>173</v>
+      </c>
+      <c r="D65" t="s">
+        <v>163</v>
+      </c>
+      <c r="E65" t="s">
+        <v>174</v>
+      </c>
+      <c r="F65" t="s">
+        <v>60</v>
+      </c>
+      <c r="G65" t="s">
+        <v>61</v>
+      </c>
+      <c r="H65" t="s">
+        <v>29</v>
+      </c>
+      <c r="I65" t="s">
+        <v>30</v>
+      </c>
+      <c r="J65" t="s">
+        <v>29</v>
+      </c>
+      <c r="K65" t="s">
+        <v>39</v>
+      </c>
+      <c r="L65" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="s">
+        <v>163</v>
+      </c>
+      <c r="B66" t="s">
+        <v>56</v>
+      </c>
+      <c r="C66" t="s">
+        <v>56</v>
+      </c>
+      <c r="D66" t="s">
+        <v>56</v>
+      </c>
+      <c r="E66" t="s">
+        <v>56</v>
+      </c>
+      <c r="F66" t="s">
+        <v>56</v>
+      </c>
+      <c r="G66" t="s">
+        <v>56</v>
+      </c>
+      <c r="H66" t="s">
+        <v>56</v>
+      </c>
+      <c r="I66" t="s">
+        <v>56</v>
+      </c>
+      <c r="J66" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="s">
+        <v>163</v>
+      </c>
+      <c r="B67" t="s">
+        <v>160</v>
+      </c>
+      <c r="C67" t="s">
+        <v>180</v>
+      </c>
+      <c r="D67" t="s">
+        <v>56</v>
+      </c>
+      <c r="E67" t="s">
+        <v>162</v>
+      </c>
+      <c r="F67" t="s">
+        <v>179</v>
+      </c>
+      <c r="G67" t="s">
+        <v>56</v>
+      </c>
+      <c r="H67" t="s">
+        <v>56</v>
+      </c>
+      <c r="I67" t="s">
+        <v>56</v>
+      </c>
+      <c r="J67" t="s">
+        <v>56</v>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
compiled report 2026-06-22: 695 election events, 279 audit entries
</commit_message>
<xml_diff>
--- a/punmonitor-compiled-report.xlsx
+++ b/punmonitor-compiled-report.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2820" uniqueCount="2820">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2828" uniqueCount="2828">
   <si>
     <t>Source Date</t>
   </si>
@@ -8074,25 +8074,412 @@
     <t>2026-06-22</t>
   </si>
   <si>
-    <t>0h 2m 18s</t>
+    <t>0h 12m 33s</t>
   </si>
   <si>
     <t>2026-06-22 22:40:40</t>
   </si>
   <si>
-    <t>25h 21m 3s</t>
-  </si>
-  <si>
-    <t>22:42:58</t>
+    <t>25h 24m 45s</t>
+  </si>
+  <si>
+    <t>22:53:13</t>
   </si>
   <si>
     <t>10.0.64</t>
   </si>
   <si>
-    <t>disconnected</t>
-  </si>
-  <si>
-    <t>offline</t>
+    <t>websocket</t>
+  </si>
+  <si>
+    <t>147.0</t>
+  </si>
+  <si>
+    <t>157835.5</t>
+  </si>
+  <si>
+    <t>0h 3m 12s</t>
+  </si>
+  <si>
+    <t>2026-06-22T22:50:59.9398109+05:30</t>
+  </si>
+  <si>
+    <t>22:50:59.939</t>
+  </si>
+  <si>
+    <t>2026-06-22T22:51:13+05:30 (2m0s ago)</t>
+  </si>
+  <si>
+    <t>651</t>
+  </si>
+  <si>
+    <t>2026-06-19T13:41:33.4313429+05:30</t>
+  </si>
+  <si>
+    <t>13:41:33.431</t>
+  </si>
+  <si>
+    <t>652</t>
+  </si>
+  <si>
+    <t>2026-06-19T13:46:33.4190791+05:30</t>
+  </si>
+  <si>
+    <t>13:46:33.419</t>
+  </si>
+  <si>
+    <t>653</t>
+  </si>
+  <si>
+    <t>2026-06-19T13:51:33.3835925+05:30</t>
+  </si>
+  <si>
+    <t>13:51:33.383</t>
+  </si>
+  <si>
+    <t>654</t>
+  </si>
+  <si>
+    <t>2026-06-19T13:56:33.4354335+05:30</t>
+  </si>
+  <si>
+    <t>13:56:33.435</t>
+  </si>
+  <si>
+    <t>655</t>
+  </si>
+  <si>
+    <t>2026-06-19T14:01:33.7407703+05:30</t>
+  </si>
+  <si>
+    <t>14:01:33.740</t>
+  </si>
+  <si>
+    <t>656</t>
+  </si>
+  <si>
+    <t>2026-06-19T14:06:33.3700386+05:30</t>
+  </si>
+  <si>
+    <t>14:06:33.370</t>
+  </si>
+  <si>
+    <t>657</t>
+  </si>
+  <si>
+    <t>2026-06-19T14:11:33.4795473+05:30</t>
+  </si>
+  <si>
+    <t>14:11:33.479</t>
+  </si>
+  <si>
+    <t>658</t>
+  </si>
+  <si>
+    <t>2026-06-19T14:16:33.5114074+05:30</t>
+  </si>
+  <si>
+    <t>14:16:33.511</t>
+  </si>
+  <si>
+    <t>659</t>
+  </si>
+  <si>
+    <t>2026-06-19T14:21:33.3706767+05:30</t>
+  </si>
+  <si>
+    <t>14:21:33.370</t>
+  </si>
+  <si>
+    <t>660</t>
+  </si>
+  <si>
+    <t>2026-06-19T14:26:33.363807+05:30</t>
+  </si>
+  <si>
+    <t>14:26:33.363</t>
+  </si>
+  <si>
+    <t>661</t>
+  </si>
+  <si>
+    <t>2026-06-19T14:31:33.5627385+05:30</t>
+  </si>
+  <si>
+    <t>14:31:33.562</t>
+  </si>
+  <si>
+    <t>662</t>
+  </si>
+  <si>
+    <t>2026-06-19T14:36:33.3229665+05:30</t>
+  </si>
+  <si>
+    <t>14:36:33.322</t>
+  </si>
+  <si>
+    <t>663</t>
+  </si>
+  <si>
+    <t>2026-06-19T14:41:33.541576+05:30</t>
+  </si>
+  <si>
+    <t>14:41:33.541</t>
+  </si>
+  <si>
+    <t>664</t>
+  </si>
+  <si>
+    <t>2026-06-19T14:46:33.3714413+05:30</t>
+  </si>
+  <si>
+    <t>14:46:33.371</t>
+  </si>
+  <si>
+    <t>665</t>
+  </si>
+  <si>
+    <t>2026-06-19T14:51:33.6029029+05:30</t>
+  </si>
+  <si>
+    <t>14:51:33.602</t>
+  </si>
+  <si>
+    <t>666</t>
+  </si>
+  <si>
+    <t>2026-06-19T14:56:33.4305433+05:30</t>
+  </si>
+  <si>
+    <t>14:56:33.430</t>
+  </si>
+  <si>
+    <t>667</t>
+  </si>
+  <si>
+    <t>2026-06-19T15:01:33.3535668+05:30</t>
+  </si>
+  <si>
+    <t>15:01:33.353</t>
+  </si>
+  <si>
+    <t>668</t>
+  </si>
+  <si>
+    <t>2026-06-19T15:06:33.3925169+05:30</t>
+  </si>
+  <si>
+    <t>15:06:33.392</t>
+  </si>
+  <si>
+    <t>669</t>
+  </si>
+  <si>
+    <t>2026-06-19T15:11:33.4331604+05:30</t>
+  </si>
+  <si>
+    <t>15:11:33.433</t>
+  </si>
+  <si>
+    <t>670</t>
+  </si>
+  <si>
+    <t>2026-06-19T15:16:33.3516037+05:30</t>
+  </si>
+  <si>
+    <t>15:16:33.351</t>
+  </si>
+  <si>
+    <t>671</t>
+  </si>
+  <si>
+    <t>2026-06-19T15:21:33.3924164+05:30</t>
+  </si>
+  <si>
+    <t>15:21:33.392</t>
+  </si>
+  <si>
+    <t>672</t>
+  </si>
+  <si>
+    <t>2026-06-19T15:26:33.4384617+05:30</t>
+  </si>
+  <si>
+    <t>15:26:33.438</t>
+  </si>
+  <si>
+    <t>673</t>
+  </si>
+  <si>
+    <t>2026-06-19T15:31:33.6068702+05:30</t>
+  </si>
+  <si>
+    <t>15:31:33.606</t>
+  </si>
+  <si>
+    <t>674</t>
+  </si>
+  <si>
+    <t>2026-06-19T15:36:33.5456911+05:30</t>
+  </si>
+  <si>
+    <t>15:36:33.545</t>
+  </si>
+  <si>
+    <t>675</t>
+  </si>
+  <si>
+    <t>2026-06-19T16:24:14.9858131+05:30</t>
+  </si>
+  <si>
+    <t>16:24:14.985</t>
+  </si>
+  <si>
+    <t>676</t>
+  </si>
+  <si>
+    <t>2026-06-19T16:24:15.02211+05:30</t>
+  </si>
+  <si>
+    <t>16:24:15.022</t>
+  </si>
+  <si>
+    <t>677</t>
+  </si>
+  <si>
+    <t>2026-06-19T16:26:33.4755019+05:30</t>
+  </si>
+  <si>
+    <t>16:26:33.475</t>
+  </si>
+  <si>
+    <t>678</t>
+  </si>
+  <si>
+    <t>2026-06-19T16:31:33.4203387+05:30</t>
+  </si>
+  <si>
+    <t>16:31:33.420</t>
+  </si>
+  <si>
+    <t>679</t>
+  </si>
+  <si>
+    <t>2026-06-19T16:36:33.3819816+05:30</t>
+  </si>
+  <si>
+    <t>16:36:33.381</t>
+  </si>
+  <si>
+    <t>680</t>
+  </si>
+  <si>
+    <t>2026-06-19T16:41:33.4184754+05:30</t>
+  </si>
+  <si>
+    <t>16:41:33.418</t>
+  </si>
+  <si>
+    <t>681</t>
+  </si>
+  <si>
+    <t>2026-06-19T16:46:33.4420373+05:30</t>
+  </si>
+  <si>
+    <t>16:46:33.442</t>
+  </si>
+  <si>
+    <t>682</t>
+  </si>
+  <si>
+    <t>2026-06-19T16:51:33.5318237+05:30</t>
+  </si>
+  <si>
+    <t>16:51:33.531</t>
+  </si>
+  <si>
+    <t>683</t>
+  </si>
+  <si>
+    <t>2026-06-19T16:56:33.6498773+05:30</t>
+  </si>
+  <si>
+    <t>16:56:33.649</t>
+  </si>
+  <si>
+    <t>684</t>
+  </si>
+  <si>
+    <t>2026-06-19T17:01:33.4809208+05:30</t>
+  </si>
+  <si>
+    <t>17:01:33.480</t>
+  </si>
+  <si>
+    <t>685</t>
+  </si>
+  <si>
+    <t>2026-06-19T17:06:33.3155595+05:30</t>
+  </si>
+  <si>
+    <t>17:06:33.315</t>
+  </si>
+  <si>
+    <t>686</t>
+  </si>
+  <si>
+    <t>2026-06-19T17:11:33.6164892+05:30</t>
+  </si>
+  <si>
+    <t>17:11:33.616</t>
+  </si>
+  <si>
+    <t>687</t>
+  </si>
+  <si>
+    <t>2026-06-19T17:16:33.5217144+05:30</t>
+  </si>
+  <si>
+    <t>17:16:33.521</t>
+  </si>
+  <si>
+    <t>688</t>
+  </si>
+  <si>
+    <t>2026-06-19T17:21:33.536392+05:30</t>
+  </si>
+  <si>
+    <t>17:21:33.536</t>
+  </si>
+  <si>
+    <t>689</t>
+  </si>
+  <si>
+    <t>2026-06-19T17:26:33.3735547+05:30</t>
+  </si>
+  <si>
+    <t>17:26:33.373</t>
+  </si>
+  <si>
+    <t>690</t>
+  </si>
+  <si>
+    <t>2026-06-19T17:31:33.4136351+05:30</t>
+  </si>
+  <si>
+    <t>17:31:33.413</t>
+  </si>
+  <si>
+    <t>691</t>
+  </si>
+  <si>
+    <t>2026-06-19T17:36:33.4154161+05:30</t>
+  </si>
+  <si>
+    <t>17:36:33.415</t>
+  </si>
+  <si>
+    <t>692</t>
   </si>
   <si>
     <t>2026-06-22T22:40:57.9979938+05:30</t>
@@ -8101,382 +8488,19 @@
     <t>22:40:57.997</t>
   </si>
   <si>
-    <t>2026-06-22T22:40:57+05:30 (2m0s ago)</t>
-  </si>
-  <si>
-    <t>651</t>
-  </si>
-  <si>
-    <t>2026-06-19T13:41:33.4313429+05:30</t>
-  </si>
-  <si>
-    <t>13:41:33.431</t>
-  </si>
-  <si>
-    <t>652</t>
-  </si>
-  <si>
-    <t>2026-06-19T13:46:33.4190791+05:30</t>
-  </si>
-  <si>
-    <t>13:46:33.419</t>
-  </si>
-  <si>
-    <t>653</t>
-  </si>
-  <si>
-    <t>2026-06-19T13:51:33.3835925+05:30</t>
-  </si>
-  <si>
-    <t>13:51:33.383</t>
-  </si>
-  <si>
-    <t>654</t>
-  </si>
-  <si>
-    <t>2026-06-19T13:56:33.4354335+05:30</t>
-  </si>
-  <si>
-    <t>13:56:33.435</t>
-  </si>
-  <si>
-    <t>655</t>
-  </si>
-  <si>
-    <t>2026-06-19T14:01:33.7407703+05:30</t>
-  </si>
-  <si>
-    <t>14:01:33.740</t>
-  </si>
-  <si>
-    <t>656</t>
-  </si>
-  <si>
-    <t>2026-06-19T14:06:33.3700386+05:30</t>
-  </si>
-  <si>
-    <t>14:06:33.370</t>
-  </si>
-  <si>
-    <t>657</t>
-  </si>
-  <si>
-    <t>2026-06-19T14:11:33.4795473+05:30</t>
-  </si>
-  <si>
-    <t>14:11:33.479</t>
-  </si>
-  <si>
-    <t>658</t>
-  </si>
-  <si>
-    <t>2026-06-19T14:16:33.5114074+05:30</t>
-  </si>
-  <si>
-    <t>14:16:33.511</t>
-  </si>
-  <si>
-    <t>659</t>
-  </si>
-  <si>
-    <t>2026-06-19T14:21:33.3706767+05:30</t>
-  </si>
-  <si>
-    <t>14:21:33.370</t>
-  </si>
-  <si>
-    <t>660</t>
-  </si>
-  <si>
-    <t>2026-06-19T14:26:33.363807+05:30</t>
-  </si>
-  <si>
-    <t>14:26:33.363</t>
-  </si>
-  <si>
-    <t>661</t>
-  </si>
-  <si>
-    <t>2026-06-19T14:31:33.5627385+05:30</t>
-  </si>
-  <si>
-    <t>14:31:33.562</t>
-  </si>
-  <si>
-    <t>662</t>
-  </si>
-  <si>
-    <t>2026-06-19T14:36:33.3229665+05:30</t>
-  </si>
-  <si>
-    <t>14:36:33.322</t>
-  </si>
-  <si>
-    <t>663</t>
-  </si>
-  <si>
-    <t>2026-06-19T14:41:33.541576+05:30</t>
-  </si>
-  <si>
-    <t>14:41:33.541</t>
-  </si>
-  <si>
-    <t>664</t>
-  </si>
-  <si>
-    <t>2026-06-19T14:46:33.3714413+05:30</t>
-  </si>
-  <si>
-    <t>14:46:33.371</t>
-  </si>
-  <si>
-    <t>665</t>
-  </si>
-  <si>
-    <t>2026-06-19T14:51:33.6029029+05:30</t>
-  </si>
-  <si>
-    <t>14:51:33.602</t>
-  </si>
-  <si>
-    <t>666</t>
-  </si>
-  <si>
-    <t>2026-06-19T14:56:33.4305433+05:30</t>
-  </si>
-  <si>
-    <t>14:56:33.430</t>
-  </si>
-  <si>
-    <t>667</t>
-  </si>
-  <si>
-    <t>2026-06-19T15:01:33.3535668+05:30</t>
-  </si>
-  <si>
-    <t>15:01:33.353</t>
-  </si>
-  <si>
-    <t>668</t>
-  </si>
-  <si>
-    <t>2026-06-19T15:06:33.3925169+05:30</t>
-  </si>
-  <si>
-    <t>15:06:33.392</t>
-  </si>
-  <si>
-    <t>669</t>
-  </si>
-  <si>
-    <t>2026-06-19T15:11:33.4331604+05:30</t>
-  </si>
-  <si>
-    <t>15:11:33.433</t>
-  </si>
-  <si>
-    <t>670</t>
-  </si>
-  <si>
-    <t>2026-06-19T15:16:33.3516037+05:30</t>
-  </si>
-  <si>
-    <t>15:16:33.351</t>
-  </si>
-  <si>
-    <t>671</t>
-  </si>
-  <si>
-    <t>2026-06-19T15:21:33.3924164+05:30</t>
-  </si>
-  <si>
-    <t>15:21:33.392</t>
-  </si>
-  <si>
-    <t>672</t>
-  </si>
-  <si>
-    <t>2026-06-19T15:26:33.4384617+05:30</t>
-  </si>
-  <si>
-    <t>15:26:33.438</t>
-  </si>
-  <si>
-    <t>673</t>
-  </si>
-  <si>
-    <t>2026-06-19T15:31:33.6068702+05:30</t>
-  </si>
-  <si>
-    <t>15:31:33.606</t>
-  </si>
-  <si>
-    <t>674</t>
-  </si>
-  <si>
-    <t>2026-06-19T15:36:33.5456911+05:30</t>
-  </si>
-  <si>
-    <t>15:36:33.545</t>
-  </si>
-  <si>
-    <t>675</t>
-  </si>
-  <si>
-    <t>2026-06-19T16:24:14.9858131+05:30</t>
-  </si>
-  <si>
-    <t>16:24:14.985</t>
-  </si>
-  <si>
-    <t>676</t>
-  </si>
-  <si>
-    <t>2026-06-19T16:24:15.02211+05:30</t>
-  </si>
-  <si>
-    <t>16:24:15.022</t>
-  </si>
-  <si>
-    <t>677</t>
-  </si>
-  <si>
-    <t>2026-06-19T16:26:33.4755019+05:30</t>
-  </si>
-  <si>
-    <t>16:26:33.475</t>
-  </si>
-  <si>
-    <t>678</t>
-  </si>
-  <si>
-    <t>2026-06-19T16:31:33.4203387+05:30</t>
-  </si>
-  <si>
-    <t>16:31:33.420</t>
-  </si>
-  <si>
-    <t>679</t>
-  </si>
-  <si>
-    <t>2026-06-19T16:36:33.3819816+05:30</t>
-  </si>
-  <si>
-    <t>16:36:33.381</t>
-  </si>
-  <si>
-    <t>680</t>
-  </si>
-  <si>
-    <t>2026-06-19T16:41:33.4184754+05:30</t>
-  </si>
-  <si>
-    <t>16:41:33.418</t>
-  </si>
-  <si>
-    <t>681</t>
-  </si>
-  <si>
-    <t>2026-06-19T16:46:33.4420373+05:30</t>
-  </si>
-  <si>
-    <t>16:46:33.442</t>
-  </si>
-  <si>
-    <t>682</t>
-  </si>
-  <si>
-    <t>2026-06-19T16:51:33.5318237+05:30</t>
-  </si>
-  <si>
-    <t>16:51:33.531</t>
-  </si>
-  <si>
-    <t>683</t>
-  </si>
-  <si>
-    <t>2026-06-19T16:56:33.6498773+05:30</t>
-  </si>
-  <si>
-    <t>16:56:33.649</t>
-  </si>
-  <si>
-    <t>684</t>
-  </si>
-  <si>
-    <t>2026-06-19T17:01:33.4809208+05:30</t>
-  </si>
-  <si>
-    <t>17:01:33.480</t>
-  </si>
-  <si>
-    <t>685</t>
-  </si>
-  <si>
-    <t>2026-06-19T17:06:33.3155595+05:30</t>
-  </si>
-  <si>
-    <t>17:06:33.315</t>
-  </si>
-  <si>
-    <t>686</t>
-  </si>
-  <si>
-    <t>2026-06-19T17:11:33.6164892+05:30</t>
-  </si>
-  <si>
-    <t>17:11:33.616</t>
-  </si>
-  <si>
-    <t>687</t>
-  </si>
-  <si>
-    <t>2026-06-19T17:16:33.5217144+05:30</t>
-  </si>
-  <si>
-    <t>17:16:33.521</t>
-  </si>
-  <si>
-    <t>688</t>
-  </si>
-  <si>
-    <t>2026-06-19T17:21:33.536392+05:30</t>
-  </si>
-  <si>
-    <t>17:21:33.536</t>
-  </si>
-  <si>
-    <t>689</t>
-  </si>
-  <si>
-    <t>2026-06-19T17:26:33.3735547+05:30</t>
-  </si>
-  <si>
-    <t>17:26:33.373</t>
-  </si>
-  <si>
-    <t>690</t>
-  </si>
-  <si>
-    <t>2026-06-19T17:31:33.4136351+05:30</t>
-  </si>
-  <si>
-    <t>17:31:33.413</t>
-  </si>
-  <si>
-    <t>691</t>
-  </si>
-  <si>
-    <t>2026-06-19T17:36:33.4154161+05:30</t>
-  </si>
-  <si>
-    <t>17:36:33.415</t>
-  </si>
-  <si>
-    <t>692</t>
-  </si>
-  <si>
-    <t>2026-06-22T22:42:58+05:30</t>
+    <t>693</t>
+  </si>
+  <si>
+    <t>2026-06-22T22:45:59.8444842+05:30</t>
+  </si>
+  <si>
+    <t>22:45:59.844</t>
+  </si>
+  <si>
+    <t>694</t>
+  </si>
+  <si>
+    <t>2026-06-22T22:53:13+05:30</t>
   </si>
 </sst>
 </file>
@@ -9649,46 +9673,46 @@
         <v>33</v>
       </c>
       <c r="G15" t="s">
-        <v>53</v>
+        <v>34</v>
       </c>
       <c r="H15" t="s">
         <v>2689</v>
       </c>
       <c r="I15" t="s">
+        <v>45</v>
+      </c>
+      <c r="J15" t="s">
         <v>2690</v>
       </c>
-      <c r="J15" t="s">
-        <v>53</v>
-      </c>
       <c r="K15" t="s">
+        <v>47</v>
+      </c>
+      <c r="L15" t="s">
         <v>2691</v>
       </c>
-      <c r="L15" t="s">
-        <v>53</v>
-      </c>
       <c r="M15" t="s">
-        <v>39</v>
+        <v>2692</v>
       </c>
       <c r="N15" t="s">
-        <v>39</v>
+        <v>1540</v>
       </c>
       <c r="O15" t="s">
-        <v>39</v>
+        <v>51</v>
       </c>
       <c r="P15" t="s">
-        <v>53</v>
+        <v>1663</v>
       </c>
       <c r="Q15" t="s">
         <v>53</v>
       </c>
       <c r="R15" t="s">
-        <v>53</v>
+        <v>189</v>
       </c>
       <c r="S15" t="s">
         <v>53</v>
       </c>
       <c r="T15" t="s">
-        <v>53</v>
+        <v>2693</v>
       </c>
       <c r="U15" t="s">
         <v>2684</v>
@@ -9755,19 +9779,19 @@
         <v>2684</v>
       </c>
       <c r="B17" t="s">
-        <v>197</v>
+        <v>57</v>
       </c>
       <c r="C17" t="s">
-        <v>2692</v>
+        <v>2694</v>
       </c>
       <c r="D17" t="s">
         <v>2684</v>
       </c>
       <c r="E17" t="s">
-        <v>2693</v>
+        <v>2695</v>
       </c>
       <c r="F17" t="s">
-        <v>146</v>
+        <v>60</v>
       </c>
       <c r="G17" t="s">
         <v>61</v>
@@ -9785,7 +9809,7 @@
         <v>39</v>
       </c>
       <c r="L17" t="s">
-        <v>146</v>
+        <v>60</v>
       </c>
       <c r="M17" t="s">
         <v>56</v>
@@ -52993,7 +53017,7 @@
         <v>101</v>
       </c>
       <c r="C744" t="s">
-        <v>2694</v>
+        <v>2696</v>
       </c>
       <c r="D744" t="s">
         <v>56</v>
@@ -53057,7 +53081,7 @@
         <v>105</v>
       </c>
       <c r="C746" t="s">
-        <v>2694</v>
+        <v>2696</v>
       </c>
       <c r="D746" t="s">
         <v>56</v>
@@ -53089,7 +53113,7 @@
         <v>106</v>
       </c>
       <c r="C747" t="s">
-        <v>107</v>
+        <v>131</v>
       </c>
       <c r="D747" t="s">
         <v>56</v>
@@ -78132,16 +78156,16 @@
         <v>2684</v>
       </c>
       <c r="B1402" t="s">
-        <v>2695</v>
+        <v>2697</v>
       </c>
       <c r="C1402" t="s">
-        <v>2696</v>
+        <v>2698</v>
       </c>
       <c r="D1402" t="s">
         <v>181</v>
       </c>
       <c r="E1402" t="s">
-        <v>2697</v>
+        <v>2699</v>
       </c>
       <c r="F1402" t="s">
         <v>60</v>
@@ -78170,16 +78194,16 @@
         <v>2684</v>
       </c>
       <c r="B1403" t="s">
-        <v>2698</v>
+        <v>2700</v>
       </c>
       <c r="C1403" t="s">
-        <v>2699</v>
+        <v>2701</v>
       </c>
       <c r="D1403" t="s">
         <v>181</v>
       </c>
       <c r="E1403" t="s">
-        <v>2700</v>
+        <v>2702</v>
       </c>
       <c r="F1403" t="s">
         <v>60</v>
@@ -78208,16 +78232,16 @@
         <v>2684</v>
       </c>
       <c r="B1404" t="s">
-        <v>2701</v>
+        <v>2703</v>
       </c>
       <c r="C1404" t="s">
-        <v>2702</v>
+        <v>2704</v>
       </c>
       <c r="D1404" t="s">
         <v>181</v>
       </c>
       <c r="E1404" t="s">
-        <v>2703</v>
+        <v>2705</v>
       </c>
       <c r="F1404" t="s">
         <v>60</v>
@@ -78246,16 +78270,16 @@
         <v>2684</v>
       </c>
       <c r="B1405" t="s">
-        <v>2704</v>
+        <v>2706</v>
       </c>
       <c r="C1405" t="s">
-        <v>2705</v>
+        <v>2707</v>
       </c>
       <c r="D1405" t="s">
         <v>181</v>
       </c>
       <c r="E1405" t="s">
-        <v>2706</v>
+        <v>2708</v>
       </c>
       <c r="F1405" t="s">
         <v>60</v>
@@ -78284,16 +78308,16 @@
         <v>2684</v>
       </c>
       <c r="B1406" t="s">
-        <v>2707</v>
+        <v>2709</v>
       </c>
       <c r="C1406" t="s">
-        <v>2708</v>
+        <v>2710</v>
       </c>
       <c r="D1406" t="s">
         <v>181</v>
       </c>
       <c r="E1406" t="s">
-        <v>2709</v>
+        <v>2711</v>
       </c>
       <c r="F1406" t="s">
         <v>60</v>
@@ -78322,16 +78346,16 @@
         <v>2684</v>
       </c>
       <c r="B1407" t="s">
-        <v>2710</v>
+        <v>2712</v>
       </c>
       <c r="C1407" t="s">
-        <v>2711</v>
+        <v>2713</v>
       </c>
       <c r="D1407" t="s">
         <v>181</v>
       </c>
       <c r="E1407" t="s">
-        <v>2712</v>
+        <v>2714</v>
       </c>
       <c r="F1407" t="s">
         <v>60</v>
@@ -78360,16 +78384,16 @@
         <v>2684</v>
       </c>
       <c r="B1408" t="s">
-        <v>2713</v>
+        <v>2715</v>
       </c>
       <c r="C1408" t="s">
-        <v>2714</v>
+        <v>2716</v>
       </c>
       <c r="D1408" t="s">
         <v>181</v>
       </c>
       <c r="E1408" t="s">
-        <v>2715</v>
+        <v>2717</v>
       </c>
       <c r="F1408" t="s">
         <v>60</v>
@@ -78398,16 +78422,16 @@
         <v>2684</v>
       </c>
       <c r="B1409" t="s">
-        <v>2716</v>
+        <v>2718</v>
       </c>
       <c r="C1409" t="s">
-        <v>2717</v>
+        <v>2719</v>
       </c>
       <c r="D1409" t="s">
         <v>181</v>
       </c>
       <c r="E1409" t="s">
-        <v>2718</v>
+        <v>2720</v>
       </c>
       <c r="F1409" t="s">
         <v>60</v>
@@ -78436,16 +78460,16 @@
         <v>2684</v>
       </c>
       <c r="B1410" t="s">
-        <v>2719</v>
+        <v>2721</v>
       </c>
       <c r="C1410" t="s">
-        <v>2720</v>
+        <v>2722</v>
       </c>
       <c r="D1410" t="s">
         <v>181</v>
       </c>
       <c r="E1410" t="s">
-        <v>2721</v>
+        <v>2723</v>
       </c>
       <c r="F1410" t="s">
         <v>60</v>
@@ -78474,16 +78498,16 @@
         <v>2684</v>
       </c>
       <c r="B1411" t="s">
-        <v>2722</v>
+        <v>2724</v>
       </c>
       <c r="C1411" t="s">
-        <v>2723</v>
+        <v>2725</v>
       </c>
       <c r="D1411" t="s">
         <v>181</v>
       </c>
       <c r="E1411" t="s">
-        <v>2724</v>
+        <v>2726</v>
       </c>
       <c r="F1411" t="s">
         <v>60</v>
@@ -78512,16 +78536,16 @@
         <v>2684</v>
       </c>
       <c r="B1412" t="s">
-        <v>2725</v>
+        <v>2727</v>
       </c>
       <c r="C1412" t="s">
-        <v>2726</v>
+        <v>2728</v>
       </c>
       <c r="D1412" t="s">
         <v>181</v>
       </c>
       <c r="E1412" t="s">
-        <v>2727</v>
+        <v>2729</v>
       </c>
       <c r="F1412" t="s">
         <v>60</v>
@@ -78550,16 +78574,16 @@
         <v>2684</v>
       </c>
       <c r="B1413" t="s">
-        <v>2728</v>
+        <v>2730</v>
       </c>
       <c r="C1413" t="s">
-        <v>2729</v>
+        <v>2731</v>
       </c>
       <c r="D1413" t="s">
         <v>181</v>
       </c>
       <c r="E1413" t="s">
-        <v>2730</v>
+        <v>2732</v>
       </c>
       <c r="F1413" t="s">
         <v>60</v>
@@ -78588,16 +78612,16 @@
         <v>2684</v>
       </c>
       <c r="B1414" t="s">
-        <v>2731</v>
+        <v>2733</v>
       </c>
       <c r="C1414" t="s">
-        <v>2732</v>
+        <v>2734</v>
       </c>
       <c r="D1414" t="s">
         <v>181</v>
       </c>
       <c r="E1414" t="s">
-        <v>2733</v>
+        <v>2735</v>
       </c>
       <c r="F1414" t="s">
         <v>60</v>
@@ -78626,16 +78650,16 @@
         <v>2684</v>
       </c>
       <c r="B1415" t="s">
-        <v>2734</v>
+        <v>2736</v>
       </c>
       <c r="C1415" t="s">
-        <v>2735</v>
+        <v>2737</v>
       </c>
       <c r="D1415" t="s">
         <v>181</v>
       </c>
       <c r="E1415" t="s">
-        <v>2736</v>
+        <v>2738</v>
       </c>
       <c r="F1415" t="s">
         <v>60</v>
@@ -78664,16 +78688,16 @@
         <v>2684</v>
       </c>
       <c r="B1416" t="s">
-        <v>2737</v>
+        <v>2739</v>
       </c>
       <c r="C1416" t="s">
-        <v>2738</v>
+        <v>2740</v>
       </c>
       <c r="D1416" t="s">
         <v>181</v>
       </c>
       <c r="E1416" t="s">
-        <v>2739</v>
+        <v>2741</v>
       </c>
       <c r="F1416" t="s">
         <v>60</v>
@@ -78702,16 +78726,16 @@
         <v>2684</v>
       </c>
       <c r="B1417" t="s">
-        <v>2740</v>
+        <v>2742</v>
       </c>
       <c r="C1417" t="s">
-        <v>2741</v>
+        <v>2743</v>
       </c>
       <c r="D1417" t="s">
         <v>181</v>
       </c>
       <c r="E1417" t="s">
-        <v>2742</v>
+        <v>2744</v>
       </c>
       <c r="F1417" t="s">
         <v>60</v>
@@ -78740,16 +78764,16 @@
         <v>2684</v>
       </c>
       <c r="B1418" t="s">
-        <v>2743</v>
+        <v>2745</v>
       </c>
       <c r="C1418" t="s">
-        <v>2744</v>
+        <v>2746</v>
       </c>
       <c r="D1418" t="s">
         <v>181</v>
       </c>
       <c r="E1418" t="s">
-        <v>2745</v>
+        <v>2747</v>
       </c>
       <c r="F1418" t="s">
         <v>60</v>
@@ -78778,16 +78802,16 @@
         <v>2684</v>
       </c>
       <c r="B1419" t="s">
-        <v>2746</v>
+        <v>2748</v>
       </c>
       <c r="C1419" t="s">
-        <v>2747</v>
+        <v>2749</v>
       </c>
       <c r="D1419" t="s">
         <v>181</v>
       </c>
       <c r="E1419" t="s">
-        <v>2748</v>
+        <v>2750</v>
       </c>
       <c r="F1419" t="s">
         <v>60</v>
@@ -78816,16 +78840,16 @@
         <v>2684</v>
       </c>
       <c r="B1420" t="s">
-        <v>2749</v>
+        <v>2751</v>
       </c>
       <c r="C1420" t="s">
-        <v>2750</v>
+        <v>2752</v>
       </c>
       <c r="D1420" t="s">
         <v>181</v>
       </c>
       <c r="E1420" t="s">
-        <v>2751</v>
+        <v>2753</v>
       </c>
       <c r="F1420" t="s">
         <v>60</v>
@@ -78854,16 +78878,16 @@
         <v>2684</v>
       </c>
       <c r="B1421" t="s">
-        <v>2752</v>
+        <v>2754</v>
       </c>
       <c r="C1421" t="s">
-        <v>2753</v>
+        <v>2755</v>
       </c>
       <c r="D1421" t="s">
         <v>181</v>
       </c>
       <c r="E1421" t="s">
-        <v>2754</v>
+        <v>2756</v>
       </c>
       <c r="F1421" t="s">
         <v>60</v>
@@ -78892,16 +78916,16 @@
         <v>2684</v>
       </c>
       <c r="B1422" t="s">
-        <v>2755</v>
+        <v>2757</v>
       </c>
       <c r="C1422" t="s">
-        <v>2756</v>
+        <v>2758</v>
       </c>
       <c r="D1422" t="s">
         <v>181</v>
       </c>
       <c r="E1422" t="s">
-        <v>2757</v>
+        <v>2759</v>
       </c>
       <c r="F1422" t="s">
         <v>60</v>
@@ -78930,16 +78954,16 @@
         <v>2684</v>
       </c>
       <c r="B1423" t="s">
-        <v>2758</v>
+        <v>2760</v>
       </c>
       <c r="C1423" t="s">
-        <v>2759</v>
+        <v>2761</v>
       </c>
       <c r="D1423" t="s">
         <v>181</v>
       </c>
       <c r="E1423" t="s">
-        <v>2760</v>
+        <v>2762</v>
       </c>
       <c r="F1423" t="s">
         <v>60</v>
@@ -78968,16 +78992,16 @@
         <v>2684</v>
       </c>
       <c r="B1424" t="s">
-        <v>2761</v>
+        <v>2763</v>
       </c>
       <c r="C1424" t="s">
-        <v>2762</v>
+        <v>2764</v>
       </c>
       <c r="D1424" t="s">
         <v>181</v>
       </c>
       <c r="E1424" t="s">
-        <v>2763</v>
+        <v>2765</v>
       </c>
       <c r="F1424" t="s">
         <v>60</v>
@@ -79006,16 +79030,16 @@
         <v>2684</v>
       </c>
       <c r="B1425" t="s">
-        <v>2764</v>
+        <v>2766</v>
       </c>
       <c r="C1425" t="s">
-        <v>2765</v>
+        <v>2767</v>
       </c>
       <c r="D1425" t="s">
         <v>181</v>
       </c>
       <c r="E1425" t="s">
-        <v>2766</v>
+        <v>2768</v>
       </c>
       <c r="F1425" t="s">
         <v>60</v>
@@ -79044,16 +79068,16 @@
         <v>2684</v>
       </c>
       <c r="B1426" t="s">
-        <v>2767</v>
+        <v>2769</v>
       </c>
       <c r="C1426" t="s">
-        <v>2768</v>
+        <v>2770</v>
       </c>
       <c r="D1426" t="s">
         <v>181</v>
       </c>
       <c r="E1426" t="s">
-        <v>2769</v>
+        <v>2771</v>
       </c>
       <c r="F1426" t="s">
         <v>750</v>
@@ -79085,16 +79109,16 @@
         <v>2684</v>
       </c>
       <c r="B1427" t="s">
-        <v>2770</v>
+        <v>2772</v>
       </c>
       <c r="C1427" t="s">
-        <v>2771</v>
+        <v>2773</v>
       </c>
       <c r="D1427" t="s">
         <v>181</v>
       </c>
       <c r="E1427" t="s">
-        <v>2772</v>
+        <v>2774</v>
       </c>
       <c r="F1427" t="s">
         <v>750</v>
@@ -79126,16 +79150,16 @@
         <v>2684</v>
       </c>
       <c r="B1428" t="s">
-        <v>2773</v>
+        <v>2775</v>
       </c>
       <c r="C1428" t="s">
-        <v>2774</v>
+        <v>2776</v>
       </c>
       <c r="D1428" t="s">
         <v>181</v>
       </c>
       <c r="E1428" t="s">
-        <v>2775</v>
+        <v>2777</v>
       </c>
       <c r="F1428" t="s">
         <v>60</v>
@@ -79164,16 +79188,16 @@
         <v>2684</v>
       </c>
       <c r="B1429" t="s">
-        <v>2776</v>
+        <v>2778</v>
       </c>
       <c r="C1429" t="s">
-        <v>2777</v>
+        <v>2779</v>
       </c>
       <c r="D1429" t="s">
         <v>181</v>
       </c>
       <c r="E1429" t="s">
-        <v>2778</v>
+        <v>2780</v>
       </c>
       <c r="F1429" t="s">
         <v>60</v>
@@ -79202,16 +79226,16 @@
         <v>2684</v>
       </c>
       <c r="B1430" t="s">
-        <v>2779</v>
+        <v>2781</v>
       </c>
       <c r="C1430" t="s">
-        <v>2780</v>
+        <v>2782</v>
       </c>
       <c r="D1430" t="s">
         <v>181</v>
       </c>
       <c r="E1430" t="s">
-        <v>2781</v>
+        <v>2783</v>
       </c>
       <c r="F1430" t="s">
         <v>60</v>
@@ -79240,16 +79264,16 @@
         <v>2684</v>
       </c>
       <c r="B1431" t="s">
-        <v>2782</v>
+        <v>2784</v>
       </c>
       <c r="C1431" t="s">
-        <v>2783</v>
+        <v>2785</v>
       </c>
       <c r="D1431" t="s">
         <v>181</v>
       </c>
       <c r="E1431" t="s">
-        <v>2784</v>
+        <v>2786</v>
       </c>
       <c r="F1431" t="s">
         <v>60</v>
@@ -79278,16 +79302,16 @@
         <v>2684</v>
       </c>
       <c r="B1432" t="s">
-        <v>2785</v>
+        <v>2787</v>
       </c>
       <c r="C1432" t="s">
-        <v>2786</v>
+        <v>2788</v>
       </c>
       <c r="D1432" t="s">
         <v>181</v>
       </c>
       <c r="E1432" t="s">
-        <v>2787</v>
+        <v>2789</v>
       </c>
       <c r="F1432" t="s">
         <v>60</v>
@@ -79316,16 +79340,16 @@
         <v>2684</v>
       </c>
       <c r="B1433" t="s">
-        <v>2788</v>
+        <v>2790</v>
       </c>
       <c r="C1433" t="s">
-        <v>2789</v>
+        <v>2791</v>
       </c>
       <c r="D1433" t="s">
         <v>181</v>
       </c>
       <c r="E1433" t="s">
-        <v>2790</v>
+        <v>2792</v>
       </c>
       <c r="F1433" t="s">
         <v>60</v>
@@ -79354,16 +79378,16 @@
         <v>2684</v>
       </c>
       <c r="B1434" t="s">
-        <v>2791</v>
+        <v>2793</v>
       </c>
       <c r="C1434" t="s">
-        <v>2792</v>
+        <v>2794</v>
       </c>
       <c r="D1434" t="s">
         <v>181</v>
       </c>
       <c r="E1434" t="s">
-        <v>2793</v>
+        <v>2795</v>
       </c>
       <c r="F1434" t="s">
         <v>60</v>
@@ -79392,16 +79416,16 @@
         <v>2684</v>
       </c>
       <c r="B1435" t="s">
-        <v>2794</v>
+        <v>2796</v>
       </c>
       <c r="C1435" t="s">
-        <v>2795</v>
+        <v>2797</v>
       </c>
       <c r="D1435" t="s">
         <v>181</v>
       </c>
       <c r="E1435" t="s">
-        <v>2796</v>
+        <v>2798</v>
       </c>
       <c r="F1435" t="s">
         <v>60</v>
@@ -79430,16 +79454,16 @@
         <v>2684</v>
       </c>
       <c r="B1436" t="s">
-        <v>2797</v>
+        <v>2799</v>
       </c>
       <c r="C1436" t="s">
-        <v>2798</v>
+        <v>2800</v>
       </c>
       <c r="D1436" t="s">
         <v>181</v>
       </c>
       <c r="E1436" t="s">
-        <v>2799</v>
+        <v>2801</v>
       </c>
       <c r="F1436" t="s">
         <v>60</v>
@@ -79468,16 +79492,16 @@
         <v>2684</v>
       </c>
       <c r="B1437" t="s">
-        <v>2800</v>
+        <v>2802</v>
       </c>
       <c r="C1437" t="s">
-        <v>2801</v>
+        <v>2803</v>
       </c>
       <c r="D1437" t="s">
         <v>181</v>
       </c>
       <c r="E1437" t="s">
-        <v>2802</v>
+        <v>2804</v>
       </c>
       <c r="F1437" t="s">
         <v>60</v>
@@ -79506,16 +79530,16 @@
         <v>2684</v>
       </c>
       <c r="B1438" t="s">
-        <v>2803</v>
+        <v>2805</v>
       </c>
       <c r="C1438" t="s">
-        <v>2804</v>
+        <v>2806</v>
       </c>
       <c r="D1438" t="s">
         <v>181</v>
       </c>
       <c r="E1438" t="s">
-        <v>2805</v>
+        <v>2807</v>
       </c>
       <c r="F1438" t="s">
         <v>60</v>
@@ -79544,16 +79568,16 @@
         <v>2684</v>
       </c>
       <c r="B1439" t="s">
-        <v>2806</v>
+        <v>2808</v>
       </c>
       <c r="C1439" t="s">
-        <v>2807</v>
+        <v>2809</v>
       </c>
       <c r="D1439" t="s">
         <v>181</v>
       </c>
       <c r="E1439" t="s">
-        <v>2808</v>
+        <v>2810</v>
       </c>
       <c r="F1439" t="s">
         <v>60</v>
@@ -79582,16 +79606,16 @@
         <v>2684</v>
       </c>
       <c r="B1440" t="s">
-        <v>2809</v>
+        <v>2811</v>
       </c>
       <c r="C1440" t="s">
-        <v>2810</v>
+        <v>2812</v>
       </c>
       <c r="D1440" t="s">
         <v>181</v>
       </c>
       <c r="E1440" t="s">
-        <v>2811</v>
+        <v>2813</v>
       </c>
       <c r="F1440" t="s">
         <v>60</v>
@@ -79620,16 +79644,16 @@
         <v>2684</v>
       </c>
       <c r="B1441" t="s">
-        <v>2812</v>
+        <v>2814</v>
       </c>
       <c r="C1441" t="s">
-        <v>2813</v>
+        <v>2815</v>
       </c>
       <c r="D1441" t="s">
         <v>181</v>
       </c>
       <c r="E1441" t="s">
-        <v>2814</v>
+        <v>2816</v>
       </c>
       <c r="F1441" t="s">
         <v>60</v>
@@ -79658,16 +79682,16 @@
         <v>2684</v>
       </c>
       <c r="B1442" t="s">
-        <v>2815</v>
+        <v>2817</v>
       </c>
       <c r="C1442" t="s">
-        <v>2816</v>
+        <v>2818</v>
       </c>
       <c r="D1442" t="s">
         <v>181</v>
       </c>
       <c r="E1442" t="s">
-        <v>2817</v>
+        <v>2819</v>
       </c>
       <c r="F1442" t="s">
         <v>60</v>
@@ -79696,16 +79720,16 @@
         <v>2684</v>
       </c>
       <c r="B1443" t="s">
-        <v>2818</v>
+        <v>2820</v>
       </c>
       <c r="C1443" t="s">
-        <v>2692</v>
+        <v>2821</v>
       </c>
       <c r="D1443" t="s">
         <v>2684</v>
       </c>
       <c r="E1443" t="s">
-        <v>2693</v>
+        <v>2822</v>
       </c>
       <c r="F1443" t="s">
         <v>146</v>
@@ -79734,31 +79758,37 @@
         <v>2684</v>
       </c>
       <c r="B1444" t="s">
-        <v>56</v>
+        <v>2823</v>
       </c>
       <c r="C1444" t="s">
-        <v>56</v>
+        <v>2824</v>
       </c>
       <c r="D1444" t="s">
-        <v>56</v>
+        <v>2684</v>
       </c>
       <c r="E1444" t="s">
-        <v>56</v>
+        <v>2825</v>
       </c>
       <c r="F1444" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="G1444" t="s">
-        <v>56</v>
+        <v>61</v>
       </c>
       <c r="H1444" t="s">
-        <v>56</v>
+        <v>182</v>
       </c>
       <c r="I1444" t="s">
-        <v>56</v>
+        <v>183</v>
       </c>
       <c r="J1444" t="s">
-        <v>56</v>
+        <v>182</v>
+      </c>
+      <c r="K1444" t="s">
+        <v>39</v>
+      </c>
+      <c r="L1444" t="s">
+        <v>60</v>
       </c>
     </row>
     <row r="1445">
@@ -79766,30 +79796,100 @@
         <v>2684</v>
       </c>
       <c r="B1445" t="s">
+        <v>2826</v>
+      </c>
+      <c r="C1445" t="s">
+        <v>2694</v>
+      </c>
+      <c r="D1445" t="s">
+        <v>2684</v>
+      </c>
+      <c r="E1445" t="s">
+        <v>2695</v>
+      </c>
+      <c r="F1445" t="s">
+        <v>60</v>
+      </c>
+      <c r="G1445" t="s">
+        <v>61</v>
+      </c>
+      <c r="H1445" t="s">
+        <v>182</v>
+      </c>
+      <c r="I1445" t="s">
+        <v>183</v>
+      </c>
+      <c r="J1445" t="s">
+        <v>182</v>
+      </c>
+      <c r="K1445" t="s">
+        <v>39</v>
+      </c>
+      <c r="L1445" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="1446">
+      <c r="A1446" t="s">
+        <v>2684</v>
+      </c>
+      <c r="B1446" t="s">
+        <v>56</v>
+      </c>
+      <c r="C1446" t="s">
+        <v>56</v>
+      </c>
+      <c r="D1446" t="s">
+        <v>56</v>
+      </c>
+      <c r="E1446" t="s">
+        <v>56</v>
+      </c>
+      <c r="F1446" t="s">
+        <v>56</v>
+      </c>
+      <c r="G1446" t="s">
+        <v>56</v>
+      </c>
+      <c r="H1446" t="s">
+        <v>56</v>
+      </c>
+      <c r="I1446" t="s">
+        <v>56</v>
+      </c>
+      <c r="J1446" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="1447">
+      <c r="A1447" t="s">
+        <v>2684</v>
+      </c>
+      <c r="B1447" t="s">
         <v>160</v>
       </c>
-      <c r="C1445" t="s">
-        <v>2819</v>
-      </c>
-      <c r="D1445" t="s">
-        <v>56</v>
-      </c>
-      <c r="E1445" t="s">
+      <c r="C1447" t="s">
+        <v>2827</v>
+      </c>
+      <c r="D1447" t="s">
+        <v>56</v>
+      </c>
+      <c r="E1447" t="s">
         <v>162</v>
       </c>
-      <c r="F1445" t="s">
-        <v>2818</v>
-      </c>
-      <c r="G1445" t="s">
-        <v>56</v>
-      </c>
-      <c r="H1445" t="s">
-        <v>56</v>
-      </c>
-      <c r="I1445" t="s">
-        <v>56</v>
-      </c>
-      <c r="J1445" t="s">
+      <c r="F1447" t="s">
+        <v>2826</v>
+      </c>
+      <c r="G1447" t="s">
+        <v>56</v>
+      </c>
+      <c r="H1447" t="s">
+        <v>56</v>
+      </c>
+      <c r="I1447" t="s">
+        <v>56</v>
+      </c>
+      <c r="J1447" t="s">
         <v>56</v>
       </c>
     </row>

</xml_diff>

<commit_message>
compiled report 2026-06-22: 696 election events, 279 audit entries
</commit_message>
<xml_diff>
--- a/punmonitor-compiled-report.xlsx
+++ b/punmonitor-compiled-report.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2828" uniqueCount="2828">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2829" uniqueCount="2829">
   <si>
     <t>Source Date</t>
   </si>
@@ -8074,31 +8074,424 @@
     <t>2026-06-22</t>
   </si>
   <si>
-    <t>0h 12m 33s</t>
+    <t>0h 17m 36s</t>
   </si>
   <si>
     <t>2026-06-22 22:40:40</t>
   </si>
   <si>
-    <t>25h 24m 45s</t>
-  </si>
-  <si>
-    <t>22:53:13</t>
+    <t>25h 26m 33s</t>
+  </si>
+  <si>
+    <t>22:58:17</t>
   </si>
   <si>
     <t>10.0.64</t>
   </si>
   <si>
-    <t>websocket</t>
-  </si>
-  <si>
-    <t>147.0</t>
-  </si>
-  <si>
-    <t>157835.5</t>
-  </si>
-  <si>
-    <t>0h 3m 12s</t>
+    <t>disconnected</t>
+  </si>
+  <si>
+    <t>offline</t>
+  </si>
+  <si>
+    <t>2026-06-22T22:56:17.1194114+05:30</t>
+  </si>
+  <si>
+    <t>22:56:17.119</t>
+  </si>
+  <si>
+    <t>2026-06-22T22:56:17+05:30 (2m0s ago)</t>
+  </si>
+  <si>
+    <t>651</t>
+  </si>
+  <si>
+    <t>2026-06-19T13:41:33.4313429+05:30</t>
+  </si>
+  <si>
+    <t>13:41:33.431</t>
+  </si>
+  <si>
+    <t>652</t>
+  </si>
+  <si>
+    <t>2026-06-19T13:46:33.4190791+05:30</t>
+  </si>
+  <si>
+    <t>13:46:33.419</t>
+  </si>
+  <si>
+    <t>653</t>
+  </si>
+  <si>
+    <t>2026-06-19T13:51:33.3835925+05:30</t>
+  </si>
+  <si>
+    <t>13:51:33.383</t>
+  </si>
+  <si>
+    <t>654</t>
+  </si>
+  <si>
+    <t>2026-06-19T13:56:33.4354335+05:30</t>
+  </si>
+  <si>
+    <t>13:56:33.435</t>
+  </si>
+  <si>
+    <t>655</t>
+  </si>
+  <si>
+    <t>2026-06-19T14:01:33.7407703+05:30</t>
+  </si>
+  <si>
+    <t>14:01:33.740</t>
+  </si>
+  <si>
+    <t>656</t>
+  </si>
+  <si>
+    <t>2026-06-19T14:06:33.3700386+05:30</t>
+  </si>
+  <si>
+    <t>14:06:33.370</t>
+  </si>
+  <si>
+    <t>657</t>
+  </si>
+  <si>
+    <t>2026-06-19T14:11:33.4795473+05:30</t>
+  </si>
+  <si>
+    <t>14:11:33.479</t>
+  </si>
+  <si>
+    <t>658</t>
+  </si>
+  <si>
+    <t>2026-06-19T14:16:33.5114074+05:30</t>
+  </si>
+  <si>
+    <t>14:16:33.511</t>
+  </si>
+  <si>
+    <t>659</t>
+  </si>
+  <si>
+    <t>2026-06-19T14:21:33.3706767+05:30</t>
+  </si>
+  <si>
+    <t>14:21:33.370</t>
+  </si>
+  <si>
+    <t>660</t>
+  </si>
+  <si>
+    <t>2026-06-19T14:26:33.363807+05:30</t>
+  </si>
+  <si>
+    <t>14:26:33.363</t>
+  </si>
+  <si>
+    <t>661</t>
+  </si>
+  <si>
+    <t>2026-06-19T14:31:33.5627385+05:30</t>
+  </si>
+  <si>
+    <t>14:31:33.562</t>
+  </si>
+  <si>
+    <t>662</t>
+  </si>
+  <si>
+    <t>2026-06-19T14:36:33.3229665+05:30</t>
+  </si>
+  <si>
+    <t>14:36:33.322</t>
+  </si>
+  <si>
+    <t>663</t>
+  </si>
+  <si>
+    <t>2026-06-19T14:41:33.541576+05:30</t>
+  </si>
+  <si>
+    <t>14:41:33.541</t>
+  </si>
+  <si>
+    <t>664</t>
+  </si>
+  <si>
+    <t>2026-06-19T14:46:33.3714413+05:30</t>
+  </si>
+  <si>
+    <t>14:46:33.371</t>
+  </si>
+  <si>
+    <t>665</t>
+  </si>
+  <si>
+    <t>2026-06-19T14:51:33.6029029+05:30</t>
+  </si>
+  <si>
+    <t>14:51:33.602</t>
+  </si>
+  <si>
+    <t>666</t>
+  </si>
+  <si>
+    <t>2026-06-19T14:56:33.4305433+05:30</t>
+  </si>
+  <si>
+    <t>14:56:33.430</t>
+  </si>
+  <si>
+    <t>667</t>
+  </si>
+  <si>
+    <t>2026-06-19T15:01:33.3535668+05:30</t>
+  </si>
+  <si>
+    <t>15:01:33.353</t>
+  </si>
+  <si>
+    <t>668</t>
+  </si>
+  <si>
+    <t>2026-06-19T15:06:33.3925169+05:30</t>
+  </si>
+  <si>
+    <t>15:06:33.392</t>
+  </si>
+  <si>
+    <t>669</t>
+  </si>
+  <si>
+    <t>2026-06-19T15:11:33.4331604+05:30</t>
+  </si>
+  <si>
+    <t>15:11:33.433</t>
+  </si>
+  <si>
+    <t>670</t>
+  </si>
+  <si>
+    <t>2026-06-19T15:16:33.3516037+05:30</t>
+  </si>
+  <si>
+    <t>15:16:33.351</t>
+  </si>
+  <si>
+    <t>671</t>
+  </si>
+  <si>
+    <t>2026-06-19T15:21:33.3924164+05:30</t>
+  </si>
+  <si>
+    <t>15:21:33.392</t>
+  </si>
+  <si>
+    <t>672</t>
+  </si>
+  <si>
+    <t>2026-06-19T15:26:33.4384617+05:30</t>
+  </si>
+  <si>
+    <t>15:26:33.438</t>
+  </si>
+  <si>
+    <t>673</t>
+  </si>
+  <si>
+    <t>2026-06-19T15:31:33.6068702+05:30</t>
+  </si>
+  <si>
+    <t>15:31:33.606</t>
+  </si>
+  <si>
+    <t>674</t>
+  </si>
+  <si>
+    <t>2026-06-19T15:36:33.5456911+05:30</t>
+  </si>
+  <si>
+    <t>15:36:33.545</t>
+  </si>
+  <si>
+    <t>675</t>
+  </si>
+  <si>
+    <t>2026-06-19T16:24:14.9858131+05:30</t>
+  </si>
+  <si>
+    <t>16:24:14.985</t>
+  </si>
+  <si>
+    <t>676</t>
+  </si>
+  <si>
+    <t>2026-06-19T16:24:15.02211+05:30</t>
+  </si>
+  <si>
+    <t>16:24:15.022</t>
+  </si>
+  <si>
+    <t>677</t>
+  </si>
+  <si>
+    <t>2026-06-19T16:26:33.4755019+05:30</t>
+  </si>
+  <si>
+    <t>16:26:33.475</t>
+  </si>
+  <si>
+    <t>678</t>
+  </si>
+  <si>
+    <t>2026-06-19T16:31:33.4203387+05:30</t>
+  </si>
+  <si>
+    <t>16:31:33.420</t>
+  </si>
+  <si>
+    <t>679</t>
+  </si>
+  <si>
+    <t>2026-06-19T16:36:33.3819816+05:30</t>
+  </si>
+  <si>
+    <t>16:36:33.381</t>
+  </si>
+  <si>
+    <t>680</t>
+  </si>
+  <si>
+    <t>2026-06-19T16:41:33.4184754+05:30</t>
+  </si>
+  <si>
+    <t>16:41:33.418</t>
+  </si>
+  <si>
+    <t>681</t>
+  </si>
+  <si>
+    <t>2026-06-19T16:46:33.4420373+05:30</t>
+  </si>
+  <si>
+    <t>16:46:33.442</t>
+  </si>
+  <si>
+    <t>682</t>
+  </si>
+  <si>
+    <t>2026-06-19T16:51:33.5318237+05:30</t>
+  </si>
+  <si>
+    <t>16:51:33.531</t>
+  </si>
+  <si>
+    <t>683</t>
+  </si>
+  <si>
+    <t>2026-06-19T16:56:33.6498773+05:30</t>
+  </si>
+  <si>
+    <t>16:56:33.649</t>
+  </si>
+  <si>
+    <t>684</t>
+  </si>
+  <si>
+    <t>2026-06-19T17:01:33.4809208+05:30</t>
+  </si>
+  <si>
+    <t>17:01:33.480</t>
+  </si>
+  <si>
+    <t>685</t>
+  </si>
+  <si>
+    <t>2026-06-19T17:06:33.3155595+05:30</t>
+  </si>
+  <si>
+    <t>17:06:33.315</t>
+  </si>
+  <si>
+    <t>686</t>
+  </si>
+  <si>
+    <t>2026-06-19T17:11:33.6164892+05:30</t>
+  </si>
+  <si>
+    <t>17:11:33.616</t>
+  </si>
+  <si>
+    <t>687</t>
+  </si>
+  <si>
+    <t>2026-06-19T17:16:33.5217144+05:30</t>
+  </si>
+  <si>
+    <t>17:16:33.521</t>
+  </si>
+  <si>
+    <t>688</t>
+  </si>
+  <si>
+    <t>2026-06-19T17:21:33.536392+05:30</t>
+  </si>
+  <si>
+    <t>17:21:33.536</t>
+  </si>
+  <si>
+    <t>689</t>
+  </si>
+  <si>
+    <t>2026-06-19T17:26:33.3735547+05:30</t>
+  </si>
+  <si>
+    <t>17:26:33.373</t>
+  </si>
+  <si>
+    <t>690</t>
+  </si>
+  <si>
+    <t>2026-06-19T17:31:33.4136351+05:30</t>
+  </si>
+  <si>
+    <t>17:31:33.413</t>
+  </si>
+  <si>
+    <t>691</t>
+  </si>
+  <si>
+    <t>2026-06-19T17:36:33.4154161+05:30</t>
+  </si>
+  <si>
+    <t>17:36:33.415</t>
+  </si>
+  <si>
+    <t>692</t>
+  </si>
+  <si>
+    <t>2026-06-22T22:40:57.9979938+05:30</t>
+  </si>
+  <si>
+    <t>22:40:57.997</t>
+  </si>
+  <si>
+    <t>693</t>
+  </si>
+  <si>
+    <t>2026-06-22T22:45:59.8444842+05:30</t>
+  </si>
+  <si>
+    <t>22:45:59.844</t>
+  </si>
+  <si>
+    <t>694</t>
   </si>
   <si>
     <t>2026-06-22T22:50:59.9398109+05:30</t>
@@ -8107,400 +8500,10 @@
     <t>22:50:59.939</t>
   </si>
   <si>
-    <t>2026-06-22T22:51:13+05:30 (2m0s ago)</t>
-  </si>
-  <si>
-    <t>651</t>
-  </si>
-  <si>
-    <t>2026-06-19T13:41:33.4313429+05:30</t>
-  </si>
-  <si>
-    <t>13:41:33.431</t>
-  </si>
-  <si>
-    <t>652</t>
-  </si>
-  <si>
-    <t>2026-06-19T13:46:33.4190791+05:30</t>
-  </si>
-  <si>
-    <t>13:46:33.419</t>
-  </si>
-  <si>
-    <t>653</t>
-  </si>
-  <si>
-    <t>2026-06-19T13:51:33.3835925+05:30</t>
-  </si>
-  <si>
-    <t>13:51:33.383</t>
-  </si>
-  <si>
-    <t>654</t>
-  </si>
-  <si>
-    <t>2026-06-19T13:56:33.4354335+05:30</t>
-  </si>
-  <si>
-    <t>13:56:33.435</t>
-  </si>
-  <si>
-    <t>655</t>
-  </si>
-  <si>
-    <t>2026-06-19T14:01:33.7407703+05:30</t>
-  </si>
-  <si>
-    <t>14:01:33.740</t>
-  </si>
-  <si>
-    <t>656</t>
-  </si>
-  <si>
-    <t>2026-06-19T14:06:33.3700386+05:30</t>
-  </si>
-  <si>
-    <t>14:06:33.370</t>
-  </si>
-  <si>
-    <t>657</t>
-  </si>
-  <si>
-    <t>2026-06-19T14:11:33.4795473+05:30</t>
-  </si>
-  <si>
-    <t>14:11:33.479</t>
-  </si>
-  <si>
-    <t>658</t>
-  </si>
-  <si>
-    <t>2026-06-19T14:16:33.5114074+05:30</t>
-  </si>
-  <si>
-    <t>14:16:33.511</t>
-  </si>
-  <si>
-    <t>659</t>
-  </si>
-  <si>
-    <t>2026-06-19T14:21:33.3706767+05:30</t>
-  </si>
-  <si>
-    <t>14:21:33.370</t>
-  </si>
-  <si>
-    <t>660</t>
-  </si>
-  <si>
-    <t>2026-06-19T14:26:33.363807+05:30</t>
-  </si>
-  <si>
-    <t>14:26:33.363</t>
-  </si>
-  <si>
-    <t>661</t>
-  </si>
-  <si>
-    <t>2026-06-19T14:31:33.5627385+05:30</t>
-  </si>
-  <si>
-    <t>14:31:33.562</t>
-  </si>
-  <si>
-    <t>662</t>
-  </si>
-  <si>
-    <t>2026-06-19T14:36:33.3229665+05:30</t>
-  </si>
-  <si>
-    <t>14:36:33.322</t>
-  </si>
-  <si>
-    <t>663</t>
-  </si>
-  <si>
-    <t>2026-06-19T14:41:33.541576+05:30</t>
-  </si>
-  <si>
-    <t>14:41:33.541</t>
-  </si>
-  <si>
-    <t>664</t>
-  </si>
-  <si>
-    <t>2026-06-19T14:46:33.3714413+05:30</t>
-  </si>
-  <si>
-    <t>14:46:33.371</t>
-  </si>
-  <si>
-    <t>665</t>
-  </si>
-  <si>
-    <t>2026-06-19T14:51:33.6029029+05:30</t>
-  </si>
-  <si>
-    <t>14:51:33.602</t>
-  </si>
-  <si>
-    <t>666</t>
-  </si>
-  <si>
-    <t>2026-06-19T14:56:33.4305433+05:30</t>
-  </si>
-  <si>
-    <t>14:56:33.430</t>
-  </si>
-  <si>
-    <t>667</t>
-  </si>
-  <si>
-    <t>2026-06-19T15:01:33.3535668+05:30</t>
-  </si>
-  <si>
-    <t>15:01:33.353</t>
-  </si>
-  <si>
-    <t>668</t>
-  </si>
-  <si>
-    <t>2026-06-19T15:06:33.3925169+05:30</t>
-  </si>
-  <si>
-    <t>15:06:33.392</t>
-  </si>
-  <si>
-    <t>669</t>
-  </si>
-  <si>
-    <t>2026-06-19T15:11:33.4331604+05:30</t>
-  </si>
-  <si>
-    <t>15:11:33.433</t>
-  </si>
-  <si>
-    <t>670</t>
-  </si>
-  <si>
-    <t>2026-06-19T15:16:33.3516037+05:30</t>
-  </si>
-  <si>
-    <t>15:16:33.351</t>
-  </si>
-  <si>
-    <t>671</t>
-  </si>
-  <si>
-    <t>2026-06-19T15:21:33.3924164+05:30</t>
-  </si>
-  <si>
-    <t>15:21:33.392</t>
-  </si>
-  <si>
-    <t>672</t>
-  </si>
-  <si>
-    <t>2026-06-19T15:26:33.4384617+05:30</t>
-  </si>
-  <si>
-    <t>15:26:33.438</t>
-  </si>
-  <si>
-    <t>673</t>
-  </si>
-  <si>
-    <t>2026-06-19T15:31:33.6068702+05:30</t>
-  </si>
-  <si>
-    <t>15:31:33.606</t>
-  </si>
-  <si>
-    <t>674</t>
-  </si>
-  <si>
-    <t>2026-06-19T15:36:33.5456911+05:30</t>
-  </si>
-  <si>
-    <t>15:36:33.545</t>
-  </si>
-  <si>
-    <t>675</t>
-  </si>
-  <si>
-    <t>2026-06-19T16:24:14.9858131+05:30</t>
-  </si>
-  <si>
-    <t>16:24:14.985</t>
-  </si>
-  <si>
-    <t>676</t>
-  </si>
-  <si>
-    <t>2026-06-19T16:24:15.02211+05:30</t>
-  </si>
-  <si>
-    <t>16:24:15.022</t>
-  </si>
-  <si>
-    <t>677</t>
-  </si>
-  <si>
-    <t>2026-06-19T16:26:33.4755019+05:30</t>
-  </si>
-  <si>
-    <t>16:26:33.475</t>
-  </si>
-  <si>
-    <t>678</t>
-  </si>
-  <si>
-    <t>2026-06-19T16:31:33.4203387+05:30</t>
-  </si>
-  <si>
-    <t>16:31:33.420</t>
-  </si>
-  <si>
-    <t>679</t>
-  </si>
-  <si>
-    <t>2026-06-19T16:36:33.3819816+05:30</t>
-  </si>
-  <si>
-    <t>16:36:33.381</t>
-  </si>
-  <si>
-    <t>680</t>
-  </si>
-  <si>
-    <t>2026-06-19T16:41:33.4184754+05:30</t>
-  </si>
-  <si>
-    <t>16:41:33.418</t>
-  </si>
-  <si>
-    <t>681</t>
-  </si>
-  <si>
-    <t>2026-06-19T16:46:33.4420373+05:30</t>
-  </si>
-  <si>
-    <t>16:46:33.442</t>
-  </si>
-  <si>
-    <t>682</t>
-  </si>
-  <si>
-    <t>2026-06-19T16:51:33.5318237+05:30</t>
-  </si>
-  <si>
-    <t>16:51:33.531</t>
-  </si>
-  <si>
-    <t>683</t>
-  </si>
-  <si>
-    <t>2026-06-19T16:56:33.6498773+05:30</t>
-  </si>
-  <si>
-    <t>16:56:33.649</t>
-  </si>
-  <si>
-    <t>684</t>
-  </si>
-  <si>
-    <t>2026-06-19T17:01:33.4809208+05:30</t>
-  </si>
-  <si>
-    <t>17:01:33.480</t>
-  </si>
-  <si>
-    <t>685</t>
-  </si>
-  <si>
-    <t>2026-06-19T17:06:33.3155595+05:30</t>
-  </si>
-  <si>
-    <t>17:06:33.315</t>
-  </si>
-  <si>
-    <t>686</t>
-  </si>
-  <si>
-    <t>2026-06-19T17:11:33.6164892+05:30</t>
-  </si>
-  <si>
-    <t>17:11:33.616</t>
-  </si>
-  <si>
-    <t>687</t>
-  </si>
-  <si>
-    <t>2026-06-19T17:16:33.5217144+05:30</t>
-  </si>
-  <si>
-    <t>17:16:33.521</t>
-  </si>
-  <si>
-    <t>688</t>
-  </si>
-  <si>
-    <t>2026-06-19T17:21:33.536392+05:30</t>
-  </si>
-  <si>
-    <t>17:21:33.536</t>
-  </si>
-  <si>
-    <t>689</t>
-  </si>
-  <si>
-    <t>2026-06-19T17:26:33.3735547+05:30</t>
-  </si>
-  <si>
-    <t>17:26:33.373</t>
-  </si>
-  <si>
-    <t>690</t>
-  </si>
-  <si>
-    <t>2026-06-19T17:31:33.4136351+05:30</t>
-  </si>
-  <si>
-    <t>17:31:33.413</t>
-  </si>
-  <si>
-    <t>691</t>
-  </si>
-  <si>
-    <t>2026-06-19T17:36:33.4154161+05:30</t>
-  </si>
-  <si>
-    <t>17:36:33.415</t>
-  </si>
-  <si>
-    <t>692</t>
-  </si>
-  <si>
-    <t>2026-06-22T22:40:57.9979938+05:30</t>
-  </si>
-  <si>
-    <t>22:40:57.997</t>
-  </si>
-  <si>
-    <t>693</t>
-  </si>
-  <si>
-    <t>2026-06-22T22:45:59.8444842+05:30</t>
-  </si>
-  <si>
-    <t>22:45:59.844</t>
-  </si>
-  <si>
-    <t>694</t>
-  </si>
-  <si>
-    <t>2026-06-22T22:53:13+05:30</t>
+    <t>695</t>
+  </si>
+  <si>
+    <t>2026-06-22T22:58:17+05:30</t>
   </si>
 </sst>
 </file>
@@ -9673,46 +9676,46 @@
         <v>33</v>
       </c>
       <c r="G15" t="s">
-        <v>34</v>
+        <v>53</v>
       </c>
       <c r="H15" t="s">
         <v>2689</v>
       </c>
       <c r="I15" t="s">
-        <v>45</v>
+        <v>2690</v>
       </c>
       <c r="J15" t="s">
-        <v>2690</v>
+        <v>53</v>
       </c>
       <c r="K15" t="s">
-        <v>47</v>
+        <v>2691</v>
       </c>
       <c r="L15" t="s">
-        <v>2691</v>
+        <v>53</v>
       </c>
       <c r="M15" t="s">
-        <v>2692</v>
+        <v>39</v>
       </c>
       <c r="N15" t="s">
-        <v>1540</v>
+        <v>39</v>
       </c>
       <c r="O15" t="s">
-        <v>51</v>
+        <v>39</v>
       </c>
       <c r="P15" t="s">
-        <v>1663</v>
+        <v>53</v>
       </c>
       <c r="Q15" t="s">
         <v>53</v>
       </c>
       <c r="R15" t="s">
-        <v>189</v>
+        <v>53</v>
       </c>
       <c r="S15" t="s">
         <v>53</v>
       </c>
       <c r="T15" t="s">
-        <v>2693</v>
+        <v>53</v>
       </c>
       <c r="U15" t="s">
         <v>2684</v>
@@ -9782,13 +9785,13 @@
         <v>57</v>
       </c>
       <c r="C17" t="s">
-        <v>2694</v>
+        <v>2692</v>
       </c>
       <c r="D17" t="s">
         <v>2684</v>
       </c>
       <c r="E17" t="s">
-        <v>2695</v>
+        <v>2693</v>
       </c>
       <c r="F17" t="s">
         <v>60</v>
@@ -53017,7 +53020,7 @@
         <v>101</v>
       </c>
       <c r="C744" t="s">
-        <v>2696</v>
+        <v>2694</v>
       </c>
       <c r="D744" t="s">
         <v>56</v>
@@ -53081,7 +53084,7 @@
         <v>105</v>
       </c>
       <c r="C746" t="s">
-        <v>2696</v>
+        <v>2694</v>
       </c>
       <c r="D746" t="s">
         <v>56</v>
@@ -53113,7 +53116,7 @@
         <v>106</v>
       </c>
       <c r="C747" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="D747" t="s">
         <v>56</v>
@@ -78156,16 +78159,16 @@
         <v>2684</v>
       </c>
       <c r="B1402" t="s">
+        <v>2695</v>
+      </c>
+      <c r="C1402" t="s">
+        <v>2696</v>
+      </c>
+      <c r="D1402" t="s">
+        <v>181</v>
+      </c>
+      <c r="E1402" t="s">
         <v>2697</v>
-      </c>
-      <c r="C1402" t="s">
-        <v>2698</v>
-      </c>
-      <c r="D1402" t="s">
-        <v>181</v>
-      </c>
-      <c r="E1402" t="s">
-        <v>2699</v>
       </c>
       <c r="F1402" t="s">
         <v>60</v>
@@ -78194,16 +78197,16 @@
         <v>2684</v>
       </c>
       <c r="B1403" t="s">
+        <v>2698</v>
+      </c>
+      <c r="C1403" t="s">
+        <v>2699</v>
+      </c>
+      <c r="D1403" t="s">
+        <v>181</v>
+      </c>
+      <c r="E1403" t="s">
         <v>2700</v>
-      </c>
-      <c r="C1403" t="s">
-        <v>2701</v>
-      </c>
-      <c r="D1403" t="s">
-        <v>181</v>
-      </c>
-      <c r="E1403" t="s">
-        <v>2702</v>
       </c>
       <c r="F1403" t="s">
         <v>60</v>
@@ -78232,16 +78235,16 @@
         <v>2684</v>
       </c>
       <c r="B1404" t="s">
+        <v>2701</v>
+      </c>
+      <c r="C1404" t="s">
+        <v>2702</v>
+      </c>
+      <c r="D1404" t="s">
+        <v>181</v>
+      </c>
+      <c r="E1404" t="s">
         <v>2703</v>
-      </c>
-      <c r="C1404" t="s">
-        <v>2704</v>
-      </c>
-      <c r="D1404" t="s">
-        <v>181</v>
-      </c>
-      <c r="E1404" t="s">
-        <v>2705</v>
       </c>
       <c r="F1404" t="s">
         <v>60</v>
@@ -78270,16 +78273,16 @@
         <v>2684</v>
       </c>
       <c r="B1405" t="s">
+        <v>2704</v>
+      </c>
+      <c r="C1405" t="s">
+        <v>2705</v>
+      </c>
+      <c r="D1405" t="s">
+        <v>181</v>
+      </c>
+      <c r="E1405" t="s">
         <v>2706</v>
-      </c>
-      <c r="C1405" t="s">
-        <v>2707</v>
-      </c>
-      <c r="D1405" t="s">
-        <v>181</v>
-      </c>
-      <c r="E1405" t="s">
-        <v>2708</v>
       </c>
       <c r="F1405" t="s">
         <v>60</v>
@@ -78308,16 +78311,16 @@
         <v>2684</v>
       </c>
       <c r="B1406" t="s">
+        <v>2707</v>
+      </c>
+      <c r="C1406" t="s">
+        <v>2708</v>
+      </c>
+      <c r="D1406" t="s">
+        <v>181</v>
+      </c>
+      <c r="E1406" t="s">
         <v>2709</v>
-      </c>
-      <c r="C1406" t="s">
-        <v>2710</v>
-      </c>
-      <c r="D1406" t="s">
-        <v>181</v>
-      </c>
-      <c r="E1406" t="s">
-        <v>2711</v>
       </c>
       <c r="F1406" t="s">
         <v>60</v>
@@ -78346,16 +78349,16 @@
         <v>2684</v>
       </c>
       <c r="B1407" t="s">
+        <v>2710</v>
+      </c>
+      <c r="C1407" t="s">
+        <v>2711</v>
+      </c>
+      <c r="D1407" t="s">
+        <v>181</v>
+      </c>
+      <c r="E1407" t="s">
         <v>2712</v>
-      </c>
-      <c r="C1407" t="s">
-        <v>2713</v>
-      </c>
-      <c r="D1407" t="s">
-        <v>181</v>
-      </c>
-      <c r="E1407" t="s">
-        <v>2714</v>
       </c>
       <c r="F1407" t="s">
         <v>60</v>
@@ -78384,16 +78387,16 @@
         <v>2684</v>
       </c>
       <c r="B1408" t="s">
+        <v>2713</v>
+      </c>
+      <c r="C1408" t="s">
+        <v>2714</v>
+      </c>
+      <c r="D1408" t="s">
+        <v>181</v>
+      </c>
+      <c r="E1408" t="s">
         <v>2715</v>
-      </c>
-      <c r="C1408" t="s">
-        <v>2716</v>
-      </c>
-      <c r="D1408" t="s">
-        <v>181</v>
-      </c>
-      <c r="E1408" t="s">
-        <v>2717</v>
       </c>
       <c r="F1408" t="s">
         <v>60</v>
@@ -78422,16 +78425,16 @@
         <v>2684</v>
       </c>
       <c r="B1409" t="s">
+        <v>2716</v>
+      </c>
+      <c r="C1409" t="s">
+        <v>2717</v>
+      </c>
+      <c r="D1409" t="s">
+        <v>181</v>
+      </c>
+      <c r="E1409" t="s">
         <v>2718</v>
-      </c>
-      <c r="C1409" t="s">
-        <v>2719</v>
-      </c>
-      <c r="D1409" t="s">
-        <v>181</v>
-      </c>
-      <c r="E1409" t="s">
-        <v>2720</v>
       </c>
       <c r="F1409" t="s">
         <v>60</v>
@@ -78460,16 +78463,16 @@
         <v>2684</v>
       </c>
       <c r="B1410" t="s">
+        <v>2719</v>
+      </c>
+      <c r="C1410" t="s">
+        <v>2720</v>
+      </c>
+      <c r="D1410" t="s">
+        <v>181</v>
+      </c>
+      <c r="E1410" t="s">
         <v>2721</v>
-      </c>
-      <c r="C1410" t="s">
-        <v>2722</v>
-      </c>
-      <c r="D1410" t="s">
-        <v>181</v>
-      </c>
-      <c r="E1410" t="s">
-        <v>2723</v>
       </c>
       <c r="F1410" t="s">
         <v>60</v>
@@ -78498,16 +78501,16 @@
         <v>2684</v>
       </c>
       <c r="B1411" t="s">
+        <v>2722</v>
+      </c>
+      <c r="C1411" t="s">
+        <v>2723</v>
+      </c>
+      <c r="D1411" t="s">
+        <v>181</v>
+      </c>
+      <c r="E1411" t="s">
         <v>2724</v>
-      </c>
-      <c r="C1411" t="s">
-        <v>2725</v>
-      </c>
-      <c r="D1411" t="s">
-        <v>181</v>
-      </c>
-      <c r="E1411" t="s">
-        <v>2726</v>
       </c>
       <c r="F1411" t="s">
         <v>60</v>
@@ -78536,16 +78539,16 @@
         <v>2684</v>
       </c>
       <c r="B1412" t="s">
+        <v>2725</v>
+      </c>
+      <c r="C1412" t="s">
+        <v>2726</v>
+      </c>
+      <c r="D1412" t="s">
+        <v>181</v>
+      </c>
+      <c r="E1412" t="s">
         <v>2727</v>
-      </c>
-      <c r="C1412" t="s">
-        <v>2728</v>
-      </c>
-      <c r="D1412" t="s">
-        <v>181</v>
-      </c>
-      <c r="E1412" t="s">
-        <v>2729</v>
       </c>
       <c r="F1412" t="s">
         <v>60</v>
@@ -78574,16 +78577,16 @@
         <v>2684</v>
       </c>
       <c r="B1413" t="s">
+        <v>2728</v>
+      </c>
+      <c r="C1413" t="s">
+        <v>2729</v>
+      </c>
+      <c r="D1413" t="s">
+        <v>181</v>
+      </c>
+      <c r="E1413" t="s">
         <v>2730</v>
-      </c>
-      <c r="C1413" t="s">
-        <v>2731</v>
-      </c>
-      <c r="D1413" t="s">
-        <v>181</v>
-      </c>
-      <c r="E1413" t="s">
-        <v>2732</v>
       </c>
       <c r="F1413" t="s">
         <v>60</v>
@@ -78612,16 +78615,16 @@
         <v>2684</v>
       </c>
       <c r="B1414" t="s">
+        <v>2731</v>
+      </c>
+      <c r="C1414" t="s">
+        <v>2732</v>
+      </c>
+      <c r="D1414" t="s">
+        <v>181</v>
+      </c>
+      <c r="E1414" t="s">
         <v>2733</v>
-      </c>
-      <c r="C1414" t="s">
-        <v>2734</v>
-      </c>
-      <c r="D1414" t="s">
-        <v>181</v>
-      </c>
-      <c r="E1414" t="s">
-        <v>2735</v>
       </c>
       <c r="F1414" t="s">
         <v>60</v>
@@ -78650,16 +78653,16 @@
         <v>2684</v>
       </c>
       <c r="B1415" t="s">
+        <v>2734</v>
+      </c>
+      <c r="C1415" t="s">
+        <v>2735</v>
+      </c>
+      <c r="D1415" t="s">
+        <v>181</v>
+      </c>
+      <c r="E1415" t="s">
         <v>2736</v>
-      </c>
-      <c r="C1415" t="s">
-        <v>2737</v>
-      </c>
-      <c r="D1415" t="s">
-        <v>181</v>
-      </c>
-      <c r="E1415" t="s">
-        <v>2738</v>
       </c>
       <c r="F1415" t="s">
         <v>60</v>
@@ -78688,16 +78691,16 @@
         <v>2684</v>
       </c>
       <c r="B1416" t="s">
+        <v>2737</v>
+      </c>
+      <c r="C1416" t="s">
+        <v>2738</v>
+      </c>
+      <c r="D1416" t="s">
+        <v>181</v>
+      </c>
+      <c r="E1416" t="s">
         <v>2739</v>
-      </c>
-      <c r="C1416" t="s">
-        <v>2740</v>
-      </c>
-      <c r="D1416" t="s">
-        <v>181</v>
-      </c>
-      <c r="E1416" t="s">
-        <v>2741</v>
       </c>
       <c r="F1416" t="s">
         <v>60</v>
@@ -78726,16 +78729,16 @@
         <v>2684</v>
       </c>
       <c r="B1417" t="s">
+        <v>2740</v>
+      </c>
+      <c r="C1417" t="s">
+        <v>2741</v>
+      </c>
+      <c r="D1417" t="s">
+        <v>181</v>
+      </c>
+      <c r="E1417" t="s">
         <v>2742</v>
-      </c>
-      <c r="C1417" t="s">
-        <v>2743</v>
-      </c>
-      <c r="D1417" t="s">
-        <v>181</v>
-      </c>
-      <c r="E1417" t="s">
-        <v>2744</v>
       </c>
       <c r="F1417" t="s">
         <v>60</v>
@@ -78764,16 +78767,16 @@
         <v>2684</v>
       </c>
       <c r="B1418" t="s">
+        <v>2743</v>
+      </c>
+      <c r="C1418" t="s">
+        <v>2744</v>
+      </c>
+      <c r="D1418" t="s">
+        <v>181</v>
+      </c>
+      <c r="E1418" t="s">
         <v>2745</v>
-      </c>
-      <c r="C1418" t="s">
-        <v>2746</v>
-      </c>
-      <c r="D1418" t="s">
-        <v>181</v>
-      </c>
-      <c r="E1418" t="s">
-        <v>2747</v>
       </c>
       <c r="F1418" t="s">
         <v>60</v>
@@ -78802,16 +78805,16 @@
         <v>2684</v>
       </c>
       <c r="B1419" t="s">
+        <v>2746</v>
+      </c>
+      <c r="C1419" t="s">
+        <v>2747</v>
+      </c>
+      <c r="D1419" t="s">
+        <v>181</v>
+      </c>
+      <c r="E1419" t="s">
         <v>2748</v>
-      </c>
-      <c r="C1419" t="s">
-        <v>2749</v>
-      </c>
-      <c r="D1419" t="s">
-        <v>181</v>
-      </c>
-      <c r="E1419" t="s">
-        <v>2750</v>
       </c>
       <c r="F1419" t="s">
         <v>60</v>
@@ -78840,16 +78843,16 @@
         <v>2684</v>
       </c>
       <c r="B1420" t="s">
+        <v>2749</v>
+      </c>
+      <c r="C1420" t="s">
+        <v>2750</v>
+      </c>
+      <c r="D1420" t="s">
+        <v>181</v>
+      </c>
+      <c r="E1420" t="s">
         <v>2751</v>
-      </c>
-      <c r="C1420" t="s">
-        <v>2752</v>
-      </c>
-      <c r="D1420" t="s">
-        <v>181</v>
-      </c>
-      <c r="E1420" t="s">
-        <v>2753</v>
       </c>
       <c r="F1420" t="s">
         <v>60</v>
@@ -78878,16 +78881,16 @@
         <v>2684</v>
       </c>
       <c r="B1421" t="s">
+        <v>2752</v>
+      </c>
+      <c r="C1421" t="s">
+        <v>2753</v>
+      </c>
+      <c r="D1421" t="s">
+        <v>181</v>
+      </c>
+      <c r="E1421" t="s">
         <v>2754</v>
-      </c>
-      <c r="C1421" t="s">
-        <v>2755</v>
-      </c>
-      <c r="D1421" t="s">
-        <v>181</v>
-      </c>
-      <c r="E1421" t="s">
-        <v>2756</v>
       </c>
       <c r="F1421" t="s">
         <v>60</v>
@@ -78916,16 +78919,16 @@
         <v>2684</v>
       </c>
       <c r="B1422" t="s">
+        <v>2755</v>
+      </c>
+      <c r="C1422" t="s">
+        <v>2756</v>
+      </c>
+      <c r="D1422" t="s">
+        <v>181</v>
+      </c>
+      <c r="E1422" t="s">
         <v>2757</v>
-      </c>
-      <c r="C1422" t="s">
-        <v>2758</v>
-      </c>
-      <c r="D1422" t="s">
-        <v>181</v>
-      </c>
-      <c r="E1422" t="s">
-        <v>2759</v>
       </c>
       <c r="F1422" t="s">
         <v>60</v>
@@ -78954,16 +78957,16 @@
         <v>2684</v>
       </c>
       <c r="B1423" t="s">
+        <v>2758</v>
+      </c>
+      <c r="C1423" t="s">
+        <v>2759</v>
+      </c>
+      <c r="D1423" t="s">
+        <v>181</v>
+      </c>
+      <c r="E1423" t="s">
         <v>2760</v>
-      </c>
-      <c r="C1423" t="s">
-        <v>2761</v>
-      </c>
-      <c r="D1423" t="s">
-        <v>181</v>
-      </c>
-      <c r="E1423" t="s">
-        <v>2762</v>
       </c>
       <c r="F1423" t="s">
         <v>60</v>
@@ -78992,16 +78995,16 @@
         <v>2684</v>
       </c>
       <c r="B1424" t="s">
+        <v>2761</v>
+      </c>
+      <c r="C1424" t="s">
+        <v>2762</v>
+      </c>
+      <c r="D1424" t="s">
+        <v>181</v>
+      </c>
+      <c r="E1424" t="s">
         <v>2763</v>
-      </c>
-      <c r="C1424" t="s">
-        <v>2764</v>
-      </c>
-      <c r="D1424" t="s">
-        <v>181</v>
-      </c>
-      <c r="E1424" t="s">
-        <v>2765</v>
       </c>
       <c r="F1424" t="s">
         <v>60</v>
@@ -79030,16 +79033,16 @@
         <v>2684</v>
       </c>
       <c r="B1425" t="s">
+        <v>2764</v>
+      </c>
+      <c r="C1425" t="s">
+        <v>2765</v>
+      </c>
+      <c r="D1425" t="s">
+        <v>181</v>
+      </c>
+      <c r="E1425" t="s">
         <v>2766</v>
-      </c>
-      <c r="C1425" t="s">
-        <v>2767</v>
-      </c>
-      <c r="D1425" t="s">
-        <v>181</v>
-      </c>
-      <c r="E1425" t="s">
-        <v>2768</v>
       </c>
       <c r="F1425" t="s">
         <v>60</v>
@@ -79068,16 +79071,16 @@
         <v>2684</v>
       </c>
       <c r="B1426" t="s">
+        <v>2767</v>
+      </c>
+      <c r="C1426" t="s">
+        <v>2768</v>
+      </c>
+      <c r="D1426" t="s">
+        <v>181</v>
+      </c>
+      <c r="E1426" t="s">
         <v>2769</v>
-      </c>
-      <c r="C1426" t="s">
-        <v>2770</v>
-      </c>
-      <c r="D1426" t="s">
-        <v>181</v>
-      </c>
-      <c r="E1426" t="s">
-        <v>2771</v>
       </c>
       <c r="F1426" t="s">
         <v>750</v>
@@ -79109,16 +79112,16 @@
         <v>2684</v>
       </c>
       <c r="B1427" t="s">
+        <v>2770</v>
+      </c>
+      <c r="C1427" t="s">
+        <v>2771</v>
+      </c>
+      <c r="D1427" t="s">
+        <v>181</v>
+      </c>
+      <c r="E1427" t="s">
         <v>2772</v>
-      </c>
-      <c r="C1427" t="s">
-        <v>2773</v>
-      </c>
-      <c r="D1427" t="s">
-        <v>181</v>
-      </c>
-      <c r="E1427" t="s">
-        <v>2774</v>
       </c>
       <c r="F1427" t="s">
         <v>750</v>
@@ -79150,16 +79153,16 @@
         <v>2684</v>
       </c>
       <c r="B1428" t="s">
+        <v>2773</v>
+      </c>
+      <c r="C1428" t="s">
+        <v>2774</v>
+      </c>
+      <c r="D1428" t="s">
+        <v>181</v>
+      </c>
+      <c r="E1428" t="s">
         <v>2775</v>
-      </c>
-      <c r="C1428" t="s">
-        <v>2776</v>
-      </c>
-      <c r="D1428" t="s">
-        <v>181</v>
-      </c>
-      <c r="E1428" t="s">
-        <v>2777</v>
       </c>
       <c r="F1428" t="s">
         <v>60</v>
@@ -79188,16 +79191,16 @@
         <v>2684</v>
       </c>
       <c r="B1429" t="s">
+        <v>2776</v>
+      </c>
+      <c r="C1429" t="s">
+        <v>2777</v>
+      </c>
+      <c r="D1429" t="s">
+        <v>181</v>
+      </c>
+      <c r="E1429" t="s">
         <v>2778</v>
-      </c>
-      <c r="C1429" t="s">
-        <v>2779</v>
-      </c>
-      <c r="D1429" t="s">
-        <v>181</v>
-      </c>
-      <c r="E1429" t="s">
-        <v>2780</v>
       </c>
       <c r="F1429" t="s">
         <v>60</v>
@@ -79226,16 +79229,16 @@
         <v>2684</v>
       </c>
       <c r="B1430" t="s">
+        <v>2779</v>
+      </c>
+      <c r="C1430" t="s">
+        <v>2780</v>
+      </c>
+      <c r="D1430" t="s">
+        <v>181</v>
+      </c>
+      <c r="E1430" t="s">
         <v>2781</v>
-      </c>
-      <c r="C1430" t="s">
-        <v>2782</v>
-      </c>
-      <c r="D1430" t="s">
-        <v>181</v>
-      </c>
-      <c r="E1430" t="s">
-        <v>2783</v>
       </c>
       <c r="F1430" t="s">
         <v>60</v>
@@ -79264,16 +79267,16 @@
         <v>2684</v>
       </c>
       <c r="B1431" t="s">
+        <v>2782</v>
+      </c>
+      <c r="C1431" t="s">
+        <v>2783</v>
+      </c>
+      <c r="D1431" t="s">
+        <v>181</v>
+      </c>
+      <c r="E1431" t="s">
         <v>2784</v>
-      </c>
-      <c r="C1431" t="s">
-        <v>2785</v>
-      </c>
-      <c r="D1431" t="s">
-        <v>181</v>
-      </c>
-      <c r="E1431" t="s">
-        <v>2786</v>
       </c>
       <c r="F1431" t="s">
         <v>60</v>
@@ -79302,16 +79305,16 @@
         <v>2684</v>
       </c>
       <c r="B1432" t="s">
+        <v>2785</v>
+      </c>
+      <c r="C1432" t="s">
+        <v>2786</v>
+      </c>
+      <c r="D1432" t="s">
+        <v>181</v>
+      </c>
+      <c r="E1432" t="s">
         <v>2787</v>
-      </c>
-      <c r="C1432" t="s">
-        <v>2788</v>
-      </c>
-      <c r="D1432" t="s">
-        <v>181</v>
-      </c>
-      <c r="E1432" t="s">
-        <v>2789</v>
       </c>
       <c r="F1432" t="s">
         <v>60</v>
@@ -79340,16 +79343,16 @@
         <v>2684</v>
       </c>
       <c r="B1433" t="s">
+        <v>2788</v>
+      </c>
+      <c r="C1433" t="s">
+        <v>2789</v>
+      </c>
+      <c r="D1433" t="s">
+        <v>181</v>
+      </c>
+      <c r="E1433" t="s">
         <v>2790</v>
-      </c>
-      <c r="C1433" t="s">
-        <v>2791</v>
-      </c>
-      <c r="D1433" t="s">
-        <v>181</v>
-      </c>
-      <c r="E1433" t="s">
-        <v>2792</v>
       </c>
       <c r="F1433" t="s">
         <v>60</v>
@@ -79378,16 +79381,16 @@
         <v>2684</v>
       </c>
       <c r="B1434" t="s">
+        <v>2791</v>
+      </c>
+      <c r="C1434" t="s">
+        <v>2792</v>
+      </c>
+      <c r="D1434" t="s">
+        <v>181</v>
+      </c>
+      <c r="E1434" t="s">
         <v>2793</v>
-      </c>
-      <c r="C1434" t="s">
-        <v>2794</v>
-      </c>
-      <c r="D1434" t="s">
-        <v>181</v>
-      </c>
-      <c r="E1434" t="s">
-        <v>2795</v>
       </c>
       <c r="F1434" t="s">
         <v>60</v>
@@ -79416,16 +79419,16 @@
         <v>2684</v>
       </c>
       <c r="B1435" t="s">
+        <v>2794</v>
+      </c>
+      <c r="C1435" t="s">
+        <v>2795</v>
+      </c>
+      <c r="D1435" t="s">
+        <v>181</v>
+      </c>
+      <c r="E1435" t="s">
         <v>2796</v>
-      </c>
-      <c r="C1435" t="s">
-        <v>2797</v>
-      </c>
-      <c r="D1435" t="s">
-        <v>181</v>
-      </c>
-      <c r="E1435" t="s">
-        <v>2798</v>
       </c>
       <c r="F1435" t="s">
         <v>60</v>
@@ -79454,16 +79457,16 @@
         <v>2684</v>
       </c>
       <c r="B1436" t="s">
+        <v>2797</v>
+      </c>
+      <c r="C1436" t="s">
+        <v>2798</v>
+      </c>
+      <c r="D1436" t="s">
+        <v>181</v>
+      </c>
+      <c r="E1436" t="s">
         <v>2799</v>
-      </c>
-      <c r="C1436" t="s">
-        <v>2800</v>
-      </c>
-      <c r="D1436" t="s">
-        <v>181</v>
-      </c>
-      <c r="E1436" t="s">
-        <v>2801</v>
       </c>
       <c r="F1436" t="s">
         <v>60</v>
@@ -79492,16 +79495,16 @@
         <v>2684</v>
       </c>
       <c r="B1437" t="s">
+        <v>2800</v>
+      </c>
+      <c r="C1437" t="s">
+        <v>2801</v>
+      </c>
+      <c r="D1437" t="s">
+        <v>181</v>
+      </c>
+      <c r="E1437" t="s">
         <v>2802</v>
-      </c>
-      <c r="C1437" t="s">
-        <v>2803</v>
-      </c>
-      <c r="D1437" t="s">
-        <v>181</v>
-      </c>
-      <c r="E1437" t="s">
-        <v>2804</v>
       </c>
       <c r="F1437" t="s">
         <v>60</v>
@@ -79530,16 +79533,16 @@
         <v>2684</v>
       </c>
       <c r="B1438" t="s">
+        <v>2803</v>
+      </c>
+      <c r="C1438" t="s">
+        <v>2804</v>
+      </c>
+      <c r="D1438" t="s">
+        <v>181</v>
+      </c>
+      <c r="E1438" t="s">
         <v>2805</v>
-      </c>
-      <c r="C1438" t="s">
-        <v>2806</v>
-      </c>
-      <c r="D1438" t="s">
-        <v>181</v>
-      </c>
-      <c r="E1438" t="s">
-        <v>2807</v>
       </c>
       <c r="F1438" t="s">
         <v>60</v>
@@ -79568,16 +79571,16 @@
         <v>2684</v>
       </c>
       <c r="B1439" t="s">
+        <v>2806</v>
+      </c>
+      <c r="C1439" t="s">
+        <v>2807</v>
+      </c>
+      <c r="D1439" t="s">
+        <v>181</v>
+      </c>
+      <c r="E1439" t="s">
         <v>2808</v>
-      </c>
-      <c r="C1439" t="s">
-        <v>2809</v>
-      </c>
-      <c r="D1439" t="s">
-        <v>181</v>
-      </c>
-      <c r="E1439" t="s">
-        <v>2810</v>
       </c>
       <c r="F1439" t="s">
         <v>60</v>
@@ -79606,16 +79609,16 @@
         <v>2684</v>
       </c>
       <c r="B1440" t="s">
+        <v>2809</v>
+      </c>
+      <c r="C1440" t="s">
+        <v>2810</v>
+      </c>
+      <c r="D1440" t="s">
+        <v>181</v>
+      </c>
+      <c r="E1440" t="s">
         <v>2811</v>
-      </c>
-      <c r="C1440" t="s">
-        <v>2812</v>
-      </c>
-      <c r="D1440" t="s">
-        <v>181</v>
-      </c>
-      <c r="E1440" t="s">
-        <v>2813</v>
       </c>
       <c r="F1440" t="s">
         <v>60</v>
@@ -79644,16 +79647,16 @@
         <v>2684</v>
       </c>
       <c r="B1441" t="s">
+        <v>2812</v>
+      </c>
+      <c r="C1441" t="s">
+        <v>2813</v>
+      </c>
+      <c r="D1441" t="s">
+        <v>181</v>
+      </c>
+      <c r="E1441" t="s">
         <v>2814</v>
-      </c>
-      <c r="C1441" t="s">
-        <v>2815</v>
-      </c>
-      <c r="D1441" t="s">
-        <v>181</v>
-      </c>
-      <c r="E1441" t="s">
-        <v>2816</v>
       </c>
       <c r="F1441" t="s">
         <v>60</v>
@@ -79682,16 +79685,16 @@
         <v>2684</v>
       </c>
       <c r="B1442" t="s">
+        <v>2815</v>
+      </c>
+      <c r="C1442" t="s">
+        <v>2816</v>
+      </c>
+      <c r="D1442" t="s">
+        <v>181</v>
+      </c>
+      <c r="E1442" t="s">
         <v>2817</v>
-      </c>
-      <c r="C1442" t="s">
-        <v>2818</v>
-      </c>
-      <c r="D1442" t="s">
-        <v>181</v>
-      </c>
-      <c r="E1442" t="s">
-        <v>2819</v>
       </c>
       <c r="F1442" t="s">
         <v>60</v>
@@ -79720,16 +79723,16 @@
         <v>2684</v>
       </c>
       <c r="B1443" t="s">
+        <v>2818</v>
+      </c>
+      <c r="C1443" t="s">
+        <v>2819</v>
+      </c>
+      <c r="D1443" t="s">
+        <v>2684</v>
+      </c>
+      <c r="E1443" t="s">
         <v>2820</v>
-      </c>
-      <c r="C1443" t="s">
-        <v>2821</v>
-      </c>
-      <c r="D1443" t="s">
-        <v>2684</v>
-      </c>
-      <c r="E1443" t="s">
-        <v>2822</v>
       </c>
       <c r="F1443" t="s">
         <v>146</v>
@@ -79758,16 +79761,16 @@
         <v>2684</v>
       </c>
       <c r="B1444" t="s">
+        <v>2821</v>
+      </c>
+      <c r="C1444" t="s">
+        <v>2822</v>
+      </c>
+      <c r="D1444" t="s">
+        <v>2684</v>
+      </c>
+      <c r="E1444" t="s">
         <v>2823</v>
-      </c>
-      <c r="C1444" t="s">
-        <v>2824</v>
-      </c>
-      <c r="D1444" t="s">
-        <v>2684</v>
-      </c>
-      <c r="E1444" t="s">
-        <v>2825</v>
       </c>
       <c r="F1444" t="s">
         <v>60</v>
@@ -79796,16 +79799,16 @@
         <v>2684</v>
       </c>
       <c r="B1445" t="s">
+        <v>2824</v>
+      </c>
+      <c r="C1445" t="s">
+        <v>2825</v>
+      </c>
+      <c r="D1445" t="s">
+        <v>2684</v>
+      </c>
+      <c r="E1445" t="s">
         <v>2826</v>
-      </c>
-      <c r="C1445" t="s">
-        <v>2694</v>
-      </c>
-      <c r="D1445" t="s">
-        <v>2684</v>
-      </c>
-      <c r="E1445" t="s">
-        <v>2695</v>
       </c>
       <c r="F1445" t="s">
         <v>60</v>
@@ -79834,31 +79837,37 @@
         <v>2684</v>
       </c>
       <c r="B1446" t="s">
-        <v>56</v>
+        <v>2827</v>
       </c>
       <c r="C1446" t="s">
-        <v>56</v>
+        <v>2692</v>
       </c>
       <c r="D1446" t="s">
-        <v>56</v>
+        <v>2684</v>
       </c>
       <c r="E1446" t="s">
-        <v>56</v>
+        <v>2693</v>
       </c>
       <c r="F1446" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="G1446" t="s">
-        <v>56</v>
+        <v>61</v>
       </c>
       <c r="H1446" t="s">
-        <v>56</v>
+        <v>182</v>
       </c>
       <c r="I1446" t="s">
-        <v>56</v>
+        <v>183</v>
       </c>
       <c r="J1446" t="s">
-        <v>56</v>
+        <v>182</v>
+      </c>
+      <c r="K1446" t="s">
+        <v>39</v>
+      </c>
+      <c r="L1446" t="s">
+        <v>60</v>
       </c>
     </row>
     <row r="1447">
@@ -79866,30 +79875,62 @@
         <v>2684</v>
       </c>
       <c r="B1447" t="s">
+        <v>56</v>
+      </c>
+      <c r="C1447" t="s">
+        <v>56</v>
+      </c>
+      <c r="D1447" t="s">
+        <v>56</v>
+      </c>
+      <c r="E1447" t="s">
+        <v>56</v>
+      </c>
+      <c r="F1447" t="s">
+        <v>56</v>
+      </c>
+      <c r="G1447" t="s">
+        <v>56</v>
+      </c>
+      <c r="H1447" t="s">
+        <v>56</v>
+      </c>
+      <c r="I1447" t="s">
+        <v>56</v>
+      </c>
+      <c r="J1447" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="1448">
+      <c r="A1448" t="s">
+        <v>2684</v>
+      </c>
+      <c r="B1448" t="s">
         <v>160</v>
       </c>
-      <c r="C1447" t="s">
+      <c r="C1448" t="s">
+        <v>2828</v>
+      </c>
+      <c r="D1448" t="s">
+        <v>56</v>
+      </c>
+      <c r="E1448" t="s">
+        <v>162</v>
+      </c>
+      <c r="F1448" t="s">
         <v>2827</v>
       </c>
-      <c r="D1447" t="s">
-        <v>56</v>
-      </c>
-      <c r="E1447" t="s">
-        <v>162</v>
-      </c>
-      <c r="F1447" t="s">
-        <v>2826</v>
-      </c>
-      <c r="G1447" t="s">
-        <v>56</v>
-      </c>
-      <c r="H1447" t="s">
-        <v>56</v>
-      </c>
-      <c r="I1447" t="s">
-        <v>56</v>
-      </c>
-      <c r="J1447" t="s">
+      <c r="G1448" t="s">
+        <v>56</v>
+      </c>
+      <c r="H1448" t="s">
+        <v>56</v>
+      </c>
+      <c r="I1448" t="s">
+        <v>56</v>
+      </c>
+      <c r="J1448" t="s">
         <v>56</v>
       </c>
     </row>

</xml_diff>